<commit_message>
Se edita el catalogo de los productos
</commit_message>
<xml_diff>
--- a/datos/productos.xlsx
+++ b/datos/productos.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1704" uniqueCount="1087">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1794" uniqueCount="1145">
   <si>
     <t>Nombre</t>
   </si>
@@ -3286,6 +3286,180 @@
   </si>
   <si>
     <t>Conjunto de Collar con Colgante de Lágrima de Cristal y Aretes</t>
+  </si>
+  <si>
+    <t>Zapatos Casuales Versátiles De Moda Con Patrón De Cocodrilo</t>
+  </si>
+  <si>
+    <t>Color: Beige, Talla: 29.5</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-1585296499-zapatos-casuales-versatiles-de-moda-con-patron-de-cocodrilo-_JM?quantity=1&amp;variation_id=179412877537</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_730419-CBT103500748521_012026-F-zapatos-casuales-versatiles-de-moda-con-patron-de-cocodrilo.webp;https://http2.mlstatic.com/D_NQ_NP_2X_996108-CBT103497713925_012026-F-zapatos-casuales-versatiles-de-moda-con-patron-de-cocodrilo.webp;https://http2.mlstatic.com/D_NQ_NP_2X_683363-CBT102983612396_012026-F-zapatos-casuales-versatiles-de-moda-con-patron-de-cocodrilo.webp</t>
+  </si>
+  <si>
+    <t>Zapato Hombre Tenis Casal Plataforma Moda Transpirable Sport</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-1863972705-zapato-hombre-tenis-casal-plataforma-moda-transpirable-sport-_JM?quantity=1&amp;variation_id=177138143622</t>
+  </si>
+  <si>
+    <t>Color: Gris, Talla: 23.5</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_936628-CBT106943681987_022026-F-zapato-hombre-tenis-casal-plataforma-moda-transpirable-sport.webp;https://http2.mlstatic.com/D_NQ_NP_2X_688210-CBT104197322259_012026-F-zapato-hombre-tenis-casal-plataforma-moda-transpirable-sport.webp;https://http2.mlstatic.com/D_NQ_NP_2X_820243-CBT74914869169_032024-F-zapato-hombre-tenis-casal-plataforma-moda-transpirable-sport.webp</t>
+  </si>
+  <si>
+    <t>Color: Caqui, Talla: 26</t>
+  </si>
+  <si>
+    <t>Botas Tacticas Hombre Zapatos De Trabajo Casual Outdoor 588</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-1907810375-botas-tacticas-hombre-zapatos-de-trabajo-casual-outdoor-588-_JM?quantity=1&amp;variation_id=178019331588</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_722244-CBT105692274218_012026-F-botas-tacticas-hombre-zapatos-de-trabajo-casual-outdoor-588.webp;https://http2.mlstatic.com/D_NQ_NP_2X_817878-CBT81532198186_012025-F-botas-tacticas-hombre-zapatos-de-trabajo-casual-outdoor-588.webp;https://http2.mlstatic.com/D_NQ_NP_2X_963367-CBT105692452258_012026-F-botas-tacticas-hombre-zapatos-de-trabajo-casual-outdoor-588.webp</t>
+  </si>
+  <si>
+    <t>Negro Talla: 25</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-1391870088-botas-de-seguridad-industrial-trabajo-casquillo-aislamiento-_JM?quantity=1&amp;variation_id=174304565690</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_952510-CBT76527863055_052024-F-botas-de-seguridad-industrial-trabajo-casquillo-aislamiento.webp;https://http2.mlstatic.com/D_NQ_NP_2X_735652-CBT93046766673_092025-F-botas-de-seguridad-industrial-trabajo-casquillo-aislamiento.webp;https://http2.mlstatic.com/D_NQ_NP_2X_931407-CBT49361572113_032022-F-botas-de-seguridad-industrial-trabajo-casquillo-aislamiento.webp</t>
+  </si>
+  <si>
+    <t>Botas De Seguridad Industrial Trabajo Casquillo Aislamiento</t>
+  </si>
+  <si>
+    <t>Botas Casquillo Hombre, Botas De Seguridad Laboral Cómodas</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-1399770488-botas-casquillo-hombre-botas-de-seguridad-laboral-comodas-_JM?quantity=1&amp;variation_id=180999225836</t>
+  </si>
+  <si>
+    <t>Color: Verde oscuro Talla: 29.5</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_650135-CBT77371017482_072024-F-botas-casquillo-hombre-botas-de-seguridad-laboral-comodas.webp;https://http2.mlstatic.com/D_NQ_NP_2X_719875-CBT77371017326_072024-F-botas-casquillo-hombre-botas-de-seguridad-laboral-comodas.webp;https://http2.mlstatic.com/D_NQ_NP_2X_824985-CBT77586643241_072024-F-botas-casquillo-hombre-botas-de-seguridad-laboral-comodas.webp</t>
+  </si>
+  <si>
+    <t>Color: Negro Talla: 31</t>
+  </si>
+  <si>
+    <t>Botas Tácticas Militares Para Exteriores Para Hombre</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-1736189418-botas-tacticas-militares-para-exteriores-para-hombre-_JM?quantity=1&amp;variation_id=176248942451</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_708527-CBT54910132787_042023-F-botas-tacticas-militares-para-exteriores-para-hombre.webp;https://http2.mlstatic.com/D_NQ_NP_2X_977035-CBT54910134985_042023-F-botas-tacticas-militares-para-exteriores-para-hombre.webp;https://http2.mlstatic.com/D_NQ_NP_2X_978862-CBT54910125531_042023-F-botas-tacticas-militares-para-exteriores-para-hombre.webp</t>
+  </si>
+  <si>
+    <t>Color: Negro Talla: 26</t>
+  </si>
+  <si>
+    <t>Bota De Seguridad Industrial Casquillo Trabajo Moda Anbaili</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-2345998809-bota-de-seguridad-industrial-casquillo-trabajo-moda-anbaili-_JM?quantity=1&amp;variation_id=183949487610</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_810360-CBT99999995999_112025-F-bota-de-seguridad-industrial-casquillo-trabajo-moda-anbaili.webp;https://http2.mlstatic.com/D_NQ_NP_2X_960862-CBT99516025326_112025-F-bota-de-seguridad-industrial-casquillo-trabajo-moda-anbaili.webp</t>
+  </si>
+  <si>
+    <t>Tenis De Seguridad Industrial Zapatos Mujer Hombre Pugood</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-3325324470-tenis-de-seguridad-industrial-zapatos-mujer-hombre-pugood-_JM?quantity=1&amp;variation_id=181446523738</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_828567-CBT93494609292_102025-F-tenis-de-seguridad-industrial-zapatos-mujer-hombre-pugood.webp;https://http2.mlstatic.com/D_NQ_NP_2X_678720-CBT78985742993_092024-F-tenis-de-seguridad-industrial-zapatos-mujer-hombre-pugood.webp;https://http2.mlstatic.com/D_NQ_NP_2X_909663-CBT78985909479_092024-F-tenis-de-seguridad-industrial-zapatos-mujer-hombre-pugood.webp</t>
+  </si>
+  <si>
+    <t>Color: Negro Talla: 25</t>
+  </si>
+  <si>
+    <t>Tenis De Seguridad Industrial Zapatos Cómodo Transpirable</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-3480729512-tenis-de-seguridad-industrial-zapatos-comodo-transpirable-_JM?quantity=1&amp;variation_id=186205261537</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_703874-CBT80747477078_112024-F-tenis-de-seguridad-industrial-zapatos-comodo-transpirable.webp;https://http2.mlstatic.com/D_NQ_NP_2X_672386-CBT80747477076_112024-F-tenis-de-seguridad-industrial-zapatos-comodo-transpirable.webp;https://http2.mlstatic.com/D_NQ_NP_2X_820311-CBT80747477074_112024-F-tenis-de-seguridad-industrial-zapatos-comodo-transpirable.webp</t>
+  </si>
+  <si>
+    <t>Regalos De Cumpleaños Para Mujeres, Cesta De Regalo Relajant Rojo</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/regalos-de-cumpleanos-para-mujeres-cesta-de-regalo-relajant/up/MLMU3473451389?pdp_filters=item_id:MLM2490113661#&amp;gid=1&amp;pid=1</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_842536-MLM106725939723_022026-F.webp</t>
+  </si>
+  <si>
+    <t>Ventiladores De Techo</t>
+  </si>
+  <si>
+    <t>Descripción: Cantidad De Aspas 6 Estructura Blanco Aspas Blanco Diámetro 52 Cm Frecuencia 60hz Material De Las Aspas Plástico</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/cozylady-lampara-de-ventilador-led-48w-e26-205-ventiladores-de-techo-cantidad-de-aspas-6-estructura-blanco-aspas-blanco-diametro-52-cm-frecuencia-60hz-material-de-las-aspas-plastico/p/MLM54407252?pdp_filters=item_id:MLM2430884049</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_711430-MLA100058619227_122025-F.webp</t>
+  </si>
+  <si>
+    <t>Audífonos Bluetooth Mini Corazón Audífonos</t>
+  </si>
+  <si>
+    <t>Descripción: Bluetooth Audífonos Cancelación Ruido</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/trymiss-k520-audifonos-bluetooth-mini-corazon-audifonos-con-microfono-audifonos-para-el-gym-manos-libres-audifonos-gamer-bluetooth-audifonos-cancelacion-ruido-14-de-febrero-regalos-para-mujer/p/MLM45453811?pdp_filters=item_id:MLM3532166646</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_827140-MLA105524534674_012026-F.webp</t>
+  </si>
+  <si>
+    <t>Pulsera De Tenis Ajustable Con Cristal Para Hombre Mujer</t>
+  </si>
+  <si>
+    <t>Largo: 19 cm, Material principal: Aleación.</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/sumlin-pulsera-de-tenis-ajustable-con-cristal-para-hombre-mujer-pulsera-de-pareja-plata-19-cm-regalos-de-san-valentin-incluye-una-hermosa-caja-de-regalo/p/MLM65215922?pdp_filters=item_id:MLM2728909083</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_840204-MLA106485769181_022026-F.webp</t>
+  </si>
+  <si>
+    <t>Marca:  Cowin</t>
+  </si>
+  <si>
+    <t>Auriculares híbridos With Ruido Activa Cancelación</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/auriculares-hibridos-cowin-e11a-with-ruido-activa-cancelacion/p/MLM65118526?pdp_filters=item_id:MLM4731897778</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_951489-MLA106257537077_012026-F.webp</t>
+  </si>
+  <si>
+    <t>Color: TK902-DY, Diseño: Sólido, Tamaño del casco: L</t>
+  </si>
+  <si>
+    <t>Casco De Moto Con Visera Abatible Y Plegable Certificado Dot</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-3853286468-casco-de-moto-con-visera-abatible-y-plegable-certificado-dot-_JM?quantity=1&amp;variation_id=189147248851</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_719669-MLM98288984742_112025-F-casco-de-moto-con-visera-abatible-y-plegable-certificado-dot.webp</t>
   </si>
 </sst>
 </file>
@@ -3321,11 +3495,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3345,8 +3522,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H302" totalsRowShown="0">
-  <autoFilter ref="A1:H302"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H317" totalsRowShown="0">
+  <autoFilter ref="A1:H317"/>
   <sortState ref="A2:H230">
     <sortCondition ref="H1:H230"/>
   </sortState>
@@ -3649,7 +3826,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H302"/>
+  <dimension ref="A1:H317"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -11105,6 +11282,393 @@
         <v>905</v>
       </c>
     </row>
+    <row r="303" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A303" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B303" t="s">
+        <v>1088</v>
+      </c>
+      <c r="C303">
+        <v>691</v>
+      </c>
+      <c r="D303">
+        <v>350</v>
+      </c>
+      <c r="E303" t="s">
+        <v>1090</v>
+      </c>
+      <c r="F303" t="s">
+        <v>1089</v>
+      </c>
+      <c r="G303" t="s">
+        <v>600</v>
+      </c>
+      <c r="H303" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="304" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A304" s="3" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B304" t="s">
+        <v>1093</v>
+      </c>
+      <c r="C304">
+        <v>555</v>
+      </c>
+      <c r="D304">
+        <v>300</v>
+      </c>
+      <c r="E304" t="s">
+        <v>1094</v>
+      </c>
+      <c r="F304" t="s">
+        <v>1092</v>
+      </c>
+      <c r="G304" t="s">
+        <v>600</v>
+      </c>
+      <c r="H304" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="305" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A305" t="s">
+        <v>1096</v>
+      </c>
+      <c r="B305" t="s">
+        <v>1095</v>
+      </c>
+      <c r="C305">
+        <v>897</v>
+      </c>
+      <c r="D305">
+        <v>570</v>
+      </c>
+      <c r="E305" t="s">
+        <v>1098</v>
+      </c>
+      <c r="F305" t="s">
+        <v>1097</v>
+      </c>
+      <c r="G305" t="s">
+        <v>600</v>
+      </c>
+      <c r="H305" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="306" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A306" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B306" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C306">
+        <v>726</v>
+      </c>
+      <c r="D306">
+        <v>500</v>
+      </c>
+      <c r="E306" t="s">
+        <v>1101</v>
+      </c>
+      <c r="F306" t="s">
+        <v>1100</v>
+      </c>
+      <c r="G306" t="s">
+        <v>600</v>
+      </c>
+      <c r="H306" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="307" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A307" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B307" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C307">
+        <v>713</v>
+      </c>
+      <c r="D307">
+        <v>530</v>
+      </c>
+      <c r="E307" t="s">
+        <v>1106</v>
+      </c>
+      <c r="F307" t="s">
+        <v>1104</v>
+      </c>
+      <c r="G307" t="s">
+        <v>600</v>
+      </c>
+      <c r="H307" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="308" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A308" t="s">
+        <v>1108</v>
+      </c>
+      <c r="B308" t="s">
+        <v>1107</v>
+      </c>
+      <c r="C308">
+        <v>1095</v>
+      </c>
+      <c r="D308">
+        <v>800</v>
+      </c>
+      <c r="E308" t="s">
+        <v>1110</v>
+      </c>
+      <c r="F308" t="s">
+        <v>1109</v>
+      </c>
+      <c r="G308" t="s">
+        <v>600</v>
+      </c>
+      <c r="H308" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="309" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A309" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B309" t="s">
+        <v>1111</v>
+      </c>
+      <c r="C309">
+        <v>890</v>
+      </c>
+      <c r="D309">
+        <v>500</v>
+      </c>
+      <c r="E309" t="s">
+        <v>1114</v>
+      </c>
+      <c r="F309" t="s">
+        <v>1113</v>
+      </c>
+      <c r="G309" t="s">
+        <v>600</v>
+      </c>
+      <c r="H309" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="310" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A310" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B310" t="s">
+        <v>1111</v>
+      </c>
+      <c r="C310">
+        <v>635</v>
+      </c>
+      <c r="D310">
+        <v>400</v>
+      </c>
+      <c r="E310" t="s">
+        <v>1117</v>
+      </c>
+      <c r="F310" t="s">
+        <v>1116</v>
+      </c>
+      <c r="G310" t="s">
+        <v>600</v>
+      </c>
+      <c r="H310" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="311" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A311" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B311" t="s">
+        <v>1118</v>
+      </c>
+      <c r="C311">
+        <v>715</v>
+      </c>
+      <c r="D311">
+        <v>550</v>
+      </c>
+      <c r="E311" t="s">
+        <v>1121</v>
+      </c>
+      <c r="F311" t="s">
+        <v>1120</v>
+      </c>
+      <c r="G311" t="s">
+        <v>600</v>
+      </c>
+      <c r="H311" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="312" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A312" t="s">
+        <v>1122</v>
+      </c>
+      <c r="B312" t="s">
+        <v>18</v>
+      </c>
+      <c r="C312">
+        <v>280</v>
+      </c>
+      <c r="E312" t="s">
+        <v>1124</v>
+      </c>
+      <c r="F312" t="s">
+        <v>1123</v>
+      </c>
+      <c r="G312" t="s">
+        <v>600</v>
+      </c>
+      <c r="H312" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="313" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A313" t="s">
+        <v>1125</v>
+      </c>
+      <c r="B313" t="s">
+        <v>1126</v>
+      </c>
+      <c r="C313">
+        <v>450</v>
+      </c>
+      <c r="D313">
+        <v>350</v>
+      </c>
+      <c r="E313" t="s">
+        <v>1128</v>
+      </c>
+      <c r="F313" t="s">
+        <v>1127</v>
+      </c>
+      <c r="G313" t="s">
+        <v>600</v>
+      </c>
+      <c r="H313" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="314" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A314" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B314" t="s">
+        <v>1130</v>
+      </c>
+      <c r="C314">
+        <v>365</v>
+      </c>
+      <c r="D314">
+        <v>200</v>
+      </c>
+      <c r="E314" t="s">
+        <v>1132</v>
+      </c>
+      <c r="F314" t="s">
+        <v>1131</v>
+      </c>
+      <c r="G314" t="s">
+        <v>600</v>
+      </c>
+      <c r="H314" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="315" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A315" t="s">
+        <v>1133</v>
+      </c>
+      <c r="B315" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C315">
+        <v>250</v>
+      </c>
+      <c r="D315">
+        <v>200</v>
+      </c>
+      <c r="E315" t="s">
+        <v>1136</v>
+      </c>
+      <c r="F315" t="s">
+        <v>1135</v>
+      </c>
+      <c r="G315" t="s">
+        <v>600</v>
+      </c>
+      <c r="H315" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="316" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A316" t="s">
+        <v>1138</v>
+      </c>
+      <c r="B316" t="s">
+        <v>1137</v>
+      </c>
+      <c r="C316">
+        <v>515</v>
+      </c>
+      <c r="D316">
+        <v>400</v>
+      </c>
+      <c r="E316" t="s">
+        <v>1140</v>
+      </c>
+      <c r="F316" t="s">
+        <v>1139</v>
+      </c>
+      <c r="G316" t="s">
+        <v>600</v>
+      </c>
+      <c r="H316" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="317" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A317" t="s">
+        <v>1142</v>
+      </c>
+      <c r="B317" t="s">
+        <v>1141</v>
+      </c>
+      <c r="C317">
+        <v>820</v>
+      </c>
+      <c r="D317">
+        <v>680</v>
+      </c>
+      <c r="E317" t="s">
+        <v>1144</v>
+      </c>
+      <c r="F317" t="s">
+        <v>1143</v>
+      </c>
+      <c r="G317" t="s">
+        <v>600</v>
+      </c>
+      <c r="H317" t="s">
+        <v>722</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Actualizar base de datos productos.xlsx y regenerar catálogo
</commit_message>
<xml_diff>
--- a/datos/productos.xlsx
+++ b/datos/productos.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2200" uniqueCount="1213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2193" uniqueCount="1211">
   <si>
     <t>Nombre</t>
   </si>
@@ -3146,12 +3146,6 @@
   </si>
   <si>
     <t>No recargable, Tamaño del producto: 34.5x12x12cm</t>
-  </si>
-  <si>
-    <t>Lámpara De Ventilador Led 48W E26 20.5 Con Mando A Distancia</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Tamaño del producto: 52x20.5x20.5</t>
   </si>
   <si>
     <t>OK</t>
@@ -3765,8 +3759,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H334" totalsRowShown="0">
-  <autoFilter ref="A1:H334"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H333" totalsRowShown="0">
+  <autoFilter ref="A1:H333"/>
   <sortState ref="A2:H340">
     <sortCondition ref="G1:G340"/>
   </sortState>
@@ -4069,7 +4063,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I334"/>
+  <dimension ref="A1:I333"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -4127,13 +4121,13 @@
         <v>392</v>
       </c>
       <c r="G2" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
       <c r="H2" t="s">
         <v>12</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -4156,13 +4150,13 @@
         <v>398</v>
       </c>
       <c r="G3" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
       <c r="H3" t="s">
         <v>12</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -4182,21 +4176,21 @@
         <v>411</v>
       </c>
       <c r="G4" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
       <c r="H4" t="s">
         <v>12</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
       <c r="C5">
         <v>589</v>
@@ -4205,24 +4199,24 @@
         <v>500</v>
       </c>
       <c r="E5" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="F5" t="s">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="G5" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H5" t="s">
         <v>602</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>173</v>
@@ -4234,24 +4228,24 @@
         <v>350</v>
       </c>
       <c r="E6" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
       <c r="F6" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="G6" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H6" t="s">
         <v>602</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>18</v>
@@ -4260,19 +4254,19 @@
         <v>250</v>
       </c>
       <c r="E7" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
       <c r="F7" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
       <c r="G7" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H7" t="s">
         <v>602</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -4280,7 +4274,7 @@
         <v>80</v>
       </c>
       <c r="B8" t="s">
-        <v>1069</v>
+        <v>1067</v>
       </c>
       <c r="C8">
         <v>250</v>
@@ -4292,13 +4286,13 @@
         <v>82</v>
       </c>
       <c r="G8" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H8" t="s">
         <v>602</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -4306,7 +4300,7 @@
         <v>83</v>
       </c>
       <c r="B9" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
       <c r="C9">
         <v>150</v>
@@ -4315,13 +4309,13 @@
         <v>84</v>
       </c>
       <c r="G9" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H9" t="s">
         <v>602</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -4329,7 +4323,7 @@
         <v>85</v>
       </c>
       <c r="B10" t="s">
-        <v>1068</v>
+        <v>1066</v>
       </c>
       <c r="C10">
         <v>250</v>
@@ -4341,13 +4335,13 @@
         <v>87</v>
       </c>
       <c r="G10" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H10" t="s">
         <v>602</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4367,13 +4361,13 @@
         <v>570</v>
       </c>
       <c r="G11" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H11" t="s">
         <v>602</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4396,13 +4390,13 @@
         <v>90</v>
       </c>
       <c r="G12" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H12" t="s">
         <v>602</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4422,13 +4416,13 @@
         <v>93</v>
       </c>
       <c r="G13" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H13" t="s">
         <v>602</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -4436,7 +4430,7 @@
         <v>94</v>
       </c>
       <c r="B14" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="C14">
         <v>250</v>
@@ -4448,7 +4442,7 @@
         <v>96</v>
       </c>
       <c r="G14" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H14" t="s">
         <v>602</v>
@@ -4459,7 +4453,7 @@
         <v>97</v>
       </c>
       <c r="B15" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
       <c r="C15">
         <v>150</v>
@@ -4471,13 +4465,13 @@
         <v>99</v>
       </c>
       <c r="G15" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H15" t="s">
         <v>602</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4485,7 +4479,7 @@
         <v>100</v>
       </c>
       <c r="B16" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="C16">
         <v>250</v>
@@ -4497,13 +4491,13 @@
         <v>102</v>
       </c>
       <c r="G16" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H16" t="s">
         <v>602</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4523,7 +4517,7 @@
         <v>105</v>
       </c>
       <c r="G17" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H17" t="s">
         <v>602</v>
@@ -4546,7 +4540,7 @@
         <v>108</v>
       </c>
       <c r="G18" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H18" t="s">
         <v>602</v>
@@ -4569,7 +4563,7 @@
         <v>560</v>
       </c>
       <c r="G19" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="H19" t="s">
         <v>602</v>
@@ -4577,10 +4571,10 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="B20" t="s">
-        <v>1110</v>
+        <v>1108</v>
       </c>
       <c r="C20">
         <v>376.51</v>
@@ -4595,21 +4589,21 @@
         <v>26</v>
       </c>
       <c r="G20" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H20" t="s">
         <v>603</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>1112</v>
+        <v>1110</v>
       </c>
       <c r="B21" t="s">
-        <v>1113</v>
+        <v>1111</v>
       </c>
       <c r="C21">
         <v>1599</v>
@@ -4618,13 +4612,13 @@
         <v>1150</v>
       </c>
       <c r="E21" t="s">
-        <v>1115</v>
+        <v>1113</v>
       </c>
       <c r="F21" t="s">
-        <v>1114</v>
+        <v>1112</v>
       </c>
       <c r="G21" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H21" t="s">
         <v>603</v>
@@ -4651,7 +4645,7 @@
         <v>969</v>
       </c>
       <c r="G22" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H22" t="s">
         <v>603</v>
@@ -4675,13 +4669,13 @@
         <v>29</v>
       </c>
       <c r="G23" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H23" t="s">
         <v>603</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4701,13 +4695,13 @@
         <v>32</v>
       </c>
       <c r="G24" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H24" t="s">
         <v>603</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4730,13 +4724,13 @@
         <v>35</v>
       </c>
       <c r="G25" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H25" t="s">
         <v>603</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4759,13 +4753,13 @@
         <v>39</v>
       </c>
       <c r="G26" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H26" t="s">
         <v>603</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4788,13 +4782,13 @@
         <v>42</v>
       </c>
       <c r="G27" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H27" t="s">
         <v>603</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4814,13 +4808,13 @@
         <v>46</v>
       </c>
       <c r="G28" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H28" t="s">
         <v>603</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4840,13 +4834,13 @@
         <v>49</v>
       </c>
       <c r="G29" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H29" t="s">
         <v>603</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4869,13 +4863,13 @@
         <v>53</v>
       </c>
       <c r="G30" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H30" t="s">
         <v>603</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -4898,13 +4892,13 @@
         <v>56</v>
       </c>
       <c r="G31" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H31" t="s">
         <v>603</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4927,13 +4921,13 @@
         <v>59</v>
       </c>
       <c r="G32" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H32" t="s">
         <v>603</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -4956,13 +4950,13 @@
         <v>62</v>
       </c>
       <c r="G33" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H33" t="s">
         <v>603</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4985,13 +4979,13 @@
         <v>65</v>
       </c>
       <c r="G34" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H34" t="s">
         <v>603</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -5011,13 +5005,13 @@
         <v>386</v>
       </c>
       <c r="G35" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="H35" t="s">
         <v>603</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -5040,13 +5034,13 @@
         <v>239</v>
       </c>
       <c r="G36" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H36" t="s">
         <v>233</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -5069,13 +5063,13 @@
         <v>242</v>
       </c>
       <c r="G37" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H37" t="s">
         <v>233</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -5098,13 +5092,13 @@
         <v>785</v>
       </c>
       <c r="G38" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H38" t="s">
         <v>233</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -5127,7 +5121,7 @@
         <v>860</v>
       </c>
       <c r="G39" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H39" t="s">
         <v>233</v>
@@ -5154,13 +5148,13 @@
         <v>727</v>
       </c>
       <c r="G40" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H40" t="s">
         <v>233</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -5180,13 +5174,13 @@
         <v>851</v>
       </c>
       <c r="G41" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H41" t="s">
         <v>233</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -5206,13 +5200,13 @@
         <v>688</v>
       </c>
       <c r="G42" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H42" t="s">
         <v>233</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -5235,7 +5229,7 @@
         <v>771</v>
       </c>
       <c r="G43" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H43" t="s">
         <v>233</v>
@@ -5259,7 +5253,7 @@
         <v>379</v>
       </c>
       <c r="G44" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H44" t="s">
         <v>233</v>
@@ -5286,13 +5280,13 @@
         <v>743</v>
       </c>
       <c r="G45" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H45" t="s">
         <v>233</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5315,13 +5309,13 @@
         <v>773</v>
       </c>
       <c r="G46" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H46" t="s">
         <v>233</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5341,13 +5335,13 @@
         <v>836</v>
       </c>
       <c r="G47" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H47" t="s">
         <v>233</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5370,13 +5364,13 @@
         <v>701</v>
       </c>
       <c r="G48" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H48" t="s">
         <v>233</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,13 +5390,13 @@
         <v>562</v>
       </c>
       <c r="G49" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H49" t="s">
         <v>233</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,13 +5419,13 @@
         <v>723</v>
       </c>
       <c r="G50" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H50" t="s">
         <v>233</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5451,13 +5445,13 @@
         <v>737</v>
       </c>
       <c r="G51" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H51" t="s">
         <v>233</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5480,13 +5474,13 @@
         <v>232</v>
       </c>
       <c r="G52" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H52" t="s">
         <v>233</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5509,13 +5503,13 @@
         <v>236</v>
       </c>
       <c r="G53" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H53" t="s">
         <v>233</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5538,13 +5532,13 @@
         <v>796</v>
       </c>
       <c r="G54" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H54" t="s">
         <v>233</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5567,13 +5561,13 @@
         <v>840</v>
       </c>
       <c r="G55" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H55" t="s">
         <v>233</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5596,13 +5590,13 @@
         <v>777</v>
       </c>
       <c r="G56" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H56" t="s">
         <v>233</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5622,13 +5616,13 @@
         <v>809</v>
       </c>
       <c r="G57" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H57" t="s">
         <v>233</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5651,13 +5645,13 @@
         <v>707</v>
       </c>
       <c r="G58" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H58" t="s">
         <v>233</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5680,13 +5674,13 @@
         <v>733</v>
       </c>
       <c r="G59" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H59" t="s">
         <v>233</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5706,13 +5700,13 @@
         <v>689</v>
       </c>
       <c r="G60" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H60" t="s">
         <v>233</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5735,13 +5729,13 @@
         <v>820</v>
       </c>
       <c r="G61" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H61" t="s">
         <v>233</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5761,13 +5755,13 @@
         <v>814</v>
       </c>
       <c r="G62" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H62" t="s">
         <v>233</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5787,13 +5781,13 @@
         <v>805</v>
       </c>
       <c r="G63" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H63" t="s">
         <v>233</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5813,13 +5807,13 @@
         <v>855</v>
       </c>
       <c r="G64" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H64" t="s">
         <v>233</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5842,13 +5836,13 @@
         <v>729</v>
       </c>
       <c r="G65" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H65" t="s">
         <v>233</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5868,13 +5862,13 @@
         <v>821</v>
       </c>
       <c r="G66" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H66" t="s">
         <v>233</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5897,7 +5891,7 @@
         <v>847</v>
       </c>
       <c r="G67" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H67" t="s">
         <v>233</v>
@@ -5921,7 +5915,7 @@
         <v>833</v>
       </c>
       <c r="G68" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H68" t="s">
         <v>233</v>
@@ -5948,7 +5942,7 @@
         <v>708</v>
       </c>
       <c r="G69" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H69" t="s">
         <v>233</v>
@@ -5975,7 +5969,7 @@
         <v>229</v>
       </c>
       <c r="G70" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H70" t="s">
         <v>233</v>
@@ -6002,7 +5996,7 @@
         <v>712</v>
       </c>
       <c r="G71" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H71" t="s">
         <v>233</v>
@@ -6026,7 +6020,7 @@
         <v>683</v>
       </c>
       <c r="G72" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H72" t="s">
         <v>233</v>
@@ -6050,13 +6044,13 @@
         <v>697</v>
       </c>
       <c r="G73" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H73" t="s">
         <v>233</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -6079,7 +6073,7 @@
         <v>750</v>
       </c>
       <c r="G74" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H74" t="s">
         <v>233</v>
@@ -6106,7 +6100,7 @@
         <v>755</v>
       </c>
       <c r="G75" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H75" t="s">
         <v>233</v>
@@ -6133,7 +6127,7 @@
         <v>757</v>
       </c>
       <c r="G76" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H76" t="s">
         <v>233</v>
@@ -6160,13 +6154,13 @@
         <v>760</v>
       </c>
       <c r="G77" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H77" t="s">
         <v>233</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -6186,13 +6180,13 @@
         <v>800</v>
       </c>
       <c r="G78" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H78" t="s">
         <v>233</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -6212,13 +6206,13 @@
         <v>803</v>
       </c>
       <c r="G79" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H79" t="s">
         <v>233</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6241,7 +6235,7 @@
         <v>747</v>
       </c>
       <c r="G80" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H80" t="s">
         <v>233</v>
@@ -6268,13 +6262,13 @@
         <v>825</v>
       </c>
       <c r="G81" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H81" t="s">
         <v>233</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6294,13 +6288,13 @@
         <v>865</v>
       </c>
       <c r="G82" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H82" t="s">
         <v>233</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6320,7 +6314,7 @@
         <v>719</v>
       </c>
       <c r="G83" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H83" t="s">
         <v>233</v>
@@ -6347,7 +6341,7 @@
         <v>717</v>
       </c>
       <c r="G84" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="H84" t="s">
         <v>233</v>
@@ -6401,7 +6395,7 @@
         <v>263</v>
       </c>
       <c r="G86" t="s">
-        <v>1211</v>
+        <v>1209</v>
       </c>
       <c r="H86" t="s">
         <v>603</v>
@@ -6428,7 +6422,7 @@
         <v>225</v>
       </c>
       <c r="G87" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="H87" t="s">
         <v>605</v>
@@ -6437,7 +6431,7 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
       <c r="B88" t="s">
         <v>18</v>
@@ -6446,13 +6440,13 @@
         <v>250</v>
       </c>
       <c r="E88" t="s">
-        <v>1094</v>
+        <v>1092</v>
       </c>
       <c r="F88" t="s">
-        <v>1093</v>
+        <v>1091</v>
       </c>
       <c r="G88" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="H88" t="s">
         <v>605</v>
@@ -6461,7 +6455,7 @@
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
       <c r="B89" t="s">
         <v>18</v>
@@ -6470,13 +6464,13 @@
         <v>250</v>
       </c>
       <c r="E89" t="s">
-        <v>1089</v>
+        <v>1087</v>
       </c>
       <c r="F89" t="s">
-        <v>1090</v>
+        <v>1088</v>
       </c>
       <c r="G89" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="H89" t="s">
         <v>605</v>
@@ -6485,7 +6479,7 @@
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
       <c r="B90" t="s">
         <v>18</v>
@@ -6494,13 +6488,13 @@
         <v>250</v>
       </c>
       <c r="E90" t="s">
-        <v>1091</v>
+        <v>1089</v>
       </c>
       <c r="F90" t="s">
-        <v>1090</v>
+        <v>1088</v>
       </c>
       <c r="G90" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="H90" t="s">
         <v>605</v>
@@ -6509,7 +6503,7 @@
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
       <c r="B91" t="s">
         <v>18</v>
@@ -6521,13 +6515,13 @@
         <v>200</v>
       </c>
       <c r="E91" t="s">
-        <v>1098</v>
+        <v>1096</v>
       </c>
       <c r="F91" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
       <c r="G91" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="H91" t="s">
         <v>605</v>
@@ -6536,7 +6530,7 @@
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
       <c r="B92" t="s">
         <v>18</v>
@@ -6545,13 +6539,13 @@
         <v>250</v>
       </c>
       <c r="E92" t="s">
-        <v>1086</v>
+        <v>1084</v>
       </c>
       <c r="F92" t="s">
-        <v>1085</v>
+        <v>1083</v>
       </c>
       <c r="G92" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="H92" t="s">
         <v>605</v>
@@ -6578,7 +6572,7 @@
         <v>372</v>
       </c>
       <c r="G93" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="H93" t="s">
         <v>605</v>
@@ -6605,7 +6599,7 @@
         <v>227</v>
       </c>
       <c r="G94" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="H94" t="s">
         <v>605</v>
@@ -6629,7 +6623,7 @@
         <v>582</v>
       </c>
       <c r="G95" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="H95" t="s">
         <v>602</v>
@@ -6638,7 +6632,7 @@
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>1103</v>
+        <v>1101</v>
       </c>
       <c r="B96" t="s">
         <v>18</v>
@@ -6650,24 +6644,24 @@
         <v>120</v>
       </c>
       <c r="E96" t="s">
-        <v>1102</v>
+        <v>1100</v>
       </c>
       <c r="F96" t="s">
-        <v>1101</v>
+        <v>1099</v>
       </c>
       <c r="G96" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="H96" t="s">
         <v>605</v>
       </c>
       <c r="I96" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B97" t="s">
         <v>18</v>
@@ -6679,13 +6673,13 @@
         <v>120</v>
       </c>
       <c r="E97" t="s">
-        <v>1106</v>
+        <v>1104</v>
       </c>
       <c r="F97" t="s">
-        <v>1104</v>
+        <v>1102</v>
       </c>
       <c r="G97" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="H97" t="s">
         <v>605</v>
@@ -6694,7 +6688,7 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
       <c r="B98" t="s">
         <v>18</v>
@@ -6706,13 +6700,13 @@
         <v>200</v>
       </c>
       <c r="E98" t="s">
-        <v>1096</v>
+        <v>1094</v>
       </c>
       <c r="F98" t="s">
-        <v>1095</v>
+        <v>1093</v>
       </c>
       <c r="G98" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="H98" t="s">
         <v>602</v>
@@ -6739,7 +6733,7 @@
         <v>20</v>
       </c>
       <c r="G99" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="H99" t="s">
         <v>602</v>
@@ -7168,7 +7162,7 @@
         <v>602</v>
       </c>
       <c r="I115" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7197,7 +7191,7 @@
         <v>602</v>
       </c>
       <c r="I116" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7307,7 +7301,7 @@
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>1209</v>
+        <v>1207</v>
       </c>
       <c r="B121" t="s">
         <v>66</v>
@@ -7325,7 +7319,7 @@
         <v>68</v>
       </c>
       <c r="G121" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
       <c r="H121" t="s">
         <v>603</v>
@@ -7348,13 +7342,13 @@
         <v>73</v>
       </c>
       <c r="G122" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
       <c r="H122" t="s">
         <v>603</v>
       </c>
       <c r="I122" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7377,13 +7371,13 @@
         <v>351</v>
       </c>
       <c r="G123" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
       <c r="H123" t="s">
         <v>603</v>
       </c>
       <c r="I123" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7406,13 +7400,13 @@
         <v>76</v>
       </c>
       <c r="G124" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
       <c r="H124" t="s">
         <v>603</v>
       </c>
       <c r="I124" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7435,13 +7429,13 @@
         <v>79</v>
       </c>
       <c r="G125" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
       <c r="H125" t="s">
         <v>603</v>
       </c>
       <c r="I125" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7470,24 +7464,24 @@
         <v>602</v>
       </c>
       <c r="I126" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
       <c r="B127" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="C127">
         <v>150</v>
       </c>
       <c r="E127" t="s">
-        <v>1063</v>
+        <v>1061</v>
       </c>
       <c r="F127" t="s">
-        <v>1064</v>
+        <v>1062</v>
       </c>
       <c r="G127" t="s">
         <v>482</v>
@@ -7498,10 +7492,10 @@
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="B128" t="s">
-        <v>1062</v>
+        <v>1060</v>
       </c>
       <c r="C128">
         <v>150</v>
@@ -7510,10 +7504,10 @@
         <v>100</v>
       </c>
       <c r="E128" t="s">
-        <v>1061</v>
+        <v>1059</v>
       </c>
       <c r="F128" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
       <c r="G128" t="s">
         <v>482</v>
@@ -7524,10 +7518,10 @@
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="B129" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
       <c r="C129">
         <v>150</v>
@@ -7536,10 +7530,10 @@
         <v>100</v>
       </c>
       <c r="E129" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="F129" t="s">
-        <v>1055</v>
+        <v>1053</v>
       </c>
       <c r="G129" t="s">
         <v>482</v>
@@ -7550,10 +7544,10 @@
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="B130" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
       <c r="C130">
         <v>120</v>
@@ -7562,10 +7556,10 @@
         <v>100</v>
       </c>
       <c r="E130" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
       <c r="F130" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
       <c r="G130" t="s">
         <v>482</v>
@@ -7663,7 +7657,7 @@
         <v>370</v>
       </c>
       <c r="E134" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
       <c r="F134" t="s">
         <v>316</v>
@@ -7700,7 +7694,7 @@
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>1047</v>
+        <v>1045</v>
       </c>
       <c r="B136" t="s">
         <v>1010</v>
@@ -7712,10 +7706,10 @@
         <v>220</v>
       </c>
       <c r="E136" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
       <c r="F136" t="s">
-        <v>1048</v>
+        <v>1046</v>
       </c>
       <c r="G136" t="s">
         <v>482</v>
@@ -7729,7 +7723,7 @@
         <v>479</v>
       </c>
       <c r="B137" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
       <c r="C137">
         <v>200</v>
@@ -7764,7 +7758,7 @@
         <v>250</v>
       </c>
       <c r="E138" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
       <c r="F138" t="s">
         <v>401</v>
@@ -7790,7 +7784,7 @@
         <v>250</v>
       </c>
       <c r="E139" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
       <c r="F139" t="s">
         <v>404</v>
@@ -7924,7 +7918,7 @@
         <v>207</v>
       </c>
       <c r="G144" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="H144" t="s">
         <v>603</v>
@@ -7950,7 +7944,7 @@
         <v>521</v>
       </c>
       <c r="G145" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="H145" t="s">
         <v>605</v>
@@ -7973,13 +7967,13 @@
         <v>209</v>
       </c>
       <c r="G146" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="H146" t="s">
         <v>605</v>
       </c>
       <c r="I146" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -8002,13 +7996,13 @@
         <v>212</v>
       </c>
       <c r="G147" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="H147" t="s">
         <v>605</v>
       </c>
       <c r="I147" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -8031,13 +8025,13 @@
         <v>215</v>
       </c>
       <c r="G148" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="H148" t="s">
         <v>605</v>
       </c>
       <c r="I148" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8060,13 +8054,13 @@
         <v>218</v>
       </c>
       <c r="G149" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="H149" t="s">
         <v>605</v>
       </c>
       <c r="I149" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8089,13 +8083,13 @@
         <v>222</v>
       </c>
       <c r="G150" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="H150" t="s">
         <v>605</v>
       </c>
       <c r="I150" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8115,13 +8109,13 @@
         <v>389</v>
       </c>
       <c r="G151" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H151" t="s">
         <v>69</v>
       </c>
       <c r="I151" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8144,13 +8138,13 @@
         <v>182</v>
       </c>
       <c r="G152" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H152" t="s">
         <v>602</v>
       </c>
       <c r="I152" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8173,13 +8167,13 @@
         <v>185</v>
       </c>
       <c r="G153" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H153" t="s">
         <v>602</v>
       </c>
       <c r="I153" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8202,13 +8196,13 @@
         <v>188</v>
       </c>
       <c r="G154" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H154" t="s">
         <v>602</v>
       </c>
       <c r="I154" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8228,13 +8222,13 @@
         <v>407</v>
       </c>
       <c r="G155" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H155" t="s">
         <v>109</v>
       </c>
       <c r="I155" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8254,7 +8248,7 @@
         <v>672</v>
       </c>
       <c r="G156" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H156" t="s">
         <v>602</v>
@@ -8280,13 +8274,13 @@
         <v>783</v>
       </c>
       <c r="G157" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H157" t="s">
         <v>69</v>
       </c>
       <c r="I157" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
@@ -8306,13 +8300,13 @@
         <v>524</v>
       </c>
       <c r="G158" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H158" t="s">
         <v>69</v>
       </c>
       <c r="I158" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8332,13 +8326,13 @@
         <v>679</v>
       </c>
       <c r="G159" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H159" t="s">
         <v>69</v>
       </c>
       <c r="I159" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8358,13 +8352,13 @@
         <v>517</v>
       </c>
       <c r="G160" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H160" t="s">
         <v>233</v>
       </c>
       <c r="I160" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8384,13 +8378,13 @@
         <v>574</v>
       </c>
       <c r="G161" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H161" t="s">
         <v>602</v>
       </c>
       <c r="I161" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8410,7 +8404,7 @@
         <v>794</v>
       </c>
       <c r="G162" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H162" t="s">
         <v>602</v>
@@ -8433,7 +8427,7 @@
         <v>594</v>
       </c>
       <c r="G163" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H163" t="s">
         <v>69</v>
@@ -8456,7 +8450,7 @@
         <v>530</v>
       </c>
       <c r="G164" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H164" t="s">
         <v>233</v>
@@ -8480,13 +8474,13 @@
         <v>543</v>
       </c>
       <c r="G165" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H165" t="s">
         <v>233</v>
       </c>
       <c r="I165" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8506,13 +8500,13 @@
         <v>540</v>
       </c>
       <c r="G166" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H166" t="s">
         <v>233</v>
       </c>
       <c r="I166" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8532,13 +8526,13 @@
         <v>601</v>
       </c>
       <c r="G167" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H167" t="s">
         <v>602</v>
       </c>
       <c r="I167" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8558,13 +8552,13 @@
         <v>566</v>
       </c>
       <c r="G168" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H168" t="s">
         <v>602</v>
       </c>
       <c r="I168" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8587,13 +8581,13 @@
         <v>590</v>
       </c>
       <c r="G169" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H169" t="s">
         <v>602</v>
       </c>
       <c r="I169" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8616,13 +8610,13 @@
         <v>965</v>
       </c>
       <c r="G170" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H170" t="s">
         <v>767</v>
       </c>
       <c r="I170" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8642,7 +8636,7 @@
         <v>954</v>
       </c>
       <c r="G171" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H171" t="s">
         <v>233</v>
@@ -8669,7 +8663,7 @@
         <v>500</v>
       </c>
       <c r="G172" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H172" t="s">
         <v>233</v>
@@ -8696,7 +8690,7 @@
         <v>869</v>
       </c>
       <c r="G173" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H173" t="s">
         <v>602</v>
@@ -8723,13 +8717,13 @@
         <v>958</v>
       </c>
       <c r="G174" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H174" t="s">
         <v>69</v>
       </c>
       <c r="I174" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8752,13 +8746,13 @@
         <v>348</v>
       </c>
       <c r="G175" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H175" t="s">
         <v>603</v>
       </c>
       <c r="I175" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8781,13 +8775,13 @@
         <v>556</v>
       </c>
       <c r="G176" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="H176" t="s">
         <v>603</v>
       </c>
       <c r="I176" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8840,7 +8834,7 @@
         <v>69</v>
       </c>
       <c r="I178" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8896,7 +8890,7 @@
         <v>69</v>
       </c>
       <c r="I180" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8952,7 +8946,7 @@
         <v>69</v>
       </c>
       <c r="I182" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8981,7 +8975,7 @@
         <v>69</v>
       </c>
       <c r="I183" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9010,7 +9004,7 @@
         <v>468</v>
       </c>
       <c r="I184" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9066,7 +9060,7 @@
         <v>603</v>
       </c>
       <c r="I186" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9092,7 +9086,7 @@
         <v>602</v>
       </c>
       <c r="I187" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="188" spans="1:9" x14ac:dyDescent="0.25">
@@ -9148,7 +9142,7 @@
         <v>602</v>
       </c>
       <c r="I189" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9204,7 +9198,7 @@
         <v>233</v>
       </c>
       <c r="I191" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.25">
@@ -9224,13 +9218,13 @@
         <v>376</v>
       </c>
       <c r="G192" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H192" t="s">
         <v>12</v>
       </c>
       <c r="I192" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,13 +9247,13 @@
         <v>11</v>
       </c>
       <c r="G193" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H193" t="s">
         <v>12</v>
       </c>
       <c r="I193" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,13 +9276,13 @@
         <v>24</v>
       </c>
       <c r="G194" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H194" t="s">
         <v>12</v>
       </c>
       <c r="I194" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
@@ -9311,13 +9305,13 @@
         <v>16</v>
       </c>
       <c r="G195" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H195" t="s">
         <v>12</v>
       </c>
       <c r="I195" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9325,7 +9319,7 @@
         <v>380</v>
       </c>
       <c r="B196" t="s">
-        <v>1187</v>
+        <v>1185</v>
       </c>
       <c r="C196">
         <v>250</v>
@@ -9340,13 +9334,13 @@
         <v>383</v>
       </c>
       <c r="G196" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H196" t="s">
         <v>12</v>
       </c>
       <c r="I196" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9366,18 +9360,18 @@
         <v>395</v>
       </c>
       <c r="G197" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H197" t="s">
         <v>12</v>
       </c>
       <c r="I197" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>1184</v>
+        <v>1182</v>
       </c>
       <c r="B198" t="s">
         <v>791</v>
@@ -9389,19 +9383,19 @@
         <v>200</v>
       </c>
       <c r="E198" t="s">
-        <v>1186</v>
+        <v>1184</v>
       </c>
       <c r="F198" t="s">
-        <v>1185</v>
+        <v>1183</v>
       </c>
       <c r="G198" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H198" t="s">
         <v>12</v>
       </c>
       <c r="I198" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9424,13 +9418,13 @@
         <v>792</v>
       </c>
       <c r="G199" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H199" t="s">
         <v>12</v>
       </c>
       <c r="I199" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9453,13 +9447,13 @@
         <v>586</v>
       </c>
       <c r="G200" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H200" t="s">
         <v>12</v>
       </c>
       <c r="I200" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9479,13 +9473,13 @@
         <v>413</v>
       </c>
       <c r="G201" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H201" t="s">
         <v>12</v>
       </c>
       <c r="I201" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.25">
@@ -9493,7 +9487,7 @@
         <v>414</v>
       </c>
       <c r="B202" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="C202">
         <v>141</v>
@@ -9508,13 +9502,13 @@
         <v>416</v>
       </c>
       <c r="G202" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H202" t="s">
         <v>12</v>
       </c>
       <c r="I202" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9537,13 +9531,13 @@
         <v>420</v>
       </c>
       <c r="G203" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H203" t="s">
         <v>12</v>
       </c>
       <c r="I203" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9566,13 +9560,13 @@
         <v>423</v>
       </c>
       <c r="G204" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H204" t="s">
         <v>12</v>
       </c>
       <c r="I204" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="205" spans="1:9" x14ac:dyDescent="0.25">
@@ -9592,7 +9586,7 @@
         <v>431</v>
       </c>
       <c r="G205" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H205" t="s">
         <v>12</v>
@@ -9619,7 +9613,7 @@
         <v>438</v>
       </c>
       <c r="G206" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H206" t="s">
         <v>12</v>
@@ -9628,10 +9622,10 @@
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="B207" t="s">
-        <v>1192</v>
+        <v>1190</v>
       </c>
       <c r="C207">
         <v>250</v>
@@ -9640,13 +9634,13 @@
         <v>200</v>
       </c>
       <c r="E207" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="F207" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
       <c r="G207" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H207" t="s">
         <v>12</v>
@@ -9655,10 +9649,10 @@
     </row>
     <row r="208" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>1183</v>
+        <v>1181</v>
       </c>
       <c r="B208" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="C208">
         <v>333</v>
@@ -9673,7 +9667,7 @@
         <v>440</v>
       </c>
       <c r="G208" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H208" t="s">
         <v>12</v>
@@ -9682,22 +9676,22 @@
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>1151</v>
+        <v>1149</v>
       </c>
       <c r="B209" t="s">
-        <v>1150</v>
+        <v>1148</v>
       </c>
       <c r="C209">
         <v>300</v>
       </c>
       <c r="E209" t="s">
-        <v>1149</v>
+        <v>1147</v>
       </c>
       <c r="F209" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
       <c r="G209" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H209" t="s">
         <v>12</v>
@@ -9706,22 +9700,22 @@
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
       <c r="B210" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
       <c r="C210">
         <v>200</v>
       </c>
       <c r="E210" t="s">
-        <v>1145</v>
+        <v>1143</v>
       </c>
       <c r="F210" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
       <c r="G210" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H210" t="s">
         <v>12</v>
@@ -9730,7 +9724,7 @@
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>1143</v>
+        <v>1141</v>
       </c>
       <c r="B211" t="s">
         <v>9</v>
@@ -9739,13 +9733,13 @@
         <v>300</v>
       </c>
       <c r="E211" t="s">
-        <v>1142</v>
+        <v>1140</v>
       </c>
       <c r="F211" t="s">
-        <v>1141</v>
+        <v>1139</v>
       </c>
       <c r="G211" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H211" t="s">
         <v>12</v>
@@ -9754,7 +9748,7 @@
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="B212" t="s">
         <v>22</v>
@@ -9763,13 +9757,13 @@
         <v>350</v>
       </c>
       <c r="E212" t="s">
-        <v>1139</v>
+        <v>1137</v>
       </c>
       <c r="F212" t="s">
-        <v>1138</v>
+        <v>1136</v>
       </c>
       <c r="G212" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="H212" t="s">
         <v>12</v>
@@ -9778,19 +9772,19 @@
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>1165</v>
+        <v>1163</v>
       </c>
       <c r="B213" t="s">
-        <v>1166</v>
+        <v>1164</v>
       </c>
       <c r="C213">
         <v>200</v>
       </c>
       <c r="E213" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="F213" t="s">
-        <v>1164</v>
+        <v>1162</v>
       </c>
       <c r="G213" t="s">
         <v>609</v>
@@ -9799,24 +9793,24 @@
         <v>608</v>
       </c>
       <c r="I213" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
       <c r="B214" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="C214">
         <v>200</v>
       </c>
       <c r="E214" t="s">
-        <v>1169</v>
+        <v>1167</v>
       </c>
       <c r="F214" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="G214" t="s">
         <v>609</v>
@@ -9828,19 +9822,19 @@
     </row>
     <row r="215" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>1162</v>
+        <v>1160</v>
       </c>
       <c r="B215" t="s">
-        <v>1163</v>
+        <v>1161</v>
       </c>
       <c r="C215">
         <v>150</v>
       </c>
       <c r="E215" t="s">
-        <v>1161</v>
+        <v>1159</v>
       </c>
       <c r="F215" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
       <c r="G215" t="s">
         <v>609</v>
@@ -9852,19 +9846,19 @@
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
       <c r="B216" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
       <c r="C216">
         <v>550</v>
       </c>
       <c r="E216" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
       <c r="F216" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="G216" t="s">
         <v>609</v>
@@ -9873,24 +9867,24 @@
         <v>608</v>
       </c>
       <c r="I216" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
       <c r="B217" t="s">
-        <v>1155</v>
+        <v>1153</v>
       </c>
       <c r="C217">
         <v>200</v>
       </c>
       <c r="E217" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
       <c r="F217" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="G217" t="s">
         <v>609</v>
@@ -9899,24 +9893,24 @@
         <v>608</v>
       </c>
       <c r="I217" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>1136</v>
+        <v>1134</v>
       </c>
       <c r="B218" t="s">
-        <v>1137</v>
+        <v>1135</v>
       </c>
       <c r="C218">
         <v>200</v>
       </c>
       <c r="E218" t="s">
-        <v>1135</v>
+        <v>1133</v>
       </c>
       <c r="F218" t="s">
-        <v>1134</v>
+        <v>1132</v>
       </c>
       <c r="G218" t="s">
         <v>609</v>
@@ -9925,24 +9919,24 @@
         <v>608</v>
       </c>
       <c r="I218" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="219" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>1132</v>
+        <v>1130</v>
       </c>
       <c r="B219" t="s">
-        <v>1133</v>
+        <v>1131</v>
       </c>
       <c r="C219">
         <v>200</v>
       </c>
       <c r="E219" t="s">
-        <v>1131</v>
+        <v>1129</v>
       </c>
       <c r="F219" t="s">
-        <v>1130</v>
+        <v>1128</v>
       </c>
       <c r="G219" t="s">
         <v>609</v>
@@ -9951,24 +9945,24 @@
         <v>608</v>
       </c>
       <c r="I219" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
       <c r="B220" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
       <c r="C220">
         <v>250</v>
       </c>
       <c r="E220" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="F220" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
       <c r="G220" t="s">
         <v>609</v>
@@ -9977,24 +9971,24 @@
         <v>608</v>
       </c>
       <c r="I220" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
       <c r="B221" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
       <c r="C221">
         <v>300</v>
       </c>
       <c r="E221" s="7" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
       <c r="F221" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
       <c r="G221" t="s">
         <v>609</v>
@@ -10003,24 +9997,24 @@
         <v>608</v>
       </c>
       <c r="I221" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>1120</v>
+        <v>1118</v>
       </c>
       <c r="B222" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="C222">
         <v>200</v>
       </c>
       <c r="E222" t="s">
-        <v>1119</v>
+        <v>1117</v>
       </c>
       <c r="F222" t="s">
-        <v>1118</v>
+        <v>1116</v>
       </c>
       <c r="G222" t="s">
         <v>609</v>
@@ -10029,7 +10023,7 @@
         <v>608</v>
       </c>
       <c r="I222" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10055,7 +10049,7 @@
         <v>608</v>
       </c>
       <c r="I223" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10081,7 +10075,7 @@
         <v>608</v>
       </c>
       <c r="I224" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.25">
@@ -10107,7 +10101,7 @@
         <v>608</v>
       </c>
       <c r="I225" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="226" spans="1:9" x14ac:dyDescent="0.25">
@@ -10133,7 +10127,7 @@
         <v>608</v>
       </c>
       <c r="I226" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10159,7 +10153,7 @@
         <v>608</v>
       </c>
       <c r="I227" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10185,7 +10179,7 @@
         <v>608</v>
       </c>
       <c r="I228" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10211,7 +10205,7 @@
         <v>608</v>
       </c>
       <c r="I229" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
@@ -10237,7 +10231,7 @@
         <v>608</v>
       </c>
       <c r="I230" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10263,7 +10257,7 @@
         <v>608</v>
       </c>
       <c r="I231" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10289,7 +10283,7 @@
         <v>608</v>
       </c>
       <c r="I232" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10315,7 +10309,7 @@
         <v>608</v>
       </c>
       <c r="I233" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="234" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -10341,7 +10335,7 @@
         <v>608</v>
       </c>
       <c r="I234" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10367,7 +10361,7 @@
         <v>608</v>
       </c>
       <c r="I235" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10505,7 +10499,7 @@
         <v>256</v>
       </c>
       <c r="G241" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H241" t="s">
         <v>109</v>
@@ -10513,7 +10507,7 @@
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>1208</v>
+        <v>1206</v>
       </c>
       <c r="B242" t="s">
         <v>515</v>
@@ -10531,7 +10525,7 @@
         <v>526</v>
       </c>
       <c r="G242" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H242" t="s">
         <v>109</v>
@@ -10557,7 +10551,7 @@
         <v>340</v>
       </c>
       <c r="G243" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H243" t="s">
         <v>109</v>
@@ -10583,7 +10577,7 @@
         <v>550</v>
       </c>
       <c r="G244" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H244" t="s">
         <v>109</v>
@@ -10609,7 +10603,7 @@
         <v>1024</v>
       </c>
       <c r="G245" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H245" t="s">
         <v>109</v>
@@ -10635,7 +10629,7 @@
         <v>1020</v>
       </c>
       <c r="G246" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H246" t="s">
         <v>109</v>
@@ -10661,7 +10655,7 @@
         <v>1015</v>
       </c>
       <c r="G247" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H247" t="s">
         <v>109</v>
@@ -10687,7 +10681,7 @@
         <v>1011</v>
       </c>
       <c r="G248" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H248" t="s">
         <v>109</v>
@@ -10713,13 +10707,13 @@
         <v>526</v>
       </c>
       <c r="G249" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H249" t="s">
         <v>109</v>
       </c>
       <c r="I249" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10742,13 +10736,13 @@
         <v>112</v>
       </c>
       <c r="G250" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H250" t="s">
         <v>109</v>
       </c>
       <c r="I250" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -10771,7 +10765,7 @@
         <v>116</v>
       </c>
       <c r="G251" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H251" t="s">
         <v>109</v>
@@ -10797,7 +10791,7 @@
         <v>532</v>
       </c>
       <c r="G252" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H252" t="s">
         <v>109</v>
@@ -10821,7 +10815,7 @@
         <v>119</v>
       </c>
       <c r="G253" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H253" t="s">
         <v>109</v>
@@ -10848,7 +10842,7 @@
         <v>994</v>
       </c>
       <c r="G254" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H254" t="s">
         <v>109</v>
@@ -10875,7 +10869,7 @@
         <v>990</v>
       </c>
       <c r="G255" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H255" t="s">
         <v>109</v>
@@ -10902,13 +10896,13 @@
         <v>988</v>
       </c>
       <c r="G256" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H256" t="s">
         <v>109</v>
       </c>
       <c r="I256" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="257" spans="1:9" x14ac:dyDescent="0.25">
@@ -10916,7 +10910,7 @@
         <v>120</v>
       </c>
       <c r="B257" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="C257">
         <v>515</v>
@@ -10931,13 +10925,13 @@
         <v>122</v>
       </c>
       <c r="G257" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H257" t="s">
         <v>109</v>
       </c>
       <c r="I257" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="258" spans="1:9" x14ac:dyDescent="0.25">
@@ -10957,13 +10951,13 @@
         <v>125</v>
       </c>
       <c r="G258" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H258" t="s">
         <v>109</v>
       </c>
       <c r="I258" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="259" spans="1:9" x14ac:dyDescent="0.25">
@@ -10986,13 +10980,13 @@
         <v>961</v>
       </c>
       <c r="G259" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H259" t="s">
         <v>109</v>
       </c>
       <c r="I259" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="260" spans="1:9" x14ac:dyDescent="0.25">
@@ -11015,13 +11009,13 @@
         <v>553</v>
       </c>
       <c r="G260" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H260" t="s">
         <v>109</v>
       </c>
       <c r="I260" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="261" spans="1:9" x14ac:dyDescent="0.25">
@@ -11044,13 +11038,13 @@
         <v>127</v>
       </c>
       <c r="G261" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H261" t="s">
         <v>109</v>
       </c>
       <c r="I261" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="262" spans="1:9" x14ac:dyDescent="0.25">
@@ -11070,13 +11064,13 @@
         <v>128</v>
       </c>
       <c r="G262" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H262" t="s">
         <v>109</v>
       </c>
       <c r="I262" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="263" spans="1:9" x14ac:dyDescent="0.25">
@@ -11099,13 +11093,13 @@
         <v>369</v>
       </c>
       <c r="G263" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H263" t="s">
         <v>109</v>
       </c>
       <c r="I263" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="264" spans="1:9" x14ac:dyDescent="0.25">
@@ -11128,13 +11122,13 @@
         <v>1031</v>
       </c>
       <c r="G264" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H264" t="s">
         <v>109</v>
       </c>
       <c r="I264" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="265" spans="1:9" x14ac:dyDescent="0.25">
@@ -11157,13 +11151,13 @@
         <v>1028</v>
       </c>
       <c r="G265" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H265" t="s">
         <v>109</v>
       </c>
       <c r="I265" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="266" spans="1:9" x14ac:dyDescent="0.25">
@@ -11186,21 +11180,21 @@
         <v>1026</v>
       </c>
       <c r="G266" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H266" t="s">
         <v>109</v>
       </c>
       <c r="I266" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="267" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
       <c r="B267" t="s">
-        <v>1199</v>
+        <v>1197</v>
       </c>
       <c r="C267">
         <v>3500</v>
@@ -11209,24 +11203,24 @@
         <v>2500</v>
       </c>
       <c r="E267" t="s">
-        <v>1201</v>
+        <v>1199</v>
       </c>
       <c r="F267" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="G267" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H267" t="s">
         <v>109</v>
       </c>
       <c r="I267" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="268" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>1194</v>
+        <v>1192</v>
       </c>
       <c r="B268" t="s">
         <v>129</v>
@@ -11244,18 +11238,18 @@
         <v>131</v>
       </c>
       <c r="G268" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H268" t="s">
         <v>109</v>
       </c>
       <c r="I268" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="269" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>1195</v>
+        <v>1193</v>
       </c>
       <c r="B269" t="s">
         <v>129</v>
@@ -11267,19 +11261,19 @@
         <v>6800</v>
       </c>
       <c r="E269" t="s">
-        <v>1197</v>
+        <v>1195</v>
       </c>
       <c r="F269" t="s">
-        <v>1196</v>
+        <v>1194</v>
       </c>
       <c r="G269" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H269" t="s">
         <v>109</v>
       </c>
       <c r="I269" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="270" spans="1:9" x14ac:dyDescent="0.25">
@@ -11302,13 +11296,13 @@
         <v>135</v>
       </c>
       <c r="G270" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H270" t="s">
         <v>109</v>
       </c>
       <c r="I270" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="271" spans="1:9" x14ac:dyDescent="0.25">
@@ -11331,13 +11325,13 @@
         <v>344</v>
       </c>
       <c r="G271" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H271" t="s">
         <v>109</v>
       </c>
       <c r="I271" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="272" spans="1:9" x14ac:dyDescent="0.25">
@@ -11357,13 +11351,13 @@
         <v>578</v>
       </c>
       <c r="G272" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H272" t="s">
         <v>109</v>
       </c>
       <c r="I272" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="273" spans="1:9" x14ac:dyDescent="0.25">
@@ -11383,18 +11377,18 @@
         <v>1000</v>
       </c>
       <c r="G273" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H273" t="s">
         <v>109</v>
       </c>
       <c r="I273" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="274" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>1203</v>
+        <v>1201</v>
       </c>
       <c r="B274" t="s">
         <v>18</v>
@@ -11412,13 +11406,13 @@
         <v>1002</v>
       </c>
       <c r="G274" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H274" t="s">
         <v>109</v>
       </c>
       <c r="I274" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="275" spans="1:9" x14ac:dyDescent="0.25">
@@ -11441,13 +11435,13 @@
         <v>997</v>
       </c>
       <c r="G275" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H275" t="s">
         <v>109</v>
       </c>
       <c r="I275" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="276" spans="1:9" x14ac:dyDescent="0.25">
@@ -11467,13 +11461,13 @@
         <v>137</v>
       </c>
       <c r="G276" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H276" t="s">
         <v>602</v>
       </c>
       <c r="I276" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="277" spans="1:9" x14ac:dyDescent="0.25">
@@ -11496,13 +11490,13 @@
         <v>979</v>
       </c>
       <c r="G277" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H277" t="s">
         <v>109</v>
       </c>
       <c r="I277" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="278" spans="1:9" x14ac:dyDescent="0.25">
@@ -11522,13 +11516,13 @@
         <v>143</v>
       </c>
       <c r="G278" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H278" t="s">
         <v>109</v>
       </c>
       <c r="I278" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="279" spans="1:9" x14ac:dyDescent="0.25">
@@ -11551,7 +11545,7 @@
         <v>144</v>
       </c>
       <c r="G279" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H279" t="s">
         <v>109</v>
@@ -11560,7 +11554,7 @@
     </row>
     <row r="280" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>1202</v>
+        <v>1200</v>
       </c>
       <c r="B280" t="s">
         <v>18</v>
@@ -11575,13 +11569,13 @@
         <v>146</v>
       </c>
       <c r="G280" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H280" t="s">
         <v>109</v>
       </c>
       <c r="I280" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="281" spans="1:9" x14ac:dyDescent="0.25">
@@ -11592,10 +11586,10 @@
         <v>677</v>
       </c>
       <c r="C281">
+        <v>600</v>
+      </c>
+      <c r="D281">
         <v>550</v>
-      </c>
-      <c r="D281">
-        <v>200</v>
       </c>
       <c r="E281" t="s">
         <v>676</v>
@@ -11604,13 +11598,13 @@
         <v>675</v>
       </c>
       <c r="G281" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H281" t="s">
         <v>109</v>
       </c>
       <c r="I281" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="282" spans="1:9" x14ac:dyDescent="0.25">
@@ -11630,13 +11624,13 @@
         <v>147</v>
       </c>
       <c r="G282" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H282" t="s">
         <v>109</v>
       </c>
       <c r="I282" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="283" spans="1:9" x14ac:dyDescent="0.25">
@@ -11659,13 +11653,13 @@
         <v>150</v>
       </c>
       <c r="G283" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H283" t="s">
         <v>109</v>
       </c>
       <c r="I283" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="284" spans="1:9" x14ac:dyDescent="0.25">
@@ -11688,13 +11682,13 @@
         <v>153</v>
       </c>
       <c r="G284" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H284" t="s">
         <v>109</v>
       </c>
       <c r="I284" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="285" spans="1:9" x14ac:dyDescent="0.25">
@@ -11717,18 +11711,18 @@
         <v>156</v>
       </c>
       <c r="G285" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H285" t="s">
         <v>109</v>
       </c>
       <c r="I285" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="286" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>1207</v>
+        <v>1205</v>
       </c>
       <c r="B286" t="s">
         <v>158</v>
@@ -11746,18 +11740,18 @@
         <v>160</v>
       </c>
       <c r="G286" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H286" t="s">
         <v>109</v>
       </c>
       <c r="I286" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="287" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>1206</v>
+        <v>1204</v>
       </c>
       <c r="B287" t="s">
         <v>161</v>
@@ -11775,18 +11769,18 @@
         <v>163</v>
       </c>
       <c r="G287" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H287" t="s">
         <v>109</v>
       </c>
       <c r="I287" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="288" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>1205</v>
+        <v>1203</v>
       </c>
       <c r="B288" t="s">
         <v>138</v>
@@ -11804,13 +11798,13 @@
         <v>140</v>
       </c>
       <c r="G288" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H288" t="s">
         <v>109</v>
       </c>
       <c r="I288" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="289" spans="1:9" x14ac:dyDescent="0.25">
@@ -11833,18 +11827,18 @@
         <v>165</v>
       </c>
       <c r="G289" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H289" t="s">
         <v>109</v>
       </c>
       <c r="I289" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="290" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A290" s="5" t="s">
-        <v>1204</v>
+        <v>1202</v>
       </c>
       <c r="B290" t="s">
         <v>117</v>
@@ -11859,13 +11853,13 @@
         <v>157</v>
       </c>
       <c r="G290" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H290" t="s">
         <v>109</v>
       </c>
       <c r="I290" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="291" spans="1:9" x14ac:dyDescent="0.25">
@@ -11888,13 +11882,13 @@
         <v>167</v>
       </c>
       <c r="G291" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H291" t="s">
         <v>603</v>
       </c>
       <c r="I291" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="292" spans="1:9" x14ac:dyDescent="0.25">
@@ -11914,13 +11908,13 @@
         <v>496</v>
       </c>
       <c r="G292" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="H292" t="s">
         <v>109</v>
       </c>
       <c r="I292" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="293" spans="1:9" x14ac:dyDescent="0.25">
@@ -11946,7 +11940,7 @@
         <v>767</v>
       </c>
       <c r="I293" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="294" spans="1:9" x14ac:dyDescent="0.25">
@@ -11972,7 +11966,7 @@
         <v>767</v>
       </c>
       <c r="I294" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="295" spans="1:9" x14ac:dyDescent="0.25">
@@ -11998,7 +11992,7 @@
         <v>767</v>
       </c>
       <c r="I295" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="296" spans="1:9" x14ac:dyDescent="0.25">
@@ -12027,7 +12021,7 @@
         <v>767</v>
       </c>
       <c r="I296" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="297" spans="1:9" x14ac:dyDescent="0.25">
@@ -12053,7 +12047,7 @@
         <v>767</v>
       </c>
       <c r="I297" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="298" spans="1:9" x14ac:dyDescent="0.25">
@@ -12079,7 +12073,7 @@
         <v>767</v>
       </c>
       <c r="I298" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="299" spans="1:9" x14ac:dyDescent="0.25">
@@ -12105,7 +12099,7 @@
         <v>767</v>
       </c>
       <c r="I299" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="300" spans="1:9" x14ac:dyDescent="0.25">
@@ -12131,7 +12125,7 @@
         <v>767</v>
       </c>
       <c r="I300" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="301" spans="1:9" x14ac:dyDescent="0.25">
@@ -12157,7 +12151,7 @@
         <v>767</v>
       </c>
       <c r="I301" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="302" spans="1:9" x14ac:dyDescent="0.25">
@@ -12354,7 +12348,7 @@
         <v>767</v>
       </c>
       <c r="I309" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="310" spans="1:9" x14ac:dyDescent="0.25">
@@ -12383,7 +12377,7 @@
         <v>767</v>
       </c>
       <c r="I310" s="4" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="311" spans="1:9" x14ac:dyDescent="0.25">
@@ -12412,7 +12406,7 @@
         <v>69</v>
       </c>
       <c r="I311" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="312" spans="1:9" x14ac:dyDescent="0.25">
@@ -12441,27 +12435,27 @@
         <v>69</v>
       </c>
       <c r="I312" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="313" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>1041</v>
+        <v>195</v>
       </c>
       <c r="B313" t="s">
-        <v>1042</v>
+        <v>1038</v>
       </c>
       <c r="C313">
-        <v>450</v>
+        <v>439</v>
       </c>
       <c r="D313">
         <v>350</v>
       </c>
       <c r="E313" t="s">
-        <v>959</v>
+        <v>196</v>
       </c>
       <c r="F313" t="s">
-        <v>958</v>
+        <v>197</v>
       </c>
       <c r="G313" t="s">
         <v>1035</v>
@@ -12470,27 +12464,27 @@
         <v>69</v>
       </c>
       <c r="I313" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="314" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>195</v>
+        <v>1210</v>
       </c>
       <c r="B314" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="C314">
-        <v>439</v>
+        <v>200</v>
       </c>
       <c r="D314">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="E314" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F314" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G314" t="s">
         <v>1035</v>
@@ -12499,27 +12493,27 @@
         <v>69</v>
       </c>
       <c r="I314" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="315" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>1212</v>
+        <v>200</v>
       </c>
       <c r="B315" t="s">
-        <v>1039</v>
+        <v>27</v>
       </c>
       <c r="C315">
-        <v>200</v>
+        <v>575</v>
       </c>
       <c r="D315">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="E315" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F315" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="G315" t="s">
         <v>1035</v>
@@ -12528,27 +12522,27 @@
         <v>69</v>
       </c>
       <c r="I315" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="316" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B316" t="s">
-        <v>27</v>
+        <v>1040</v>
       </c>
       <c r="C316">
-        <v>575</v>
+        <v>650</v>
       </c>
       <c r="D316">
-        <v>250</v>
+        <v>350</v>
       </c>
       <c r="E316" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="F316" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="G316" t="s">
         <v>1035</v>
@@ -12557,56 +12551,56 @@
         <v>69</v>
       </c>
       <c r="I316" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="317" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>203</v>
+        <v>934</v>
       </c>
       <c r="B317" t="s">
-        <v>1040</v>
+        <v>936</v>
       </c>
       <c r="C317">
-        <v>650</v>
+        <v>735</v>
       </c>
       <c r="D317">
-        <v>350</v>
+        <v>450</v>
       </c>
       <c r="E317" t="s">
-        <v>204</v>
+        <v>937</v>
       </c>
       <c r="F317" t="s">
-        <v>205</v>
+        <v>935</v>
       </c>
       <c r="G317" t="s">
-        <v>1035</v>
+        <v>501</v>
       </c>
       <c r="H317" t="s">
-        <v>69</v>
+        <v>12</v>
       </c>
       <c r="I317" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="318" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>934</v>
+        <v>943</v>
       </c>
       <c r="B318" t="s">
-        <v>936</v>
+        <v>942</v>
       </c>
       <c r="C318">
-        <v>735</v>
+        <v>890</v>
       </c>
       <c r="D318">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="E318" t="s">
-        <v>937</v>
+        <v>945</v>
       </c>
       <c r="F318" t="s">
-        <v>935</v>
+        <v>944</v>
       </c>
       <c r="G318" t="s">
         <v>501</v>
@@ -12615,27 +12609,27 @@
         <v>12</v>
       </c>
       <c r="I318" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="319" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>943</v>
+        <v>933</v>
       </c>
       <c r="B319" t="s">
-        <v>942</v>
+        <v>930</v>
       </c>
       <c r="C319">
-        <v>890</v>
+        <v>749</v>
       </c>
       <c r="D319">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="E319" t="s">
-        <v>945</v>
+        <v>932</v>
       </c>
       <c r="F319" t="s">
-        <v>944</v>
+        <v>931</v>
       </c>
       <c r="G319" t="s">
         <v>501</v>
@@ -12644,27 +12638,27 @@
         <v>12</v>
       </c>
       <c r="I319" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="320" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>933</v>
+        <v>939</v>
       </c>
       <c r="B320" t="s">
-        <v>930</v>
+        <v>938</v>
       </c>
       <c r="C320">
-        <v>749</v>
+        <v>879</v>
       </c>
       <c r="D320">
-        <v>400</v>
+        <v>650</v>
       </c>
       <c r="E320" t="s">
-        <v>932</v>
+        <v>941</v>
       </c>
       <c r="F320" t="s">
-        <v>931</v>
+        <v>940</v>
       </c>
       <c r="G320" t="s">
         <v>501</v>
@@ -12673,27 +12667,27 @@
         <v>12</v>
       </c>
       <c r="I320" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="321" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>939</v>
+        <v>950</v>
       </c>
       <c r="B321" t="s">
-        <v>938</v>
+        <v>949</v>
       </c>
       <c r="C321">
-        <v>879</v>
+        <v>715</v>
       </c>
       <c r="D321">
-        <v>650</v>
+        <v>450</v>
       </c>
       <c r="E321" t="s">
-        <v>941</v>
+        <v>952</v>
       </c>
       <c r="F321" t="s">
-        <v>940</v>
+        <v>951</v>
       </c>
       <c r="G321" t="s">
         <v>501</v>
@@ -12702,27 +12696,27 @@
         <v>12</v>
       </c>
       <c r="I321" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="322" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>950</v>
+        <v>946</v>
       </c>
       <c r="B322" t="s">
-        <v>949</v>
+        <v>942</v>
       </c>
       <c r="C322">
-        <v>715</v>
+        <v>635</v>
       </c>
       <c r="D322">
-        <v>450</v>
+        <v>400</v>
       </c>
       <c r="E322" t="s">
-        <v>952</v>
+        <v>948</v>
       </c>
       <c r="F322" t="s">
-        <v>951</v>
+        <v>947</v>
       </c>
       <c r="G322" t="s">
         <v>501</v>
@@ -12731,27 +12725,27 @@
         <v>12</v>
       </c>
       <c r="I322" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="323" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A323" t="s">
-        <v>946</v>
+      <c r="A323" s="3" t="s">
+        <v>926</v>
       </c>
       <c r="B323" t="s">
-        <v>942</v>
+        <v>928</v>
       </c>
       <c r="C323">
-        <v>635</v>
+        <v>570</v>
       </c>
       <c r="D323">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E323" t="s">
-        <v>948</v>
+        <v>929</v>
       </c>
       <c r="F323" t="s">
-        <v>947</v>
+        <v>927</v>
       </c>
       <c r="G323" t="s">
         <v>501</v>
@@ -12760,27 +12754,27 @@
         <v>12</v>
       </c>
       <c r="I323" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="324" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A324" s="3" t="s">
-        <v>926</v>
+      <c r="A324" t="s">
+        <v>922</v>
       </c>
       <c r="B324" t="s">
-        <v>928</v>
+        <v>923</v>
       </c>
       <c r="C324">
-        <v>570</v>
+        <v>497</v>
       </c>
       <c r="D324">
         <v>300</v>
       </c>
       <c r="E324" t="s">
-        <v>929</v>
+        <v>925</v>
       </c>
       <c r="F324" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="G324" t="s">
         <v>501</v>
@@ -12789,27 +12783,27 @@
         <v>12</v>
       </c>
       <c r="I324" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="325" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>922</v>
+        <v>247</v>
       </c>
       <c r="B325" t="s">
-        <v>923</v>
+        <v>1179</v>
       </c>
       <c r="C325">
-        <v>497</v>
+        <v>678</v>
       </c>
       <c r="D325">
-        <v>300</v>
+        <v>450</v>
       </c>
       <c r="E325" t="s">
-        <v>925</v>
+        <v>248</v>
       </c>
       <c r="F325" t="s">
-        <v>924</v>
+        <v>249</v>
       </c>
       <c r="G325" t="s">
         <v>501</v>
@@ -12818,27 +12812,24 @@
         <v>12</v>
       </c>
       <c r="I325" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="326" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>247</v>
+        <v>432</v>
       </c>
       <c r="B326" t="s">
-        <v>1181</v>
+        <v>433</v>
       </c>
       <c r="C326">
-        <v>678</v>
-      </c>
-      <c r="D326">
-        <v>450</v>
+        <v>100</v>
       </c>
       <c r="E326" t="s">
-        <v>248</v>
+        <v>434</v>
       </c>
       <c r="F326" t="s">
-        <v>249</v>
+        <v>435</v>
       </c>
       <c r="G326" t="s">
         <v>501</v>
@@ -12847,24 +12838,27 @@
         <v>12</v>
       </c>
       <c r="I326" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="327" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>432</v>
+        <v>243</v>
       </c>
       <c r="B327" t="s">
-        <v>433</v>
+        <v>244</v>
       </c>
       <c r="C327">
-        <v>100</v>
+        <v>419.19</v>
+      </c>
+      <c r="D327">
+        <v>300</v>
       </c>
       <c r="E327" t="s">
-        <v>434</v>
+        <v>245</v>
       </c>
       <c r="F327" t="s">
-        <v>435</v>
+        <v>246</v>
       </c>
       <c r="G327" t="s">
         <v>501</v>
@@ -12873,27 +12867,27 @@
         <v>12</v>
       </c>
       <c r="I327" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="328" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="B328" t="s">
-        <v>244</v>
+        <v>1180</v>
       </c>
       <c r="C328">
-        <v>419.19</v>
+        <v>600</v>
       </c>
       <c r="D328">
         <v>300</v>
       </c>
       <c r="E328" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F328" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="G328" t="s">
         <v>501</v>
@@ -12902,27 +12896,27 @@
         <v>12</v>
       </c>
       <c r="I328" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="329" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>250</v>
+        <v>502</v>
       </c>
       <c r="B329" t="s">
-        <v>1182</v>
+        <v>503</v>
       </c>
       <c r="C329">
-        <v>600</v>
+        <v>911</v>
       </c>
       <c r="D329">
-        <v>300</v>
+        <v>540</v>
       </c>
       <c r="E329" t="s">
-        <v>251</v>
+        <v>504</v>
       </c>
       <c r="F329" t="s">
-        <v>252</v>
+        <v>505</v>
       </c>
       <c r="G329" t="s">
         <v>501</v>
@@ -12931,27 +12925,27 @@
         <v>12</v>
       </c>
       <c r="I329" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="330" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B330" t="s">
-        <v>503</v>
+        <v>511</v>
       </c>
       <c r="C330">
-        <v>911</v>
+        <v>800</v>
       </c>
       <c r="D330">
-        <v>540</v>
+        <v>400</v>
       </c>
       <c r="E330" t="s">
-        <v>504</v>
+        <v>512</v>
       </c>
       <c r="F330" t="s">
-        <v>505</v>
+        <v>513</v>
       </c>
       <c r="G330" t="s">
         <v>501</v>
@@ -12960,27 +12954,27 @@
         <v>12</v>
       </c>
       <c r="I330" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="331" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="B331" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="C331">
-        <v>800</v>
+        <v>365</v>
       </c>
       <c r="D331">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E331" t="s">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="F331" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="G331" t="s">
         <v>501</v>
@@ -12989,27 +12983,24 @@
         <v>12</v>
       </c>
       <c r="I331" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="332" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>506</v>
+        <v>1170</v>
       </c>
       <c r="B332" t="s">
-        <v>507</v>
+        <v>1171</v>
       </c>
       <c r="C332">
-        <v>365</v>
-      </c>
-      <c r="D332">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="E332" t="s">
-        <v>508</v>
+        <v>1173</v>
       </c>
       <c r="F332" t="s">
-        <v>509</v>
+        <v>1172</v>
       </c>
       <c r="G332" t="s">
         <v>501</v>
@@ -13018,24 +13009,27 @@
         <v>12</v>
       </c>
       <c r="I332" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="333" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>1172</v>
+        <v>1174</v>
       </c>
       <c r="B333" t="s">
-        <v>1173</v>
+        <v>1177</v>
       </c>
       <c r="C333">
-        <v>350</v>
+        <v>200</v>
+      </c>
+      <c r="D333">
+        <v>170</v>
       </c>
       <c r="E333" t="s">
         <v>1175</v>
       </c>
       <c r="F333" t="s">
-        <v>1174</v>
+        <v>1176</v>
       </c>
       <c r="G333" t="s">
         <v>501</v>
@@ -13044,36 +13038,7 @@
         <v>12</v>
       </c>
       <c r="I333" s="6" t="s">
-        <v>1043</v>
-      </c>
-    </row>
-    <row r="334" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A334" t="s">
-        <v>1176</v>
-      </c>
-      <c r="B334" t="s">
-        <v>1179</v>
-      </c>
-      <c r="C334">
-        <v>200</v>
-      </c>
-      <c r="D334">
-        <v>170</v>
-      </c>
-      <c r="E334" t="s">
-        <v>1177</v>
-      </c>
-      <c r="F334" t="s">
-        <v>1178</v>
-      </c>
-      <c r="G334" t="s">
-        <v>501</v>
-      </c>
-      <c r="H334" t="s">
-        <v>12</v>
-      </c>
-      <c r="I334" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualiza proyecto (2 modificados, 14 nuevos): productos.xlsx, index.html, D_NQ_NP_2X_647415-CBT111501198724_062026-F-espejo-luz-led-touch-pared-bano-decorativo-tocador-3-luces.webp
</commit_message>
<xml_diff>
--- a/datos/productos.xlsx
+++ b/datos/productos.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Proyecto\Catalogo\datos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Respaldo\Catalogo\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2420" uniqueCount="1354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2486" uniqueCount="1395">
   <si>
     <t>Nombre</t>
   </si>
@@ -4091,6 +4091,133 @@
   </si>
   <si>
     <t>https://panchochacharas.netlify.app/imagenes/4aaa7507c541c0dc0aac5e2393fb2c31.jpeg</t>
+  </si>
+  <si>
+    <t>Aluminio Negro con Mango de Madera, Set de 3 Unidades (24 y 28 cm)</t>
+  </si>
+  <si>
+    <t>Pack de Sartenes Antiadherentes</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_718669-MLA109014019546_032026-F.webp</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/pack-de-sartenes-antiadherentes-xinest-de-aluminio-negro-con-mango-de-madera-set-de-3-unidades-24-y-28-cm/p/MLM67441876?pdp_filters=item_id%3AMLM5595517674#&amp;gid=1&amp;pid=1</t>
+  </si>
+  <si>
+    <t>Pistola Para Pintar Eléctrica</t>
+  </si>
+  <si>
+    <t>1500 W con Tanque de 1 L y 4 Boquillas</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/pistola-para-pintar-electrica-kozfule-1500-w-con-tanque-de-1-l-y-4-boquillas/p/MLM74444635?pdp_filters=item_id:MLM5570051942#&amp;gid=1&amp;pid=1</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_766896-MLA112984703506_072026-F.webp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pistola Pintar Inalámbrica </t>
+  </si>
+  <si>
+    <t>24v 3 Baterías Profesional Hvlp</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-5179674838-pistola-pintar-inalambrica-24v-3-baterias-profesional-hvlp-_JM?quantity=1#&amp;gid=1&amp;pid=1</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_693699-CBT113902483621_062026-F-pistola-pintar-inalambrica-24v-3-baterias-profesional-hvlp.webp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set De Bloques Bonsái Flor Cerezo </t>
+  </si>
+  <si>
+    <t>775 Piezas</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-5457979378-set-de-bloques-bonsai-flor-cerezo-775-piezas-_JM?quantity=1#&amp;gid=1&amp;pid=1</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_980602-CBT111696934142_062026-F-set-de-bloques-bonsai-flor-cerezo-775-piezas.webp</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-2999989219-set-de-bloques-de-construccion-de-bote-482-piezas-ninos-_JM?quantity=1</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_676962-CBT111935393828_062026-F-set-de-bloques-de-construccion-de-bote-482-piezas-ninos.webp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set De Bloques De Construcción De Bote </t>
+  </si>
+  <si>
+    <t>482 Piezas</t>
+  </si>
+  <si>
+    <t>Epicentro Restaurador De Bajos Audishako MAX-MX Ecualizador Para Sistema De Audio Auto, Pickup Y Suv, Para Subwoofer, Incluye Control Remoto Y Accesorios De Instalación</t>
+  </si>
+  <si>
+    <t>Sistema de audio</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/epicentro-restaurador-de-bajos-audishako-max-mx-ecualizador-para-sistema-de-audio-auto-pickup-y-suv-para-subwoofer-incluye-control-remoto-y-accesorios-de-instalacion/p/MLM51149598?pdp_filters=item_id:MLM2546220371</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_831886-MLA99444153134_112025-F.webp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epicentro Audishako Max-02 Restaurador De Bajos Para Auto, Subwoofer Para Carro, Pickups Y Suv, Accesorios Para Auto Audio Diseño En Relieve 3d, Incluye Dash Remoto Control De Bajos
+</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/epicentro-audishako-max-02-restaurador-de-bajos-para-auto-subwoofer-para-carro-pickups-y-suv-accesorios-para-auto-audio-diseno-en-relieve-3d-incluye-dash-remoto-control-de-bajos/p/MLM64640099?pdp_filters=item_id:MLM4697020282</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_801469-MLA105455425099_012026-F.webp</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-5166780854-espejo-luz-led-touch-pared-bano-decorativo-tocador-3-luces-_JM?quantity=1&amp;variation_id=192915215412</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_647415-CBT111501198724_062026-F-espejo-luz-led-touch-pared-bano-decorativo-tocador-3-luces.webp</t>
+  </si>
+  <si>
+    <t>Espejo Luz Led Touch Pared Baño Decorativo Tocador 3 Luces</t>
+  </si>
+  <si>
+    <t>Altura: 52.5 cm, Ancho: 37.5 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inversor Hzero 600W de Onda Senoidal Modificada para Auto con 2 Salidas AC y 2 USB
+</t>
+  </si>
+  <si>
+    <t>Inversor</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/inversor-hzero-600w-de-onda-senoidal-modificada-para-auto-con-2-salidas-ac-y-2-usb/p/MLM52856540?pdp_filters=item_id:MLM2587727551</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_996228-MLA110110565683_042026-F.webp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hzero Inversor De Corriente 1000W 12v A 110v, Transformador Portatil Para Coche Con 2 Ac Y 2 Usb, Ideal Para Respaldo Eléctrico Hogar, Protección Eléctrica Múltiple
+</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/hzero-inversor-de-corriente-1000w-12v-a-110v-transformador-portatil-para-coche-con-2-ac-y-2-usb-ideal-para-respaldo-electrico-hogar-proteccion-electrica-multiple/p/MLM57806893?pdp_filters=item_id:MLM2587781837</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_911255-MLA109065062914_032026-F.webp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hzero Convertidor Inversor De Corriente 4000W 12v-110v Para Herramientas Eléctricas Feria Exterior, Transformador Portatil 2 AC+ 2 USB, Protección Eléctrica Múltiple
+</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/hzero-convertidor-inversor-de-corriente-4000w-12v-110v-para-herramientas-electricas-feria-exterior-transformador-portatil-2-ac-2-usb-proteccion-electrica-multiple/p/MLM68452917?pdp_filters=item_id:MLM5235134128</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_987469-MLA110791222267_042026-F.webp</t>
   </si>
 </sst>
 </file>
@@ -4264,8 +4391,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H367" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A1:H367"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H378" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A1:H378"/>
   <sortState ref="A2:H342">
     <sortCondition ref="A1:A342"/>
   </sortState>
@@ -4568,7 +4695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I367"/>
+  <dimension ref="A1:I378"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="70" style="1" customWidth="1"/>
@@ -14501,13 +14628,299 @@
         <v>1346</v>
       </c>
       <c r="G367" s="7" t="s">
-        <v>1338</v>
+        <v>441</v>
       </c>
       <c r="H367" s="7" t="s">
         <v>66</v>
       </c>
       <c r="I367" s="14" t="s">
         <v>903</v>
+      </c>
+    </row>
+    <row r="368" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A368" s="1" t="s">
+        <v>1355</v>
+      </c>
+      <c r="B368" s="1" t="s">
+        <v>1354</v>
+      </c>
+      <c r="C368" s="7">
+        <v>1383</v>
+      </c>
+      <c r="D368" s="7">
+        <v>630</v>
+      </c>
+      <c r="E368" s="15" t="s">
+        <v>1356</v>
+      </c>
+      <c r="F368" s="15" t="s">
+        <v>1357</v>
+      </c>
+      <c r="G368" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="H368" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="369" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A369" s="1" t="s">
+        <v>1358</v>
+      </c>
+      <c r="B369" s="1" t="s">
+        <v>1359</v>
+      </c>
+      <c r="C369" s="7">
+        <v>899</v>
+      </c>
+      <c r="D369" s="7">
+        <v>485</v>
+      </c>
+      <c r="E369" s="15" t="s">
+        <v>1361</v>
+      </c>
+      <c r="F369" s="15" t="s">
+        <v>1360</v>
+      </c>
+      <c r="G369" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="H369" s="7" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="370" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A370" s="1" t="s">
+        <v>1362</v>
+      </c>
+      <c r="B370" s="1" t="s">
+        <v>1363</v>
+      </c>
+      <c r="C370" s="7">
+        <v>1050</v>
+      </c>
+      <c r="D370" s="7">
+        <v>600</v>
+      </c>
+      <c r="E370" s="15" t="s">
+        <v>1365</v>
+      </c>
+      <c r="F370" s="15" t="s">
+        <v>1364</v>
+      </c>
+      <c r="G370" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="H370" s="7" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="371" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A371" s="1" t="s">
+        <v>1366</v>
+      </c>
+      <c r="B371" s="1" t="s">
+        <v>1367</v>
+      </c>
+      <c r="C371" s="7">
+        <v>1084</v>
+      </c>
+      <c r="D371" s="7">
+        <v>650</v>
+      </c>
+      <c r="E371" s="15" t="s">
+        <v>1369</v>
+      </c>
+      <c r="F371" s="15" t="s">
+        <v>1368</v>
+      </c>
+      <c r="G371" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="H371" s="7" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="372" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A372" s="1" t="s">
+        <v>1372</v>
+      </c>
+      <c r="B372" s="1" t="s">
+        <v>1373</v>
+      </c>
+      <c r="C372" s="7">
+        <v>1265</v>
+      </c>
+      <c r="D372" s="7">
+        <v>650</v>
+      </c>
+      <c r="E372" s="15" t="s">
+        <v>1371</v>
+      </c>
+      <c r="F372" s="15" t="s">
+        <v>1370</v>
+      </c>
+      <c r="G372" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="H372" s="7" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="373" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A373" s="1" t="s">
+        <v>1374</v>
+      </c>
+      <c r="B373" s="1" t="s">
+        <v>1375</v>
+      </c>
+      <c r="C373" s="7">
+        <v>1225</v>
+      </c>
+      <c r="D373" s="7">
+        <v>700</v>
+      </c>
+      <c r="E373" s="15" t="s">
+        <v>1377</v>
+      </c>
+      <c r="F373" s="15" t="s">
+        <v>1376</v>
+      </c>
+      <c r="G373" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="H373" s="7" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="374" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A374" s="1" t="s">
+        <v>1378</v>
+      </c>
+      <c r="B374" s="1" t="s">
+        <v>1375</v>
+      </c>
+      <c r="C374" s="7">
+        <v>1225</v>
+      </c>
+      <c r="D374" s="7">
+        <v>700</v>
+      </c>
+      <c r="E374" s="15" t="s">
+        <v>1380</v>
+      </c>
+      <c r="F374" s="15" t="s">
+        <v>1379</v>
+      </c>
+      <c r="G374" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="H374" s="7" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="375" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A375" s="1" t="s">
+        <v>1383</v>
+      </c>
+      <c r="B375" s="1" t="s">
+        <v>1384</v>
+      </c>
+      <c r="C375" s="7">
+        <v>535</v>
+      </c>
+      <c r="D375" s="7">
+        <v>400</v>
+      </c>
+      <c r="E375" s="15" t="s">
+        <v>1382</v>
+      </c>
+      <c r="F375" s="15" t="s">
+        <v>1381</v>
+      </c>
+      <c r="G375" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="H375" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="376" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A376" s="1" t="s">
+        <v>1385</v>
+      </c>
+      <c r="B376" s="1" t="s">
+        <v>1386</v>
+      </c>
+      <c r="C376" s="7">
+        <v>1033</v>
+      </c>
+      <c r="D376" s="7">
+        <v>675</v>
+      </c>
+      <c r="E376" s="15" t="s">
+        <v>1388</v>
+      </c>
+      <c r="F376" s="15" t="s">
+        <v>1387</v>
+      </c>
+      <c r="G376" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="H376" s="7" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="377" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A377" s="1" t="s">
+        <v>1389</v>
+      </c>
+      <c r="B377" s="1" t="s">
+        <v>1386</v>
+      </c>
+      <c r="C377" s="7">
+        <v>614</v>
+      </c>
+      <c r="D377" s="7">
+        <v>375</v>
+      </c>
+      <c r="E377" s="15" t="s">
+        <v>1391</v>
+      </c>
+      <c r="F377" s="15" t="s">
+        <v>1390</v>
+      </c>
+      <c r="G377" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="H377" s="7" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="378" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A378" s="1" t="s">
+        <v>1392</v>
+      </c>
+      <c r="B378" s="1" t="s">
+        <v>1386</v>
+      </c>
+      <c r="C378" s="7">
+        <v>946</v>
+      </c>
+      <c r="D378" s="7">
+        <v>575</v>
+      </c>
+      <c r="E378" s="15" t="s">
+        <v>1394</v>
+      </c>
+      <c r="F378" s="15" t="s">
+        <v>1393</v>
+      </c>
+      <c r="G378" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="H378" s="7" t="s">
+        <v>535</v>
       </c>
     </row>
   </sheetData>
@@ -14521,11 +14934,33 @@
     <hyperlink ref="E263" r:id="rId7"/>
     <hyperlink ref="E343" r:id="rId8"/>
     <hyperlink ref="E157" r:id="rId9"/>
+    <hyperlink ref="E368" r:id="rId10"/>
+    <hyperlink ref="F368" r:id="rId11" location="&amp;gid=1&amp;pid=1"/>
+    <hyperlink ref="F369" r:id="rId12" location="&amp;gid=1&amp;pid=1"/>
+    <hyperlink ref="E369" r:id="rId13"/>
+    <hyperlink ref="F370" r:id="rId14" location="&amp;gid=1&amp;pid=1"/>
+    <hyperlink ref="E370" r:id="rId15"/>
+    <hyperlink ref="F371" r:id="rId16" location="&amp;gid=1&amp;pid=1"/>
+    <hyperlink ref="E371" r:id="rId17"/>
+    <hyperlink ref="F372" r:id="rId18"/>
+    <hyperlink ref="E372" r:id="rId19"/>
+    <hyperlink ref="F373" r:id="rId20"/>
+    <hyperlink ref="E373" r:id="rId21"/>
+    <hyperlink ref="F374"/>
+    <hyperlink ref="E374" r:id="rId22"/>
+    <hyperlink ref="F375" r:id="rId23"/>
+    <hyperlink ref="E375" r:id="rId24"/>
+    <hyperlink ref="F376" r:id="rId25"/>
+    <hyperlink ref="E376" r:id="rId26"/>
+    <hyperlink ref="F377" r:id="rId27"/>
+    <hyperlink ref="E377" r:id="rId28"/>
+    <hyperlink ref="F378" r:id="rId29"/>
+    <hyperlink ref="E378" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId10"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId31"/>
   <tableParts count="1">
-    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId32"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualiza proyecto (2 modificados, 1 nuevo): productos.xlsx, index.html, D_NQ_NP_2X_715614-MLA103111958883_122025-F.webp
</commit_message>
<xml_diff>
--- a/datos/productos.xlsx
+++ b/datos/productos.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2533" uniqueCount="1430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2539" uniqueCount="1434">
   <si>
     <t>Nombre</t>
   </si>
@@ -4325,6 +4325,19 @@
   </si>
   <si>
     <t>Dimensiones: 21.5 cm x 24.5 cm x 27.5 cm</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/triciclo-electrico-para-ninos-ykioea-de-drift-con-control-remoto-bluetooth-y-3-velocidades/p/MLM63671276</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_715614-MLA103111958883_122025-F.webp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Velocidad máxima: 20 km/h, Peso máximo soportado. 85 kg
+</t>
+  </si>
+  <si>
+    <t>Triciclo Eléctrico para Niños, Adolescentes y Adultos de Drift con Control Remoto, Bluetooth y 3 Velocidades</t>
   </si>
 </sst>
 </file>
@@ -4498,8 +4511,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H386" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A1:H386"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H387" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A1:H387"/>
   <sortState ref="A2:H342">
     <sortCondition ref="A1:A342"/>
   </sortState>
@@ -4802,7 +4815,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I386"/>
+  <dimension ref="A1:I387"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="70" style="1" customWidth="1"/>
@@ -15235,6 +15248,32 @@
       </c>
       <c r="H386" s="7" t="s">
         <v>211</v>
+      </c>
+    </row>
+    <row r="387" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A387" s="1" t="s">
+        <v>1433</v>
+      </c>
+      <c r="B387" s="1" t="s">
+        <v>1432</v>
+      </c>
+      <c r="C387" s="7">
+        <v>4699</v>
+      </c>
+      <c r="D387" s="7">
+        <v>2832</v>
+      </c>
+      <c r="E387" s="15" t="s">
+        <v>1431</v>
+      </c>
+      <c r="F387" s="15" t="s">
+        <v>1430</v>
+      </c>
+      <c r="G387" s="7" t="s">
+        <v>892</v>
+      </c>
+      <c r="H387" s="7" t="s">
+        <v>531</v>
       </c>
     </row>
   </sheetData>
@@ -15292,11 +15331,13 @@
     <hyperlink ref="E385" r:id="rId50" display="https://http2.mlstatic.com/D_NQ_NP_2X_984373-MLA112451559563_052026-F.webp"/>
     <hyperlink ref="F386" r:id="rId51"/>
     <hyperlink ref="E386" r:id="rId52"/>
+    <hyperlink ref="F387" r:id="rId53"/>
+    <hyperlink ref="E387" r:id="rId54"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId53"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId55"/>
   <tableParts count="1">
-    <tablePart r:id="rId54"/>
+    <tablePart r:id="rId56"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualiza proyecto (2 modificados, 1 nuevo): productos.xlsx, index.html, ~$productos.xlsx
</commit_message>
<xml_diff>
--- a/datos/productos.xlsx
+++ b/datos/productos.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2539" uniqueCount="1434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2547" uniqueCount="1438">
   <si>
     <t>Nombre</t>
   </si>
@@ -4338,6 +4338,18 @@
   </si>
   <si>
     <t>Triciclo Eléctrico para Niños, Adolescentes y Adultos de Drift con Control Remoto, Bluetooth y 3 Velocidades</t>
+  </si>
+  <si>
+    <t>Batidora De Inmersión Trituradora Electrodomesticos</t>
+  </si>
+  <si>
+    <t>De 1000w</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-5261364026-batidora-de-inmersion-trituradora-de-1000w-electrodomesticos-_JM?quantity=1&amp;sid=purchases</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_816888-CBT110109284844_042026-F-batidora-de-inmersion-trituradora-de-1000w-electrodomesticos.webp</t>
   </si>
 </sst>
 </file>
@@ -4382,7 +4394,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4404,6 +4416,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4432,7 +4450,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4461,6 +4479,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -4511,8 +4530,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H387" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A1:H387"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H388" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A1:H388"/>
   <sortState ref="A2:H342">
     <sortCondition ref="A1:A342"/>
   </sortState>
@@ -4815,7 +4834,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I387"/>
+  <dimension ref="A1:I388"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="70" style="1" customWidth="1"/>
@@ -4866,7 +4885,7 @@
         <v>350</v>
       </c>
       <c r="D2" s="7">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>1055</v>
@@ -6120,7 +6139,7 @@
         <v>399</v>
       </c>
       <c r="D48" s="7">
-        <v>320</v>
+        <v>300</v>
       </c>
       <c r="E48" s="7" t="s">
         <v>471</v>
@@ -6805,10 +6824,10 @@
         <v>865</v>
       </c>
       <c r="C73" s="7">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="D73" s="7">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="E73" s="7" t="s">
         <v>898</v>
@@ -8608,7 +8627,7 @@
         <v>1069</v>
       </c>
       <c r="C140" s="7">
-        <v>398</v>
+        <v>599</v>
       </c>
       <c r="D140" s="7">
         <v>300</v>
@@ -9103,6 +9122,9 @@
       <c r="C158" s="7">
         <v>350</v>
       </c>
+      <c r="D158" s="7">
+        <v>300</v>
+      </c>
       <c r="E158" s="7" t="s">
         <v>481</v>
       </c>
@@ -9110,12 +9132,14 @@
         <v>482</v>
       </c>
       <c r="G158" s="7" t="s">
-        <v>438</v>
+        <v>1326</v>
       </c>
       <c r="H158" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I158" s="9"/>
+      <c r="I158" s="16" t="s">
+        <v>892</v>
+      </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
@@ -9958,7 +9982,7 @@
         <v>347</v>
       </c>
       <c r="D190" s="7">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="E190" s="7" t="s">
         <v>191</v>
@@ -9987,7 +10011,7 @@
         <v>498</v>
       </c>
       <c r="D191" s="7">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="E191" s="7" t="s">
         <v>194</v>
@@ -10302,7 +10326,7 @@
         <v>398</v>
       </c>
       <c r="D203" s="7">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="E203" s="7" t="s">
         <v>201</v>
@@ -12506,10 +12530,10 @@
         <v>367</v>
       </c>
       <c r="C282" s="7">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D282" s="7">
-        <v>250</v>
+        <v>220</v>
       </c>
       <c r="E282" s="7" t="s">
         <v>893</v>
@@ -13170,7 +13194,7 @@
         <v>350</v>
       </c>
       <c r="D306" s="7">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="E306" s="7" t="s">
         <v>1096</v>
@@ -13196,10 +13220,10 @@
         <v>1193</v>
       </c>
       <c r="C307" s="7">
-        <v>250</v>
+        <v>220</v>
       </c>
       <c r="D307" s="7">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="E307" s="7" t="s">
         <v>1098</v>
@@ -14111,7 +14135,7 @@
         <v>850</v>
       </c>
       <c r="D343" s="7">
-        <v>550</v>
+        <v>500</v>
       </c>
       <c r="E343" s="7" t="s">
         <v>1236</v>
@@ -14434,7 +14458,7 @@
         <v>399</v>
       </c>
       <c r="D356" s="7">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="E356" s="7" t="s">
         <v>1284</v>
@@ -15198,7 +15222,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="385" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A385" s="1" t="s">
         <v>1423</v>
       </c>
@@ -15224,7 +15248,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="386" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A386" s="1" t="s">
         <v>1428</v>
       </c>
@@ -15250,7 +15274,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="387" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A387" s="1" t="s">
         <v>1433</v>
       </c>
@@ -15274,6 +15298,35 @@
       </c>
       <c r="H387" s="7" t="s">
         <v>531</v>
+      </c>
+    </row>
+    <row r="388" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A388" s="1" t="s">
+        <v>1434</v>
+      </c>
+      <c r="B388" s="1" t="s">
+        <v>1435</v>
+      </c>
+      <c r="C388" s="7">
+        <v>349</v>
+      </c>
+      <c r="D388" s="7">
+        <v>295</v>
+      </c>
+      <c r="E388" s="15" t="s">
+        <v>1437</v>
+      </c>
+      <c r="F388" s="15" t="s">
+        <v>1436</v>
+      </c>
+      <c r="G388" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="H388" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="I388" s="14" t="s">
+        <v>892</v>
       </c>
     </row>
   </sheetData>
@@ -15333,11 +15386,13 @@
     <hyperlink ref="E386" r:id="rId52"/>
     <hyperlink ref="F387" r:id="rId53"/>
     <hyperlink ref="E387" r:id="rId54"/>
+    <hyperlink ref="F388" r:id="rId55"/>
+    <hyperlink ref="E388" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId55"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId57"/>
   <tableParts count="1">
-    <tablePart r:id="rId56"/>
+    <tablePart r:id="rId58"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualiza proyecto (2 modificados): productos.xlsx, index.html
</commit_message>
<xml_diff>
--- a/datos/productos.xlsx
+++ b/datos/productos.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2307" uniqueCount="1457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2325" uniqueCount="1475">
   <si>
     <t>Nombre</t>
   </si>
@@ -4407,6 +4407,60 @@
   </si>
   <si>
     <t>https://http2.mlstatic.com/D_NQ_NP_2X_870766-MLA111944165952_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_637261-MLA111944285568_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_835091-MLA112882459449_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_865807-MLA113706863262_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_881890-MLA115108214329_072026-F.webp</t>
+  </si>
+  <si>
+    <t>https://video-vod-clips.mms.mlstatic.com/v1/video/hls/cli_04xzu0y81ntclips/019f1a4ceb3b7612b8229efa46d49f6b/master.m3u8</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_650019-MLA112598239078_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_694102-MLA111420836191_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_960139-MLA111232526403_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_654633-MLA111232677355_052026-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_908039-MLA112874706206_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_922341-MLA112874942992_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_668896-MLA114078462461_072026-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_761866-MLA76203783381_052024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_967910-MLA76082310461_042024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_699850-MLA76082339489_042024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_688162-MLA77258607126_072024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_987664-MLA73443046442_122023-F.webp</t>
+  </si>
+  <si>
+    <t>https://video-static-clips.mms.mlstatic.com/62c82f1f923a3f082b72612d/019ec7172f297018bc87b285605c79fd/packaging/static/master.m3u8</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_937988-MLA100214376229_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_839463-MLA100214244569_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_878239-MLA100214347283_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_746732-MLA100214337393_122025-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_853469-MLA73479850047_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_636371-MLA72966055893_112023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_647337-MLA74448293715_022024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_843886-MLA73007265330_112023-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_838661-MLA114043475512_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_997422-MLA111845686244_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_946430-MLA112856485647_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_885165-MLA111740080984_062026-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_700050-MLA90330537717_082025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_810830-MLA92985348779_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_611435-MLA103169335415_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_770740-MLA102656875022_122025-F.webp</t>
+  </si>
+  <si>
+    <t>https://video-vod-clips.mms.mlstatic.com/v1/video/hls/cli_04xzu0y81ntclips/019fbae051fa719da9d306536dceb684/master.m3u8</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_972461-MLA108765590667_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_959062-MLA111287287492_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_702439-MLA108999676116_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_991088-MLA108999765964_032026-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_772336-MLA83215360667_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_641687-MLA82926894938_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_686941-MLA80851161221_112024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_788718-MLA101812695971_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_703043-MLA79489338416_102024-F.webp</t>
+  </si>
+  <si>
+    <t>https://video-vod-clips.mms.mlstatic.com/v1/video/hls/cli_04xzu0y81ntclips/019eedaef42876b0b4c1468e5ea4c162/master.m3u8</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_918751-MLA113089268495_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_972829-MLA114388137831_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_739083-MLA113884890489_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_823404-MLA110625955659_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_668792-MLA111243248596_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_665158-MLA114050953663_072026-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_622982-MLA91998379772_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_918567-MLA93316673763_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_951409-MLA93316693351_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_873847-MLA99429346773_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_754609-MLA92520544449_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_981089-MLA107665597095_022026-F.webp</t>
+  </si>
+  <si>
+    <t>https://video-vod-clips.mms.mlstatic.com/v1/video/hls/cli_04xzu0y81ntclips/019f7cd765587bb9b171a45689bab017/master.m3u8</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_860421-MLA111296936608_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_731074-MLA113783205421_062026-F.webp</t>
+  </si>
+  <si>
+    <t>https://video-static-clips.mms.mlstatic.com/62c82f1f923a3f082b72612d/019ed9394d7a72dc8adc7f349c65987a/packaging/static/master.m3u8</t>
   </si>
 </sst>
 </file>
@@ -4569,7 +4623,7 @@
   <autoFilter ref="A1:J388">
     <filterColumn colId="0">
       <filters>
-        <filter val="Bebedero Para mascotas 4.5L, Fuente de Agua Dispensador Automático Silencioso"/>
+        <filter val="Epicentro Max-02 Restaurador De Bajos Para Auto, Ecualizador para sistema de audio_x000a_"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -5300,7 +5354,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>856</v>
       </c>
@@ -5323,7 +5377,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>763</v>
       </c>
@@ -5349,7 +5403,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>578</v>
       </c>
@@ -5372,7 +5426,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>789</v>
       </c>
@@ -5395,7 +5449,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>765</v>
       </c>
@@ -5421,7 +5475,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>533</v>
       </c>
@@ -5444,7 +5498,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>533</v>
       </c>
@@ -5467,7 +5521,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>533</v>
       </c>
@@ -5490,7 +5544,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>495</v>
       </c>
@@ -5516,7 +5570,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>111</v>
       </c>
@@ -5542,7 +5596,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>850</v>
       </c>
@@ -5568,7 +5622,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>839</v>
       </c>
@@ -5594,7 +5648,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>114</v>
       </c>
@@ -5617,7 +5671,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>840</v>
       </c>
@@ -5643,7 +5697,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>849</v>
       </c>
@@ -5669,7 +5723,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>841</v>
       </c>
@@ -5693,6 +5747,12 @@
       </c>
       <c r="H32" s="7" t="s">
         <v>100</v>
+      </c>
+      <c r="I32" s="12" t="s">
+        <v>1462</v>
+      </c>
+      <c r="J32" s="12" t="s">
+        <v>1461</v>
       </c>
     </row>
     <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
@@ -6084,7 +6144,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>203</v>
       </c>
@@ -6110,7 +6170,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>337</v>
       </c>
@@ -6136,7 +6196,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>188</v>
       </c>
@@ -6159,7 +6219,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>808</v>
       </c>
@@ -6185,7 +6245,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>807</v>
       </c>
@@ -6211,7 +6271,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>457</v>
       </c>
@@ -6237,7 +6297,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>221</v>
       </c>
@@ -6263,7 +6323,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>813</v>
       </c>
@@ -6289,7 +6349,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>899</v>
       </c>
@@ -6315,7 +6375,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>1328</v>
       </c>
@@ -6341,7 +6401,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>978</v>
       </c>
@@ -6364,7 +6424,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>796</v>
       </c>
@@ -6387,7 +6447,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>1063</v>
       </c>
@@ -6412,8 +6472,14 @@
       <c r="H61" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I61" s="12" t="s">
+        <v>1458</v>
+      </c>
+      <c r="J61" s="12" t="s">
+        <v>1457</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>340</v>
       </c>
@@ -6436,7 +6502,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>974</v>
       </c>
@@ -6459,7 +6525,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>853</v>
       </c>
@@ -7296,7 +7362,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>646</v>
       </c>
@@ -7322,7 +7388,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="98" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>646</v>
       </c>
@@ -7345,7 +7411,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>308</v>
       </c>
@@ -7371,7 +7437,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>208</v>
       </c>
@@ -7397,7 +7463,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>243</v>
       </c>
@@ -7423,7 +7489,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="102" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>173</v>
       </c>
@@ -7449,7 +7515,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="103" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>176</v>
       </c>
@@ -7472,7 +7538,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>329</v>
       </c>
@@ -7497,8 +7563,11 @@
       <c r="H104" s="7" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I104" s="12" t="s">
+        <v>1463</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>464</v>
       </c>
@@ -7521,7 +7590,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>918</v>
       </c>
@@ -7547,7 +7616,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>212</v>
       </c>
@@ -7573,7 +7642,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>1003</v>
       </c>
@@ -7599,7 +7668,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>347</v>
       </c>
@@ -7625,7 +7694,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>1004</v>
       </c>
@@ -7651,7 +7720,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>1073</v>
       </c>
@@ -7677,7 +7746,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>28</v>
       </c>
@@ -8490,7 +8559,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>486</v>
       </c>
@@ -8513,7 +8582,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>482</v>
       </c>
@@ -8536,7 +8605,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>255</v>
       </c>
@@ -8562,7 +8631,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>97</v>
       </c>
@@ -8585,7 +8654,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>33</v>
       </c>
@@ -8610,8 +8679,11 @@
       <c r="H149" s="7" t="s">
         <v>531</v>
       </c>
-    </row>
-    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I149" s="12" t="s">
+        <v>1465</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>36</v>
       </c>
@@ -8637,7 +8709,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>40</v>
       </c>
@@ -8663,7 +8735,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>164</v>
       </c>
@@ -8689,7 +8761,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>167</v>
       </c>
@@ -8715,7 +8787,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>170</v>
       </c>
@@ -8741,7 +8813,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>613</v>
       </c>
@@ -8767,7 +8839,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>391</v>
       </c>
@@ -8793,7 +8865,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>642</v>
       </c>
@@ -8819,7 +8891,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>478</v>
       </c>
@@ -8845,7 +8917,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>351</v>
       </c>
@@ -8868,7 +8940,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>871</v>
       </c>
@@ -10480,7 +10552,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="225" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>670</v>
       </c>
@@ -10506,7 +10578,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="226" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>723</v>
       </c>
@@ -10532,7 +10604,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="227" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>1027</v>
       </c>
@@ -10558,7 +10630,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="228" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>884</v>
       </c>
@@ -10584,7 +10656,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="229" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>863</v>
       </c>
@@ -10610,7 +10682,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="230" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>57</v>
       </c>
@@ -10636,7 +10708,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="231" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>395</v>
       </c>
@@ -10659,7 +10731,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="232" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>298</v>
       </c>
@@ -10685,7 +10757,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="233" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>311</v>
       </c>
@@ -10710,8 +10782,11 @@
       <c r="H233" s="7" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="234" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I233" s="12" t="s">
+        <v>1460</v>
+      </c>
+    </row>
+    <row r="234" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A234" s="1" t="s">
         <v>74</v>
       </c>
@@ -10737,7 +10812,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="235" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A235" s="1" t="s">
         <v>671</v>
       </c>
@@ -10763,7 +10838,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="236" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A236" s="1" t="s">
         <v>793</v>
       </c>
@@ -10789,7 +10864,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="237" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A237" s="1" t="s">
         <v>1316</v>
       </c>
@@ -10815,7 +10890,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="238" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A238" s="1" t="s">
         <v>1028</v>
       </c>
@@ -10841,7 +10916,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="239" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A239" s="1" t="s">
         <v>1031</v>
       </c>
@@ -10867,7 +10942,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="240" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
         <v>672</v>
       </c>
@@ -10893,7 +10968,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="241" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
         <v>321</v>
       </c>
@@ -10919,7 +10994,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="242" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>360</v>
       </c>
@@ -10942,7 +11017,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="243" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>235</v>
       </c>
@@ -10968,7 +11043,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="244" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>820</v>
       </c>
@@ -10991,7 +11066,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="245" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
         <v>272</v>
       </c>
@@ -11017,7 +11092,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="246" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
         <v>1018</v>
       </c>
@@ -11040,7 +11115,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="247" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>450</v>
       </c>
@@ -11063,7 +11138,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="248" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>542</v>
       </c>
@@ -11086,7 +11161,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="249" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>656</v>
       </c>
@@ -11112,7 +11187,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="250" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
         <v>259</v>
       </c>
@@ -11135,7 +11210,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="251" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
         <v>135</v>
       </c>
@@ -11161,7 +11236,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="252" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
         <v>138</v>
       </c>
@@ -11186,8 +11261,11 @@
       <c r="H252" s="7" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="253" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I252" s="12" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="253" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
         <v>141</v>
       </c>
@@ -11213,7 +11291,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="254" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
         <v>720</v>
       </c>
@@ -11239,7 +11317,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="255" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
         <v>399</v>
       </c>
@@ -11265,7 +11343,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="256" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
         <v>913</v>
       </c>
@@ -13677,7 +13755,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="353" spans="1:8" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:10" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A353" s="1" t="s">
         <v>1270</v>
       </c>
@@ -13699,8 +13777,14 @@
       <c r="H353" s="7" t="s">
         <v>530</v>
       </c>
-    </row>
-    <row r="354" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I353" s="12" t="s">
+        <v>1467</v>
+      </c>
+      <c r="J353" s="12" t="s">
+        <v>1466</v>
+      </c>
+    </row>
+    <row r="354" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A354" s="1" t="s">
         <v>1276</v>
       </c>
@@ -13723,7 +13807,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="355" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A355" s="1" t="s">
         <v>1326</v>
       </c>
@@ -13749,7 +13833,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="356" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A356" s="1" t="s">
         <v>1327</v>
       </c>
@@ -13775,7 +13859,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="357" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A357" s="1" t="s">
         <v>1292</v>
       </c>
@@ -13801,7 +13885,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="358" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A358" s="1" t="s">
         <v>1295</v>
       </c>
@@ -13827,7 +13911,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="359" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A359" s="1" t="s">
         <v>1300</v>
       </c>
@@ -13853,7 +13937,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="360" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A360" s="1" t="s">
         <v>1303</v>
       </c>
@@ -13879,7 +13963,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="361" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A361" s="1" t="s">
         <v>1308</v>
       </c>
@@ -13905,7 +13989,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="362" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A362" s="1" t="s">
         <v>1313</v>
       </c>
@@ -13925,7 +14009,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="363" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A363" s="1" t="s">
         <v>1321</v>
       </c>
@@ -13951,7 +14035,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="364" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
         <v>1331</v>
       </c>
@@ -13977,7 +14061,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="365" spans="1:8" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:10" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
         <v>1342</v>
       </c>
@@ -14003,7 +14087,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="366" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A366" s="1" t="s">
         <v>1345</v>
       </c>
@@ -14029,7 +14113,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="367" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A367" s="1" t="s">
         <v>1349</v>
       </c>
@@ -14055,7 +14139,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="368" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A368" s="1" t="s">
         <v>1353</v>
       </c>
@@ -14081,7 +14165,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="369" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A369" s="1" t="s">
         <v>1359</v>
       </c>
@@ -14107,7 +14191,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="370" spans="1:8" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:10" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A370" s="1" t="s">
         <v>1378</v>
       </c>
@@ -14132,8 +14216,14 @@
       <c r="H370" s="7" t="s">
         <v>531</v>
       </c>
-    </row>
-    <row r="371" spans="1:8" ht="87" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I370" s="12" t="s">
+        <v>1471</v>
+      </c>
+      <c r="J370" s="12" t="s">
+        <v>1472</v>
+      </c>
+    </row>
+    <row r="371" spans="1:10" ht="87" x14ac:dyDescent="0.35">
       <c r="A371" s="1" t="s">
         <v>1377</v>
       </c>
@@ -14158,8 +14248,14 @@
       <c r="H371" s="7" t="s">
         <v>531</v>
       </c>
-    </row>
-    <row r="372" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I371" s="12" t="s">
+        <v>1473</v>
+      </c>
+      <c r="J371" s="12" t="s">
+        <v>1474</v>
+      </c>
+    </row>
+    <row r="372" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A372" s="1" t="s">
         <v>1367</v>
       </c>
@@ -14185,7 +14281,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="373" spans="1:8" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:10" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A373" s="1" t="s">
         <v>1383</v>
       </c>
@@ -14211,7 +14307,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="374" spans="1:8" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:10" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A374" s="1" t="s">
         <v>1385</v>
       </c>
@@ -14237,7 +14333,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="375" spans="1:8" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:10" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A375" s="1" t="s">
         <v>1387</v>
       </c>
@@ -14263,7 +14359,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="376" spans="1:8" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:10" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A376" s="1" t="s">
         <v>1379</v>
       </c>
@@ -14288,8 +14384,14 @@
       <c r="H376" s="7" t="s">
         <v>531</v>
       </c>
-    </row>
-    <row r="377" spans="1:8" ht="58" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I376" s="12" t="s">
+        <v>1470</v>
+      </c>
+      <c r="J376" s="12" t="s">
+        <v>1469</v>
+      </c>
+    </row>
+    <row r="377" spans="1:10" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A377" s="1" t="s">
         <v>1389</v>
       </c>
@@ -14314,8 +14416,11 @@
       <c r="H377" s="7" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="378" spans="1:8" ht="58" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I377" s="12" t="s">
+        <v>1459</v>
+      </c>
+    </row>
+    <row r="378" spans="1:10" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A378" s="1" t="s">
         <v>1393</v>
       </c>
@@ -14341,7 +14446,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="379" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A379" s="1" t="s">
         <v>1397</v>
       </c>
@@ -14367,7 +14472,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="380" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A380" s="1" t="s">
         <v>1401</v>
       </c>
@@ -14393,7 +14498,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="381" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A381" s="1" t="s">
         <v>1405</v>
       </c>
@@ -14419,7 +14524,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="382" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A382" s="1" t="s">
         <v>1409</v>
       </c>
@@ -14445,7 +14550,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="383" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A383" s="1" t="s">
         <v>1413</v>
       </c>
@@ -14471,7 +14576,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="384" spans="1:8" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:10" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A384" s="1" t="s">
         <v>1419</v>
       </c>
@@ -14497,7 +14602,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="385" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A385" s="1" t="s">
         <v>1422</v>
       </c>
@@ -14550,6 +14655,9 @@
       </c>
       <c r="H386" s="7" t="s">
         <v>211</v>
+      </c>
+      <c r="I386" s="12" t="s">
+        <v>1464</v>
       </c>
     </row>
     <row r="387" spans="1:10" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
@@ -14687,11 +14795,29 @@
     <hyperlink ref="J258" r:id="rId64"/>
     <hyperlink ref="I36" r:id="rId65"/>
     <hyperlink ref="I385"/>
+    <hyperlink ref="J61" r:id="rId66"/>
+    <hyperlink ref="I61"/>
+    <hyperlink ref="I377" r:id="rId67"/>
+    <hyperlink ref="I233"/>
+    <hyperlink ref="J32" r:id="rId68"/>
+    <hyperlink ref="I32"/>
+    <hyperlink ref="I104"/>
+    <hyperlink ref="I386"/>
+    <hyperlink ref="I149"/>
+    <hyperlink ref="J353" r:id="rId69"/>
+    <hyperlink ref="I353"/>
+    <hyperlink ref="I252"/>
+    <hyperlink ref="J376" r:id="rId70"/>
+    <hyperlink ref="I376"/>
+    <hyperlink ref="J370" r:id="rId71"/>
+    <hyperlink ref="I370"/>
+    <hyperlink ref="I371" r:id="rId72"/>
+    <hyperlink ref="J371" r:id="rId73"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId66"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId74"/>
   <tableParts count="1">
-    <tablePart r:id="rId67"/>
+    <tablePart r:id="rId75"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualiza proyecto (2 modificados, 1 eliminado): productos.xlsx, ~$productos.xlsx, index.html
</commit_message>
<xml_diff>
--- a/datos/productos.xlsx
+++ b/datos/productos.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2325" uniqueCount="1475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2331" uniqueCount="1483">
   <si>
     <t>Nombre</t>
   </si>
@@ -4054,18 +4054,6 @@
     <t>https://panchochacharas.netlify.app/imagenes/4aaa7507c541c0dc0aac5e2393fb2c31.jpeg</t>
   </si>
   <si>
-    <t>Aluminio Negro con Mango de Madera, Set de 3 Unidades (24 y 28 cm)</t>
-  </si>
-  <si>
-    <t>Pack de Sartenes Antiadherentes</t>
-  </si>
-  <si>
-    <t>https://http2.mlstatic.com/D_NQ_NP_2X_718669-MLA109014019546_032026-F.webp</t>
-  </si>
-  <si>
-    <t>https://www.mercadolibre.com.mx/pack-de-sartenes-antiadherentes-xinest-de-aluminio-negro-con-mango-de-madera-set-de-3-unidades-24-y-28-cm/p/MLM67441876?pdp_filters=item_id%3AMLM5595517674#&amp;gid=1&amp;pid=1</t>
-  </si>
-  <si>
     <t>Pistola Para Pintar Eléctrica</t>
   </si>
   <si>
@@ -4391,9 +4379,6 @@
     <t>https://http2.mlstatic.com/D_NQ_NP_2X_704682-MLA112632086794_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_648062-MLA114215908179_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_721338-MLA112631444306_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_666014-MLA110019279904_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_747141-MLA110928994963_042026-F.webp</t>
   </si>
   <si>
-    <t>https://http2.mlstatic.com/D_NQ_NP_2X_885715-MLA103257094455_122025-F.webp;</t>
-  </si>
-  <si>
     <t>https://http2.mlstatic.com/D_NQ_NP_2X_679078-MLA106513626675_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_867289-MLA106513332881_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_837213-MLA106512862341_022026-F.webp</t>
   </si>
   <si>
@@ -4403,9 +4388,6 @@
     <t>https://http2.mlstatic.com/D_NQ_NP_2X_877039-MLA114231711531_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_669195-MLA111691242302_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_694108-MLA111868098195_052026-F.webp</t>
   </si>
   <si>
-    <t xml:space="preserve">https://http2.mlstatic.com/D_NQ_NP_2X_984373-MLA112451559563_052026-F.webp; </t>
-  </si>
-  <si>
     <t>https://http2.mlstatic.com/D_NQ_NP_2X_870766-MLA111944165952_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_637261-MLA111944285568_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_835091-MLA112882459449_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_865807-MLA113706863262_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_881890-MLA115108214329_072026-F.webp</t>
   </si>
   <si>
@@ -4461,6 +4443,48 @@
   </si>
   <si>
     <t>https://video-static-clips.mms.mlstatic.com/62c82f1f923a3f082b72612d/019ed9394d7a72dc8adc7f349c65987a/packaging/static/master.m3u8</t>
+  </si>
+  <si>
+    <t>https://video-vod-clips.mms.mlstatic.com/v1/video/hls/cli_04xzu0y81ntclips/019f6363325b7280806cc57c579f2933/master.m3u8</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_630634-MLA83929492736_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_826427-MLA83875691856_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_778506-MLA83875632066_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_734315-MLA83875642068_042025-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_601798-MLA74779553000_032024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_784677-MLA71729912500_092023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_982997-MLA73375012815_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_982999-MLA70028199790_062023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_830261-MLA70048397883_062023-F.webp</t>
+  </si>
+  <si>
+    <t>https://video-vod-clips.mms.mlstatic.com/v1/video/hls/cli_04xzu0y81ntclips/019f29451c3876a8969ca32011081a6b/master.m3u8</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_743943-MLA113720575198_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_652343-MLA98742656086_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_688496-MLA89833143459_082025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_980015-MLA111245266119_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_676086-MLA108251244515_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_743943-MLA113720575198_072026-F.webp</t>
+  </si>
+  <si>
+    <t>https://video-vod-clips.mms.mlstatic.com/v1/video/hls/cli_04xzu0y81ntclips/019eec50ebdc7581aaf884c109615b29/master.m3u8</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_842998-MLA109635418200_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_655182-MLA88058609951_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_931498-MLA73993836353_012024-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_892154-MLA114436130385_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_641144-MLA114436417313_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_829930-MLA114436306203_072026-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_726152-MLA113045385176_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_848969-MLA113204126664_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_715603-MLA113204126666_072026-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_854442-MLA81845510730_012025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_966885-MLA81845471952_012025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_982348-MLA81845471950_012025-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_933354-MLA113160110934_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_644822-MLA114391216509_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_679253-MLA114391531429_072026-F.webp</t>
+  </si>
+  <si>
+    <t>https://video-vod-clips.mms.mlstatic.com/v1/video/hls/cli_04xzu0y81ntclips/019f9f72c531799fa159fcfdf4ceaee9/master.m3u8</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_885715-MLA103257094455_122025-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_984373-MLA112451559563_052026-F.webp</t>
   </si>
 </sst>
 </file>
@@ -4619,14 +4643,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:J388" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J388">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Epicentro Max-02 Restaurador De Bajos Para Auto, Ecualizador para sistema de audio_x000a_"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:J387" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J387"/>
   <sortState ref="A2:H342">
     <sortCondition ref="A1:A342"/>
   </sortState>
@@ -4931,7 +4949,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J388"/>
+  <dimension ref="A1:J387"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="70" style="1" customWidth="1"/>
@@ -4971,13 +4989,13 @@
         <v>7</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>1436</v>
+        <v>1432</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>1437</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+        <v>1433</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>1082</v>
       </c>
@@ -5005,7 +5023,7 @@
       <c r="I2" s="12"/>
       <c r="J2" s="12"/>
     </row>
-    <row r="3" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1084</v>
       </c>
@@ -5031,7 +5049,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>588</v>
       </c>
@@ -5054,7 +5072,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>155</v>
       </c>
@@ -5080,7 +5098,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>406</v>
       </c>
@@ -5103,7 +5121,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>862</v>
       </c>
@@ -5129,7 +5147,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>104</v>
       </c>
@@ -5155,7 +5173,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>693</v>
       </c>
@@ -5181,7 +5199,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>861</v>
       </c>
@@ -5207,7 +5225,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>238</v>
       </c>
@@ -5233,7 +5251,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>750</v>
       </c>
@@ -5259,7 +5277,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>971</v>
       </c>
@@ -5282,7 +5300,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>632</v>
       </c>
@@ -5308,7 +5326,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>992</v>
       </c>
@@ -5331,7 +5349,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>109</v>
       </c>
@@ -5354,7 +5372,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>856</v>
       </c>
@@ -5377,7 +5395,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>763</v>
       </c>
@@ -5403,7 +5421,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>578</v>
       </c>
@@ -5426,7 +5444,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>789</v>
       </c>
@@ -5449,7 +5467,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>765</v>
       </c>
@@ -5475,7 +5493,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>533</v>
       </c>
@@ -5498,7 +5516,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>533</v>
       </c>
@@ -5521,7 +5539,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>533</v>
       </c>
@@ -5544,7 +5562,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>495</v>
       </c>
@@ -5570,7 +5588,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>111</v>
       </c>
@@ -5596,7 +5614,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>850</v>
       </c>
@@ -5622,7 +5640,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>839</v>
       </c>
@@ -5648,7 +5666,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>114</v>
       </c>
@@ -5671,7 +5689,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>840</v>
       </c>
@@ -5697,7 +5715,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>849</v>
       </c>
@@ -5723,7 +5741,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>841</v>
       </c>
@@ -5749,13 +5767,13 @@
         <v>100</v>
       </c>
       <c r="I32" s="12" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="J32" s="12" t="s">
-        <v>1461</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+        <v>1455</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>844</v>
       </c>
@@ -5781,7 +5799,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>842</v>
       </c>
@@ -5807,7 +5825,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>843</v>
       </c>
@@ -5830,7 +5848,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>1061</v>
       </c>
@@ -5856,10 +5874,10 @@
         <v>66</v>
       </c>
       <c r="I36" s="12" t="s">
-        <v>1454</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+        <v>1449</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>1329</v>
       </c>
@@ -5885,7 +5903,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>1000</v>
       </c>
@@ -5908,7 +5926,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>598</v>
       </c>
@@ -5931,7 +5949,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>922</v>
       </c>
@@ -5957,7 +5975,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>77</v>
       </c>
@@ -5977,7 +5995,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>186</v>
       </c>
@@ -6000,7 +6018,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>159</v>
       </c>
@@ -6026,7 +6044,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>929</v>
       </c>
@@ -6049,7 +6067,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>934</v>
       </c>
@@ -6072,7 +6090,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>930</v>
       </c>
@@ -6095,7 +6113,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>930</v>
       </c>
@@ -6118,7 +6136,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>468</v>
       </c>
@@ -6144,7 +6162,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>203</v>
       </c>
@@ -6170,7 +6188,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>337</v>
       </c>
@@ -6196,7 +6214,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>188</v>
       </c>
@@ -6219,7 +6237,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="52" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>808</v>
       </c>
@@ -6245,7 +6263,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>807</v>
       </c>
@@ -6271,7 +6289,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>457</v>
       </c>
@@ -6297,7 +6315,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="55" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>221</v>
       </c>
@@ -6323,7 +6341,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="56" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>813</v>
       </c>
@@ -6348,8 +6366,14 @@
       <c r="H56" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I56" s="12" t="s">
+        <v>1475</v>
+      </c>
+      <c r="J56" s="12" t="s">
+        <v>1474</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>899</v>
       </c>
@@ -6375,7 +6399,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>1328</v>
       </c>
@@ -6401,7 +6425,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>978</v>
       </c>
@@ -6424,7 +6448,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>796</v>
       </c>
@@ -6447,7 +6471,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>1063</v>
       </c>
@@ -6473,13 +6497,13 @@
         <v>12</v>
       </c>
       <c r="I61" s="12" t="s">
-        <v>1458</v>
+        <v>1452</v>
       </c>
       <c r="J61" s="12" t="s">
-        <v>1457</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+        <v>1451</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>340</v>
       </c>
@@ -6502,7 +6526,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>974</v>
       </c>
@@ -6525,7 +6549,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>853</v>
       </c>
@@ -6551,7 +6575,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>942</v>
       </c>
@@ -6577,7 +6601,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>944</v>
       </c>
@@ -6603,7 +6627,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>1077</v>
       </c>
@@ -6629,13 +6653,13 @@
         <v>100</v>
       </c>
       <c r="I67" s="12" t="s">
-        <v>1443</v>
+        <v>1439</v>
       </c>
       <c r="J67" s="12" t="s">
-        <v>1444</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>120</v>
       </c>
@@ -6661,10 +6685,10 @@
         <v>100</v>
       </c>
       <c r="I68" s="12" t="s">
-        <v>1445</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>746</v>
       </c>
@@ -6687,7 +6711,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>676</v>
       </c>
@@ -6713,7 +6737,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="71" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>344</v>
       </c>
@@ -6736,7 +6760,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="72" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>410</v>
       </c>
@@ -6762,7 +6786,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="73" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>895</v>
       </c>
@@ -6788,10 +6812,10 @@
         <v>66</v>
       </c>
       <c r="I73" s="12" t="s">
-        <v>1438</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+        <v>1434</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>379</v>
       </c>
@@ -6814,7 +6838,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="75" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>375</v>
       </c>
@@ -6837,7 +6861,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="76" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>413</v>
       </c>
@@ -6863,7 +6887,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="77" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>786</v>
       </c>
@@ -6889,7 +6913,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>774</v>
       </c>
@@ -6912,7 +6936,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="79" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>785</v>
       </c>
@@ -6935,7 +6959,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="80" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>1034</v>
       </c>
@@ -6961,7 +6985,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>771</v>
       </c>
@@ -6987,7 +7011,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>575</v>
       </c>
@@ -7010,7 +7034,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>569</v>
       </c>
@@ -7033,7 +7057,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>1040</v>
       </c>
@@ -7059,7 +7083,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>1048</v>
       </c>
@@ -7085,7 +7109,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>314</v>
       </c>
@@ -7111,7 +7135,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>601</v>
       </c>
@@ -7134,7 +7158,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>381</v>
       </c>
@@ -7160,7 +7184,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>1318</v>
       </c>
@@ -7186,7 +7210,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>906</v>
       </c>
@@ -7212,7 +7236,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="91" spans="1:8" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>651</v>
       </c>
@@ -7238,7 +7262,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>682</v>
       </c>
@@ -7264,7 +7288,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="93" spans="1:8" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>731</v>
       </c>
@@ -7287,7 +7311,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>231</v>
       </c>
@@ -7313,7 +7337,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>611</v>
       </c>
@@ -7339,7 +7363,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="96" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>648</v>
       </c>
@@ -7362,7 +7386,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>646</v>
       </c>
@@ -7388,7 +7412,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>646</v>
       </c>
@@ -7411,7 +7435,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>308</v>
       </c>
@@ -7437,7 +7461,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>208</v>
       </c>
@@ -7463,7 +7487,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>243</v>
       </c>
@@ -7489,7 +7513,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>173</v>
       </c>
@@ -7515,7 +7539,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>176</v>
       </c>
@@ -7538,7 +7562,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>329</v>
       </c>
@@ -7564,10 +7588,10 @@
         <v>66</v>
       </c>
       <c r="I104" s="12" t="s">
-        <v>1463</v>
-      </c>
-    </row>
-    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+        <v>1457</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>464</v>
       </c>
@@ -7590,7 +7614,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>918</v>
       </c>
@@ -7616,7 +7640,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>212</v>
       </c>
@@ -7642,7 +7666,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>1003</v>
       </c>
@@ -7668,7 +7692,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>347</v>
       </c>
@@ -7694,7 +7718,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>1004</v>
       </c>
@@ -7720,7 +7744,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>1073</v>
       </c>
@@ -7746,7 +7770,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>28</v>
       </c>
@@ -7769,7 +7793,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>30</v>
       </c>
@@ -7792,7 +7816,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>508</v>
       </c>
@@ -7815,7 +7839,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>524</v>
       </c>
@@ -7838,7 +7862,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>417</v>
       </c>
@@ -7864,7 +7888,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>875</v>
       </c>
@@ -7890,7 +7914,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>867</v>
       </c>
@@ -7916,7 +7940,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>421</v>
       </c>
@@ -7942,7 +7966,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>79</v>
       </c>
@@ -7968,7 +7992,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="121" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>700</v>
       </c>
@@ -7994,7 +8018,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="122" spans="1:8" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>734</v>
       </c>
@@ -8020,7 +8044,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="123" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>686</v>
       </c>
@@ -8046,7 +8070,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="124" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>708</v>
       </c>
@@ -8069,7 +8093,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>8</v>
       </c>
@@ -8095,7 +8119,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>512</v>
       </c>
@@ -8118,7 +8142,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>695</v>
       </c>
@@ -8141,7 +8165,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="128" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>565</v>
       </c>
@@ -8164,7 +8188,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="129" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>246</v>
       </c>
@@ -8187,7 +8211,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="130" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>249</v>
       </c>
@@ -8213,7 +8237,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="131" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>252</v>
       </c>
@@ -8239,7 +8263,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="132" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>384</v>
       </c>
@@ -8265,7 +8289,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>388</v>
       </c>
@@ -8291,7 +8315,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>82</v>
       </c>
@@ -8314,10 +8338,10 @@
         <v>530</v>
       </c>
       <c r="I134" s="12" t="s">
-        <v>1442</v>
-      </c>
-    </row>
-    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+        <v>1438</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>1024</v>
       </c>
@@ -8342,8 +8366,11 @@
       <c r="H135" s="7" t="s">
         <v>531</v>
       </c>
-    </row>
-    <row r="136" spans="1:9" ht="58" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I135" s="12" t="s">
+        <v>1478</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9" ht="58" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>989</v>
       </c>
@@ -8366,7 +8393,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>446</v>
       </c>
@@ -8392,7 +8419,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>85</v>
       </c>
@@ -8415,7 +8442,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>288</v>
       </c>
@@ -8441,7 +8468,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>1319</v>
       </c>
@@ -8467,7 +8494,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="141" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>88</v>
       </c>
@@ -8490,7 +8517,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="142" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>91</v>
       </c>
@@ -8513,7 +8540,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="143" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>94</v>
       </c>
@@ -8536,7 +8563,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>472</v>
       </c>
@@ -8559,7 +8586,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="145" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>486</v>
       </c>
@@ -8582,7 +8609,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="146" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>482</v>
       </c>
@@ -8605,7 +8632,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="147" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>255</v>
       </c>
@@ -8631,7 +8658,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="148" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>97</v>
       </c>
@@ -8654,7 +8681,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="149" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>33</v>
       </c>
@@ -8680,10 +8707,10 @@
         <v>531</v>
       </c>
       <c r="I149" s="12" t="s">
-        <v>1465</v>
-      </c>
-    </row>
-    <row r="150" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+        <v>1459</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>36</v>
       </c>
@@ -8709,7 +8736,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="151" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>40</v>
       </c>
@@ -8735,7 +8762,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="152" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>164</v>
       </c>
@@ -8761,7 +8788,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="153" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>167</v>
       </c>
@@ -8787,7 +8814,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="154" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>170</v>
       </c>
@@ -8813,7 +8840,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="155" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>613</v>
       </c>
@@ -8839,7 +8866,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="156" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>391</v>
       </c>
@@ -8865,7 +8892,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>642</v>
       </c>
@@ -8891,7 +8918,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>478</v>
       </c>
@@ -8917,7 +8944,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>351</v>
       </c>
@@ -8940,7 +8967,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>871</v>
       </c>
@@ -8966,7 +8993,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="161" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>607</v>
       </c>
@@ -8989,7 +9016,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="162" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>43</v>
       </c>
@@ -9012,7 +9039,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
         <v>714</v>
       </c>
@@ -9038,7 +9065,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="164" spans="1:8" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>712</v>
       </c>
@@ -9061,7 +9088,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="165" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>704</v>
       </c>
@@ -9084,7 +9111,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="166" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>291</v>
       </c>
@@ -9110,7 +9137,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>498</v>
       </c>
@@ -9133,7 +9160,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="168" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>304</v>
       </c>
@@ -9159,7 +9186,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="169" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
         <v>124</v>
       </c>
@@ -9182,7 +9209,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="170" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>1080</v>
       </c>
@@ -9205,7 +9232,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="171" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>67</v>
       </c>
@@ -9228,7 +9255,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="172" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>318</v>
       </c>
@@ -9254,7 +9281,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="173" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>71</v>
       </c>
@@ -9279,8 +9306,14 @@
       <c r="H173" s="7" t="s">
         <v>531</v>
       </c>
-    </row>
-    <row r="174" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I173" s="12" t="s">
+        <v>1470</v>
+      </c>
+      <c r="J173" s="12" t="s">
+        <v>1469</v>
+      </c>
+    </row>
+    <row r="174" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>760</v>
       </c>
@@ -9306,7 +9339,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>775</v>
       </c>
@@ -9329,7 +9362,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>504</v>
       </c>
@@ -9352,7 +9385,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>47</v>
       </c>
@@ -9375,7 +9408,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>50</v>
       </c>
@@ -9401,7 +9434,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="179" spans="1:8" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>639</v>
       </c>
@@ -9427,7 +9460,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>54</v>
       </c>
@@ -9453,7 +9486,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>557</v>
       </c>
@@ -9476,7 +9509,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>557</v>
       </c>
@@ -9499,7 +9532,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="183" spans="1:8" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>995</v>
       </c>
@@ -9522,7 +9555,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="184" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>1065</v>
       </c>
@@ -9548,7 +9581,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="185" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>955</v>
       </c>
@@ -9571,7 +9604,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="186" spans="1:8" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>742</v>
       </c>
@@ -9597,7 +9630,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="187" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>554</v>
       </c>
@@ -9620,7 +9653,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="188" spans="1:8" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>425</v>
       </c>
@@ -9646,7 +9679,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="189" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>836</v>
       </c>
@@ -9672,7 +9705,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="190" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>190</v>
       </c>
@@ -9698,7 +9731,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="191" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>193</v>
       </c>
@@ -9724,7 +9757,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="192" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>196</v>
       </c>
@@ -9750,7 +9783,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="193" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A193" s="1" t="s">
         <v>354</v>
       </c>
@@ -9773,7 +9806,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="194" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>939</v>
       </c>
@@ -9799,7 +9832,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="195" spans="1:9" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>227</v>
       </c>
@@ -9825,10 +9858,10 @@
         <v>100</v>
       </c>
       <c r="I195" s="12" t="s">
-        <v>1441</v>
-      </c>
-    </row>
-    <row r="196" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+        <v>1437</v>
+      </c>
+    </row>
+    <row r="196" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>577</v>
       </c>
@@ -9851,7 +9884,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="197" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>577</v>
       </c>
@@ -9874,7 +9907,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="198" spans="1:9" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>959</v>
       </c>
@@ -9897,7 +9930,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="199" spans="1:9" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>961</v>
       </c>
@@ -9920,7 +9953,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="200" spans="1:9" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>594</v>
       </c>
@@ -9943,7 +9976,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="201" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>269</v>
       </c>
@@ -9969,7 +10002,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="202" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>1009</v>
       </c>
@@ -9995,7 +10028,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="203" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A203" s="1" t="s">
         <v>199</v>
       </c>
@@ -10021,7 +10054,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>724</v>
       </c>
@@ -10044,7 +10077,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>17</v>
       </c>
@@ -10070,7 +10103,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="206" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>1047</v>
       </c>
@@ -10096,7 +10129,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>617</v>
       </c>
@@ -10122,7 +10155,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="208" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>737</v>
       </c>
@@ -10148,7 +10181,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="209" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>621</v>
       </c>
@@ -10174,7 +10207,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>780</v>
       </c>
@@ -10197,7 +10230,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
         <v>21</v>
       </c>
@@ -10223,7 +10256,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A212" s="1" t="s">
         <v>357</v>
       </c>
@@ -10249,7 +10282,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>604</v>
       </c>
@@ -10272,7 +10305,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>295</v>
       </c>
@@ -10298,7 +10331,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A215" s="1" t="s">
         <v>428</v>
       </c>
@@ -10321,7 +10354,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>950</v>
       </c>
@@ -10347,7 +10380,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>516</v>
       </c>
@@ -10373,7 +10406,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="218" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
         <v>13</v>
       </c>
@@ -10399,7 +10432,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="219" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
         <v>129</v>
       </c>
@@ -10422,7 +10455,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="220" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>832</v>
       </c>
@@ -10448,7 +10481,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="221" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>520</v>
       </c>
@@ -10474,7 +10507,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="222" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>660</v>
       </c>
@@ -10500,7 +10533,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="223" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>660</v>
       </c>
@@ -10526,7 +10559,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="224" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>660</v>
       </c>
@@ -10552,7 +10585,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="225" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>670</v>
       </c>
@@ -10578,7 +10611,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="226" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>723</v>
       </c>
@@ -10604,7 +10637,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="227" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>1027</v>
       </c>
@@ -10630,7 +10663,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="228" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>884</v>
       </c>
@@ -10656,7 +10689,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="229" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>863</v>
       </c>
@@ -10682,7 +10715,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="230" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>57</v>
       </c>
@@ -10708,7 +10741,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="231" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>395</v>
       </c>
@@ -10731,7 +10764,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="232" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>298</v>
       </c>
@@ -10757,7 +10790,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="233" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>311</v>
       </c>
@@ -10783,10 +10816,10 @@
         <v>100</v>
       </c>
       <c r="I233" s="12" t="s">
-        <v>1460</v>
-      </c>
-    </row>
-    <row r="234" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+        <v>1454</v>
+      </c>
+    </row>
+    <row r="234" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A234" s="1" t="s">
         <v>74</v>
       </c>
@@ -10812,7 +10845,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="235" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A235" s="1" t="s">
         <v>671</v>
       </c>
@@ -10838,7 +10871,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="236" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A236" s="1" t="s">
         <v>793</v>
       </c>
@@ -10864,7 +10897,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="237" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A237" s="1" t="s">
         <v>1316</v>
       </c>
@@ -10890,7 +10923,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="238" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A238" s="1" t="s">
         <v>1028</v>
       </c>
@@ -10916,7 +10949,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="239" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A239" s="1" t="s">
         <v>1031</v>
       </c>
@@ -10942,7 +10975,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="240" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
         <v>672</v>
       </c>
@@ -10968,7 +11001,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="241" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
         <v>321</v>
       </c>
@@ -10994,7 +11027,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="242" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>360</v>
       </c>
@@ -11017,7 +11050,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="243" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>235</v>
       </c>
@@ -11043,7 +11076,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="244" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>820</v>
       </c>
@@ -11066,7 +11099,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="245" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
         <v>272</v>
       </c>
@@ -11092,7 +11125,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="246" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
         <v>1018</v>
       </c>
@@ -11115,7 +11148,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="247" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>450</v>
       </c>
@@ -11138,7 +11171,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="248" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>542</v>
       </c>
@@ -11161,7 +11194,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="249" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>656</v>
       </c>
@@ -11187,7 +11220,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="250" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
         <v>259</v>
       </c>
@@ -11210,7 +11243,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
         <v>135</v>
       </c>
@@ -11236,7 +11269,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="252" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
         <v>138</v>
       </c>
@@ -11262,10 +11295,10 @@
         <v>100</v>
       </c>
       <c r="I252" s="12" t="s">
-        <v>1468</v>
-      </c>
-    </row>
-    <row r="253" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+        <v>1462</v>
+      </c>
+    </row>
+    <row r="253" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
         <v>141</v>
       </c>
@@ -11291,7 +11324,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
         <v>720</v>
       </c>
@@ -11317,7 +11350,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="255" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
         <v>399</v>
       </c>
@@ -11343,7 +11376,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="256" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
         <v>913</v>
       </c>
@@ -11366,7 +11399,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="257" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A257" s="1" t="s">
         <v>1049</v>
       </c>
@@ -11392,7 +11425,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="258" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
         <v>453</v>
       </c>
@@ -11406,7 +11439,7 @@
         <v>1300</v>
       </c>
       <c r="E258" s="12" t="s">
-        <v>1451</v>
+        <v>1481</v>
       </c>
       <c r="F258" s="7" t="s">
         <v>455</v>
@@ -11418,13 +11451,13 @@
         <v>211</v>
       </c>
       <c r="I258" s="12" t="s">
-        <v>1452</v>
+        <v>1447</v>
       </c>
       <c r="J258" s="12" t="s">
-        <v>1453</v>
-      </c>
-    </row>
-    <row r="259" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+        <v>1448</v>
+      </c>
+    </row>
+    <row r="259" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
         <v>276</v>
       </c>
@@ -11450,7 +11483,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="260" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
         <v>752</v>
       </c>
@@ -11473,7 +11506,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="261" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
         <v>301</v>
       </c>
@@ -11496,7 +11529,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="262" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
         <v>628</v>
       </c>
@@ -11519,7 +11552,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="263" spans="1:10" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A263" s="1" t="s">
         <v>756</v>
       </c>
@@ -11545,7 +11578,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="264" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
         <v>431</v>
       </c>
@@ -11571,7 +11604,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="265" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
         <v>1019</v>
       </c>
@@ -11597,7 +11630,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="266" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
         <v>879</v>
       </c>
@@ -11623,7 +11656,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="267" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
         <v>279</v>
       </c>
@@ -11649,7 +11682,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="268" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
         <v>262</v>
       </c>
@@ -11675,7 +11708,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="269" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
         <v>363</v>
       </c>
@@ -11701,7 +11734,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="270" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A270" s="1" t="s">
         <v>1290</v>
       </c>
@@ -11724,7 +11757,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="271" spans="1:10" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
         <v>967</v>
       </c>
@@ -11747,7 +11780,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="272" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A272" s="1" t="s">
         <v>266</v>
       </c>
@@ -11770,7 +11803,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="273" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A273" s="1" t="s">
         <v>1014</v>
       </c>
@@ -11796,10 +11829,10 @@
         <v>100</v>
       </c>
       <c r="I273" s="12" t="s">
-        <v>1446</v>
-      </c>
-    </row>
-    <row r="274" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="274" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A274" s="1" t="s">
         <v>435</v>
       </c>
@@ -11825,7 +11858,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="275" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A275" s="1" t="s">
         <v>282</v>
       </c>
@@ -11851,7 +11884,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="276" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A276" s="1" t="s">
         <v>285</v>
       </c>
@@ -11877,7 +11910,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="277" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A277" s="1" t="s">
         <v>817</v>
       </c>
@@ -11903,7 +11936,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="278" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A278" s="1" t="s">
         <v>461</v>
       </c>
@@ -11929,7 +11962,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="279" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A279" s="1" t="s">
         <v>218</v>
       </c>
@@ -11955,7 +11988,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="280" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A280" s="1" t="s">
         <v>224</v>
       </c>
@@ -11981,7 +12014,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="281" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A281" s="1" t="s">
         <v>1070</v>
       </c>
@@ -12007,7 +12040,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="282" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A282" s="1" t="s">
         <v>366</v>
       </c>
@@ -12033,7 +12066,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="283" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>369</v>
       </c>
@@ -12059,7 +12092,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="284" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A284" s="1" t="s">
         <v>439</v>
       </c>
@@ -12085,7 +12118,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="285" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A285" s="1" t="s">
         <v>1023</v>
       </c>
@@ -12111,7 +12144,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="286" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>1022</v>
       </c>
@@ -12137,7 +12170,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="287" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A287" s="1" t="s">
         <v>1021</v>
       </c>
@@ -12163,7 +12196,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="288" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
         <v>833</v>
       </c>
@@ -12189,7 +12222,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="289" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A289" s="2" t="s">
         <v>1020</v>
       </c>
@@ -12212,7 +12245,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="290" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A290" s="1" t="s">
         <v>834</v>
       </c>
@@ -12238,7 +12271,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="291" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A291" s="1" t="s">
         <v>60</v>
       </c>
@@ -12264,7 +12297,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="292" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A292" s="1" t="s">
         <v>372</v>
       </c>
@@ -12288,7 +12321,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="293" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A293" s="1" t="s">
         <v>215</v>
       </c>
@@ -12314,7 +12347,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="294" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
         <v>180</v>
       </c>
@@ -12340,7 +12373,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="295" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
         <v>325</v>
       </c>
@@ -12365,8 +12398,11 @@
       <c r="H295" s="7" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="296" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I295" s="12" t="s">
+        <v>1471</v>
+      </c>
+    </row>
+    <row r="296" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
         <v>183</v>
       </c>
@@ -12392,7 +12428,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="297" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
         <v>443</v>
       </c>
@@ -12418,7 +12454,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="298" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
         <v>622</v>
       </c>
@@ -12444,7 +12480,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="299" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>984</v>
       </c>
@@ -12467,7 +12503,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="300" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
         <v>562</v>
       </c>
@@ -12490,7 +12526,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="301" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
         <v>585</v>
       </c>
@@ -12513,7 +12549,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="302" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>800</v>
       </c>
@@ -12539,7 +12575,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="303" spans="1:8" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>1291</v>
       </c>
@@ -12565,7 +12601,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="304" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
         <v>1085</v>
       </c>
@@ -12591,7 +12627,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="305" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
         <v>1089</v>
       </c>
@@ -12617,7 +12653,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="306" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>1093</v>
       </c>
@@ -12643,7 +12679,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="307" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>1193</v>
       </c>
@@ -12669,7 +12705,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="308" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>1098</v>
       </c>
@@ -12695,13 +12731,13 @@
         <v>532</v>
       </c>
       <c r="I308" s="12" t="s">
-        <v>1439</v>
+        <v>1435</v>
       </c>
       <c r="J308" s="12" t="s">
-        <v>1440</v>
-      </c>
-    </row>
-    <row r="309" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+        <v>1436</v>
+      </c>
+    </row>
+    <row r="309" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>1102</v>
       </c>
@@ -12727,7 +12763,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="310" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
         <v>1106</v>
       </c>
@@ -12753,7 +12789,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="311" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
         <v>1108</v>
       </c>
@@ -12779,7 +12815,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="312" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A312" s="1" t="s">
         <v>1114</v>
       </c>
@@ -12805,7 +12841,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="313" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A313" s="1" t="s">
         <v>1118</v>
       </c>
@@ -12831,7 +12867,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="314" spans="1:10" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
         <v>1126</v>
       </c>
@@ -12851,7 +12887,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="315" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
         <v>1128</v>
       </c>
@@ -12871,7 +12907,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="316" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A316" s="1" t="s">
         <v>1132</v>
       </c>
@@ -12894,7 +12930,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="317" spans="1:10" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A317" s="1" t="s">
         <v>1136</v>
       </c>
@@ -12914,7 +12950,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="318" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
         <v>1140</v>
       </c>
@@ -12937,7 +12973,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="319" spans="1:10" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
         <v>1144</v>
       </c>
@@ -12960,7 +12996,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="320" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
         <v>1148</v>
       </c>
@@ -12980,7 +13016,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="321" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
         <v>1288</v>
       </c>
@@ -13006,7 +13042,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="322" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
         <v>1155</v>
       </c>
@@ -13032,7 +13068,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="323" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>1159</v>
       </c>
@@ -13052,7 +13088,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="324" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>1163</v>
       </c>
@@ -13075,7 +13111,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="325" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
         <v>1167</v>
       </c>
@@ -13101,7 +13137,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="326" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>1171</v>
       </c>
@@ -13127,7 +13163,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="327" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>1175</v>
       </c>
@@ -13150,7 +13186,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="328" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A328" s="1" t="s">
         <v>1179</v>
       </c>
@@ -13176,7 +13212,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="329" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A329" s="1" t="s">
         <v>1182</v>
       </c>
@@ -13196,7 +13232,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="330" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A330" s="1" t="s">
         <v>1317</v>
       </c>
@@ -13219,7 +13255,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="331" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A331" s="1" t="s">
         <v>1188</v>
       </c>
@@ -13242,7 +13278,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="332" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A332" s="1" t="s">
         <v>1284</v>
       </c>
@@ -13268,7 +13304,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="333" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A333" s="1" t="s">
         <v>1197</v>
       </c>
@@ -13294,7 +13330,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="334" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
         <v>1201</v>
       </c>
@@ -13320,7 +13356,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="335" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
         <v>1204</v>
       </c>
@@ -13346,7 +13382,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="336" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A336" s="1" t="s">
         <v>1208</v>
       </c>
@@ -13369,7 +13405,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="337" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A337" s="1" t="s">
         <v>1211</v>
       </c>
@@ -13395,7 +13431,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="338" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A338" s="1" t="s">
         <v>1215</v>
       </c>
@@ -13421,7 +13457,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="339" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A339" s="1" t="s">
         <v>1220</v>
       </c>
@@ -13444,7 +13480,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="340" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A340" s="1" t="s">
         <v>1222</v>
       </c>
@@ -13467,10 +13503,10 @@
         <v>530</v>
       </c>
       <c r="I340" s="12" t="s">
-        <v>1447</v>
-      </c>
-    </row>
-    <row r="341" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="341" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A341" s="1" t="s">
         <v>1223</v>
       </c>
@@ -13490,7 +13526,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="342" spans="1:9" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A342" s="1" t="s">
         <v>1228</v>
       </c>
@@ -13513,10 +13549,10 @@
         <v>100</v>
       </c>
       <c r="I342" s="12" t="s">
-        <v>1450</v>
-      </c>
-    </row>
-    <row r="343" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+        <v>1446</v>
+      </c>
+    </row>
+    <row r="343" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A343" s="1" t="s">
         <v>1232</v>
       </c>
@@ -13542,7 +13578,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="344" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A344" s="1" t="s">
         <v>1237</v>
       </c>
@@ -13568,7 +13604,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="345" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A345" s="1" t="s">
         <v>1240</v>
       </c>
@@ -13591,7 +13627,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="346" spans="1:9" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A346" s="1" t="s">
         <v>1241</v>
       </c>
@@ -13614,7 +13650,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="347" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A347" s="1" t="s">
         <v>1246</v>
       </c>
@@ -13637,7 +13673,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="348" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A348" s="1" t="s">
         <v>1252</v>
       </c>
@@ -13660,7 +13696,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="349" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A349" s="1" t="s">
         <v>1254</v>
       </c>
@@ -13683,7 +13719,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="350" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A350" s="1" t="s">
         <v>1258</v>
       </c>
@@ -13709,7 +13745,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="351" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A351" s="1" t="s">
         <v>1264</v>
       </c>
@@ -13732,7 +13768,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="352" spans="1:9" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A352" s="1" t="s">
         <v>1266</v>
       </c>
@@ -13755,7 +13791,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="353" spans="1:10" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A353" s="1" t="s">
         <v>1270</v>
       </c>
@@ -13778,13 +13814,13 @@
         <v>530</v>
       </c>
       <c r="I353" s="12" t="s">
-        <v>1467</v>
+        <v>1461</v>
       </c>
       <c r="J353" s="12" t="s">
-        <v>1466</v>
-      </c>
-    </row>
-    <row r="354" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+        <v>1460</v>
+      </c>
+    </row>
+    <row r="354" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A354" s="1" t="s">
         <v>1276</v>
       </c>
@@ -13807,7 +13843,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="355" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A355" s="1" t="s">
         <v>1326</v>
       </c>
@@ -13833,7 +13869,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="356" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A356" s="1" t="s">
         <v>1327</v>
       </c>
@@ -13859,7 +13895,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="357" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A357" s="1" t="s">
         <v>1292</v>
       </c>
@@ -13885,7 +13921,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="358" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A358" s="1" t="s">
         <v>1295</v>
       </c>
@@ -13911,7 +13947,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="359" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A359" s="1" t="s">
         <v>1300</v>
       </c>
@@ -13937,7 +13973,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="360" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A360" s="1" t="s">
         <v>1303</v>
       </c>
@@ -13963,7 +13999,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="361" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A361" s="1" t="s">
         <v>1308</v>
       </c>
@@ -13989,7 +14025,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="362" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A362" s="1" t="s">
         <v>1313</v>
       </c>
@@ -14009,7 +14045,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="363" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A363" s="1" t="s">
         <v>1321</v>
       </c>
@@ -14035,7 +14071,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="364" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
         <v>1331</v>
       </c>
@@ -14061,33 +14097,33 @@
         <v>66</v>
       </c>
     </row>
-    <row r="365" spans="1:10" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B365" s="1" t="s">
         <v>1342</v>
       </c>
-      <c r="B365" s="1" t="s">
-        <v>1341</v>
-      </c>
       <c r="C365" s="7">
-        <v>1383</v>
+        <v>899</v>
       </c>
       <c r="D365" s="7">
-        <v>630</v>
+        <v>485</v>
       </c>
       <c r="E365" s="12" t="s">
+        <v>1344</v>
+      </c>
+      <c r="F365" s="12" t="s">
         <v>1343</v>
-      </c>
-      <c r="F365" s="12" t="s">
-        <v>1344</v>
       </c>
       <c r="G365" s="7" t="s">
         <v>891</v>
       </c>
       <c r="H365" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="366" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="366" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A366" s="1" t="s">
         <v>1345</v>
       </c>
@@ -14095,10 +14131,10 @@
         <v>1346</v>
       </c>
       <c r="C366" s="7">
-        <v>899</v>
+        <v>1050</v>
       </c>
       <c r="D366" s="7">
-        <v>485</v>
+        <v>600</v>
       </c>
       <c r="E366" s="12" t="s">
         <v>1348</v>
@@ -14112,8 +14148,14 @@
       <c r="H366" s="7" t="s">
         <v>531</v>
       </c>
-    </row>
-    <row r="367" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I366" s="12" t="s">
+        <v>1479</v>
+      </c>
+      <c r="J366" s="12" t="s">
+        <v>1480</v>
+      </c>
+    </row>
+    <row r="367" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A367" s="1" t="s">
         <v>1349</v>
       </c>
@@ -14121,10 +14163,10 @@
         <v>1350</v>
       </c>
       <c r="C367" s="7">
-        <v>1050</v>
+        <v>1084</v>
       </c>
       <c r="D367" s="7">
-        <v>600</v>
+        <v>650</v>
       </c>
       <c r="E367" s="12" t="s">
         <v>1352</v>
@@ -14136,27 +14178,30 @@
         <v>891</v>
       </c>
       <c r="H367" s="7" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="368" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+        <v>530</v>
+      </c>
+      <c r="I367" s="12" t="s">
+        <v>1476</v>
+      </c>
+    </row>
+    <row r="368" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A368" s="1" t="s">
-        <v>1353</v>
+        <v>1355</v>
       </c>
       <c r="B368" s="1" t="s">
-        <v>1354</v>
+        <v>1356</v>
       </c>
       <c r="C368" s="7">
-        <v>1084</v>
+        <v>1265</v>
       </c>
       <c r="D368" s="7">
         <v>650</v>
       </c>
       <c r="E368" s="12" t="s">
-        <v>1356</v>
+        <v>1354</v>
       </c>
       <c r="F368" s="12" t="s">
-        <v>1355</v>
+        <v>1353</v>
       </c>
       <c r="G368" s="7" t="s">
         <v>891</v>
@@ -14164,19 +14209,22 @@
       <c r="H368" s="7" t="s">
         <v>530</v>
       </c>
-    </row>
-    <row r="369" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I368" s="12" t="s">
+        <v>1477</v>
+      </c>
+    </row>
+    <row r="369" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A369" s="1" t="s">
-        <v>1359</v>
+        <v>1374</v>
       </c>
       <c r="B369" s="1" t="s">
-        <v>1360</v>
+        <v>1371</v>
       </c>
       <c r="C369" s="7">
-        <v>1265</v>
+        <v>1225</v>
       </c>
       <c r="D369" s="7">
-        <v>650</v>
+        <v>700</v>
       </c>
       <c r="E369" s="12" t="s">
         <v>1358</v>
@@ -14188,15 +14236,21 @@
         <v>891</v>
       </c>
       <c r="H369" s="7" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="370" spans="1:10" ht="58" hidden="1" x14ac:dyDescent="0.35">
+        <v>531</v>
+      </c>
+      <c r="I369" s="12" t="s">
+        <v>1465</v>
+      </c>
+      <c r="J369" s="12" t="s">
+        <v>1466</v>
+      </c>
+    </row>
+    <row r="370" spans="1:10" ht="87" x14ac:dyDescent="0.35">
       <c r="A370" s="1" t="s">
-        <v>1378</v>
+        <v>1373</v>
       </c>
       <c r="B370" s="1" t="s">
-        <v>1375</v>
+        <v>1372</v>
       </c>
       <c r="C370" s="7">
         <v>1225</v>
@@ -14205,10 +14259,10 @@
         <v>700</v>
       </c>
       <c r="E370" s="12" t="s">
-        <v>1362</v>
+        <v>1360</v>
       </c>
       <c r="F370" s="12" t="s">
-        <v>1361</v>
+        <v>1359</v>
       </c>
       <c r="G370" s="7" t="s">
         <v>891</v>
@@ -14217,56 +14271,50 @@
         <v>531</v>
       </c>
       <c r="I370" s="12" t="s">
-        <v>1471</v>
+        <v>1467</v>
       </c>
       <c r="J370" s="12" t="s">
-        <v>1472</v>
-      </c>
-    </row>
-    <row r="371" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="371" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A371" s="1" t="s">
-        <v>1377</v>
+        <v>1363</v>
       </c>
       <c r="B371" s="1" t="s">
-        <v>1376</v>
+        <v>1364</v>
       </c>
       <c r="C371" s="7">
-        <v>1225</v>
+        <v>535</v>
       </c>
       <c r="D371" s="7">
-        <v>700</v>
+        <v>400</v>
       </c>
       <c r="E371" s="12" t="s">
-        <v>1364</v>
+        <v>1362</v>
       </c>
       <c r="F371" s="12" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
       <c r="G371" s="7" t="s">
         <v>891</v>
       </c>
       <c r="H371" s="7" t="s">
-        <v>531</v>
-      </c>
-      <c r="I371" s="12" t="s">
-        <v>1473</v>
-      </c>
-      <c r="J371" s="12" t="s">
-        <v>1474</v>
-      </c>
-    </row>
-    <row r="372" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="372" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A372" s="1" t="s">
-        <v>1367</v>
+        <v>1379</v>
       </c>
       <c r="B372" s="1" t="s">
-        <v>1368</v>
+        <v>1380</v>
       </c>
       <c r="C372" s="7">
-        <v>535</v>
+        <v>1033</v>
       </c>
       <c r="D372" s="7">
-        <v>400</v>
+        <v>675</v>
       </c>
       <c r="E372" s="12" t="s">
         <v>1366</v>
@@ -14278,27 +14326,33 @@
         <v>891</v>
       </c>
       <c r="H372" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="373" spans="1:10" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+        <v>531</v>
+      </c>
+      <c r="I372" s="12" t="s">
+        <v>1473</v>
+      </c>
+      <c r="J372" s="12" t="s">
+        <v>1472</v>
+      </c>
+    </row>
+    <row r="373" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A373" s="1" t="s">
-        <v>1383</v>
+        <v>1381</v>
       </c>
       <c r="B373" s="1" t="s">
-        <v>1384</v>
+        <v>1382</v>
       </c>
       <c r="C373" s="7">
-        <v>1033</v>
+        <v>614</v>
       </c>
       <c r="D373" s="7">
-        <v>675</v>
+        <v>375</v>
       </c>
       <c r="E373" s="12" t="s">
-        <v>1370</v>
+        <v>1368</v>
       </c>
       <c r="F373" s="12" t="s">
-        <v>1369</v>
+        <v>1367</v>
       </c>
       <c r="G373" s="7" t="s">
         <v>891</v>
@@ -14307,24 +14361,24 @@
         <v>531</v>
       </c>
     </row>
-    <row r="374" spans="1:10" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A374" s="1" t="s">
-        <v>1385</v>
+        <v>1383</v>
       </c>
       <c r="B374" s="1" t="s">
-        <v>1386</v>
+        <v>1384</v>
       </c>
       <c r="C374" s="7">
-        <v>614</v>
+        <v>946</v>
       </c>
       <c r="D374" s="7">
-        <v>375</v>
+        <v>575</v>
       </c>
       <c r="E374" s="12" t="s">
-        <v>1372</v>
+        <v>1370</v>
       </c>
       <c r="F374" s="12" t="s">
-        <v>1371</v>
+        <v>1369</v>
       </c>
       <c r="G374" s="7" t="s">
         <v>891</v>
@@ -14333,24 +14387,24 @@
         <v>531</v>
       </c>
     </row>
-    <row r="375" spans="1:10" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A375" s="1" t="s">
-        <v>1387</v>
+        <v>1375</v>
       </c>
       <c r="B375" s="1" t="s">
-        <v>1388</v>
+        <v>1376</v>
       </c>
       <c r="C375" s="7">
-        <v>946</v>
+        <v>1174</v>
       </c>
       <c r="D375" s="7">
-        <v>575</v>
+        <v>700</v>
       </c>
       <c r="E375" s="12" t="s">
-        <v>1374</v>
+        <v>1378</v>
       </c>
       <c r="F375" s="12" t="s">
-        <v>1373</v>
+        <v>1377</v>
       </c>
       <c r="G375" s="7" t="s">
         <v>891</v>
@@ -14358,40 +14412,43 @@
       <c r="H375" s="7" t="s">
         <v>531</v>
       </c>
-    </row>
-    <row r="376" spans="1:10" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I375" s="12" t="s">
+        <v>1464</v>
+      </c>
+      <c r="J375" s="12" t="s">
+        <v>1463</v>
+      </c>
+    </row>
+    <row r="376" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A376" s="1" t="s">
-        <v>1379</v>
+        <v>1385</v>
       </c>
       <c r="B376" s="1" t="s">
-        <v>1380</v>
+        <v>1386</v>
       </c>
       <c r="C376" s="7">
-        <v>1174</v>
+        <v>1395</v>
       </c>
       <c r="D376" s="7">
-        <v>700</v>
+        <v>920</v>
       </c>
       <c r="E376" s="12" t="s">
-        <v>1382</v>
+        <v>1388</v>
       </c>
       <c r="F376" s="12" t="s">
-        <v>1381</v>
+        <v>1387</v>
       </c>
       <c r="G376" s="7" t="s">
         <v>891</v>
       </c>
       <c r="H376" s="7" t="s">
-        <v>531</v>
+        <v>66</v>
       </c>
       <c r="I376" s="12" t="s">
-        <v>1470</v>
-      </c>
-      <c r="J376" s="12" t="s">
-        <v>1469</v>
-      </c>
-    </row>
-    <row r="377" spans="1:10" ht="58" hidden="1" x14ac:dyDescent="0.35">
+        <v>1453</v>
+      </c>
+    </row>
+    <row r="377" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A377" s="1" t="s">
         <v>1389</v>
       </c>
@@ -14399,10 +14456,10 @@
         <v>1390</v>
       </c>
       <c r="C377" s="7">
-        <v>1395</v>
+        <v>488</v>
       </c>
       <c r="D377" s="7">
-        <v>920</v>
+        <v>400</v>
       </c>
       <c r="E377" s="12" t="s">
         <v>1392</v>
@@ -14414,39 +14471,36 @@
         <v>891</v>
       </c>
       <c r="H377" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="I377" s="12" t="s">
-        <v>1459</v>
-      </c>
-    </row>
-    <row r="378" spans="1:10" ht="58" hidden="1" x14ac:dyDescent="0.35">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="378" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A378" s="1" t="s">
         <v>1393</v>
       </c>
       <c r="B378" s="1" t="s">
+        <v>1396</v>
+      </c>
+      <c r="C378" s="7">
+        <v>554</v>
+      </c>
+      <c r="D378" s="7">
+        <v>200</v>
+      </c>
+      <c r="E378" s="12" t="s">
+        <v>1395</v>
+      </c>
+      <c r="F378" s="12" t="s">
         <v>1394</v>
-      </c>
-      <c r="C378" s="7">
-        <v>488</v>
-      </c>
-      <c r="D378" s="7">
-        <v>400</v>
-      </c>
-      <c r="E378" s="12" t="s">
-        <v>1396</v>
-      </c>
-      <c r="F378" s="12" t="s">
-        <v>1395</v>
       </c>
       <c r="G378" s="7" t="s">
         <v>891</v>
       </c>
       <c r="H378" s="7" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="379" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="379" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A379" s="1" t="s">
         <v>1397</v>
       </c>
@@ -14454,10 +14508,10 @@
         <v>1400</v>
       </c>
       <c r="C379" s="7">
-        <v>554</v>
+        <v>398</v>
       </c>
       <c r="D379" s="7">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="E379" s="12" t="s">
         <v>1399</v>
@@ -14469,36 +14523,36 @@
         <v>891</v>
       </c>
       <c r="H379" s="7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="380" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="380" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A380" s="1" t="s">
         <v>1401</v>
       </c>
       <c r="B380" s="1" t="s">
+        <v>1402</v>
+      </c>
+      <c r="C380" s="7">
+        <v>399</v>
+      </c>
+      <c r="D380" s="7">
+        <v>120</v>
+      </c>
+      <c r="E380" s="12" t="s">
         <v>1404</v>
       </c>
-      <c r="C380" s="7">
-        <v>398</v>
-      </c>
-      <c r="D380" s="7">
-        <v>250</v>
-      </c>
-      <c r="E380" s="12" t="s">
+      <c r="F380" s="12" t="s">
         <v>1403</v>
-      </c>
-      <c r="F380" s="12" t="s">
-        <v>1402</v>
       </c>
       <c r="G380" s="7" t="s">
         <v>891</v>
       </c>
       <c r="H380" s="7" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="381" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="381" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A381" s="1" t="s">
         <v>1405</v>
       </c>
@@ -14506,10 +14560,10 @@
         <v>1406</v>
       </c>
       <c r="C381" s="7">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D381" s="7">
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="E381" s="12" t="s">
         <v>1408</v>
@@ -14521,10 +14575,10 @@
         <v>891</v>
       </c>
       <c r="H381" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="382" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="382" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A382" s="1" t="s">
         <v>1409</v>
       </c>
@@ -14532,7 +14586,7 @@
         <v>1410</v>
       </c>
       <c r="C382" s="7">
-        <v>397</v>
+        <v>350</v>
       </c>
       <c r="D382" s="7">
         <v>300</v>
@@ -14547,27 +14601,27 @@
         <v>891</v>
       </c>
       <c r="H382" s="7" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="383" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="383" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A383" s="1" t="s">
-        <v>1413</v>
+        <v>1415</v>
       </c>
       <c r="B383" s="1" t="s">
-        <v>1414</v>
+        <v>1416</v>
       </c>
       <c r="C383" s="7">
-        <v>350</v>
+        <v>385</v>
       </c>
       <c r="D383" s="7">
         <v>300</v>
       </c>
       <c r="E383" s="12" t="s">
-        <v>1416</v>
+        <v>1414</v>
       </c>
       <c r="F383" s="12" t="s">
-        <v>1415</v>
+        <v>1413</v>
       </c>
       <c r="G383" s="7" t="s">
         <v>891</v>
@@ -14576,24 +14630,24 @@
         <v>66</v>
       </c>
     </row>
-    <row r="384" spans="1:10" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A384" s="1" t="s">
+        <v>1418</v>
+      </c>
+      <c r="B384" s="1" t="s">
+        <v>1417</v>
+      </c>
+      <c r="C384" s="7">
+        <v>1690</v>
+      </c>
+      <c r="D384" s="7">
+        <v>1090</v>
+      </c>
+      <c r="E384" s="12" t="s">
+        <v>1482</v>
+      </c>
+      <c r="F384" s="12" t="s">
         <v>1419</v>
-      </c>
-      <c r="B384" s="1" t="s">
-        <v>1420</v>
-      </c>
-      <c r="C384" s="7">
-        <v>385</v>
-      </c>
-      <c r="D384" s="7">
-        <v>300</v>
-      </c>
-      <c r="E384" s="12" t="s">
-        <v>1418</v>
-      </c>
-      <c r="F384" s="12" t="s">
-        <v>1417</v>
       </c>
       <c r="G384" s="7" t="s">
         <v>891</v>
@@ -14601,48 +14655,51 @@
       <c r="H384" s="7" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="385" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+      <c r="I384" s="12" t="s">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="385" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A385" s="1" t="s">
         <v>1422</v>
       </c>
       <c r="B385" s="1" t="s">
+        <v>1423</v>
+      </c>
+      <c r="C385" s="7">
+        <v>1999</v>
+      </c>
+      <c r="D385" s="7">
+        <v>800</v>
+      </c>
+      <c r="E385" s="12" t="s">
         <v>1421</v>
       </c>
-      <c r="C385" s="7">
-        <v>1690</v>
-      </c>
-      <c r="D385" s="7">
-        <v>1090</v>
-      </c>
-      <c r="E385" s="12" t="s">
-        <v>1455</v>
-      </c>
       <c r="F385" s="12" t="s">
-        <v>1423</v>
+        <v>1420</v>
       </c>
       <c r="G385" s="7" t="s">
         <v>891</v>
       </c>
       <c r="H385" s="7" t="s">
-        <v>66</v>
+        <v>211</v>
       </c>
       <c r="I385" s="12" t="s">
-        <v>1456</v>
-      </c>
-    </row>
-    <row r="386" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
+        <v>1458</v>
+      </c>
+    </row>
+    <row r="386" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A386" s="1" t="s">
+        <v>1427</v>
+      </c>
+      <c r="B386" s="1" t="s">
         <v>1426</v>
       </c>
-      <c r="B386" s="1" t="s">
-        <v>1427</v>
-      </c>
       <c r="C386" s="7">
-        <v>1999</v>
+        <v>4699</v>
       </c>
       <c r="D386" s="7">
-        <v>800</v>
+        <v>2832</v>
       </c>
       <c r="E386" s="12" t="s">
         <v>1425</v>
@@ -14654,67 +14711,38 @@
         <v>891</v>
       </c>
       <c r="H386" s="7" t="s">
-        <v>211</v>
+        <v>530</v>
       </c>
       <c r="I386" s="12" t="s">
-        <v>1464</v>
-      </c>
-    </row>
-    <row r="387" spans="1:10" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+        <v>1445</v>
+      </c>
+      <c r="J386" s="12" t="s">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="387" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A387" s="1" t="s">
+        <v>1428</v>
+      </c>
+      <c r="B387" s="1" t="s">
+        <v>1429</v>
+      </c>
+      <c r="C387" s="7">
+        <v>349</v>
+      </c>
+      <c r="D387" s="7">
+        <v>295</v>
+      </c>
+      <c r="E387" s="12" t="s">
         <v>1431</v>
       </c>
-      <c r="B387" s="1" t="s">
+      <c r="F387" s="12" t="s">
         <v>1430</v>
       </c>
-      <c r="C387" s="7">
-        <v>4699</v>
-      </c>
-      <c r="D387" s="7">
-        <v>2832</v>
-      </c>
-      <c r="E387" s="12" t="s">
-        <v>1429</v>
-      </c>
-      <c r="F387" s="12" t="s">
-        <v>1428</v>
-      </c>
       <c r="G387" s="7" t="s">
-        <v>891</v>
+        <v>438</v>
       </c>
       <c r="H387" s="7" t="s">
-        <v>530</v>
-      </c>
-      <c r="I387" s="12" t="s">
-        <v>1449</v>
-      </c>
-      <c r="J387" s="12" t="s">
-        <v>1448</v>
-      </c>
-    </row>
-    <row r="388" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A388" s="1" t="s">
-        <v>1432</v>
-      </c>
-      <c r="B388" s="1" t="s">
-        <v>1433</v>
-      </c>
-      <c r="C388" s="7">
-        <v>349</v>
-      </c>
-      <c r="D388" s="7">
-        <v>295</v>
-      </c>
-      <c r="E388" s="12" t="s">
-        <v>1435</v>
-      </c>
-      <c r="F388" s="12" t="s">
-        <v>1434</v>
-      </c>
-      <c r="G388" s="7" t="s">
-        <v>438</v>
-      </c>
-      <c r="H388" s="7" t="s">
         <v>66</v>
       </c>
     </row>
@@ -14729,19 +14757,19 @@
     <hyperlink ref="E261" r:id="rId7"/>
     <hyperlink ref="E340" r:id="rId8"/>
     <hyperlink ref="E155" r:id="rId9"/>
-    <hyperlink ref="E365" r:id="rId10"/>
-    <hyperlink ref="F365" r:id="rId11" location="&amp;gid=1&amp;pid=1"/>
+    <hyperlink ref="F365" r:id="rId10" location="&amp;gid=1&amp;pid=1"/>
+    <hyperlink ref="E365" r:id="rId11"/>
     <hyperlink ref="F366" r:id="rId12" location="&amp;gid=1&amp;pid=1"/>
     <hyperlink ref="E366" r:id="rId13"/>
     <hyperlink ref="F367" r:id="rId14" location="&amp;gid=1&amp;pid=1"/>
     <hyperlink ref="E367" r:id="rId15"/>
-    <hyperlink ref="F368" r:id="rId16" location="&amp;gid=1&amp;pid=1"/>
+    <hyperlink ref="F368" r:id="rId16"/>
     <hyperlink ref="E368" r:id="rId17"/>
     <hyperlink ref="F369" r:id="rId18"/>
     <hyperlink ref="E369" r:id="rId19"/>
-    <hyperlink ref="F370" r:id="rId20"/>
-    <hyperlink ref="E370" r:id="rId21"/>
-    <hyperlink ref="F371" display="https://www.mercadolibre.com.mx/epicentro-audishako-max-02-restaurador-de-bajos-para-auto-subwoofer-para-carro-pickups-y-suv-accesorios-para-auto-audio-diseno-en-relieve-3d-incluye-dash-remoto-control-de-bajos/p/MLM64640099?pdp_filters=item_id:MLM46970202"/>
+    <hyperlink ref="F370" display="https://www.mercadolibre.com.mx/epicentro-audishako-max-02-restaurador-de-bajos-para-auto-subwoofer-para-carro-pickups-y-suv-accesorios-para-auto-audio-diseno-en-relieve-3d-incluye-dash-remoto-control-de-bajos/p/MLM64640099?pdp_filters=item_id:MLM46970202"/>
+    <hyperlink ref="E370" r:id="rId20"/>
+    <hyperlink ref="F371" r:id="rId21"/>
     <hyperlink ref="E371" r:id="rId22"/>
     <hyperlink ref="F372" r:id="rId23"/>
     <hyperlink ref="E372" r:id="rId24"/>
@@ -14753,9 +14781,9 @@
     <hyperlink ref="E375" r:id="rId30"/>
     <hyperlink ref="F376" r:id="rId31"/>
     <hyperlink ref="E376" r:id="rId32"/>
-    <hyperlink ref="F377" r:id="rId33"/>
+    <hyperlink ref="F377" r:id="rId33" location="reviews"/>
     <hyperlink ref="E377" r:id="rId34"/>
-    <hyperlink ref="F378" r:id="rId35" location="reviews"/>
+    <hyperlink ref="F378" r:id="rId35"/>
     <hyperlink ref="E378" r:id="rId36"/>
     <hyperlink ref="F379" r:id="rId37"/>
     <hyperlink ref="E379" r:id="rId38"/>
@@ -14775,49 +14803,59 @@
     <hyperlink ref="E386" r:id="rId52"/>
     <hyperlink ref="F387" r:id="rId53"/>
     <hyperlink ref="E387" r:id="rId54"/>
-    <hyperlink ref="F388" r:id="rId55"/>
-    <hyperlink ref="E388" r:id="rId56"/>
-    <hyperlink ref="I73"/>
-    <hyperlink ref="I308" r:id="rId57"/>
-    <hyperlink ref="J308" r:id="rId58"/>
-    <hyperlink ref="I195"/>
-    <hyperlink ref="I134"/>
-    <hyperlink ref="I67"/>
-    <hyperlink ref="J67" r:id="rId59"/>
-    <hyperlink ref="I68"/>
-    <hyperlink ref="I273"/>
-    <hyperlink ref="I340"/>
-    <hyperlink ref="J387" r:id="rId60"/>
-    <hyperlink ref="I387" r:id="rId61"/>
-    <hyperlink ref="I342"/>
-    <hyperlink ref="E258" r:id="rId62"/>
-    <hyperlink ref="I258" r:id="rId63"/>
-    <hyperlink ref="J258" r:id="rId64"/>
-    <hyperlink ref="I36" r:id="rId65"/>
-    <hyperlink ref="I385"/>
-    <hyperlink ref="J61" r:id="rId66"/>
-    <hyperlink ref="I61"/>
-    <hyperlink ref="I377" r:id="rId67"/>
-    <hyperlink ref="I233"/>
-    <hyperlink ref="J32" r:id="rId68"/>
-    <hyperlink ref="I32"/>
-    <hyperlink ref="I104"/>
-    <hyperlink ref="I386"/>
-    <hyperlink ref="I149"/>
-    <hyperlink ref="J353" r:id="rId69"/>
-    <hyperlink ref="I353"/>
-    <hyperlink ref="I252"/>
-    <hyperlink ref="J376" r:id="rId70"/>
-    <hyperlink ref="I376"/>
+    <hyperlink ref="I73" display="https://http2.mlstatic.com/D_NQ_NP_2X_977864-MLA82522530268_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_728802-MLA82808708997_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_714871-MLA82808836891_032025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
+    <hyperlink ref="I308" r:id="rId55"/>
+    <hyperlink ref="J308" r:id="rId56"/>
+    <hyperlink ref="I195" display="https://http2.mlstatic.com/D_NQ_NP_2X_881622-MLA100107482214_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_853470-MLA83211986807_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_889429-MLA82708797484_032025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
+    <hyperlink ref="I134" display="https://http2.mlstatic.com/D_NQ_NP_2X_691159-MLA74393127536_022024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_797614-MLA74213272750_012024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_768655-MLA74336317695_012024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
+    <hyperlink ref="I67" display="https://http2.mlstatic.com/D_NQ_NP_2X_665383-MLA110622349795_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_998155-MLA109812957268_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_967066-MLA109813016698_042026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="J67" r:id="rId57"/>
+    <hyperlink ref="I68" display="https://http2.mlstatic.com/D_NQ_NP_2X_754117-MLA87918629604_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_955266-MLA88256438081_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_924778-MLA88256272783_072025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
+    <hyperlink ref="I273" display="https://http2.mlstatic.com/D_NQ_NP_2X_651538-MLA109474609027_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_786870-MLA109384870397_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_877937-MLA109385877631_032026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I340" display="https://http2.mlstatic.com/D_NQ_NP_2X_659872-MLA110558100656_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_654212-MLA110558217136_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_728798-MLA110558100602_052026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="J386" r:id="rId58"/>
+    <hyperlink ref="I386" r:id="rId59"/>
+    <hyperlink ref="I342" display="https://http2.mlstatic.com/D_NQ_NP_2X_704682-MLA112632086794_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_648062-MLA114215908179_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_721338-MLA112631444306_062026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="E258" r:id="rId60"/>
+    <hyperlink ref="I258" r:id="rId61"/>
+    <hyperlink ref="J258" r:id="rId62"/>
+    <hyperlink ref="I36" r:id="rId63"/>
+    <hyperlink ref="I384" display="https://http2.mlstatic.com/D_NQ_NP_2X_870766-MLA111944165952_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_637261-MLA111944285568_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_835091-MLA112882459449_062026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="J61" r:id="rId64"/>
+    <hyperlink ref="I61" display="https://http2.mlstatic.com/D_NQ_NP_2X_650019-MLA112598239078_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_694102-MLA111420836191_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_960139-MLA111232526403_052026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I376" r:id="rId65"/>
+    <hyperlink ref="I233" display="https://http2.mlstatic.com/D_NQ_NP_2X_761866-MLA76203783381_052024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_967910-MLA76082310461_042024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_699850-MLA76082339489_042024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
+    <hyperlink ref="J32" r:id="rId66"/>
+    <hyperlink ref="I32" display="https://http2.mlstatic.com/D_NQ_NP_2X_937988-MLA100214376229_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_839463-MLA100214244569_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_878239-MLA100214347283_122025-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I104" display="https://http2.mlstatic.com/D_NQ_NP_2X_853469-MLA73479850047_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_636371-MLA72966055893_112023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_647337-MLA74448293715_022024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
+    <hyperlink ref="I385" display="https://http2.mlstatic.com/D_NQ_NP_2X_838661-MLA114043475512_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_997422-MLA111845686244_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_946430-MLA112856485647_062026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I149" display="https://http2.mlstatic.com/D_NQ_NP_2X_700050-MLA90330537717_082025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_810830-MLA92985348779_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_611435-MLA103169335415_122025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
+    <hyperlink ref="J353" r:id="rId67"/>
+    <hyperlink ref="I353" display="https://http2.mlstatic.com/D_NQ_NP_2X_972461-MLA108765590667_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_959062-MLA111287287492_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_702439-MLA108999676116_032026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I252" display="https://http2.mlstatic.com/D_NQ_NP_2X_772336-MLA83215360667_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_641687-MLA82926894938_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_686941-MLA80851161221_112024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
+    <hyperlink ref="J375" r:id="rId68"/>
+    <hyperlink ref="I375" display="https://http2.mlstatic.com/D_NQ_NP_2X_918751-MLA113089268495_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_972829-MLA114388137831_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_739083-MLA113884890489_062026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="J369" r:id="rId69"/>
+    <hyperlink ref="I369" display="https://http2.mlstatic.com/D_NQ_NP_2X_622982-MLA91998379772_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_918567-MLA93316673763_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_951409-MLA93316693351_092025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
+    <hyperlink ref="I370" r:id="rId70"/>
     <hyperlink ref="J370" r:id="rId71"/>
-    <hyperlink ref="I370"/>
-    <hyperlink ref="I371" r:id="rId72"/>
-    <hyperlink ref="J371" r:id="rId73"/>
+    <hyperlink ref="J173" r:id="rId72"/>
+    <hyperlink ref="I173" display="https://http2.mlstatic.com/D_NQ_NP_2X_630634-MLA83929492736_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_826427-MLA83875691856_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_778506-MLA83875632066_042025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
+    <hyperlink ref="I295" display="https://http2.mlstatic.com/D_NQ_NP_2X_601798-MLA74779553000_032024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_784677-MLA71729912500_092023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_982997-MLA73375012815_122023-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
+    <hyperlink ref="J372" r:id="rId73"/>
+    <hyperlink ref="I372" display="https://http2.mlstatic.com/D_NQ_NP_2X_743943-MLA113720575198_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_652343-MLA98742656086_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_688496-MLA89833143459_082025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
+    <hyperlink ref="J56" r:id="rId74"/>
+    <hyperlink ref="I56" r:id="rId75"/>
+    <hyperlink ref="I367" r:id="rId76"/>
+    <hyperlink ref="I368" r:id="rId77"/>
+    <hyperlink ref="I135" r:id="rId78"/>
+    <hyperlink ref="I366" r:id="rId79"/>
+    <hyperlink ref="J366" r:id="rId80"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId74"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId81"/>
   <tableParts count="1">
-    <tablePart r:id="rId75"/>
+    <tablePart r:id="rId82"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualiza proyecto (3 modificados, 1 eliminado, 475 nuevos): DescargarImagenes.py, productos.xlsx, ~$productos.xlsx
</commit_message>
<xml_diff>
--- a/datos/productos.xlsx
+++ b/datos/productos.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2403" uniqueCount="1580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2412" uniqueCount="1587">
   <si>
     <t>Nombre</t>
   </si>
@@ -4776,6 +4776,27 @@
   </si>
   <si>
     <t>https://http2.mlstatic.com/D_NQ_NP_2X_973200-MLA111559842713_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_705535-MLA110612658098_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_743702-MLA110611090138_052026-F.webp</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_701490-MLA108653774761_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_910611-MLA87584829978_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_761367-MLA87718920709_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_607798-MLA107642299882_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_656127-MLA114825035763_072026-F.webp</t>
+  </si>
+  <si>
+    <t>Espejo De Baño Led Tri Color Tira De Luz</t>
+  </si>
+  <si>
+    <t>Radio: 50cm</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_861035-MLM110725392715_042026-F-espejo-de-bano-led-tri-color-tira-de-luz-defogging-time5050.webp</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-2900477235-espejo-de-bano-led-tri-color-tira-de-luz-defogging-time5050-_JM?quantity=1&amp;sid=purchases</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_957897-MLA114152946760_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_988648-MLA114781488773_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_938364-MLA113693419924_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_714728-MLA115205021849_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_675499-MLA115386756969_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_808617-MLA114152032962_082026-F.webp</t>
+  </si>
+  <si>
+    <t>https://video-vod-clips.mms.mlstatic.com/v1/video/hls/cli_04xzu0y81ntclips/019f90e3cbb27ae8a7448a824f49eed7/master.m3u8</t>
   </si>
 </sst>
 </file>
@@ -4934,8 +4955,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:J375" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J375"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:J376" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J376"/>
   <sortState ref="A2:H342">
     <sortCondition ref="A1:A342"/>
   </sortState>
@@ -5240,7 +5261,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J375"/>
+  <dimension ref="A1:J376"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="70" style="1" customWidth="1"/>
@@ -7906,6 +7927,9 @@
       <c r="H102" s="7" t="s">
         <v>198</v>
       </c>
+      <c r="I102" s="12" t="s">
+        <v>1580</v>
+      </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
@@ -14656,22 +14680,22 @@
     </row>
     <row r="359" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A359" s="1" t="s">
-        <v>1315</v>
+        <v>1581</v>
       </c>
       <c r="B359" s="1" t="s">
-        <v>1316</v>
+        <v>1582</v>
       </c>
       <c r="C359" s="7">
-        <v>535</v>
+        <v>590</v>
       </c>
       <c r="D359" s="7">
         <v>400</v>
       </c>
       <c r="E359" s="12" t="s">
-        <v>1314</v>
+        <v>1583</v>
       </c>
       <c r="F359" s="12" t="s">
-        <v>1313</v>
+        <v>1584</v>
       </c>
       <c r="G359" s="7" t="s">
         <v>861</v>
@@ -14680,62 +14704,62 @@
         <v>66</v>
       </c>
       <c r="I359" s="12" t="s">
-        <v>1552</v>
+        <v>1585</v>
       </c>
       <c r="J359" s="12" t="s">
-        <v>1551</v>
-      </c>
-    </row>
-    <row r="360" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>1586</v>
+      </c>
+    </row>
+    <row r="360" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A360" s="1" t="s">
-        <v>1331</v>
+        <v>1315</v>
       </c>
       <c r="B360" s="1" t="s">
-        <v>1332</v>
+        <v>1316</v>
       </c>
       <c r="C360" s="7">
-        <v>1033</v>
+        <v>535</v>
       </c>
       <c r="D360" s="7">
-        <v>675</v>
+        <v>400</v>
       </c>
       <c r="E360" s="12" t="s">
-        <v>1318</v>
+        <v>1314</v>
       </c>
       <c r="F360" s="12" t="s">
-        <v>1317</v>
+        <v>1313</v>
       </c>
       <c r="G360" s="7" t="s">
         <v>861</v>
       </c>
       <c r="H360" s="7" t="s">
-        <v>512</v>
+        <v>66</v>
       </c>
       <c r="I360" s="12" t="s">
-        <v>1424</v>
+        <v>1552</v>
       </c>
       <c r="J360" s="12" t="s">
-        <v>1423</v>
-      </c>
-    </row>
-    <row r="361" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+        <v>1551</v>
+      </c>
+    </row>
+    <row r="361" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A361" s="1" t="s">
-        <v>1333</v>
+        <v>1331</v>
       </c>
       <c r="B361" s="1" t="s">
-        <v>1334</v>
+        <v>1332</v>
       </c>
       <c r="C361" s="7">
-        <v>614</v>
+        <v>1033</v>
       </c>
       <c r="D361" s="7">
-        <v>375</v>
+        <v>675</v>
       </c>
       <c r="E361" s="12" t="s">
-        <v>1320</v>
+        <v>1318</v>
       </c>
       <c r="F361" s="12" t="s">
-        <v>1319</v>
+        <v>1317</v>
       </c>
       <c r="G361" s="7" t="s">
         <v>861</v>
@@ -14743,25 +14767,31 @@
       <c r="H361" s="7" t="s">
         <v>512</v>
       </c>
-    </row>
-    <row r="362" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="I361" s="12" t="s">
+        <v>1424</v>
+      </c>
+      <c r="J361" s="12" t="s">
+        <v>1423</v>
+      </c>
+    </row>
+    <row r="362" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A362" s="1" t="s">
-        <v>1335</v>
+        <v>1333</v>
       </c>
       <c r="B362" s="1" t="s">
-        <v>1336</v>
+        <v>1334</v>
       </c>
       <c r="C362" s="7">
-        <v>946</v>
+        <v>614</v>
       </c>
       <c r="D362" s="7">
-        <v>575</v>
+        <v>375</v>
       </c>
       <c r="E362" s="12" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="F362" s="12" t="s">
-        <v>1321</v>
+        <v>1319</v>
       </c>
       <c r="G362" s="7" t="s">
         <v>861</v>
@@ -14769,31 +14799,25 @@
       <c r="H362" s="7" t="s">
         <v>512</v>
       </c>
-      <c r="I362" s="12" t="s">
-        <v>1534</v>
-      </c>
-      <c r="J362" s="12" t="s">
-        <v>1533</v>
-      </c>
-    </row>
-    <row r="363" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="363" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A363" s="1" t="s">
-        <v>1327</v>
+        <v>1335</v>
       </c>
       <c r="B363" s="1" t="s">
-        <v>1328</v>
+        <v>1336</v>
       </c>
       <c r="C363" s="7">
-        <v>1174</v>
+        <v>946</v>
       </c>
       <c r="D363" s="7">
-        <v>700</v>
+        <v>575</v>
       </c>
       <c r="E363" s="12" t="s">
-        <v>1330</v>
+        <v>1322</v>
       </c>
       <c r="F363" s="12" t="s">
-        <v>1329</v>
+        <v>1321</v>
       </c>
       <c r="G363" s="7" t="s">
         <v>861</v>
@@ -14802,242 +14826,242 @@
         <v>512</v>
       </c>
       <c r="I363" s="12" t="s">
-        <v>1415</v>
+        <v>1534</v>
       </c>
       <c r="J363" s="12" t="s">
-        <v>1414</v>
-      </c>
-    </row>
-    <row r="364" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+        <v>1533</v>
+      </c>
+    </row>
+    <row r="364" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
-        <v>1337</v>
+        <v>1327</v>
       </c>
       <c r="B364" s="1" t="s">
-        <v>1338</v>
+        <v>1328</v>
       </c>
       <c r="C364" s="7">
-        <v>1395</v>
+        <v>1174</v>
       </c>
       <c r="D364" s="7">
-        <v>920</v>
+        <v>700</v>
       </c>
       <c r="E364" s="12" t="s">
-        <v>1340</v>
+        <v>1330</v>
       </c>
       <c r="F364" s="12" t="s">
-        <v>1339</v>
+        <v>1329</v>
       </c>
       <c r="G364" s="7" t="s">
         <v>861</v>
       </c>
       <c r="H364" s="7" t="s">
-        <v>66</v>
+        <v>512</v>
       </c>
       <c r="I364" s="12" t="s">
-        <v>1404</v>
+        <v>1415</v>
+      </c>
+      <c r="J364" s="12" t="s">
+        <v>1414</v>
       </c>
     </row>
     <row r="365" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
-        <v>1527</v>
+        <v>1337</v>
       </c>
       <c r="B365" s="1" t="s">
-        <v>1341</v>
+        <v>1338</v>
       </c>
       <c r="C365" s="7">
-        <v>488</v>
+        <v>1395</v>
       </c>
       <c r="D365" s="7">
-        <v>400</v>
+        <v>920</v>
       </c>
       <c r="E365" s="12" t="s">
-        <v>1343</v>
+        <v>1340</v>
       </c>
       <c r="F365" s="12" t="s">
-        <v>1342</v>
+        <v>1339</v>
       </c>
       <c r="G365" s="7" t="s">
         <v>861</v>
       </c>
       <c r="H365" s="7" t="s">
-        <v>512</v>
+        <v>66</v>
       </c>
       <c r="I365" s="12" t="s">
-        <v>1482</v>
-      </c>
-      <c r="J365" s="12" t="s">
-        <v>1528</v>
-      </c>
-    </row>
-    <row r="366" spans="1:10" x14ac:dyDescent="0.35">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="366" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A366" s="1" t="s">
-        <v>1344</v>
+        <v>1527</v>
       </c>
       <c r="B366" s="1" t="s">
-        <v>1347</v>
+        <v>1341</v>
       </c>
       <c r="C366" s="7">
-        <v>554</v>
+        <v>488</v>
       </c>
       <c r="D366" s="7">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="E366" s="12" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="F366" s="12" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
       <c r="G366" s="7" t="s">
         <v>861</v>
       </c>
       <c r="H366" s="7" t="s">
-        <v>12</v>
+        <v>512</v>
       </c>
       <c r="I366" s="12" t="s">
-        <v>1458</v>
+        <v>1482</v>
       </c>
       <c r="J366" s="12" t="s">
-        <v>1457</v>
-      </c>
-    </row>
-    <row r="367" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="367" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A367" s="1" t="s">
-        <v>1348</v>
+        <v>1344</v>
       </c>
       <c r="B367" s="1" t="s">
-        <v>1351</v>
+        <v>1347</v>
       </c>
       <c r="C367" s="7">
-        <v>398</v>
+        <v>554</v>
       </c>
       <c r="D367" s="7">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="E367" s="12" t="s">
-        <v>1350</v>
+        <v>1346</v>
       </c>
       <c r="F367" s="12" t="s">
-        <v>1349</v>
+        <v>1345</v>
       </c>
       <c r="G367" s="7" t="s">
         <v>861</v>
       </c>
       <c r="H367" s="7" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="368" spans="1:10" x14ac:dyDescent="0.35">
+        <v>12</v>
+      </c>
+      <c r="I367" s="12" t="s">
+        <v>1458</v>
+      </c>
+      <c r="J367" s="12" t="s">
+        <v>1457</v>
+      </c>
+    </row>
+    <row r="368" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A368" s="1" t="s">
-        <v>1352</v>
+        <v>1348</v>
       </c>
       <c r="B368" s="1" t="s">
-        <v>1353</v>
+        <v>1351</v>
       </c>
       <c r="C368" s="7">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D368" s="7">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="E368" s="12" t="s">
-        <v>1355</v>
+        <v>1350</v>
       </c>
       <c r="F368" s="12" t="s">
-        <v>1354</v>
+        <v>1349</v>
       </c>
       <c r="G368" s="7" t="s">
         <v>861</v>
       </c>
       <c r="H368" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="I368" s="12" t="s">
-        <v>1548</v>
-      </c>
-    </row>
-    <row r="369" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="369" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A369" s="1" t="s">
-        <v>1356</v>
+        <v>1352</v>
       </c>
       <c r="B369" s="1" t="s">
-        <v>1357</v>
+        <v>1353</v>
       </c>
       <c r="C369" s="7">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="D369" s="7">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="E369" s="12" t="s">
-        <v>1359</v>
+        <v>1355</v>
       </c>
       <c r="F369" s="12" t="s">
-        <v>1358</v>
+        <v>1354</v>
       </c>
       <c r="G369" s="7" t="s">
         <v>861</v>
       </c>
       <c r="H369" s="7" t="s">
-        <v>198</v>
+        <v>66</v>
       </c>
       <c r="I369" s="12" t="s">
-        <v>1438</v>
-      </c>
-      <c r="J369" s="12" t="s">
-        <v>1439</v>
-      </c>
-    </row>
-    <row r="370" spans="1:10" x14ac:dyDescent="0.35">
+        <v>1548</v>
+      </c>
+    </row>
+    <row r="370" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A370" s="1" t="s">
-        <v>1360</v>
+        <v>1356</v>
       </c>
       <c r="B370" s="1" t="s">
-        <v>1361</v>
+        <v>1357</v>
       </c>
       <c r="C370" s="7">
-        <v>350</v>
+        <v>397</v>
       </c>
       <c r="D370" s="7">
         <v>300</v>
       </c>
       <c r="E370" s="12" t="s">
-        <v>1363</v>
+        <v>1359</v>
       </c>
       <c r="F370" s="12" t="s">
-        <v>1362</v>
+        <v>1358</v>
       </c>
       <c r="G370" s="7" t="s">
         <v>861</v>
       </c>
       <c r="H370" s="7" t="s">
-        <v>66</v>
+        <v>198</v>
       </c>
       <c r="I370" s="12" t="s">
-        <v>1543</v>
+        <v>1438</v>
       </c>
       <c r="J370" s="12" t="s">
-        <v>1542</v>
-      </c>
-    </row>
-    <row r="371" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+        <v>1439</v>
+      </c>
+    </row>
+    <row r="371" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A371" s="1" t="s">
-        <v>1366</v>
+        <v>1360</v>
       </c>
       <c r="B371" s="1" t="s">
-        <v>1367</v>
+        <v>1361</v>
       </c>
       <c r="C371" s="7">
-        <v>385</v>
+        <v>350</v>
       </c>
       <c r="D371" s="7">
         <v>300</v>
       </c>
       <c r="E371" s="12" t="s">
-        <v>1365</v>
+        <v>1363</v>
       </c>
       <c r="F371" s="12" t="s">
-        <v>1364</v>
+        <v>1362</v>
       </c>
       <c r="G371" s="7" t="s">
         <v>861</v>
@@ -15046,27 +15070,30 @@
         <v>66</v>
       </c>
       <c r="I371" s="12" t="s">
-        <v>1434</v>
-      </c>
-    </row>
-    <row r="372" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>1543</v>
+      </c>
+      <c r="J371" s="12" t="s">
+        <v>1542</v>
+      </c>
+    </row>
+    <row r="372" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A372" s="1" t="s">
-        <v>1369</v>
+        <v>1366</v>
       </c>
       <c r="B372" s="1" t="s">
-        <v>1368</v>
+        <v>1367</v>
       </c>
       <c r="C372" s="7">
-        <v>1690</v>
+        <v>385</v>
       </c>
       <c r="D372" s="7">
-        <v>1090</v>
+        <v>300</v>
       </c>
       <c r="E372" s="12" t="s">
-        <v>1433</v>
+        <v>1365</v>
       </c>
       <c r="F372" s="12" t="s">
-        <v>1370</v>
+        <v>1364</v>
       </c>
       <c r="G372" s="7" t="s">
         <v>861</v>
@@ -15075,99 +15102,128 @@
         <v>66</v>
       </c>
       <c r="I372" s="12" t="s">
-        <v>1401</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="373" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A373" s="1" t="s">
-        <v>1373</v>
+        <v>1369</v>
       </c>
       <c r="B373" s="1" t="s">
-        <v>1374</v>
+        <v>1368</v>
       </c>
       <c r="C373" s="7">
-        <v>1999</v>
+        <v>1690</v>
       </c>
       <c r="D373" s="7">
-        <v>800</v>
+        <v>1090</v>
       </c>
       <c r="E373" s="12" t="s">
-        <v>1372</v>
+        <v>1433</v>
       </c>
       <c r="F373" s="12" t="s">
-        <v>1371</v>
+        <v>1370</v>
       </c>
       <c r="G373" s="7" t="s">
         <v>861</v>
       </c>
       <c r="H373" s="7" t="s">
-        <v>198</v>
+        <v>66</v>
       </c>
       <c r="I373" s="12" t="s">
-        <v>1409</v>
-      </c>
-    </row>
-    <row r="374" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>1401</v>
+      </c>
+    </row>
+    <row r="374" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A374" s="1" t="s">
-        <v>1378</v>
+        <v>1373</v>
       </c>
       <c r="B374" s="1" t="s">
-        <v>1377</v>
+        <v>1374</v>
       </c>
       <c r="C374" s="7">
-        <v>4699</v>
+        <v>1999</v>
       </c>
       <c r="D374" s="7">
-        <v>2832</v>
+        <v>800</v>
       </c>
       <c r="E374" s="12" t="s">
-        <v>1376</v>
+        <v>1372</v>
       </c>
       <c r="F374" s="12" t="s">
-        <v>1375</v>
+        <v>1371</v>
       </c>
       <c r="G374" s="7" t="s">
         <v>861</v>
       </c>
       <c r="H374" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="I374" s="12" t="s">
+        <v>1409</v>
+      </c>
+    </row>
+    <row r="375" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A375" s="1" t="s">
+        <v>1378</v>
+      </c>
+      <c r="B375" s="1" t="s">
+        <v>1377</v>
+      </c>
+      <c r="C375" s="7">
+        <v>4699</v>
+      </c>
+      <c r="D375" s="7">
+        <v>2832</v>
+      </c>
+      <c r="E375" s="12" t="s">
+        <v>1376</v>
+      </c>
+      <c r="F375" s="12" t="s">
+        <v>1375</v>
+      </c>
+      <c r="G375" s="7" t="s">
+        <v>861</v>
+      </c>
+      <c r="H375" s="7" t="s">
         <v>511</v>
       </c>
-      <c r="I374" s="12" t="s">
+      <c r="I375" s="12" t="s">
         <v>1396</v>
       </c>
-      <c r="J374" s="12" t="s">
+      <c r="J375" s="12" t="s">
         <v>1395</v>
       </c>
     </row>
-    <row r="375" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A375" s="1" t="s">
+    <row r="376" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A376" s="1" t="s">
         <v>1379</v>
       </c>
-      <c r="B375" s="1" t="s">
+      <c r="B376" s="1" t="s">
         <v>1380</v>
       </c>
-      <c r="C375" s="7">
+      <c r="C376" s="7">
         <v>349</v>
       </c>
-      <c r="D375" s="7">
+      <c r="D376" s="7">
         <v>295</v>
       </c>
-      <c r="E375" s="12" t="s">
+      <c r="E376" s="12" t="s">
         <v>1382</v>
       </c>
-      <c r="F375" s="12" t="s">
+      <c r="F376" s="12" t="s">
         <v>1381</v>
       </c>
-      <c r="G375" s="7" t="s">
+      <c r="G376" s="7" t="s">
         <v>420</v>
       </c>
-      <c r="H375" s="7" t="s">
+      <c r="H376" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I375" s="12" t="s">
+      <c r="I376" s="12" t="s">
         <v>1493</v>
       </c>
-      <c r="J375" s="12" t="s">
+      <c r="J376" s="12" t="s">
         <v>1492</v>
       </c>
     </row>
@@ -15194,40 +15250,40 @@
     <hyperlink ref="E357" r:id="rId19"/>
     <hyperlink ref="F358" display="https://www.mercadolibre.com.mx/epicentro-audishako-max-02-restaurador-de-bajos-para-auto-subwoofer-para-carro-pickups-y-suv-accesorios-para-auto-audio-diseno-en-relieve-3d-incluye-dash-remoto-control-de-bajos/p/MLM64640099?pdp_filters=item_id:MLM46970202"/>
     <hyperlink ref="E358" r:id="rId20"/>
-    <hyperlink ref="F359" r:id="rId21"/>
-    <hyperlink ref="E359" r:id="rId22"/>
-    <hyperlink ref="F360" r:id="rId23"/>
-    <hyperlink ref="E360" r:id="rId24"/>
-    <hyperlink ref="F361" r:id="rId25"/>
-    <hyperlink ref="E361" r:id="rId26"/>
-    <hyperlink ref="F362" r:id="rId27"/>
-    <hyperlink ref="E362" r:id="rId28"/>
-    <hyperlink ref="F363" r:id="rId29"/>
-    <hyperlink ref="E363" r:id="rId30"/>
-    <hyperlink ref="F364" r:id="rId31"/>
-    <hyperlink ref="E364" r:id="rId32"/>
-    <hyperlink ref="F365" r:id="rId33" location="reviews"/>
-    <hyperlink ref="E365" r:id="rId34"/>
-    <hyperlink ref="F366" r:id="rId35"/>
-    <hyperlink ref="E366" r:id="rId36"/>
-    <hyperlink ref="F367" r:id="rId37"/>
-    <hyperlink ref="E367" r:id="rId38"/>
-    <hyperlink ref="F368" r:id="rId39"/>
-    <hyperlink ref="E368" r:id="rId40"/>
-    <hyperlink ref="F369" r:id="rId41"/>
-    <hyperlink ref="E369" r:id="rId42"/>
-    <hyperlink ref="F370" r:id="rId43"/>
-    <hyperlink ref="E370" r:id="rId44"/>
-    <hyperlink ref="F371" r:id="rId45"/>
-    <hyperlink ref="E371" r:id="rId46"/>
-    <hyperlink ref="F372" r:id="rId47"/>
-    <hyperlink ref="E372" r:id="rId48"/>
-    <hyperlink ref="F373" r:id="rId49"/>
-    <hyperlink ref="E373" r:id="rId50"/>
-    <hyperlink ref="F374" r:id="rId51"/>
-    <hyperlink ref="E374" r:id="rId52"/>
-    <hyperlink ref="F375" r:id="rId53"/>
-    <hyperlink ref="E375" r:id="rId54"/>
+    <hyperlink ref="F360" r:id="rId21"/>
+    <hyperlink ref="E360" r:id="rId22"/>
+    <hyperlink ref="F361" r:id="rId23"/>
+    <hyperlink ref="E361" r:id="rId24"/>
+    <hyperlink ref="F362" r:id="rId25"/>
+    <hyperlink ref="E362" r:id="rId26"/>
+    <hyperlink ref="F363" r:id="rId27"/>
+    <hyperlink ref="E363" r:id="rId28"/>
+    <hyperlink ref="F364" r:id="rId29"/>
+    <hyperlink ref="E364" r:id="rId30"/>
+    <hyperlink ref="F365" r:id="rId31"/>
+    <hyperlink ref="E365" r:id="rId32"/>
+    <hyperlink ref="F366" r:id="rId33" location="reviews"/>
+    <hyperlink ref="E366" r:id="rId34"/>
+    <hyperlink ref="F367" r:id="rId35"/>
+    <hyperlink ref="E367" r:id="rId36"/>
+    <hyperlink ref="F368" r:id="rId37"/>
+    <hyperlink ref="E368" r:id="rId38"/>
+    <hyperlink ref="F369" r:id="rId39"/>
+    <hyperlink ref="E369" r:id="rId40"/>
+    <hyperlink ref="F370" r:id="rId41"/>
+    <hyperlink ref="E370" r:id="rId42"/>
+    <hyperlink ref="F371" r:id="rId43"/>
+    <hyperlink ref="E371" r:id="rId44"/>
+    <hyperlink ref="F372" r:id="rId45"/>
+    <hyperlink ref="E372" r:id="rId46"/>
+    <hyperlink ref="F373" r:id="rId47"/>
+    <hyperlink ref="E373" r:id="rId48"/>
+    <hyperlink ref="F374" r:id="rId49"/>
+    <hyperlink ref="E374" r:id="rId50"/>
+    <hyperlink ref="F375" r:id="rId51"/>
+    <hyperlink ref="E375" r:id="rId52"/>
+    <hyperlink ref="F376" r:id="rId53"/>
+    <hyperlink ref="E376" r:id="rId54"/>
     <hyperlink ref="I72" display="https://http2.mlstatic.com/D_NQ_NP_2X_977864-MLA82522530268_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_728802-MLA82808708997_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_714871-MLA82808836891_032025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I299" r:id="rId55"/>
     <hyperlink ref="J299" r:id="rId56"/>
@@ -15238,28 +15294,28 @@
     <hyperlink ref="I67" display="https://http2.mlstatic.com/D_NQ_NP_2X_754117-MLA87918629604_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_955266-MLA88256438081_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_924778-MLA88256272783_072025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I265" display="https://http2.mlstatic.com/D_NQ_NP_2X_651538-MLA109474609027_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_786870-MLA109384870397_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_877937-MLA109385877631_032026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I328" display="https://http2.mlstatic.com/D_NQ_NP_2X_659872-MLA110558100656_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_654212-MLA110558217136_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_728798-MLA110558100602_052026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J374" r:id="rId58"/>
-    <hyperlink ref="I374" r:id="rId59"/>
+    <hyperlink ref="J375" r:id="rId58"/>
+    <hyperlink ref="I375" r:id="rId59"/>
     <hyperlink ref="I330" display="https://http2.mlstatic.com/D_NQ_NP_2X_704682-MLA112632086794_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_648062-MLA114215908179_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_721338-MLA112631444306_062026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="E250" r:id="rId60"/>
     <hyperlink ref="I250" r:id="rId61"/>
     <hyperlink ref="J250" r:id="rId62"/>
     <hyperlink ref="I36" r:id="rId63"/>
-    <hyperlink ref="I372" display="https://http2.mlstatic.com/D_NQ_NP_2X_870766-MLA111944165952_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_637261-MLA111944285568_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_835091-MLA112882459449_062026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I373" display="https://http2.mlstatic.com/D_NQ_NP_2X_870766-MLA111944165952_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_637261-MLA111944285568_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_835091-MLA112882459449_062026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="J60" r:id="rId64"/>
     <hyperlink ref="I60" display="https://http2.mlstatic.com/D_NQ_NP_2X_650019-MLA112598239078_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_694102-MLA111420836191_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_960139-MLA111232526403_052026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I364" r:id="rId65"/>
+    <hyperlink ref="I365" r:id="rId65"/>
     <hyperlink ref="I225" display="https://http2.mlstatic.com/D_NQ_NP_2X_761866-MLA76203783381_052024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_967910-MLA76082310461_042024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_699850-MLA76082339489_042024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="J32" r:id="rId66"/>
     <hyperlink ref="I32" display="https://http2.mlstatic.com/D_NQ_NP_2X_937988-MLA100214376229_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_839463-MLA100214244569_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_878239-MLA100214347283_122025-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I101" display="https://http2.mlstatic.com/D_NQ_NP_2X_853469-MLA73479850047_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_636371-MLA72966055893_112023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_647337-MLA74448293715_022024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="I373" display="https://http2.mlstatic.com/D_NQ_NP_2X_838661-MLA114043475512_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_997422-MLA111845686244_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_946430-MLA112856485647_062026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I374" display="https://http2.mlstatic.com/D_NQ_NP_2X_838661-MLA114043475512_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_997422-MLA111845686244_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_946430-MLA112856485647_062026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I146" display="https://http2.mlstatic.com/D_NQ_NP_2X_700050-MLA90330537717_082025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_810830-MLA92985348779_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_611435-MLA103169335415_122025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
     <hyperlink ref="J341" r:id="rId67"/>
     <hyperlink ref="I341" display="https://http2.mlstatic.com/D_NQ_NP_2X_972461-MLA108765590667_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_959062-MLA111287287492_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_702439-MLA108999676116_032026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I244" display="https://http2.mlstatic.com/D_NQ_NP_2X_772336-MLA83215360667_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_641687-MLA82926894938_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_686941-MLA80851161221_112024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J363" r:id="rId68"/>
-    <hyperlink ref="I363" display="https://http2.mlstatic.com/D_NQ_NP_2X_918751-MLA113089268495_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_972829-MLA114388137831_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_739083-MLA113884890489_062026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="J364" r:id="rId68"/>
+    <hyperlink ref="I364" display="https://http2.mlstatic.com/D_NQ_NP_2X_918751-MLA113089268495_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_972829-MLA114388137831_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_739083-MLA113884890489_062026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="J357" r:id="rId69"/>
     <hyperlink ref="I357" display="https://http2.mlstatic.com/D_NQ_NP_2X_622982-MLA91998379772_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_918567-MLA93316673763_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_951409-MLA93316693351_092025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I358" r:id="rId70"/>
@@ -15267,8 +15323,8 @@
     <hyperlink ref="J169" r:id="rId72"/>
     <hyperlink ref="I169" display="https://http2.mlstatic.com/D_NQ_NP_2X_630634-MLA83929492736_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_826427-MLA83875691856_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_778506-MLA83875632066_042025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I286" display="https://http2.mlstatic.com/D_NQ_NP_2X_601798-MLA74779553000_032024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_784677-MLA71729912500_092023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_982997-MLA73375012815_122023-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J360" r:id="rId73"/>
-    <hyperlink ref="I360" display="https://http2.mlstatic.com/D_NQ_NP_2X_743943-MLA113720575198_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_652343-MLA98742656086_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_688496-MLA89833143459_082025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
+    <hyperlink ref="J361" r:id="rId73"/>
+    <hyperlink ref="I361" display="https://http2.mlstatic.com/D_NQ_NP_2X_743943-MLA113720575198_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_652343-MLA98742656086_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_688496-MLA89833143459_082025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
     <hyperlink ref="J56" r:id="rId74"/>
     <hyperlink ref="I56" r:id="rId75"/>
     <hyperlink ref="I355" r:id="rId76"/>
@@ -15276,12 +15332,12 @@
     <hyperlink ref="I132" r:id="rId78"/>
     <hyperlink ref="I354" r:id="rId79"/>
     <hyperlink ref="J354" r:id="rId80"/>
-    <hyperlink ref="I371" display="https://http2.mlstatic.com/D_NQ_NP_2X_730160-MLA112550162587_062026-F.webp;http://http2.mlstatic.com/D_NQ_NP_2X_748872-MLA113290799753_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_824232-MLA112954608093_062026-F.webp;https://http2.mlstatic.com/D_NQ"/>
+    <hyperlink ref="I372" display="https://http2.mlstatic.com/D_NQ_NP_2X_730160-MLA112550162587_062026-F.webp;http://http2.mlstatic.com/D_NQ_NP_2X_748872-MLA113290799753_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_824232-MLA112954608093_062026-F.webp;https://http2.mlstatic.com/D_NQ"/>
     <hyperlink ref="I107" r:id="rId81"/>
     <hyperlink ref="I2" display="https://http2.mlstatic.com/D_NQ_NP_2X_644970-MLA111138624893_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_618974-MLA113557256809_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_849248-MLA111414716285_052026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I11" r:id="rId82"/>
-    <hyperlink ref="I369" r:id="rId83"/>
-    <hyperlink ref="J369" r:id="rId84"/>
+    <hyperlink ref="I370" r:id="rId83"/>
+    <hyperlink ref="J370" r:id="rId84"/>
     <hyperlink ref="E145" r:id="rId85"/>
     <hyperlink ref="I145" r:id="rId86"/>
     <hyperlink ref="J180" r:id="rId87"/>
@@ -15301,8 +15357,8 @@
     <hyperlink ref="I54" r:id="rId101"/>
     <hyperlink ref="I353" r:id="rId102"/>
     <hyperlink ref="I325" r:id="rId103"/>
-    <hyperlink ref="J366" r:id="rId104"/>
-    <hyperlink ref="I366" r:id="rId105"/>
+    <hyperlink ref="J367" r:id="rId104"/>
+    <hyperlink ref="I367" r:id="rId105"/>
     <hyperlink ref="I337" display="https://http2.mlstatic.com/D_NQ_NP_2X_871513-MLA105683275105_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_921467-MLA106225093215_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_768089-MLA111241397693_052026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I273" r:id="rId106"/>
     <hyperlink ref="J268" r:id="rId107"/>
@@ -15326,7 +15382,7 @@
     <hyperlink ref="I197" display="https://http2.mlstatic.com/D_NQ_NP_2X_882824-MLA78038279945_072024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_628505-MLA80605999965_112024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_605405-MLA79717879214_102024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="J108" r:id="rId121"/>
     <hyperlink ref="I108" r:id="rId122"/>
-    <hyperlink ref="I365" r:id="rId123"/>
+    <hyperlink ref="I366" r:id="rId123"/>
     <hyperlink ref="I174" display="https://http2.mlstatic.com/D_NQ_NP_2X_671282-MLA88303913955_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_751626-MLA88304056333_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_928886-MLA111461620111_052026-F.webp;https://http2.mlstatic.com/D_NQ_"/>
     <hyperlink ref="I85" r:id="rId124"/>
     <hyperlink ref="I212" r:id="rId125"/>
@@ -15336,8 +15392,8 @@
     <hyperlink ref="J271" r:id="rId128"/>
     <hyperlink ref="I271" r:id="rId129"/>
     <hyperlink ref="I324" r:id="rId130"/>
-    <hyperlink ref="J375" r:id="rId131"/>
-    <hyperlink ref="I375" r:id="rId132"/>
+    <hyperlink ref="J376" r:id="rId131"/>
+    <hyperlink ref="I376" r:id="rId132"/>
     <hyperlink ref="J53" r:id="rId133"/>
     <hyperlink ref="I53" r:id="rId134"/>
     <hyperlink ref="I222" display="https://http2.mlstatic.com/D_NQ_NP_2X_931197-MLA111097282025_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_647752-MLA86304062244_062025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_697099-MLA86808814199_062025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
@@ -15371,13 +15427,13 @@
     <hyperlink ref="J143" r:id="rId148"/>
     <hyperlink ref="J87" r:id="rId149"/>
     <hyperlink ref="I87" r:id="rId150"/>
-    <hyperlink ref="J365" r:id="rId151"/>
+    <hyperlink ref="J366" r:id="rId151"/>
     <hyperlink ref="J235" r:id="rId152"/>
     <hyperlink ref="I235" display="https://http2.mlstatic.com/D_NQ_NP_2X_786831-MLA112508605409_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_945451-MLA106951088919_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_942407-MLA79868078780_102024-F.webp;https://http2.mlstatic.com/D_NQ"/>
     <hyperlink ref="J25" r:id="rId153"/>
     <hyperlink ref="I156" r:id="rId154"/>
-    <hyperlink ref="J362" r:id="rId155"/>
-    <hyperlink ref="I362" display="https://http2.mlstatic.com/D_NQ_NP_2X_654570-MLA114163554383_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_820669-MLA112176540320_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_827402-MLA113697495744_072026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="J363" r:id="rId155"/>
+    <hyperlink ref="I363" display="https://http2.mlstatic.com/D_NQ_NP_2X_654570-MLA114163554383_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_820669-MLA112176540320_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_827402-MLA113697495744_072026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="J283" r:id="rId156"/>
     <hyperlink ref="I283" r:id="rId157"/>
     <hyperlink ref="I147" r:id="rId158"/>
@@ -15385,48 +15441,53 @@
     <hyperlink ref="I167" display="https://http2.mlstatic.com/D_NQ_NP_2X_949414-MLA115597206229_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_781530-MLA115596590455_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_794977-MLA113865153424_072026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I242" r:id="rId160"/>
     <hyperlink ref="I336" r:id="rId161"/>
-    <hyperlink ref="J370" r:id="rId162"/>
-    <hyperlink ref="I370" r:id="rId163"/>
+    <hyperlink ref="J371" r:id="rId162"/>
+    <hyperlink ref="I371" r:id="rId163"/>
     <hyperlink ref="I113" display="https://http2.mlstatic.com/D_NQ_NP_2X_602967-MLA106207657120_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_937184-MLA99857184303_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_615655-MLA93805615686_102025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
     <hyperlink ref="J113" r:id="rId164"/>
     <hyperlink ref="I274" display="https://http2.mlstatic.com/D_NQ_NP_2X_811367-MLA96964641173_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_724534-MLA95972455447_102025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_862711-MLA94582890276_102025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I188" r:id="rId165"/>
-    <hyperlink ref="I368" r:id="rId166"/>
+    <hyperlink ref="I369" r:id="rId166"/>
     <hyperlink ref="I112" display="https://http2.mlstatic.com/D_NQ_NP_2X_832809-MLA100859657141_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_651615-MLA104572148023_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_683702-MLA104248384382_012026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I321" r:id="rId167"/>
-    <hyperlink ref="J359" r:id="rId168"/>
-    <hyperlink ref="I359" display="https://http2.mlstatic.com/D_NQ_NP_2X_986254-MLA113898749317_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_998498-MLA115220256263_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_611119-MLA113912677208_072026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I297"/>
+    <hyperlink ref="J360" r:id="rId168"/>
+    <hyperlink ref="I360" display="https://http2.mlstatic.com/D_NQ_NP_2X_986254-MLA113898749317_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_998498-MLA115220256263_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_611119-MLA113912677208_072026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I297" display="https://http2.mlstatic.com/D_NQ_NP_2X_672294-MLA110281902509_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_995715-MLA110918042491_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_936537-MLA110364709430_052026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="J297" r:id="rId169"/>
     <hyperlink ref="J326" r:id="rId170"/>
-    <hyperlink ref="I326"/>
+    <hyperlink ref="I326" display="https://http2.mlstatic.com/D_NQ_NP_2X_623123-MLA111040290746_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_934760-MLA111878498611_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_790070-MLA112661729675_062026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="J338" r:id="rId171"/>
-    <hyperlink ref="I338"/>
+    <hyperlink ref="I338" display="https://http2.mlstatic.com/D_NQ_NP_2X_637815-MLA110916194519_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_643077-MLA110749031212_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_708016-MLA112321199072_062026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I320" r:id="rId172"/>
     <hyperlink ref="I122" r:id="rId173"/>
     <hyperlink ref="J55" r:id="rId174"/>
-    <hyperlink ref="I55"/>
+    <hyperlink ref="I55" display="https://http2.mlstatic.com/D_NQ_NP_2X_707272-MLA81406001662_122024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_992452-MLA71699440818_092023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_616985-MLA84032409756_052025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="J293" r:id="rId175"/>
-    <hyperlink ref="I293"/>
+    <hyperlink ref="I293" display="https://http2.mlstatic.com/D_NQ_NP_2X_699847-MLA83204192108_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_847455-MLA79932861627_102024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_823994-MLA70105011582_062023-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="J247" r:id="rId176"/>
-    <hyperlink ref="I247"/>
+    <hyperlink ref="I247" display="https://http2.mlstatic.com/D_NQ_NP_2X_896395-MLA74651133358_022024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_757231-MLA73307952803_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_773664-MLA113844190574_072026-F.webp;https://http2.mlstatic.com/D_NQ_"/>
     <hyperlink ref="I269" r:id="rId177"/>
     <hyperlink ref="J214" r:id="rId178"/>
-    <hyperlink ref="I214"/>
+    <hyperlink ref="I214" display="https://http2.mlstatic.com/D_NQ_NP_2X_857704-MLA105910693631_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_785878-MLA115684445439_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_732723-MLA114610870605_072026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I124" r:id="rId179"/>
-    <hyperlink ref="I139"/>
-    <hyperlink ref="I151"/>
+    <hyperlink ref="I139" display="https://http2.mlstatic.com/D_NQ_NP_2X_731885-MLA81735782871_012025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_877502-MLA81736505623_012025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_739624-MLA81735782869_012025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
+    <hyperlink ref="I151" display="https://http2.mlstatic.com/D_NQ_NP_2X_852777-MLA73231184100_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_953229-MLA74068746840_012024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_727505-MLA74823139724_032024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I163" r:id="rId180"/>
     <hyperlink ref="J163" r:id="rId181"/>
     <hyperlink ref="F111" r:id="rId182" location="reviews"/>
     <hyperlink ref="I111" r:id="rId183"/>
     <hyperlink ref="I323" r:id="rId184"/>
     <hyperlink ref="I327" r:id="rId185"/>
+    <hyperlink ref="I102"/>
+    <hyperlink ref="E359" r:id="rId186"/>
+    <hyperlink ref="F359" r:id="rId187"/>
+    <hyperlink ref="I359"/>
+    <hyperlink ref="J359" r:id="rId188"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId186"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId189"/>
   <tableParts count="1">
-    <tablePart r:id="rId187"/>
+    <tablePart r:id="rId190"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualiza proyecto (4 modificados, 2 nuevos): GenerarCatalogo.py, productos.xlsx, index.html
</commit_message>
<xml_diff>
--- a/datos/productos.xlsx
+++ b/datos/productos.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2427" uniqueCount="1602">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2419" uniqueCount="1596">
   <si>
     <t>Nombre</t>
   </si>
@@ -3973,12 +3973,6 @@
     <t>Altura: 52.5 cm, Ancho: 37.5 cm</t>
   </si>
   <si>
-    <t>https://www.mercadolibre.com.mx/inversor-hzero-600w-de-onda-senoidal-modificada-para-auto-con-2-salidas-ac-y-2-usb/p/MLM52856540?pdp_filters=item_id:MLM2587727551</t>
-  </si>
-  <si>
-    <t>https://http2.mlstatic.com/D_NQ_NP_2X_996228-MLA110110565683_042026-F.webp</t>
-  </si>
-  <si>
     <t>https://www.mercadolibre.com.mx/hzero-inversor-de-corriente-1000w-12v-a-110v-transformador-portatil-para-coche-con-2-ac-y-2-usb-ideal-para-respaldo-electrico-hogar-proteccion-electrica-multiple/p/MLM57806893?pdp_filters=item_id:MLM2587781837</t>
   </si>
   <si>
@@ -4017,13 +4011,6 @@
     <t>https://http2.mlstatic.com/D_NQ_NP_2X_824026-MLA102603004510_122025-F.webp</t>
   </si>
   <si>
-    <t xml:space="preserve">Inversor convertidor de corriente 600W
-</t>
-  </si>
-  <si>
-    <t>Marca: Hzero Descripcion: Onda Senoidal Modificada para Auto con 2 Salidas AC y 2 USB</t>
-  </si>
-  <si>
     <t xml:space="preserve">Inversor Convertidor De Corriente 1000W 12v A 110v
 </t>
   </si>
@@ -4296,12 +4283,6 @@
   </si>
   <si>
     <t>https://http2.mlstatic.com/D_NQ_NP_2X_601798-MLA74779553000_032024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_784677-MLA71729912500_092023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_982997-MLA73375012815_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_982999-MLA70028199790_062023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_830261-MLA70048397883_062023-F.webp</t>
-  </si>
-  <si>
-    <t>https://video-vod-clips.mms.mlstatic.com/v1/video/hls/cli_04xzu0y81ntclips/019f29451c3876a8969ca32011081a6b/master.m3u8</t>
-  </si>
-  <si>
-    <t>https://http2.mlstatic.com/D_NQ_NP_2X_743943-MLA113720575198_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_652343-MLA98742656086_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_688496-MLA89833143459_082025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_980015-MLA111245266119_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_676086-MLA108251244515_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_743943-MLA113720575198_072026-F.webp</t>
   </si>
   <si>
     <t>https://video-vod-clips.mms.mlstatic.com/v1/video/hls/cli_04xzu0y81ntclips/019eec50ebdc7581aaf884c109615b29/master.m3u8</t>
@@ -5009,8 +4990,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:J377" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J377"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:J376" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J376"/>
   <sortState ref="A2:H342">
     <sortCondition ref="A1:A342"/>
   </sortState>
@@ -5315,7 +5296,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J377"/>
+  <dimension ref="A1:J376"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="70" style="1" customWidth="1"/>
@@ -5355,10 +5336,10 @@
         <v>7</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>1380</v>
+        <v>1376</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>1381</v>
+        <v>1377</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -5387,7 +5368,7 @@
         <v>66</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>1433</v>
+        <v>1427</v>
       </c>
       <c r="J2" s="12"/>
     </row>
@@ -5417,7 +5398,7 @@
         <v>66</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>1509</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -5469,7 +5450,7 @@
         <v>510</v>
       </c>
       <c r="I5" s="12" t="s">
-        <v>1497</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -5625,7 +5606,7 @@
         <v>66</v>
       </c>
       <c r="I11" s="12" t="s">
-        <v>1434</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
@@ -5965,7 +5946,7 @@
         <v>511</v>
       </c>
       <c r="J25" s="12" t="s">
-        <v>1526</v>
+        <v>1520</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
@@ -5994,7 +5975,7 @@
         <v>99</v>
       </c>
       <c r="I26" s="12" t="s">
-        <v>1468</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
@@ -6063,7 +6044,7 @@
         <v>114</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>1587</v>
+        <v>1581</v>
       </c>
       <c r="G29" s="7" t="s">
         <v>912</v>
@@ -6150,10 +6131,10 @@
         <v>99</v>
       </c>
       <c r="I32" s="12" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="J32" s="12" t="s">
-        <v>1403</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
@@ -6257,7 +6238,7 @@
         <v>66</v>
       </c>
       <c r="I36" s="12" t="s">
-        <v>1397</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
@@ -6545,10 +6526,10 @@
         <v>512</v>
       </c>
       <c r="I48" s="12" t="s">
-        <v>1503</v>
+        <v>1497</v>
       </c>
       <c r="J48" s="12" t="s">
-        <v>1502</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
@@ -6652,10 +6633,10 @@
         <v>12</v>
       </c>
       <c r="I52" s="12" t="s">
-        <v>1511</v>
+        <v>1505</v>
       </c>
       <c r="J52" s="12" t="s">
-        <v>1510</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.35">
@@ -6684,10 +6665,10 @@
         <v>12</v>
       </c>
       <c r="I53" s="12" t="s">
-        <v>1490</v>
+        <v>1484</v>
       </c>
       <c r="J53" s="12" t="s">
-        <v>1489</v>
+        <v>1483</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
@@ -6716,10 +6697,10 @@
         <v>12</v>
       </c>
       <c r="I54" s="12" t="s">
-        <v>1451</v>
+        <v>1445</v>
       </c>
       <c r="J54" s="12" t="s">
-        <v>1450</v>
+        <v>1444</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
@@ -6748,10 +6729,10 @@
         <v>12</v>
       </c>
       <c r="I55" s="12" t="s">
-        <v>1557</v>
+        <v>1551</v>
       </c>
       <c r="J55" s="12" t="s">
-        <v>1556</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.35">
@@ -6780,10 +6761,10 @@
         <v>12</v>
       </c>
       <c r="I56" s="12" t="s">
-        <v>1423</v>
+        <v>1417</v>
       </c>
       <c r="J56" s="12" t="s">
-        <v>1422</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.35">
@@ -6884,10 +6865,10 @@
         <v>12</v>
       </c>
       <c r="I60" s="12" t="s">
-        <v>1400</v>
+        <v>1396</v>
       </c>
       <c r="J60" s="12" t="s">
-        <v>1399</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.35">
@@ -7017,7 +6998,7 @@
         <v>512</v>
       </c>
       <c r="I65" s="12" t="s">
-        <v>1514</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="66" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -7046,10 +7027,10 @@
         <v>99</v>
       </c>
       <c r="I66" s="12" t="s">
-        <v>1387</v>
+        <v>1383</v>
       </c>
       <c r="J66" s="12" t="s">
-        <v>1388</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -7078,7 +7059,7 @@
         <v>99</v>
       </c>
       <c r="I67" s="12" t="s">
-        <v>1389</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.35">
@@ -7153,10 +7134,10 @@
         <v>197</v>
       </c>
       <c r="I70" s="12" t="s">
-        <v>1443</v>
+        <v>1437</v>
       </c>
       <c r="J70" s="12" t="s">
-        <v>1444</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.35">
@@ -7211,7 +7192,7 @@
         <v>66</v>
       </c>
       <c r="I72" s="12" t="s">
-        <v>1382</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.35">
@@ -7260,10 +7241,10 @@
         <v>12</v>
       </c>
       <c r="I74" s="12" t="s">
-        <v>1446</v>
+        <v>1440</v>
       </c>
       <c r="J74" s="12" t="s">
-        <v>1445</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.35">
@@ -7292,7 +7273,7 @@
         <v>405</v>
       </c>
       <c r="I75" s="12" t="s">
-        <v>1496</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.35">
@@ -7543,7 +7524,7 @@
         <v>99</v>
       </c>
       <c r="I85" s="12" t="s">
-        <v>1479</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.35">
@@ -7560,7 +7541,7 @@
         <v>579</v>
       </c>
       <c r="F86" s="12" t="s">
-        <v>1600</v>
+        <v>1594</v>
       </c>
       <c r="G86" s="7" t="s">
         <v>990</v>
@@ -7569,10 +7550,10 @@
         <v>510</v>
       </c>
       <c r="I86" s="12" t="s">
-        <v>1599</v>
+        <v>1593</v>
       </c>
       <c r="J86" s="12" t="s">
-        <v>1598</v>
+        <v>1592</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.35">
@@ -7601,10 +7582,10 @@
         <v>66</v>
       </c>
       <c r="I87" s="12" t="s">
-        <v>1521</v>
+        <v>1515</v>
       </c>
       <c r="J87" s="12" t="s">
-        <v>1520</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.35">
@@ -7962,7 +7943,7 @@
         <v>66</v>
       </c>
       <c r="I101" s="12" t="s">
-        <v>1405</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.35">
@@ -7988,7 +7969,7 @@
         <v>197</v>
       </c>
       <c r="I102" s="12" t="s">
-        <v>1575</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.35">
@@ -8095,7 +8076,7 @@
         <v>12</v>
       </c>
       <c r="I106" s="12" t="s">
-        <v>1459</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.35">
@@ -8124,7 +8105,7 @@
         <v>12</v>
       </c>
       <c r="I107" s="12" t="s">
-        <v>1432</v>
+        <v>1426</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.35">
@@ -8153,10 +8134,10 @@
         <v>511</v>
       </c>
       <c r="I108" s="12" t="s">
-        <v>1476</v>
+        <v>1470</v>
       </c>
       <c r="J108" s="12" t="s">
-        <v>1475</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.35">
@@ -8219,7 +8200,7 @@
         <v>491</v>
       </c>
       <c r="F111" s="12" t="s">
-        <v>1570</v>
+        <v>1564</v>
       </c>
       <c r="G111" s="7" t="s">
         <v>879</v>
@@ -8228,7 +8209,7 @@
         <v>510</v>
       </c>
       <c r="I111" s="12" t="s">
-        <v>1571</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.35">
@@ -8254,7 +8235,7 @@
         <v>66</v>
       </c>
       <c r="I112" s="12" t="s">
-        <v>1544</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.35">
@@ -8283,10 +8264,10 @@
         <v>66</v>
       </c>
       <c r="I113" s="12" t="s">
-        <v>1540</v>
+        <v>1534</v>
       </c>
       <c r="J113" s="12" t="s">
-        <v>1539</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.35">
@@ -8367,10 +8348,10 @@
         <v>66</v>
       </c>
       <c r="I116" s="12" t="s">
-        <v>1493</v>
+        <v>1487</v>
       </c>
       <c r="J116" s="12" t="s">
-        <v>1492</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.35">
@@ -8526,7 +8507,7 @@
         <v>12</v>
       </c>
       <c r="I122" s="12" t="s">
-        <v>1555</v>
+        <v>1549</v>
       </c>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.35">
@@ -8575,7 +8556,7 @@
         <v>510</v>
       </c>
       <c r="I124" s="12" t="s">
-        <v>1565</v>
+        <v>1559</v>
       </c>
     </row>
     <row r="125" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -8751,7 +8732,7 @@
         <v>510</v>
       </c>
       <c r="I131" s="12" t="s">
-        <v>1386</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.35">
@@ -8780,7 +8761,7 @@
         <v>511</v>
       </c>
       <c r="I132" s="12" t="s">
-        <v>1426</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="133" spans="1:10" ht="58" x14ac:dyDescent="0.35">
@@ -8855,7 +8836,7 @@
         <v>510</v>
       </c>
       <c r="I135" s="12" t="s">
-        <v>1501</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.35">
@@ -8910,10 +8891,10 @@
         <v>66</v>
       </c>
       <c r="I137" s="12" t="s">
-        <v>1470</v>
+        <v>1464</v>
       </c>
       <c r="J137" s="12" t="s">
-        <v>1469</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.35">
@@ -8962,7 +8943,7 @@
         <v>510</v>
       </c>
       <c r="I139" s="12" t="s">
-        <v>1566</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.35">
@@ -9011,7 +8992,7 @@
         <v>197</v>
       </c>
       <c r="I141" s="12" t="s">
-        <v>1594</v>
+        <v>1588</v>
       </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.35">
@@ -9037,10 +9018,10 @@
         <v>197</v>
       </c>
       <c r="I142" s="12" t="s">
-        <v>1596</v>
+        <v>1590</v>
       </c>
       <c r="J142" s="12" t="s">
-        <v>1595</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.35">
@@ -9066,10 +9047,10 @@
         <v>197</v>
       </c>
       <c r="I143" s="12" t="s">
-        <v>1519</v>
+        <v>1513</v>
       </c>
       <c r="J143" s="12" t="s">
-        <v>1518</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="144" spans="1:10" x14ac:dyDescent="0.35">
@@ -9109,7 +9090,7 @@
         <v>250</v>
       </c>
       <c r="E145" s="12" t="s">
-        <v>1572</v>
+        <v>1566</v>
       </c>
       <c r="F145" s="7" t="s">
         <v>98</v>
@@ -9121,7 +9102,7 @@
         <v>510</v>
       </c>
       <c r="I145" s="12" t="s">
-        <v>1437</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.35">
@@ -9150,7 +9131,7 @@
         <v>511</v>
       </c>
       <c r="I146" s="12" t="s">
-        <v>1407</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.35">
@@ -9179,7 +9160,7 @@
         <v>511</v>
       </c>
       <c r="I147" s="12" t="s">
-        <v>1532</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.35">
@@ -9208,7 +9189,7 @@
         <v>511</v>
       </c>
       <c r="I148" s="12" t="s">
-        <v>1458</v>
+        <v>1452</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.35">
@@ -9237,7 +9218,7 @@
         <v>510</v>
       </c>
       <c r="I149" s="12" t="s">
-        <v>1467</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.35">
@@ -9292,7 +9273,7 @@
         <v>510</v>
       </c>
       <c r="I151" s="12" t="s">
-        <v>1567</v>
+        <v>1561</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.35">
@@ -9422,7 +9403,7 @@
         <v>511</v>
       </c>
       <c r="I156" s="12" t="s">
-        <v>1527</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="157" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -9569,10 +9550,10 @@
         <v>510</v>
       </c>
       <c r="I162" s="12" t="s">
-        <v>1592</v>
+        <v>1586</v>
       </c>
       <c r="J162" s="12" t="s">
-        <v>1593</v>
+        <v>1587</v>
       </c>
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.35">
@@ -9598,10 +9579,10 @@
         <v>510</v>
       </c>
       <c r="I163" s="12" t="s">
-        <v>1568</v>
+        <v>1562</v>
       </c>
       <c r="J163" s="12" t="s">
-        <v>1569</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.35">
@@ -9699,10 +9680,10 @@
         <v>511</v>
       </c>
       <c r="I167" s="12" t="s">
-        <v>1534</v>
+        <v>1528</v>
       </c>
       <c r="J167" s="12" t="s">
-        <v>1533</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.35">
@@ -9757,10 +9738,10 @@
         <v>511</v>
       </c>
       <c r="I169" s="12" t="s">
-        <v>1418</v>
+        <v>1414</v>
       </c>
       <c r="J169" s="12" t="s">
-        <v>1417</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.35">
@@ -9884,7 +9865,7 @@
         <v>511</v>
       </c>
       <c r="I174" s="12" t="s">
-        <v>1478</v>
+        <v>1472</v>
       </c>
     </row>
     <row r="175" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -10034,10 +10015,10 @@
         <v>66</v>
       </c>
       <c r="I180" s="12" t="s">
-        <v>1439</v>
+        <v>1433</v>
       </c>
       <c r="J180" s="12" t="s">
-        <v>1438</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="181" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -10164,7 +10145,7 @@
         <v>99</v>
       </c>
       <c r="I185" s="12" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="186" spans="1:10" x14ac:dyDescent="0.35">
@@ -10242,7 +10223,7 @@
         <v>66</v>
       </c>
       <c r="I188" s="12" t="s">
-        <v>1542</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="189" spans="1:10" x14ac:dyDescent="0.35">
@@ -10297,7 +10278,7 @@
         <v>99</v>
       </c>
       <c r="I190" s="12" t="s">
-        <v>1385</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="191" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -10441,7 +10422,7 @@
         <v>66</v>
       </c>
       <c r="I196" s="12" t="s">
-        <v>1483</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="197" spans="1:10" x14ac:dyDescent="0.35">
@@ -10470,10 +10451,10 @@
         <v>12</v>
       </c>
       <c r="I197" s="12" t="s">
-        <v>1474</v>
+        <v>1468</v>
       </c>
       <c r="J197" s="12" t="s">
-        <v>1473</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="198" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -10681,7 +10662,7 @@
         <v>12</v>
       </c>
       <c r="I205" s="12" t="s">
-        <v>1515</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="206" spans="1:10" x14ac:dyDescent="0.35">
@@ -10808,7 +10789,7 @@
         <v>511</v>
       </c>
       <c r="I210" s="12" t="s">
-        <v>1513</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="211" spans="1:10" x14ac:dyDescent="0.35">
@@ -10863,7 +10844,7 @@
         <v>12</v>
       </c>
       <c r="I212" s="12" t="s">
-        <v>1480</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="213" spans="1:10" x14ac:dyDescent="0.35">
@@ -10915,10 +10896,10 @@
         <v>510</v>
       </c>
       <c r="I214" s="12" t="s">
-        <v>1564</v>
+        <v>1558</v>
       </c>
       <c r="J214" s="12" t="s">
-        <v>1563</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="215" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -11129,7 +11110,7 @@
         <v>511</v>
       </c>
       <c r="I222" s="12" t="s">
-        <v>1491</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="223" spans="1:10" x14ac:dyDescent="0.35">
@@ -11207,7 +11188,7 @@
         <v>99</v>
       </c>
       <c r="I225" s="12" t="s">
-        <v>1402</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="226" spans="1:10" x14ac:dyDescent="0.35">
@@ -11354,7 +11335,7 @@
         <v>440</v>
       </c>
       <c r="E231" s="12" t="s">
-        <v>1582</v>
+        <v>1576</v>
       </c>
       <c r="F231" s="7" t="s">
         <v>997</v>
@@ -11366,7 +11347,7 @@
         <v>653</v>
       </c>
       <c r="I231" s="12" t="s">
-        <v>1583</v>
+        <v>1577</v>
       </c>
     </row>
     <row r="232" spans="1:10" x14ac:dyDescent="0.35">
@@ -11473,10 +11454,10 @@
         <v>511</v>
       </c>
       <c r="I235" s="12" t="s">
-        <v>1525</v>
+        <v>1519</v>
       </c>
       <c r="J235" s="12" t="s">
-        <v>1524</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="236" spans="1:10" x14ac:dyDescent="0.35">
@@ -11551,7 +11532,7 @@
         <v>99</v>
       </c>
       <c r="I238" s="12" t="s">
-        <v>1442</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="239" spans="1:10" x14ac:dyDescent="0.35">
@@ -11649,7 +11630,7 @@
         <v>66</v>
       </c>
       <c r="I242" s="12" t="s">
-        <v>1535</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="243" spans="1:10" x14ac:dyDescent="0.35">
@@ -11704,7 +11685,7 @@
         <v>99</v>
       </c>
       <c r="I244" s="12" t="s">
-        <v>1410</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="245" spans="1:10" x14ac:dyDescent="0.35">
@@ -11733,10 +11714,10 @@
         <v>99</v>
       </c>
       <c r="I245" s="12" t="s">
-        <v>1471</v>
+        <v>1465</v>
       </c>
       <c r="J245" s="12" t="s">
-        <v>1472</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="246" spans="1:10" x14ac:dyDescent="0.35">
@@ -11791,10 +11772,10 @@
         <v>12</v>
       </c>
       <c r="I247" s="12" t="s">
-        <v>1561</v>
+        <v>1555</v>
       </c>
       <c r="J247" s="12" t="s">
-        <v>1560</v>
+        <v>1554</v>
       </c>
     </row>
     <row r="248" spans="1:10" x14ac:dyDescent="0.35">
@@ -11860,7 +11841,7 @@
         <v>1300</v>
       </c>
       <c r="E250" s="12" t="s">
-        <v>1429</v>
+        <v>1423</v>
       </c>
       <c r="F250" s="7" t="s">
         <v>436</v>
@@ -11872,10 +11853,10 @@
         <v>197</v>
       </c>
       <c r="I250" s="12" t="s">
-        <v>1395</v>
+        <v>1391</v>
       </c>
       <c r="J250" s="12" t="s">
-        <v>1396</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="251" spans="1:10" x14ac:dyDescent="0.35">
@@ -12103,7 +12084,7 @@
         <v>99</v>
       </c>
       <c r="I259" s="12" t="s">
-        <v>1441</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="260" spans="1:10" x14ac:dyDescent="0.35">
@@ -12132,10 +12113,10 @@
         <v>66</v>
       </c>
       <c r="I260" s="12" t="s">
-        <v>1495</v>
+        <v>1489</v>
       </c>
       <c r="J260" s="12" t="s">
-        <v>1494</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="261" spans="1:10" x14ac:dyDescent="0.35">
@@ -12259,7 +12240,7 @@
         <v>99</v>
       </c>
       <c r="I265" s="12" t="s">
-        <v>1390</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="266" spans="1:10" x14ac:dyDescent="0.35">
@@ -12314,7 +12295,7 @@
         <v>99</v>
       </c>
       <c r="I267" s="12" t="s">
-        <v>1447</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="268" spans="1:10" x14ac:dyDescent="0.35">
@@ -12343,10 +12324,10 @@
         <v>99</v>
       </c>
       <c r="I268" s="12" t="s">
-        <v>1457</v>
+        <v>1451</v>
       </c>
       <c r="J268" s="12" t="s">
-        <v>1456</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="269" spans="1:10" x14ac:dyDescent="0.35">
@@ -12375,7 +12356,7 @@
         <v>12</v>
       </c>
       <c r="I269" s="12" t="s">
-        <v>1562</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="270" spans="1:10" x14ac:dyDescent="0.35">
@@ -12430,10 +12411,10 @@
         <v>12</v>
       </c>
       <c r="I271" s="12" t="s">
-        <v>1485</v>
+        <v>1479</v>
       </c>
       <c r="J271" s="12" t="s">
-        <v>1484</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="272" spans="1:10" x14ac:dyDescent="0.35">
@@ -12462,7 +12443,7 @@
         <v>12</v>
       </c>
       <c r="I272" s="12" t="s">
-        <v>1440</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="273" spans="1:10" x14ac:dyDescent="0.35">
@@ -12491,7 +12472,7 @@
         <v>66</v>
       </c>
       <c r="I273" s="12" t="s">
-        <v>1455</v>
+        <v>1449</v>
       </c>
     </row>
     <row r="274" spans="1:10" x14ac:dyDescent="0.35">
@@ -12520,7 +12501,7 @@
         <v>66</v>
       </c>
       <c r="I274" s="12" t="s">
-        <v>1541</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="275" spans="1:10" x14ac:dyDescent="0.35">
@@ -12549,7 +12530,7 @@
         <v>66</v>
       </c>
       <c r="I275" s="12" t="s">
-        <v>1504</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="276" spans="1:10" x14ac:dyDescent="0.35">
@@ -12630,7 +12611,7 @@
         <v>99</v>
       </c>
       <c r="I278" s="12" t="s">
-        <v>1586</v>
+        <v>1580</v>
       </c>
     </row>
     <row r="279" spans="1:10" x14ac:dyDescent="0.35">
@@ -12659,10 +12640,10 @@
         <v>99</v>
       </c>
       <c r="I279" s="12" t="s">
-        <v>1591</v>
+        <v>1585</v>
       </c>
       <c r="J279" s="12" t="s">
-        <v>1590</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="280" spans="1:10" x14ac:dyDescent="0.35">
@@ -12766,10 +12747,10 @@
         <v>511</v>
       </c>
       <c r="I283" s="12" t="s">
-        <v>1531</v>
+        <v>1525</v>
       </c>
       <c r="J283" s="12" t="s">
-        <v>1530</v>
+        <v>1524</v>
       </c>
     </row>
     <row r="284" spans="1:10" x14ac:dyDescent="0.35">
@@ -12822,7 +12803,7 @@
         <v>197</v>
       </c>
       <c r="I285" s="12" t="s">
-        <v>1508</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="286" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -12851,7 +12832,7 @@
         <v>66</v>
       </c>
       <c r="I286" s="12" t="s">
-        <v>1419</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="287" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -12906,7 +12887,7 @@
         <v>197</v>
       </c>
       <c r="I288" s="12" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="289" spans="1:10" x14ac:dyDescent="0.35">
@@ -13030,10 +13011,10 @@
         <v>12</v>
       </c>
       <c r="I293" s="12" t="s">
-        <v>1559</v>
+        <v>1553</v>
       </c>
       <c r="J293" s="12" t="s">
-        <v>1558</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="294" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -13114,10 +13095,10 @@
         <v>99</v>
       </c>
       <c r="I296" s="12" t="s">
-        <v>1507</v>
+        <v>1501</v>
       </c>
       <c r="J296" s="12" t="s">
-        <v>1601</v>
+        <v>1595</v>
       </c>
     </row>
     <row r="297" spans="1:10" x14ac:dyDescent="0.35">
@@ -13146,10 +13127,10 @@
         <v>66</v>
       </c>
       <c r="I297" s="12" t="s">
-        <v>1549</v>
+        <v>1543</v>
       </c>
       <c r="J297" s="12" t="s">
-        <v>1548</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="298" spans="1:10" x14ac:dyDescent="0.35">
@@ -13178,10 +13159,10 @@
         <v>66</v>
       </c>
       <c r="I298" s="12" t="s">
-        <v>1482</v>
+        <v>1476</v>
       </c>
       <c r="J298" s="12" t="s">
-        <v>1481</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="299" spans="1:10" x14ac:dyDescent="0.35">
@@ -13210,10 +13191,10 @@
         <v>512</v>
       </c>
       <c r="I299" s="12" t="s">
-        <v>1383</v>
+        <v>1379</v>
       </c>
       <c r="J299" s="12" t="s">
-        <v>1384</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="300" spans="1:10" x14ac:dyDescent="0.35">
@@ -13242,10 +13223,10 @@
         <v>510</v>
       </c>
       <c r="I300" s="12" t="s">
-        <v>1465</v>
+        <v>1459</v>
       </c>
       <c r="J300" s="12" t="s">
-        <v>1464</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="301" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -13274,7 +13255,7 @@
         <v>510</v>
       </c>
       <c r="I301" s="12" t="s">
-        <v>1498</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="302" spans="1:10" x14ac:dyDescent="0.35">
@@ -13329,10 +13310,10 @@
         <v>12</v>
       </c>
       <c r="I303" s="12" t="s">
-        <v>1500</v>
+        <v>1494</v>
       </c>
       <c r="J303" s="12" t="s">
-        <v>1499</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="304" spans="1:10" x14ac:dyDescent="0.35">
@@ -13726,7 +13707,7 @@
         <v>12</v>
       </c>
       <c r="I320" s="12" t="s">
-        <v>1554</v>
+        <v>1548</v>
       </c>
     </row>
     <row r="321" spans="1:10" x14ac:dyDescent="0.35">
@@ -13755,7 +13736,7 @@
         <v>66</v>
       </c>
       <c r="I321" s="12" t="s">
-        <v>1545</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="322" spans="1:10" x14ac:dyDescent="0.35">
@@ -13784,10 +13765,10 @@
         <v>66</v>
       </c>
       <c r="I322" s="12" t="s">
-        <v>1449</v>
+        <v>1443</v>
       </c>
       <c r="J322" s="12" t="s">
-        <v>1448</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="323" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -13816,7 +13797,7 @@
         <v>99</v>
       </c>
       <c r="I323" s="12" t="s">
-        <v>1573</v>
+        <v>1567</v>
       </c>
     </row>
     <row r="324" spans="1:10" x14ac:dyDescent="0.35">
@@ -13842,7 +13823,7 @@
         <v>512</v>
       </c>
       <c r="I324" s="12" t="s">
-        <v>1486</v>
+        <v>1480</v>
       </c>
     </row>
     <row r="325" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -13871,7 +13852,7 @@
         <v>66</v>
       </c>
       <c r="I325" s="12" t="s">
-        <v>1453</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="326" spans="1:10" x14ac:dyDescent="0.35">
@@ -13900,10 +13881,10 @@
         <v>12</v>
       </c>
       <c r="I326" s="12" t="s">
-        <v>1551</v>
+        <v>1545</v>
       </c>
       <c r="J326" s="12" t="s">
-        <v>1550</v>
+        <v>1544</v>
       </c>
     </row>
     <row r="327" spans="1:10" x14ac:dyDescent="0.35">
@@ -13929,7 +13910,7 @@
         <v>99</v>
       </c>
       <c r="I327" s="12" t="s">
-        <v>1574</v>
+        <v>1568</v>
       </c>
     </row>
     <row r="328" spans="1:10" x14ac:dyDescent="0.35">
@@ -13955,7 +13936,7 @@
         <v>510</v>
       </c>
       <c r="I328" s="12" t="s">
-        <v>1391</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="329" spans="1:10" x14ac:dyDescent="0.35">
@@ -13978,7 +13959,7 @@
         <v>66</v>
       </c>
       <c r="I329" s="12" t="s">
-        <v>1466</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="330" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -14004,7 +13985,7 @@
         <v>99</v>
       </c>
       <c r="I330" s="12" t="s">
-        <v>1394</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="331" spans="1:10" x14ac:dyDescent="0.35">
@@ -14033,7 +14014,7 @@
         <v>66</v>
       </c>
       <c r="I331" s="12" t="s">
-        <v>1512</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="332" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -14062,10 +14043,10 @@
         <v>510</v>
       </c>
       <c r="I332" s="12" t="s">
-        <v>1517</v>
+        <v>1511</v>
       </c>
       <c r="J332" s="12" t="s">
-        <v>1516</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="333" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -14091,10 +14072,10 @@
         <v>99</v>
       </c>
       <c r="I333" s="12" t="s">
-        <v>1588</v>
+        <v>1582</v>
       </c>
       <c r="J333" s="12" t="s">
-        <v>1589</v>
+        <v>1583</v>
       </c>
     </row>
     <row r="334" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -14120,10 +14101,10 @@
         <v>99</v>
       </c>
       <c r="I334" s="12" t="s">
-        <v>1506</v>
+        <v>1500</v>
       </c>
       <c r="J334" s="12" t="s">
-        <v>1505</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="335" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -14172,7 +14153,7 @@
         <v>66</v>
       </c>
       <c r="I336" s="12" t="s">
-        <v>1536</v>
+        <v>1530</v>
       </c>
     </row>
     <row r="337" spans="1:10" x14ac:dyDescent="0.35">
@@ -14198,7 +14179,7 @@
         <v>66</v>
       </c>
       <c r="I337" s="12" t="s">
-        <v>1454</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="338" spans="1:10" x14ac:dyDescent="0.35">
@@ -14227,10 +14208,10 @@
         <v>12</v>
       </c>
       <c r="I338" s="12" t="s">
-        <v>1553</v>
+        <v>1547</v>
       </c>
       <c r="J338" s="12" t="s">
-        <v>1552</v>
+        <v>1546</v>
       </c>
     </row>
     <row r="339" spans="1:10" x14ac:dyDescent="0.35">
@@ -14302,10 +14283,10 @@
         <v>510</v>
       </c>
       <c r="I341" s="12" t="s">
-        <v>1409</v>
+        <v>1405</v>
       </c>
       <c r="J341" s="12" t="s">
-        <v>1408</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="342" spans="1:10" x14ac:dyDescent="0.35">
@@ -14331,10 +14312,10 @@
         <v>66</v>
       </c>
       <c r="I342" s="12" t="s">
-        <v>1463</v>
+        <v>1457</v>
       </c>
       <c r="J342" s="12" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
     </row>
     <row r="343" spans="1:10" x14ac:dyDescent="0.35">
@@ -14617,7 +14598,7 @@
         <v>511</v>
       </c>
       <c r="I353" s="12" t="s">
-        <v>1452</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="354" spans="1:10" x14ac:dyDescent="0.35">
@@ -14646,10 +14627,10 @@
         <v>511</v>
       </c>
       <c r="I354" s="12" t="s">
-        <v>1427</v>
+        <v>1421</v>
       </c>
       <c r="J354" s="12" t="s">
-        <v>1428</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="355" spans="1:10" x14ac:dyDescent="0.35">
@@ -14678,7 +14659,7 @@
         <v>510</v>
       </c>
       <c r="I355" s="12" t="s">
-        <v>1424</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="356" spans="1:10" x14ac:dyDescent="0.35">
@@ -14707,15 +14688,15 @@
         <v>510</v>
       </c>
       <c r="I356" s="12" t="s">
-        <v>1425</v>
+        <v>1419</v>
       </c>
     </row>
     <row r="357" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A357" s="1" t="s">
-        <v>1323</v>
+        <v>1321</v>
       </c>
       <c r="B357" s="1" t="s">
-        <v>1320</v>
+        <v>1318</v>
       </c>
       <c r="C357" s="7">
         <v>1225</v>
@@ -14736,18 +14717,18 @@
         <v>511</v>
       </c>
       <c r="I357" s="12" t="s">
-        <v>1413</v>
+        <v>1409</v>
       </c>
       <c r="J357" s="12" t="s">
-        <v>1414</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="358" spans="1:10" ht="87" x14ac:dyDescent="0.35">
       <c r="A358" s="1" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B358" s="1" t="s">
-        <v>1321</v>
+        <v>1319</v>
       </c>
       <c r="C358" s="7">
         <v>1225</v>
@@ -14768,18 +14749,18 @@
         <v>511</v>
       </c>
       <c r="I358" s="12" t="s">
-        <v>1415</v>
+        <v>1411</v>
       </c>
       <c r="J358" s="12" t="s">
-        <v>1416</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="359" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A359" s="1" t="s">
-        <v>1576</v>
+        <v>1570</v>
       </c>
       <c r="B359" s="1" t="s">
-        <v>1577</v>
+        <v>1571</v>
       </c>
       <c r="C359" s="7">
         <v>590</v>
@@ -14788,10 +14769,10 @@
         <v>400</v>
       </c>
       <c r="E359" s="12" t="s">
-        <v>1578</v>
+        <v>1572</v>
       </c>
       <c r="F359" s="12" t="s">
-        <v>1579</v>
+        <v>1573</v>
       </c>
       <c r="G359" s="7" t="s">
         <v>859</v>
@@ -14800,10 +14781,10 @@
         <v>66</v>
       </c>
       <c r="I359" s="12" t="s">
-        <v>1580</v>
+        <v>1574</v>
       </c>
       <c r="J359" s="12" t="s">
-        <v>1581</v>
+        <v>1575</v>
       </c>
     </row>
     <row r="360" spans="1:10" x14ac:dyDescent="0.35">
@@ -14832,24 +14813,24 @@
         <v>66</v>
       </c>
       <c r="I360" s="12" t="s">
-        <v>1547</v>
+        <v>1541</v>
       </c>
       <c r="J360" s="12" t="s">
-        <v>1546</v>
-      </c>
-    </row>
-    <row r="361" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>1540</v>
+      </c>
+    </row>
+    <row r="361" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A361" s="1" t="s">
-        <v>1328</v>
+        <v>1326</v>
       </c>
       <c r="B361" s="1" t="s">
-        <v>1329</v>
+        <v>1327</v>
       </c>
       <c r="C361" s="7">
-        <v>1033</v>
+        <v>614</v>
       </c>
       <c r="D361" s="7">
-        <v>675</v>
+        <v>375</v>
       </c>
       <c r="E361" s="12" t="s">
         <v>1315</v>
@@ -14863,25 +14844,19 @@
       <c r="H361" s="7" t="s">
         <v>511</v>
       </c>
-      <c r="I361" s="12" t="s">
-        <v>1421</v>
-      </c>
-      <c r="J361" s="12" t="s">
-        <v>1420</v>
-      </c>
-    </row>
-    <row r="362" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="362" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A362" s="1" t="s">
-        <v>1330</v>
+        <v>1328</v>
       </c>
       <c r="B362" s="1" t="s">
-        <v>1331</v>
+        <v>1329</v>
       </c>
       <c r="C362" s="7">
-        <v>614</v>
+        <v>946</v>
       </c>
       <c r="D362" s="7">
-        <v>375</v>
+        <v>575</v>
       </c>
       <c r="E362" s="12" t="s">
         <v>1317</v>
@@ -14895,25 +14870,31 @@
       <c r="H362" s="7" t="s">
         <v>511</v>
       </c>
-    </row>
-    <row r="363" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="I362" s="12" t="s">
+        <v>1523</v>
+      </c>
+      <c r="J362" s="12" t="s">
+        <v>1522</v>
+      </c>
+    </row>
+    <row r="363" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A363" s="1" t="s">
-        <v>1332</v>
+        <v>1322</v>
       </c>
       <c r="B363" s="1" t="s">
-        <v>1333</v>
+        <v>1323</v>
       </c>
       <c r="C363" s="7">
-        <v>946</v>
+        <v>1174</v>
       </c>
       <c r="D363" s="7">
-        <v>575</v>
+        <v>700</v>
       </c>
       <c r="E363" s="12" t="s">
-        <v>1319</v>
+        <v>1325</v>
       </c>
       <c r="F363" s="12" t="s">
-        <v>1318</v>
+        <v>1324</v>
       </c>
       <c r="G363" s="7" t="s">
         <v>859</v>
@@ -14922,106 +14903,106 @@
         <v>511</v>
       </c>
       <c r="I363" s="12" t="s">
-        <v>1529</v>
+        <v>1408</v>
       </c>
       <c r="J363" s="12" t="s">
-        <v>1528</v>
-      </c>
-    </row>
-    <row r="364" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+        <v>1407</v>
+      </c>
+    </row>
+    <row r="364" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
-        <v>1324</v>
+        <v>1330</v>
       </c>
       <c r="B364" s="1" t="s">
-        <v>1325</v>
+        <v>1331</v>
       </c>
       <c r="C364" s="7">
-        <v>1174</v>
+        <v>1395</v>
       </c>
       <c r="D364" s="7">
-        <v>700</v>
+        <v>920</v>
       </c>
       <c r="E364" s="12" t="s">
-        <v>1327</v>
+        <v>1333</v>
       </c>
       <c r="F364" s="12" t="s">
-        <v>1326</v>
+        <v>1332</v>
       </c>
       <c r="G364" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H364" s="7" t="s">
-        <v>511</v>
+        <v>66</v>
       </c>
       <c r="I364" s="12" t="s">
-        <v>1412</v>
-      </c>
-      <c r="J364" s="12" t="s">
-        <v>1411</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="365" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
+        <v>1516</v>
+      </c>
+      <c r="B365" s="1" t="s">
         <v>1334</v>
       </c>
-      <c r="B365" s="1" t="s">
+      <c r="C365" s="7">
+        <v>488</v>
+      </c>
+      <c r="D365" s="7">
+        <v>400</v>
+      </c>
+      <c r="E365" s="12" t="s">
+        <v>1336</v>
+      </c>
+      <c r="F365" s="12" t="s">
         <v>1335</v>
-      </c>
-      <c r="C365" s="7">
-        <v>1395</v>
-      </c>
-      <c r="D365" s="7">
-        <v>920</v>
-      </c>
-      <c r="E365" s="12" t="s">
-        <v>1337</v>
-      </c>
-      <c r="F365" s="12" t="s">
-        <v>1336</v>
       </c>
       <c r="G365" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H365" s="7" t="s">
-        <v>66</v>
+        <v>511</v>
       </c>
       <c r="I365" s="12" t="s">
-        <v>1401</v>
-      </c>
-    </row>
-    <row r="366" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+        <v>1471</v>
+      </c>
+      <c r="J365" s="12" t="s">
+        <v>1517</v>
+      </c>
+    </row>
+    <row r="366" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A366" s="1" t="s">
-        <v>1522</v>
+        <v>1337</v>
       </c>
       <c r="B366" s="1" t="s">
+        <v>1340</v>
+      </c>
+      <c r="C366" s="7">
+        <v>554</v>
+      </c>
+      <c r="D366" s="7">
+        <v>200</v>
+      </c>
+      <c r="E366" s="12" t="s">
+        <v>1339</v>
+      </c>
+      <c r="F366" s="12" t="s">
         <v>1338</v>
-      </c>
-      <c r="C366" s="7">
-        <v>488</v>
-      </c>
-      <c r="D366" s="7">
-        <v>400</v>
-      </c>
-      <c r="E366" s="12" t="s">
-        <v>1340</v>
-      </c>
-      <c r="F366" s="12" t="s">
-        <v>1339</v>
       </c>
       <c r="G366" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H366" s="7" t="s">
-        <v>511</v>
+        <v>12</v>
       </c>
       <c r="I366" s="12" t="s">
-        <v>1477</v>
+        <v>1579</v>
       </c>
       <c r="J366" s="12" t="s">
-        <v>1523</v>
-      </c>
-    </row>
-    <row r="367" spans="1:10" x14ac:dyDescent="0.35">
+        <v>1578</v>
+      </c>
+    </row>
+    <row r="367" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A367" s="1" t="s">
         <v>1341</v>
       </c>
@@ -15029,10 +15010,10 @@
         <v>1344</v>
       </c>
       <c r="C367" s="7">
-        <v>554</v>
+        <v>398</v>
       </c>
       <c r="D367" s="7">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="E367" s="12" t="s">
         <v>1343</v>
@@ -15044,42 +15025,39 @@
         <v>859</v>
       </c>
       <c r="H367" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I367" s="12" t="s">
-        <v>1585</v>
-      </c>
-      <c r="J367" s="12" t="s">
-        <v>1584</v>
-      </c>
-    </row>
-    <row r="368" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="368" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A368" s="1" t="s">
         <v>1345</v>
       </c>
       <c r="B368" s="1" t="s">
+        <v>1346</v>
+      </c>
+      <c r="C368" s="7">
+        <v>399</v>
+      </c>
+      <c r="D368" s="7">
+        <v>100</v>
+      </c>
+      <c r="E368" s="12" t="s">
         <v>1348</v>
       </c>
-      <c r="C368" s="7">
-        <v>398</v>
-      </c>
-      <c r="D368" s="7">
-        <v>250</v>
-      </c>
-      <c r="E368" s="12" t="s">
+      <c r="F368" s="12" t="s">
         <v>1347</v>
-      </c>
-      <c r="F368" s="12" t="s">
-        <v>1346</v>
       </c>
       <c r="G368" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H368" s="7" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="369" spans="1:10" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+      <c r="I368" s="12" t="s">
+        <v>1537</v>
+      </c>
+    </row>
+    <row r="369" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A369" s="1" t="s">
         <v>1349</v>
       </c>
@@ -15087,10 +15065,10 @@
         <v>1350</v>
       </c>
       <c r="C369" s="7">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D369" s="7">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="E369" s="12" t="s">
         <v>1352</v>
@@ -15102,13 +15080,16 @@
         <v>859</v>
       </c>
       <c r="H369" s="7" t="s">
-        <v>66</v>
+        <v>197</v>
       </c>
       <c r="I369" s="12" t="s">
-        <v>1543</v>
-      </c>
-    </row>
-    <row r="370" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>1429</v>
+      </c>
+      <c r="J369" s="12" t="s">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="370" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A370" s="1" t="s">
         <v>1353</v>
       </c>
@@ -15116,7 +15097,7 @@
         <v>1354</v>
       </c>
       <c r="C370" s="7">
-        <v>397</v>
+        <v>350</v>
       </c>
       <c r="D370" s="7">
         <v>300</v>
@@ -15131,33 +15112,33 @@
         <v>859</v>
       </c>
       <c r="H370" s="7" t="s">
-        <v>197</v>
+        <v>66</v>
       </c>
       <c r="I370" s="12" t="s">
-        <v>1435</v>
+        <v>1532</v>
       </c>
       <c r="J370" s="12" t="s">
-        <v>1436</v>
-      </c>
-    </row>
-    <row r="371" spans="1:10" x14ac:dyDescent="0.35">
+        <v>1531</v>
+      </c>
+    </row>
+    <row r="371" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A371" s="1" t="s">
-        <v>1357</v>
+        <v>1359</v>
       </c>
       <c r="B371" s="1" t="s">
-        <v>1358</v>
+        <v>1360</v>
       </c>
       <c r="C371" s="7">
-        <v>350</v>
+        <v>385</v>
       </c>
       <c r="D371" s="7">
         <v>300</v>
       </c>
       <c r="E371" s="12" t="s">
-        <v>1360</v>
+        <v>1358</v>
       </c>
       <c r="F371" s="12" t="s">
-        <v>1359</v>
+        <v>1357</v>
       </c>
       <c r="G371" s="7" t="s">
         <v>859</v>
@@ -15166,30 +15147,27 @@
         <v>66</v>
       </c>
       <c r="I371" s="12" t="s">
-        <v>1538</v>
-      </c>
-      <c r="J371" s="12" t="s">
-        <v>1537</v>
-      </c>
-    </row>
-    <row r="372" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+        <v>1425</v>
+      </c>
+    </row>
+    <row r="372" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A372" s="1" t="s">
+        <v>1362</v>
+      </c>
+      <c r="B372" s="1" t="s">
+        <v>1361</v>
+      </c>
+      <c r="C372" s="7">
+        <v>1690</v>
+      </c>
+      <c r="D372" s="7">
+        <v>1090</v>
+      </c>
+      <c r="E372" s="12" t="s">
+        <v>1424</v>
+      </c>
+      <c r="F372" s="12" t="s">
         <v>1363</v>
-      </c>
-      <c r="B372" s="1" t="s">
-        <v>1364</v>
-      </c>
-      <c r="C372" s="7">
-        <v>385</v>
-      </c>
-      <c r="D372" s="7">
-        <v>300</v>
-      </c>
-      <c r="E372" s="12" t="s">
-        <v>1362</v>
-      </c>
-      <c r="F372" s="12" t="s">
-        <v>1361</v>
       </c>
       <c r="G372" s="7" t="s">
         <v>859</v>
@@ -15198,7 +15176,7 @@
         <v>66</v>
       </c>
       <c r="I372" s="12" t="s">
-        <v>1431</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="373" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -15206,42 +15184,42 @@
         <v>1366</v>
       </c>
       <c r="B373" s="1" t="s">
+        <v>1367</v>
+      </c>
+      <c r="C373" s="7">
+        <v>1999</v>
+      </c>
+      <c r="D373" s="7">
+        <v>800</v>
+      </c>
+      <c r="E373" s="12" t="s">
         <v>1365</v>
       </c>
-      <c r="C373" s="7">
-        <v>1690</v>
-      </c>
-      <c r="D373" s="7">
-        <v>1090</v>
-      </c>
-      <c r="E373" s="12" t="s">
-        <v>1430</v>
-      </c>
       <c r="F373" s="12" t="s">
-        <v>1367</v>
+        <v>1364</v>
       </c>
       <c r="G373" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H373" s="7" t="s">
-        <v>66</v>
+        <v>197</v>
       </c>
       <c r="I373" s="12" t="s">
-        <v>1398</v>
-      </c>
-    </row>
-    <row r="374" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>1402</v>
+      </c>
+    </row>
+    <row r="374" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A374" s="1" t="s">
+        <v>1371</v>
+      </c>
+      <c r="B374" s="1" t="s">
         <v>1370</v>
       </c>
-      <c r="B374" s="1" t="s">
-        <v>1371</v>
-      </c>
       <c r="C374" s="7">
-        <v>1999</v>
+        <v>4699</v>
       </c>
       <c r="D374" s="7">
-        <v>800</v>
+        <v>2832</v>
       </c>
       <c r="E374" s="12" t="s">
         <v>1369</v>
@@ -15253,81 +15231,52 @@
         <v>859</v>
       </c>
       <c r="H374" s="7" t="s">
-        <v>197</v>
+        <v>510</v>
       </c>
       <c r="I374" s="12" t="s">
-        <v>1406</v>
-      </c>
-    </row>
-    <row r="375" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>1389</v>
+      </c>
+      <c r="J374" s="12" t="s">
+        <v>1388</v>
+      </c>
+    </row>
+    <row r="375" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A375" s="1" t="s">
+        <v>1372</v>
+      </c>
+      <c r="B375" s="1" t="s">
+        <v>1373</v>
+      </c>
+      <c r="C375" s="7">
+        <v>349</v>
+      </c>
+      <c r="D375" s="7">
+        <v>295</v>
+      </c>
+      <c r="E375" s="12" t="s">
         <v>1375</v>
       </c>
-      <c r="B375" s="1" t="s">
+      <c r="F375" s="12" t="s">
         <v>1374</v>
       </c>
-      <c r="C375" s="7">
-        <v>4699</v>
-      </c>
-      <c r="D375" s="7">
-        <v>2832</v>
-      </c>
-      <c r="E375" s="12" t="s">
-        <v>1373</v>
-      </c>
-      <c r="F375" s="12" t="s">
-        <v>1372</v>
-      </c>
       <c r="G375" s="7" t="s">
-        <v>859</v>
+        <v>419</v>
       </c>
       <c r="H375" s="7" t="s">
-        <v>510</v>
+        <v>66</v>
       </c>
       <c r="I375" s="12" t="s">
-        <v>1393</v>
+        <v>1482</v>
       </c>
       <c r="J375" s="12" t="s">
-        <v>1392</v>
+        <v>1481</v>
       </c>
     </row>
     <row r="376" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A376" s="1" t="s">
-        <v>1376</v>
-      </c>
-      <c r="B376" s="1" t="s">
-        <v>1377</v>
-      </c>
-      <c r="C376" s="7">
-        <v>349</v>
-      </c>
-      <c r="D376" s="7">
-        <v>295</v>
-      </c>
-      <c r="E376" s="12" t="s">
-        <v>1379</v>
-      </c>
-      <c r="F376" s="12" t="s">
-        <v>1378</v>
-      </c>
-      <c r="G376" s="7" t="s">
-        <v>419</v>
-      </c>
-      <c r="H376" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="I376" s="12" t="s">
-        <v>1488</v>
-      </c>
-      <c r="J376" s="12" t="s">
-        <v>1487</v>
-      </c>
-    </row>
-    <row r="377" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A377" s="13" t="s">
-        <v>1597</v>
-      </c>
-      <c r="B377" s="1"/>
+      <c r="A376" s="13" t="s">
+        <v>1591</v>
+      </c>
+      <c r="B376" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -15358,255 +15307,247 @@
     <hyperlink ref="E361" r:id="rId24"/>
     <hyperlink ref="F362" r:id="rId25"/>
     <hyperlink ref="E362" r:id="rId26"/>
-    <hyperlink ref="F363" r:id="rId27"/>
-    <hyperlink ref="E363" r:id="rId28"/>
-    <hyperlink ref="F364" r:id="rId29"/>
-    <hyperlink ref="E364" r:id="rId30"/>
-    <hyperlink ref="F365" r:id="rId31"/>
-    <hyperlink ref="E365" r:id="rId32"/>
-    <hyperlink ref="F366" r:id="rId33" location="reviews"/>
-    <hyperlink ref="E366" r:id="rId34"/>
-    <hyperlink ref="F367" r:id="rId35"/>
-    <hyperlink ref="E367" r:id="rId36"/>
-    <hyperlink ref="F368" r:id="rId37"/>
-    <hyperlink ref="E368" r:id="rId38"/>
-    <hyperlink ref="F369" r:id="rId39"/>
-    <hyperlink ref="E369" r:id="rId40"/>
-    <hyperlink ref="F370" r:id="rId41"/>
-    <hyperlink ref="E370" r:id="rId42"/>
-    <hyperlink ref="F371" r:id="rId43"/>
-    <hyperlink ref="E371" r:id="rId44"/>
-    <hyperlink ref="F372" r:id="rId45"/>
-    <hyperlink ref="E372" r:id="rId46"/>
-    <hyperlink ref="F373" r:id="rId47"/>
-    <hyperlink ref="E373" r:id="rId48"/>
-    <hyperlink ref="F374" r:id="rId49"/>
-    <hyperlink ref="E374" r:id="rId50"/>
-    <hyperlink ref="F375" r:id="rId51"/>
-    <hyperlink ref="E375" r:id="rId52"/>
-    <hyperlink ref="F376" r:id="rId53"/>
-    <hyperlink ref="E376" r:id="rId54"/>
+    <hyperlink ref="F364" r:id="rId27"/>
+    <hyperlink ref="E364" r:id="rId28"/>
+    <hyperlink ref="F365" r:id="rId29" location="reviews"/>
+    <hyperlink ref="E365" r:id="rId30"/>
+    <hyperlink ref="F366" r:id="rId31"/>
+    <hyperlink ref="E366" r:id="rId32"/>
+    <hyperlink ref="F367" r:id="rId33"/>
+    <hyperlink ref="E367" r:id="rId34"/>
+    <hyperlink ref="F368" r:id="rId35"/>
+    <hyperlink ref="E368" r:id="rId36"/>
+    <hyperlink ref="F369" r:id="rId37"/>
+    <hyperlink ref="E369" r:id="rId38"/>
+    <hyperlink ref="F370" r:id="rId39"/>
+    <hyperlink ref="E370" r:id="rId40"/>
+    <hyperlink ref="F371" r:id="rId41"/>
+    <hyperlink ref="E371" r:id="rId42"/>
+    <hyperlink ref="F372" r:id="rId43"/>
+    <hyperlink ref="E372" r:id="rId44"/>
+    <hyperlink ref="F373" r:id="rId45"/>
+    <hyperlink ref="E373" r:id="rId46"/>
+    <hyperlink ref="F374" r:id="rId47"/>
+    <hyperlink ref="E374" r:id="rId48"/>
+    <hyperlink ref="F375" r:id="rId49"/>
+    <hyperlink ref="E375" r:id="rId50"/>
     <hyperlink ref="I72" display="https://http2.mlstatic.com/D_NQ_NP_2X_977864-MLA82522530268_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_728802-MLA82808708997_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_714871-MLA82808836891_032025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="I299" r:id="rId55"/>
-    <hyperlink ref="J299" r:id="rId56"/>
+    <hyperlink ref="I299" r:id="rId51"/>
+    <hyperlink ref="J299" r:id="rId52"/>
     <hyperlink ref="I190" display="https://http2.mlstatic.com/D_NQ_NP_2X_881622-MLA100107482214_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_853470-MLA83211986807_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_889429-MLA82708797484_032025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
     <hyperlink ref="I131" display="https://http2.mlstatic.com/D_NQ_NP_2X_691159-MLA74393127536_022024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_797614-MLA74213272750_012024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_768655-MLA74336317695_012024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I66" display="https://http2.mlstatic.com/D_NQ_NP_2X_665383-MLA110622349795_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_998155-MLA109812957268_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_967066-MLA109813016698_042026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J66" r:id="rId57"/>
+    <hyperlink ref="J66" r:id="rId53"/>
     <hyperlink ref="I67" display="https://http2.mlstatic.com/D_NQ_NP_2X_754117-MLA87918629604_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_955266-MLA88256438081_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_924778-MLA88256272783_072025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I265" display="https://http2.mlstatic.com/D_NQ_NP_2X_651538-MLA109474609027_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_786870-MLA109384870397_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_877937-MLA109385877631_032026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I328" display="https://http2.mlstatic.com/D_NQ_NP_2X_659872-MLA110558100656_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_654212-MLA110558217136_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_728798-MLA110558100602_052026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J375" r:id="rId58"/>
-    <hyperlink ref="I375" r:id="rId59"/>
+    <hyperlink ref="J374" r:id="rId54"/>
+    <hyperlink ref="I374" r:id="rId55"/>
     <hyperlink ref="I330" display="https://http2.mlstatic.com/D_NQ_NP_2X_704682-MLA112632086794_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_648062-MLA114215908179_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_721338-MLA112631444306_062026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="E250" r:id="rId60"/>
-    <hyperlink ref="I250" r:id="rId61"/>
-    <hyperlink ref="J250" r:id="rId62"/>
-    <hyperlink ref="I36" r:id="rId63"/>
-    <hyperlink ref="I373" display="https://http2.mlstatic.com/D_NQ_NP_2X_870766-MLA111944165952_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_637261-MLA111944285568_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_835091-MLA112882459449_062026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J60" r:id="rId64"/>
+    <hyperlink ref="E250" r:id="rId56"/>
+    <hyperlink ref="I250" r:id="rId57"/>
+    <hyperlink ref="J250" r:id="rId58"/>
+    <hyperlink ref="I36" r:id="rId59"/>
+    <hyperlink ref="I372" display="https://http2.mlstatic.com/D_NQ_NP_2X_870766-MLA111944165952_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_637261-MLA111944285568_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_835091-MLA112882459449_062026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="J60" r:id="rId60"/>
     <hyperlink ref="I60" display="https://http2.mlstatic.com/D_NQ_NP_2X_650019-MLA112598239078_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_694102-MLA111420836191_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_960139-MLA111232526403_052026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I365" r:id="rId65"/>
+    <hyperlink ref="I364" r:id="rId61"/>
     <hyperlink ref="I225" display="https://http2.mlstatic.com/D_NQ_NP_2X_761866-MLA76203783381_052024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_967910-MLA76082310461_042024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_699850-MLA76082339489_042024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J32" r:id="rId66"/>
+    <hyperlink ref="J32" r:id="rId62"/>
     <hyperlink ref="I32" display="https://http2.mlstatic.com/D_NQ_NP_2X_937988-MLA100214376229_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_839463-MLA100214244569_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_878239-MLA100214347283_122025-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I101" display="https://http2.mlstatic.com/D_NQ_NP_2X_853469-MLA73479850047_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_636371-MLA72966055893_112023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_647337-MLA74448293715_022024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="I374" display="https://http2.mlstatic.com/D_NQ_NP_2X_838661-MLA114043475512_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_997422-MLA111845686244_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_946430-MLA112856485647_062026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I373" display="https://http2.mlstatic.com/D_NQ_NP_2X_838661-MLA114043475512_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_997422-MLA111845686244_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_946430-MLA112856485647_062026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I146" display="https://http2.mlstatic.com/D_NQ_NP_2X_700050-MLA90330537717_082025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_810830-MLA92985348779_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_611435-MLA103169335415_122025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="J341" r:id="rId67"/>
+    <hyperlink ref="J341" r:id="rId63"/>
     <hyperlink ref="I341" display="https://http2.mlstatic.com/D_NQ_NP_2X_972461-MLA108765590667_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_959062-MLA111287287492_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_702439-MLA108999676116_032026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I244" display="https://http2.mlstatic.com/D_NQ_NP_2X_772336-MLA83215360667_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_641687-MLA82926894938_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_686941-MLA80851161221_112024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J364" r:id="rId68"/>
-    <hyperlink ref="I364" display="https://http2.mlstatic.com/D_NQ_NP_2X_918751-MLA113089268495_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_972829-MLA114388137831_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_739083-MLA113884890489_062026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J357" r:id="rId69"/>
+    <hyperlink ref="J362" r:id="rId64"/>
+    <hyperlink ref="I362" display="https://http2.mlstatic.com/D_NQ_NP_2X_654570-MLA114163554383_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_820669-MLA112176540320_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_827402-MLA113697495744_072026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="J357" r:id="rId65"/>
     <hyperlink ref="I357" display="https://http2.mlstatic.com/D_NQ_NP_2X_622982-MLA91998379772_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_918567-MLA93316673763_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_951409-MLA93316693351_092025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="I358" r:id="rId70"/>
-    <hyperlink ref="J358" r:id="rId71"/>
-    <hyperlink ref="J169" r:id="rId72"/>
+    <hyperlink ref="I358" r:id="rId66"/>
+    <hyperlink ref="J358" r:id="rId67"/>
+    <hyperlink ref="J169" r:id="rId68"/>
     <hyperlink ref="I169" display="https://http2.mlstatic.com/D_NQ_NP_2X_630634-MLA83929492736_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_826427-MLA83875691856_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_778506-MLA83875632066_042025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I286" display="https://http2.mlstatic.com/D_NQ_NP_2X_601798-MLA74779553000_032024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_784677-MLA71729912500_092023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_982997-MLA73375012815_122023-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J361" r:id="rId73"/>
-    <hyperlink ref="I361" display="https://http2.mlstatic.com/D_NQ_NP_2X_743943-MLA113720575198_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_652343-MLA98742656086_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_688496-MLA89833143459_082025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="J56" r:id="rId74"/>
-    <hyperlink ref="I56" r:id="rId75"/>
-    <hyperlink ref="I355" r:id="rId76"/>
-    <hyperlink ref="I356" r:id="rId77"/>
-    <hyperlink ref="I132" r:id="rId78"/>
-    <hyperlink ref="I354" r:id="rId79"/>
-    <hyperlink ref="J354" r:id="rId80"/>
-    <hyperlink ref="I372" display="https://http2.mlstatic.com/D_NQ_NP_2X_730160-MLA112550162587_062026-F.webp;http://http2.mlstatic.com/D_NQ_NP_2X_748872-MLA113290799753_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_824232-MLA112954608093_062026-F.webp;https://http2.mlstatic.com/D_NQ"/>
-    <hyperlink ref="I107" r:id="rId81"/>
+    <hyperlink ref="J56" r:id="rId69"/>
+    <hyperlink ref="I56" r:id="rId70"/>
+    <hyperlink ref="I355" r:id="rId71"/>
+    <hyperlink ref="I356" r:id="rId72"/>
+    <hyperlink ref="I132" r:id="rId73"/>
+    <hyperlink ref="I354" r:id="rId74"/>
+    <hyperlink ref="J354" r:id="rId75"/>
+    <hyperlink ref="I371" display="https://http2.mlstatic.com/D_NQ_NP_2X_730160-MLA112550162587_062026-F.webp;http://http2.mlstatic.com/D_NQ_NP_2X_748872-MLA113290799753_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_824232-MLA112954608093_062026-F.webp;https://http2.mlstatic.com/D_NQ"/>
+    <hyperlink ref="I107" r:id="rId76"/>
     <hyperlink ref="I2" display="https://http2.mlstatic.com/D_NQ_NP_2X_644970-MLA111138624893_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_618974-MLA113557256809_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_849248-MLA111414716285_052026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I11" r:id="rId82"/>
-    <hyperlink ref="I370" r:id="rId83"/>
-    <hyperlink ref="J370" r:id="rId84"/>
-    <hyperlink ref="E145" r:id="rId85"/>
-    <hyperlink ref="I145" r:id="rId86"/>
-    <hyperlink ref="J180" r:id="rId87"/>
-    <hyperlink ref="I180" r:id="rId88"/>
-    <hyperlink ref="I272" r:id="rId89"/>
-    <hyperlink ref="I259" r:id="rId90"/>
-    <hyperlink ref="I238" r:id="rId91"/>
-    <hyperlink ref="J70" r:id="rId92"/>
-    <hyperlink ref="I70" r:id="rId93"/>
-    <hyperlink ref="J74" r:id="rId94"/>
-    <hyperlink ref="I74" r:id="rId95"/>
-    <hyperlink ref="I267" r:id="rId96"/>
-    <hyperlink ref="E251" r:id="rId97"/>
-    <hyperlink ref="J322" r:id="rId98"/>
-    <hyperlink ref="I322" r:id="rId99"/>
-    <hyperlink ref="J54" r:id="rId100"/>
-    <hyperlink ref="I54" r:id="rId101"/>
-    <hyperlink ref="I353" r:id="rId102"/>
-    <hyperlink ref="I325" r:id="rId103"/>
-    <hyperlink ref="J367" r:id="rId104"/>
-    <hyperlink ref="I367"/>
+    <hyperlink ref="I11" r:id="rId77"/>
+    <hyperlink ref="I369" r:id="rId78"/>
+    <hyperlink ref="J369" r:id="rId79"/>
+    <hyperlink ref="E145" r:id="rId80"/>
+    <hyperlink ref="I145" r:id="rId81"/>
+    <hyperlink ref="J180" r:id="rId82"/>
+    <hyperlink ref="I180" r:id="rId83"/>
+    <hyperlink ref="I272" r:id="rId84"/>
+    <hyperlink ref="I259" r:id="rId85"/>
+    <hyperlink ref="I238" r:id="rId86"/>
+    <hyperlink ref="J70" r:id="rId87"/>
+    <hyperlink ref="I70" r:id="rId88"/>
+    <hyperlink ref="J74" r:id="rId89"/>
+    <hyperlink ref="I74" r:id="rId90"/>
+    <hyperlink ref="I267" r:id="rId91"/>
+    <hyperlink ref="E251" r:id="rId92"/>
+    <hyperlink ref="J322" r:id="rId93"/>
+    <hyperlink ref="I322" r:id="rId94"/>
+    <hyperlink ref="J54" r:id="rId95"/>
+    <hyperlink ref="I54" r:id="rId96"/>
+    <hyperlink ref="I353" r:id="rId97"/>
+    <hyperlink ref="I325" r:id="rId98"/>
+    <hyperlink ref="J366" r:id="rId99"/>
+    <hyperlink ref="I366" display="https://http2.mlstatic.com/D_NQ_NP_2X_967252-MLA112857017004_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_802434-MLA114058497103_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_904877-MLA112857136140_072026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I337" display="https://http2.mlstatic.com/D_NQ_NP_2X_871513-MLA105683275105_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_921467-MLA106225093215_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_768089-MLA111241397693_052026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I273" r:id="rId105"/>
-    <hyperlink ref="J268" r:id="rId106"/>
+    <hyperlink ref="I273" r:id="rId100"/>
+    <hyperlink ref="J268" r:id="rId101"/>
     <hyperlink ref="I268" display="https://http2.mlstatic.com/D_NQ_NP_2X_723996-MLA101839595031_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_648298-MLA100279286785_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_899562-MLA105452243109_012026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I148" r:id="rId107"/>
+    <hyperlink ref="I148" r:id="rId102"/>
     <hyperlink ref="I106" display="https://http2.mlstatic.com/D_NQ_NP_2X_986480-MLA92403239851_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_992851-MLA91999385090_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_790783-MLA94732447073_102025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I185" display="https://http2.mlstatic.com/D_NQ_NP_2X_714527-MLA94159366454_102025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_847366-MLA97737335743_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_618907-MLA100261323194_122025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="I288" r:id="rId108"/>
-    <hyperlink ref="J342" r:id="rId109"/>
-    <hyperlink ref="I342" r:id="rId110"/>
-    <hyperlink ref="J300" r:id="rId111"/>
-    <hyperlink ref="I300" r:id="rId112"/>
+    <hyperlink ref="I288" r:id="rId103"/>
+    <hyperlink ref="J342" r:id="rId104"/>
+    <hyperlink ref="I342" r:id="rId105"/>
+    <hyperlink ref="J300" r:id="rId106"/>
+    <hyperlink ref="I300" r:id="rId107"/>
     <hyperlink ref="I329" display="https://http2.mlstatic.com/D_NQ_NP_2X_886751-MLA110760597980_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_722285-MLA111072136212_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_745568-MLA111456288976_052026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I149" r:id="rId113"/>
-    <hyperlink ref="I26" r:id="rId114"/>
-    <hyperlink ref="J137" r:id="rId115"/>
-    <hyperlink ref="I137" r:id="rId116"/>
-    <hyperlink ref="I245" r:id="rId117"/>
-    <hyperlink ref="J245" r:id="rId118"/>
-    <hyperlink ref="J197" r:id="rId119"/>
+    <hyperlink ref="I149" r:id="rId108"/>
+    <hyperlink ref="I26" r:id="rId109"/>
+    <hyperlink ref="J137" r:id="rId110"/>
+    <hyperlink ref="I137" r:id="rId111"/>
+    <hyperlink ref="I245" r:id="rId112"/>
+    <hyperlink ref="J245" r:id="rId113"/>
+    <hyperlink ref="J197" r:id="rId114"/>
     <hyperlink ref="I197" display="https://http2.mlstatic.com/D_NQ_NP_2X_882824-MLA78038279945_072024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_628505-MLA80605999965_112024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_605405-MLA79717879214_102024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J108" r:id="rId120"/>
-    <hyperlink ref="I108" r:id="rId121"/>
-    <hyperlink ref="I366" r:id="rId122"/>
+    <hyperlink ref="J108" r:id="rId115"/>
+    <hyperlink ref="I108" r:id="rId116"/>
+    <hyperlink ref="I365" r:id="rId117"/>
     <hyperlink ref="I174" display="https://http2.mlstatic.com/D_NQ_NP_2X_671282-MLA88303913955_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_751626-MLA88304056333_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_928886-MLA111461620111_052026-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="I85" r:id="rId123"/>
-    <hyperlink ref="I212" r:id="rId124"/>
-    <hyperlink ref="J298" r:id="rId125"/>
+    <hyperlink ref="I85" r:id="rId118"/>
+    <hyperlink ref="I212" r:id="rId119"/>
+    <hyperlink ref="J298" r:id="rId120"/>
     <hyperlink ref="I298" display="https://http2.mlstatic.com/D_NQ_NP_2X_700210-MLA112568199673_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_802525-MLA112567847565_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_792468-MLA109485788846_042026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I196" r:id="rId126"/>
-    <hyperlink ref="J271" r:id="rId127"/>
-    <hyperlink ref="I271" r:id="rId128"/>
-    <hyperlink ref="I324" r:id="rId129"/>
-    <hyperlink ref="J376" r:id="rId130"/>
-    <hyperlink ref="I376" r:id="rId131"/>
-    <hyperlink ref="J53" r:id="rId132"/>
-    <hyperlink ref="I53" r:id="rId133"/>
+    <hyperlink ref="I196" r:id="rId121"/>
+    <hyperlink ref="J271" r:id="rId122"/>
+    <hyperlink ref="I271" r:id="rId123"/>
+    <hyperlink ref="I324" r:id="rId124"/>
+    <hyperlink ref="J375" r:id="rId125"/>
+    <hyperlink ref="I375" r:id="rId126"/>
+    <hyperlink ref="J53" r:id="rId127"/>
+    <hyperlink ref="I53" r:id="rId128"/>
     <hyperlink ref="I222" display="https://http2.mlstatic.com/D_NQ_NP_2X_931197-MLA111097282025_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_647752-MLA86304062244_062025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_697099-MLA86808814199_062025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="J116" r:id="rId134"/>
+    <hyperlink ref="J116" r:id="rId129"/>
     <hyperlink ref="I116" display="https://http2.mlstatic.com/D_NQ_NP_2X_745425-MLA103761528641_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_974089-MLA111955152709_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_981681-MLA94488043029_102025-F.webp;https://http2.mlstatic.com/D_NQ"/>
-    <hyperlink ref="J260" r:id="rId135"/>
+    <hyperlink ref="J260" r:id="rId130"/>
     <hyperlink ref="I260" display="https://http2.mlstatic.com/D_NQ_NP_2X_990444-MLA85056951766_052025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_988969-MLA85056892306_052025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_982610-MLA112201389146_062026-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="I75" r:id="rId136"/>
+    <hyperlink ref="I75" r:id="rId131"/>
     <hyperlink ref="I5" display="https://http2.mlstatic.com/D_NQ_NP_2X_694398-MLA79165334679_092024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_601148-MLA79165686217_092024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_993833-MLA78690991305_082024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I301" display="https://http2.mlstatic.com/D_NQ_NP_2X_767186-MLA109412110946_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_863859-MLA110084692769_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_611180-MLA109193207080_042026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J303" r:id="rId137"/>
-    <hyperlink ref="I303" r:id="rId138"/>
+    <hyperlink ref="J303" r:id="rId132"/>
+    <hyperlink ref="I303" r:id="rId133"/>
     <hyperlink ref="I135" display="https://http2.mlstatic.com/D_NQ_NP_2X_839510-MLA85369833245_052025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_984239-MLA85369833247_052025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_909408-MLA85370025445_052025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J48" r:id="rId139"/>
+    <hyperlink ref="J48" r:id="rId134"/>
     <hyperlink ref="I48" display="https://http2.mlstatic.com/D_NQ_NP_2X_615383-MLA106283983813_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_637244-MLA106762003457_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_647036-MLA106069021004_022026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I275" r:id="rId140"/>
-    <hyperlink ref="J334" r:id="rId141"/>
+    <hyperlink ref="I275" r:id="rId135"/>
+    <hyperlink ref="J334" r:id="rId136"/>
     <hyperlink ref="I334" display="https://http2.mlstatic.com/D_NQ_NP_2X_694390-MLA103915605591_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_901157-MLA112027651816_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_930408-MLA112027361550_062026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I296" display="https://http2.mlstatic.com/D_NQ_NP_2X_877410-MLA86700953698_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_621602-MLA110823348827_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_945418-MLA86701516062_072025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="I285" r:id="rId142"/>
+    <hyperlink ref="I285" r:id="rId137"/>
     <hyperlink ref="I3" display="https://http2.mlstatic.com/D_NQ_NP_2X_652387-MLA81262109420_122024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_964100-MLA74205385415_012024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_663926-MLA71594815900_092023-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J52" r:id="rId143"/>
+    <hyperlink ref="J52" r:id="rId138"/>
     <hyperlink ref="I52" display="https://http2.mlstatic.com/D_NQ_NP_2X_787566-MLA112208805453_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_610420-MLA108420590498_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_778316-MLA108420330866_032026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I331" display="https://http2.mlstatic.com/D_NQ_NP_2X_811172-MLA108871819192_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_673692-MLA109653928111_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_807085-MLA109742422391_032026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I210" display="https://http2.mlstatic.com/D_NQ_NP_2X_787733-MLA73258839528_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_702415-MLA111282425851_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_934591-MLA108763618671_032026-F.webp;https://http2.mlstatic.com/D_NQ"/>
     <hyperlink ref="I65" display="https://http2.mlstatic.com/D_NQ_NP_2X_822004-MLA83792590685_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_922399-MLA83499949924_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_741644-MLA73913804094_012024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="I205" r:id="rId144"/>
-    <hyperlink ref="J332" r:id="rId145"/>
-    <hyperlink ref="I332" r:id="rId146"/>
+    <hyperlink ref="I205" r:id="rId139"/>
+    <hyperlink ref="J332" r:id="rId140"/>
+    <hyperlink ref="I332" r:id="rId141"/>
     <hyperlink ref="I143" display="https://http2.mlstatic.com/D_NQ_NP_2X_951908-MLA106095526036_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_697058-MLA92029170496_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_770689-MLA112170606647_052026-F.webp;https://http2.mlstatic.com/D_NQ"/>
-    <hyperlink ref="J143" r:id="rId147"/>
-    <hyperlink ref="J87" r:id="rId148"/>
-    <hyperlink ref="I87" r:id="rId149"/>
-    <hyperlink ref="J366" r:id="rId150"/>
-    <hyperlink ref="J235" r:id="rId151"/>
+    <hyperlink ref="J143" r:id="rId142"/>
+    <hyperlink ref="J87" r:id="rId143"/>
+    <hyperlink ref="I87" r:id="rId144"/>
+    <hyperlink ref="J365" r:id="rId145"/>
+    <hyperlink ref="J235" r:id="rId146"/>
     <hyperlink ref="I235" display="https://http2.mlstatic.com/D_NQ_NP_2X_786831-MLA112508605409_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_945451-MLA106951088919_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_942407-MLA79868078780_102024-F.webp;https://http2.mlstatic.com/D_NQ"/>
-    <hyperlink ref="J25" r:id="rId152"/>
-    <hyperlink ref="I156" r:id="rId153"/>
-    <hyperlink ref="J363" r:id="rId154"/>
-    <hyperlink ref="I363" display="https://http2.mlstatic.com/D_NQ_NP_2X_654570-MLA114163554383_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_820669-MLA112176540320_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_827402-MLA113697495744_072026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J283" r:id="rId155"/>
-    <hyperlink ref="I283" r:id="rId156"/>
-    <hyperlink ref="I147" r:id="rId157"/>
-    <hyperlink ref="J167" r:id="rId158"/>
+    <hyperlink ref="J25" r:id="rId147"/>
+    <hyperlink ref="I156" r:id="rId148"/>
+    <hyperlink ref="J283" r:id="rId149"/>
+    <hyperlink ref="I283" r:id="rId150"/>
+    <hyperlink ref="I147" r:id="rId151"/>
+    <hyperlink ref="J167" r:id="rId152"/>
     <hyperlink ref="I167" display="https://http2.mlstatic.com/D_NQ_NP_2X_949414-MLA115597206229_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_781530-MLA115596590455_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_794977-MLA113865153424_072026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I242" r:id="rId159"/>
-    <hyperlink ref="I336" r:id="rId160"/>
-    <hyperlink ref="J371" r:id="rId161"/>
-    <hyperlink ref="I371" r:id="rId162"/>
+    <hyperlink ref="I242" r:id="rId153"/>
+    <hyperlink ref="I336" r:id="rId154"/>
+    <hyperlink ref="J370" r:id="rId155"/>
+    <hyperlink ref="I370" r:id="rId156"/>
     <hyperlink ref="I113" display="https://http2.mlstatic.com/D_NQ_NP_2X_602967-MLA106207657120_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_937184-MLA99857184303_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_615655-MLA93805615686_102025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="J113" r:id="rId163"/>
+    <hyperlink ref="J113" r:id="rId157"/>
     <hyperlink ref="I274" display="https://http2.mlstatic.com/D_NQ_NP_2X_811367-MLA96964641173_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_724534-MLA95972455447_102025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_862711-MLA94582890276_102025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="I188" r:id="rId164"/>
-    <hyperlink ref="I369" r:id="rId165"/>
+    <hyperlink ref="I188" r:id="rId158"/>
+    <hyperlink ref="I368" r:id="rId159"/>
     <hyperlink ref="I112" display="https://http2.mlstatic.com/D_NQ_NP_2X_832809-MLA100859657141_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_651615-MLA104572148023_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_683702-MLA104248384382_012026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I321" r:id="rId166"/>
-    <hyperlink ref="J360" r:id="rId167"/>
+    <hyperlink ref="I321" r:id="rId160"/>
+    <hyperlink ref="J360" r:id="rId161"/>
     <hyperlink ref="I360" display="https://http2.mlstatic.com/D_NQ_NP_2X_986254-MLA113898749317_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_998498-MLA115220256263_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_611119-MLA113912677208_072026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I297" display="https://http2.mlstatic.com/D_NQ_NP_2X_672294-MLA110281902509_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_995715-MLA110918042491_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_936537-MLA110364709430_052026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J297" r:id="rId168"/>
-    <hyperlink ref="J326" r:id="rId169"/>
+    <hyperlink ref="J297" r:id="rId162"/>
+    <hyperlink ref="J326" r:id="rId163"/>
     <hyperlink ref="I326" display="https://http2.mlstatic.com/D_NQ_NP_2X_623123-MLA111040290746_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_934760-MLA111878498611_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_790070-MLA112661729675_062026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J338" r:id="rId170"/>
+    <hyperlink ref="J338" r:id="rId164"/>
     <hyperlink ref="I338" display="https://http2.mlstatic.com/D_NQ_NP_2X_637815-MLA110916194519_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_643077-MLA110749031212_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_708016-MLA112321199072_062026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I320" r:id="rId171"/>
-    <hyperlink ref="I122" r:id="rId172"/>
-    <hyperlink ref="J55" r:id="rId173"/>
+    <hyperlink ref="I320" r:id="rId165"/>
+    <hyperlink ref="I122" r:id="rId166"/>
+    <hyperlink ref="J55" r:id="rId167"/>
     <hyperlink ref="I55" display="https://http2.mlstatic.com/D_NQ_NP_2X_707272-MLA81406001662_122024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_992452-MLA71699440818_092023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_616985-MLA84032409756_052025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J293" r:id="rId174"/>
+    <hyperlink ref="J293" r:id="rId168"/>
     <hyperlink ref="I293" display="https://http2.mlstatic.com/D_NQ_NP_2X_699847-MLA83204192108_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_847455-MLA79932861627_102024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_823994-MLA70105011582_062023-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J247" r:id="rId175"/>
+    <hyperlink ref="J247" r:id="rId169"/>
     <hyperlink ref="I247" display="https://http2.mlstatic.com/D_NQ_NP_2X_896395-MLA74651133358_022024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_757231-MLA73307952803_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_773664-MLA113844190574_072026-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="I269" r:id="rId176"/>
-    <hyperlink ref="J214" r:id="rId177"/>
+    <hyperlink ref="I269" r:id="rId170"/>
+    <hyperlink ref="J214" r:id="rId171"/>
     <hyperlink ref="I214" display="https://http2.mlstatic.com/D_NQ_NP_2X_857704-MLA105910693631_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_785878-MLA115684445439_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_732723-MLA114610870605_072026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I124" r:id="rId178"/>
+    <hyperlink ref="I124" r:id="rId172"/>
     <hyperlink ref="I139" display="https://http2.mlstatic.com/D_NQ_NP_2X_731885-MLA81735782871_012025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_877502-MLA81736505623_012025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_739624-MLA81735782869_012025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I151" display="https://http2.mlstatic.com/D_NQ_NP_2X_852777-MLA73231184100_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_953229-MLA74068746840_012024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_727505-MLA74823139724_032024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="I163" r:id="rId179"/>
-    <hyperlink ref="J163" r:id="rId180"/>
-    <hyperlink ref="F111" r:id="rId181" location="reviews"/>
-    <hyperlink ref="I111" r:id="rId182"/>
-    <hyperlink ref="I323" r:id="rId183"/>
-    <hyperlink ref="I327" r:id="rId184"/>
+    <hyperlink ref="I163" r:id="rId173"/>
+    <hyperlink ref="J163" r:id="rId174"/>
+    <hyperlink ref="F111" r:id="rId175" location="reviews"/>
+    <hyperlink ref="I111" r:id="rId176"/>
+    <hyperlink ref="I323" r:id="rId177"/>
+    <hyperlink ref="I327" r:id="rId178"/>
     <hyperlink ref="I102" display="https://http2.mlstatic.com/D_NQ_NP_2X_701490-MLA108653774761_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_910611-MLA87584829978_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_761367-MLA87718920709_072025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="E359" r:id="rId185"/>
-    <hyperlink ref="F359" r:id="rId186"/>
+    <hyperlink ref="E359" r:id="rId179"/>
+    <hyperlink ref="F359" r:id="rId180"/>
     <hyperlink ref="I359" display="https://http2.mlstatic.com/D_NQ_NP_2X_957897-MLA114152946760_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_988648-MLA114781488773_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_938364-MLA113693419924_072026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J359" r:id="rId187"/>
-    <hyperlink ref="E231" r:id="rId188"/>
-    <hyperlink ref="I231" r:id="rId189"/>
-    <hyperlink ref="I278" r:id="rId190"/>
-    <hyperlink ref="F29" r:id="rId191"/>
-    <hyperlink ref="I333"/>
-    <hyperlink ref="J333" r:id="rId192"/>
-    <hyperlink ref="J279" r:id="rId193"/>
-    <hyperlink ref="I279"/>
-    <hyperlink ref="I162" r:id="rId194"/>
-    <hyperlink ref="J162" r:id="rId195"/>
-    <hyperlink ref="I141" r:id="rId196"/>
-    <hyperlink ref="J142" r:id="rId197"/>
-    <hyperlink ref="I142"/>
-    <hyperlink ref="J86" r:id="rId198"/>
-    <hyperlink ref="I86"/>
-    <hyperlink ref="F86" r:id="rId199"/>
-    <hyperlink ref="J296" r:id="rId200"/>
+    <hyperlink ref="J359" r:id="rId181"/>
+    <hyperlink ref="E231" r:id="rId182"/>
+    <hyperlink ref="I231" r:id="rId183"/>
+    <hyperlink ref="I278" r:id="rId184"/>
+    <hyperlink ref="F29" r:id="rId185"/>
+    <hyperlink ref="I333" display="https://http2.mlstatic.com/D_NQ_NP_2X_661292-MLA98293086467_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_907390-MLA106707175024_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_876338-MLA108047534008_032026-F.webp;https://http2.mlstatic.com/D_NQ"/>
+    <hyperlink ref="J333" r:id="rId186"/>
+    <hyperlink ref="J279" r:id="rId187"/>
+    <hyperlink ref="I279" display="https://http2.mlstatic.com/D_NQ_NP_2X_609731-MLA83282009211_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_965155-MLA83841127402_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_758965-MLA85304541601_052025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
+    <hyperlink ref="I162" r:id="rId188"/>
+    <hyperlink ref="J162" r:id="rId189"/>
+    <hyperlink ref="I141" r:id="rId190"/>
+    <hyperlink ref="J142" r:id="rId191"/>
+    <hyperlink ref="I142" display="https://http2.mlstatic.com/D_NQ_NP_2X_863418-MLA109994960812_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_927650-MLA105811665406_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_743624-MLA105810281830_022026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="J86" r:id="rId192"/>
+    <hyperlink ref="I86" display="https://http2.mlstatic.com/D_NQ_NP_2X_929447-MLA114868215933_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_688697-MLA113791320300_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_631693-MLA113790881904_072026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="F86" r:id="rId193"/>
+    <hyperlink ref="J296" r:id="rId194"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId201"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId195"/>
   <tableParts count="1">
-    <tablePart r:id="rId202"/>
+    <tablePart r:id="rId196"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualiza proyecto (2 modificados, 1 eliminado, 2 nuevos): productos.xlsx, ~$productos.xlsx, index.html
</commit_message>
<xml_diff>
--- a/datos/productos.xlsx
+++ b/datos/productos.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2419" uniqueCount="1596">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2412" uniqueCount="1591">
   <si>
     <t>Nombre</t>
   </si>
@@ -3603,20 +3603,10 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Transmisor Y Receptor Auxiliar Bluetooth 5.3 Laptop Y Coche C25 Plug C25 Negro , Adaptado Inalámbric Estéreo, Audi Alta Calidad, Conexió 3.5mm
-</t>
-  </si>
-  <si>
     <t>https://www.mercadolibre.com.mx/adaptador-bluetooth-auto-llamadas-y-musica-para-movil/up/MLMU3814435585</t>
   </si>
   <si>
     <t>https://http2.mlstatic.com/D_NQ_NP_2X_987611-MLM107926464043_032026-F.webp</t>
-  </si>
-  <si>
-    <t>https://www.mercadolibre.com.mx/naiwant-transmisor-y-receptor-auxiliar-bluetooth-53-laptop-y-coche-c25-plug-c25-negro-adaptado-inalambric-estereo-audi-alta-calidad-conexio-35mm/p/MLM65201623?pdp_filters=item_id:MLM2843434933#&amp;gid=1&amp;pid=1</t>
-  </si>
-  <si>
-    <t>https://http2.mlstatic.com/D_NQ_NP_2X_983873-MLA109780349159_032026-F.webp</t>
   </si>
   <si>
     <t xml:space="preserve">Gafas De Sol Polarizadas Con Montura Cuadrada Para Hombre
@@ -4532,12 +4522,6 @@
   </si>
   <si>
     <t>https://http2.mlstatic.com/D_NQ_NP_2X_841625-MLA90322371395_082025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_931928-MLA90286123036_082025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_613327-MLA90322341537_082025-F.webp</t>
-  </si>
-  <si>
-    <t>https://video-static-clips.mms.mlstatic.com/62c82f1f923a3f082b72612d/019e8b58f7327dada9733a33bdb6d5be/packaging/static/master.m3u8</t>
-  </si>
-  <si>
-    <t>https://http2.mlstatic.com/D_NQ_NP_2X_694390-MLA103915605591_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_901157-MLA112027651816_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_930408-MLA112027361550_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_648399-MLA112027885812_062026-F.webp</t>
   </si>
   <si>
     <t>https://http2.mlstatic.com/D_NQ_NP_2X_877410-MLA86700953698_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_621602-MLA110823348827_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_945418-MLA86701516062_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_924886-MLA109781041828_042026-F.webp</t>
@@ -4990,8 +4974,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:J376" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J376"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:J375" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J375"/>
   <sortState ref="A2:H342">
     <sortCondition ref="A1:A342"/>
   </sortState>
@@ -5296,7 +5280,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J376"/>
+  <dimension ref="A1:J375"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="70" style="1" customWidth="1"/>
@@ -5336,10 +5320,10 @@
         <v>7</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>1376</v>
+        <v>1373</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>1377</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -5362,13 +5346,13 @@
         <v>1017</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="H2" s="7" t="s">
         <v>66</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>1427</v>
+        <v>1424</v>
       </c>
       <c r="J2" s="12"/>
     </row>
@@ -5398,7 +5382,7 @@
         <v>66</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>1503</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -5450,7 +5434,7 @@
         <v>510</v>
       </c>
       <c r="I5" s="12" t="s">
-        <v>1491</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -5559,7 +5543,7 @@
         <v>834</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>1256</v>
+        <v>1253</v>
       </c>
       <c r="C10" s="7">
         <v>300</v>
@@ -5606,7 +5590,7 @@
         <v>66</v>
       </c>
       <c r="I11" s="12" t="s">
-        <v>1428</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
@@ -5946,7 +5930,7 @@
         <v>511</v>
       </c>
       <c r="J25" s="12" t="s">
-        <v>1520</v>
+        <v>1515</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
@@ -5975,7 +5959,7 @@
         <v>99</v>
       </c>
       <c r="I26" s="12" t="s">
-        <v>1462</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
@@ -6044,7 +6028,7 @@
         <v>114</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>1581</v>
+        <v>1576</v>
       </c>
       <c r="G29" s="7" t="s">
         <v>912</v>
@@ -6131,10 +6115,10 @@
         <v>99</v>
       </c>
       <c r="I32" s="12" t="s">
-        <v>1400</v>
+        <v>1397</v>
       </c>
       <c r="J32" s="12" t="s">
-        <v>1399</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
@@ -6238,15 +6222,15 @@
         <v>66</v>
       </c>
       <c r="I36" s="12" t="s">
-        <v>1393</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
-        <v>1278</v>
+        <v>1275</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>1279</v>
+        <v>1276</v>
       </c>
       <c r="C37" s="7">
         <v>300</v>
@@ -6261,7 +6245,7 @@
         <v>390</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="H37" s="7" t="s">
         <v>66</v>
@@ -6526,10 +6510,10 @@
         <v>512</v>
       </c>
       <c r="I48" s="12" t="s">
-        <v>1497</v>
+        <v>1494</v>
       </c>
       <c r="J48" s="12" t="s">
-        <v>1496</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
@@ -6633,10 +6617,10 @@
         <v>12</v>
       </c>
       <c r="I52" s="12" t="s">
-        <v>1505</v>
+        <v>1500</v>
       </c>
       <c r="J52" s="12" t="s">
-        <v>1504</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.35">
@@ -6665,10 +6649,10 @@
         <v>12</v>
       </c>
       <c r="I53" s="12" t="s">
-        <v>1484</v>
+        <v>1481</v>
       </c>
       <c r="J53" s="12" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
@@ -6697,10 +6681,10 @@
         <v>12</v>
       </c>
       <c r="I54" s="12" t="s">
-        <v>1445</v>
+        <v>1442</v>
       </c>
       <c r="J54" s="12" t="s">
-        <v>1444</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
@@ -6708,7 +6692,7 @@
         <v>207</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>1237</v>
+        <v>1234</v>
       </c>
       <c r="C55" s="7">
         <v>652</v>
@@ -6729,10 +6713,10 @@
         <v>12</v>
       </c>
       <c r="I55" s="12" t="s">
-        <v>1551</v>
+        <v>1546</v>
       </c>
       <c r="J55" s="12" t="s">
-        <v>1550</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.35">
@@ -6761,10 +6745,10 @@
         <v>12</v>
       </c>
       <c r="I56" s="12" t="s">
-        <v>1417</v>
+        <v>1414</v>
       </c>
       <c r="J56" s="12" t="s">
-        <v>1416</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.35">
@@ -6787,7 +6771,7 @@
         <v>869</v>
       </c>
       <c r="G57" s="7" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="H57" s="7" t="s">
         <v>66</v>
@@ -6853,7 +6837,7 @@
         <v>1000</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>1284</v>
+        <v>1281</v>
       </c>
       <c r="F60" s="12" t="s">
         <v>1028</v>
@@ -6865,10 +6849,10 @@
         <v>12</v>
       </c>
       <c r="I60" s="12" t="s">
-        <v>1396</v>
+        <v>1393</v>
       </c>
       <c r="J60" s="12" t="s">
-        <v>1395</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.35">
@@ -6998,7 +6982,7 @@
         <v>512</v>
       </c>
       <c r="I65" s="12" t="s">
-        <v>1508</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="66" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -7027,10 +7011,10 @@
         <v>99</v>
       </c>
       <c r="I66" s="12" t="s">
-        <v>1383</v>
+        <v>1380</v>
       </c>
       <c r="J66" s="12" t="s">
-        <v>1384</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -7059,7 +7043,7 @@
         <v>99</v>
       </c>
       <c r="I67" s="12" t="s">
-        <v>1385</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.35">
@@ -7134,10 +7118,10 @@
         <v>197</v>
       </c>
       <c r="I70" s="12" t="s">
-        <v>1437</v>
+        <v>1434</v>
       </c>
       <c r="J70" s="12" t="s">
-        <v>1438</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.35">
@@ -7192,7 +7176,7 @@
         <v>66</v>
       </c>
       <c r="I72" s="12" t="s">
-        <v>1378</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.35">
@@ -7241,10 +7225,10 @@
         <v>12</v>
       </c>
       <c r="I74" s="12" t="s">
-        <v>1440</v>
+        <v>1437</v>
       </c>
       <c r="J74" s="12" t="s">
-        <v>1439</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.35">
@@ -7273,7 +7257,7 @@
         <v>405</v>
       </c>
       <c r="I75" s="12" t="s">
-        <v>1490</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.35">
@@ -7524,7 +7508,7 @@
         <v>99</v>
       </c>
       <c r="I85" s="12" t="s">
-        <v>1473</v>
+        <v>1470</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.35">
@@ -7541,7 +7525,7 @@
         <v>579</v>
       </c>
       <c r="F86" s="12" t="s">
-        <v>1594</v>
+        <v>1589</v>
       </c>
       <c r="G86" s="7" t="s">
         <v>990</v>
@@ -7550,15 +7534,15 @@
         <v>510</v>
       </c>
       <c r="I86" s="12" t="s">
-        <v>1593</v>
+        <v>1588</v>
       </c>
       <c r="J86" s="12" t="s">
-        <v>1592</v>
+        <v>1587</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
-        <v>1268</v>
+        <v>1265</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>667</v>
@@ -7582,10 +7566,10 @@
         <v>66</v>
       </c>
       <c r="I87" s="12" t="s">
-        <v>1515</v>
+        <v>1510</v>
       </c>
       <c r="J87" s="12" t="s">
-        <v>1514</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.35">
@@ -7943,7 +7927,7 @@
         <v>66</v>
       </c>
       <c r="I101" s="12" t="s">
-        <v>1401</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.35">
@@ -7969,7 +7953,7 @@
         <v>197</v>
       </c>
       <c r="I102" s="12" t="s">
-        <v>1569</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.35">
@@ -8076,7 +8060,7 @@
         <v>12</v>
       </c>
       <c r="I106" s="12" t="s">
-        <v>1453</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.35">
@@ -8105,7 +8089,7 @@
         <v>12</v>
       </c>
       <c r="I107" s="12" t="s">
-        <v>1426</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.35">
@@ -8134,10 +8118,10 @@
         <v>511</v>
       </c>
       <c r="I108" s="12" t="s">
-        <v>1470</v>
+        <v>1467</v>
       </c>
       <c r="J108" s="12" t="s">
-        <v>1469</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.35">
@@ -8200,7 +8184,7 @@
         <v>491</v>
       </c>
       <c r="F111" s="12" t="s">
-        <v>1564</v>
+        <v>1559</v>
       </c>
       <c r="G111" s="7" t="s">
         <v>879</v>
@@ -8209,7 +8193,7 @@
         <v>510</v>
       </c>
       <c r="I111" s="12" t="s">
-        <v>1565</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.35">
@@ -8235,7 +8219,7 @@
         <v>66</v>
       </c>
       <c r="I112" s="12" t="s">
-        <v>1538</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.35">
@@ -8264,10 +8248,10 @@
         <v>66</v>
       </c>
       <c r="I113" s="12" t="s">
-        <v>1534</v>
+        <v>1529</v>
       </c>
       <c r="J113" s="12" t="s">
-        <v>1533</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.35">
@@ -8348,10 +8332,10 @@
         <v>66</v>
       </c>
       <c r="I116" s="12" t="s">
-        <v>1487</v>
+        <v>1484</v>
       </c>
       <c r="J116" s="12" t="s">
-        <v>1486</v>
+        <v>1483</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.35">
@@ -8507,7 +8491,7 @@
         <v>12</v>
       </c>
       <c r="I122" s="12" t="s">
-        <v>1549</v>
+        <v>1544</v>
       </c>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.35">
@@ -8556,7 +8540,7 @@
         <v>510</v>
       </c>
       <c r="I124" s="12" t="s">
-        <v>1559</v>
+        <v>1554</v>
       </c>
     </row>
     <row r="125" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -8732,7 +8716,7 @@
         <v>510</v>
       </c>
       <c r="I131" s="12" t="s">
-        <v>1382</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.35">
@@ -8761,7 +8745,7 @@
         <v>511</v>
       </c>
       <c r="I132" s="12" t="s">
-        <v>1420</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="133" spans="1:10" ht="58" x14ac:dyDescent="0.35">
@@ -8836,7 +8820,7 @@
         <v>510</v>
       </c>
       <c r="I135" s="12" t="s">
-        <v>1495</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.35">
@@ -8867,7 +8851,7 @@
     </row>
     <row r="137" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
-        <v>1269</v>
+        <v>1266</v>
       </c>
       <c r="B137" s="1" t="s">
         <v>1032</v>
@@ -8891,10 +8875,10 @@
         <v>66</v>
       </c>
       <c r="I137" s="12" t="s">
-        <v>1464</v>
+        <v>1461</v>
       </c>
       <c r="J137" s="12" t="s">
-        <v>1463</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.35">
@@ -8943,7 +8927,7 @@
         <v>510</v>
       </c>
       <c r="I139" s="12" t="s">
-        <v>1560</v>
+        <v>1555</v>
       </c>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.35">
@@ -8992,7 +8976,7 @@
         <v>197</v>
       </c>
       <c r="I141" s="12" t="s">
-        <v>1588</v>
+        <v>1583</v>
       </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.35">
@@ -9018,10 +9002,10 @@
         <v>197</v>
       </c>
       <c r="I142" s="12" t="s">
-        <v>1590</v>
+        <v>1585</v>
       </c>
       <c r="J142" s="12" t="s">
-        <v>1589</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.35">
@@ -9047,10 +9031,10 @@
         <v>197</v>
       </c>
       <c r="I143" s="12" t="s">
-        <v>1513</v>
+        <v>1508</v>
       </c>
       <c r="J143" s="12" t="s">
-        <v>1512</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="144" spans="1:10" x14ac:dyDescent="0.35">
@@ -9090,7 +9074,7 @@
         <v>250</v>
       </c>
       <c r="E145" s="12" t="s">
-        <v>1566</v>
+        <v>1561</v>
       </c>
       <c r="F145" s="7" t="s">
         <v>98</v>
@@ -9102,7 +9086,7 @@
         <v>510</v>
       </c>
       <c r="I145" s="12" t="s">
-        <v>1431</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.35">
@@ -9131,7 +9115,7 @@
         <v>511</v>
       </c>
       <c r="I146" s="12" t="s">
-        <v>1403</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.35">
@@ -9160,7 +9144,7 @@
         <v>511</v>
       </c>
       <c r="I147" s="12" t="s">
-        <v>1526</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.35">
@@ -9189,7 +9173,7 @@
         <v>511</v>
       </c>
       <c r="I148" s="12" t="s">
-        <v>1452</v>
+        <v>1449</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.35">
@@ -9218,7 +9202,7 @@
         <v>510</v>
       </c>
       <c r="I149" s="12" t="s">
-        <v>1461</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.35">
@@ -9273,7 +9257,7 @@
         <v>510</v>
       </c>
       <c r="I151" s="12" t="s">
-        <v>1561</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.35">
@@ -9290,7 +9274,7 @@
         <v>150</v>
       </c>
       <c r="E152" s="12" t="s">
-        <v>1289</v>
+        <v>1286</v>
       </c>
       <c r="F152" s="7" t="s">
         <v>593</v>
@@ -9374,7 +9358,7 @@
         <v>462</v>
       </c>
       <c r="G155" s="7" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="H155" s="7" t="s">
         <v>66</v>
@@ -9403,7 +9387,7 @@
         <v>511</v>
       </c>
       <c r="I156" s="12" t="s">
-        <v>1521</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="157" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -9550,10 +9534,10 @@
         <v>510</v>
       </c>
       <c r="I162" s="12" t="s">
-        <v>1586</v>
+        <v>1581</v>
       </c>
       <c r="J162" s="12" t="s">
-        <v>1587</v>
+        <v>1582</v>
       </c>
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.35">
@@ -9579,10 +9563,10 @@
         <v>510</v>
       </c>
       <c r="I163" s="12" t="s">
-        <v>1562</v>
+        <v>1557</v>
       </c>
       <c r="J163" s="12" t="s">
-        <v>1563</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.35">
@@ -9680,10 +9664,10 @@
         <v>511</v>
       </c>
       <c r="I167" s="12" t="s">
-        <v>1528</v>
+        <v>1523</v>
       </c>
       <c r="J167" s="12" t="s">
-        <v>1527</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.35">
@@ -9738,10 +9722,10 @@
         <v>511</v>
       </c>
       <c r="I169" s="12" t="s">
-        <v>1414</v>
+        <v>1411</v>
       </c>
       <c r="J169" s="12" t="s">
-        <v>1413</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.35">
@@ -9865,7 +9849,7 @@
         <v>511</v>
       </c>
       <c r="I174" s="12" t="s">
-        <v>1472</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="175" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -10015,10 +9999,10 @@
         <v>66</v>
       </c>
       <c r="I180" s="12" t="s">
-        <v>1433</v>
+        <v>1430</v>
       </c>
       <c r="J180" s="12" t="s">
-        <v>1432</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="181" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -10145,7 +10129,7 @@
         <v>99</v>
       </c>
       <c r="I185" s="12" t="s">
-        <v>1454</v>
+        <v>1451</v>
       </c>
     </row>
     <row r="186" spans="1:10" x14ac:dyDescent="0.35">
@@ -10223,7 +10207,7 @@
         <v>66</v>
       </c>
       <c r="I188" s="12" t="s">
-        <v>1536</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="189" spans="1:10" x14ac:dyDescent="0.35">
@@ -10278,7 +10262,7 @@
         <v>99</v>
       </c>
       <c r="I190" s="12" t="s">
-        <v>1381</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="191" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -10422,7 +10406,7 @@
         <v>66</v>
       </c>
       <c r="I196" s="12" t="s">
-        <v>1477</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="197" spans="1:10" x14ac:dyDescent="0.35">
@@ -10451,10 +10435,10 @@
         <v>12</v>
       </c>
       <c r="I197" s="12" t="s">
-        <v>1468</v>
+        <v>1465</v>
       </c>
       <c r="J197" s="12" t="s">
-        <v>1467</v>
+        <v>1464</v>
       </c>
     </row>
     <row r="198" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -10662,7 +10646,7 @@
         <v>12</v>
       </c>
       <c r="I205" s="12" t="s">
-        <v>1509</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="206" spans="1:10" x14ac:dyDescent="0.35">
@@ -10789,7 +10773,7 @@
         <v>511</v>
       </c>
       <c r="I210" s="12" t="s">
-        <v>1507</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="211" spans="1:10" x14ac:dyDescent="0.35">
@@ -10844,7 +10828,7 @@
         <v>12</v>
       </c>
       <c r="I212" s="12" t="s">
-        <v>1474</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="213" spans="1:10" x14ac:dyDescent="0.35">
@@ -10896,10 +10880,10 @@
         <v>510</v>
       </c>
       <c r="I214" s="12" t="s">
-        <v>1558</v>
+        <v>1553</v>
       </c>
       <c r="J214" s="12" t="s">
-        <v>1557</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="215" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -11110,7 +11094,7 @@
         <v>511</v>
       </c>
       <c r="I222" s="12" t="s">
-        <v>1485</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="223" spans="1:10" x14ac:dyDescent="0.35">
@@ -11188,7 +11172,7 @@
         <v>99</v>
       </c>
       <c r="I225" s="12" t="s">
-        <v>1398</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="226" spans="1:10" x14ac:dyDescent="0.35">
@@ -11271,7 +11255,7 @@
     </row>
     <row r="229" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
-        <v>1266</v>
+        <v>1263</v>
       </c>
       <c r="B229" s="1" t="s">
         <v>799</v>
@@ -11335,7 +11319,7 @@
         <v>440</v>
       </c>
       <c r="E231" s="12" t="s">
-        <v>1576</v>
+        <v>1571</v>
       </c>
       <c r="F231" s="7" t="s">
         <v>997</v>
@@ -11347,7 +11331,7 @@
         <v>653</v>
       </c>
       <c r="I231" s="12" t="s">
-        <v>1577</v>
+        <v>1572</v>
       </c>
     </row>
     <row r="232" spans="1:10" x14ac:dyDescent="0.35">
@@ -11454,10 +11438,10 @@
         <v>511</v>
       </c>
       <c r="I235" s="12" t="s">
-        <v>1519</v>
+        <v>1514</v>
       </c>
       <c r="J235" s="12" t="s">
-        <v>1518</v>
+        <v>1513</v>
       </c>
     </row>
     <row r="236" spans="1:10" x14ac:dyDescent="0.35">
@@ -11532,7 +11516,7 @@
         <v>99</v>
       </c>
       <c r="I238" s="12" t="s">
-        <v>1436</v>
+        <v>1433</v>
       </c>
     </row>
     <row r="239" spans="1:10" x14ac:dyDescent="0.35">
@@ -11630,7 +11614,7 @@
         <v>66</v>
       </c>
       <c r="I242" s="12" t="s">
-        <v>1529</v>
+        <v>1524</v>
       </c>
     </row>
     <row r="243" spans="1:10" x14ac:dyDescent="0.35">
@@ -11685,7 +11669,7 @@
         <v>99</v>
       </c>
       <c r="I244" s="12" t="s">
-        <v>1406</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="245" spans="1:10" x14ac:dyDescent="0.35">
@@ -11714,10 +11698,10 @@
         <v>99</v>
       </c>
       <c r="I245" s="12" t="s">
-        <v>1465</v>
+        <v>1462</v>
       </c>
       <c r="J245" s="12" t="s">
-        <v>1466</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="246" spans="1:10" x14ac:dyDescent="0.35">
@@ -11772,10 +11756,10 @@
         <v>12</v>
       </c>
       <c r="I247" s="12" t="s">
-        <v>1555</v>
+        <v>1550</v>
       </c>
       <c r="J247" s="12" t="s">
-        <v>1554</v>
+        <v>1549</v>
       </c>
     </row>
     <row r="248" spans="1:10" x14ac:dyDescent="0.35">
@@ -11841,7 +11825,7 @@
         <v>1300</v>
       </c>
       <c r="E250" s="12" t="s">
-        <v>1423</v>
+        <v>1420</v>
       </c>
       <c r="F250" s="7" t="s">
         <v>436</v>
@@ -11853,10 +11837,10 @@
         <v>197</v>
       </c>
       <c r="I250" s="12" t="s">
-        <v>1391</v>
+        <v>1388</v>
       </c>
       <c r="J250" s="12" t="s">
-        <v>1392</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="251" spans="1:10" x14ac:dyDescent="0.35">
@@ -11922,7 +11906,7 @@
         <v>600</v>
       </c>
       <c r="E253" s="12" t="s">
-        <v>1287</v>
+        <v>1284</v>
       </c>
       <c r="G253" s="7" t="s">
         <v>289</v>
@@ -11959,7 +11943,7 @@
         <v>729</v>
       </c>
       <c r="B255" s="1" t="s">
-        <v>1239</v>
+        <v>1236</v>
       </c>
       <c r="C255" s="7">
         <v>200</v>
@@ -12084,7 +12068,7 @@
         <v>99</v>
       </c>
       <c r="I259" s="12" t="s">
-        <v>1435</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="260" spans="1:10" x14ac:dyDescent="0.35">
@@ -12113,10 +12097,10 @@
         <v>66</v>
       </c>
       <c r="I260" s="12" t="s">
-        <v>1489</v>
+        <v>1486</v>
       </c>
       <c r="J260" s="12" t="s">
-        <v>1488</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="261" spans="1:10" x14ac:dyDescent="0.35">
@@ -12147,7 +12131,7 @@
     </row>
     <row r="262" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
-        <v>1240</v>
+        <v>1237</v>
       </c>
       <c r="B262" s="1" t="s">
         <v>946</v>
@@ -12240,7 +12224,7 @@
         <v>99</v>
       </c>
       <c r="I265" s="12" t="s">
-        <v>1386</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="266" spans="1:10" x14ac:dyDescent="0.35">
@@ -12295,7 +12279,7 @@
         <v>99</v>
       </c>
       <c r="I267" s="12" t="s">
-        <v>1441</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="268" spans="1:10" x14ac:dyDescent="0.35">
@@ -12324,10 +12308,10 @@
         <v>99</v>
       </c>
       <c r="I268" s="12" t="s">
-        <v>1451</v>
+        <v>1448</v>
       </c>
       <c r="J268" s="12" t="s">
-        <v>1450</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="269" spans="1:10" x14ac:dyDescent="0.35">
@@ -12356,7 +12340,7 @@
         <v>12</v>
       </c>
       <c r="I269" s="12" t="s">
-        <v>1556</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="270" spans="1:10" x14ac:dyDescent="0.35">
@@ -12373,7 +12357,7 @@
         <v>380</v>
       </c>
       <c r="E270" s="7" t="s">
-        <v>1265</v>
+        <v>1262</v>
       </c>
       <c r="F270" s="7" t="s">
         <v>444</v>
@@ -12390,7 +12374,7 @@
         <v>204</v>
       </c>
       <c r="B271" s="1" t="s">
-        <v>1235</v>
+        <v>1232</v>
       </c>
       <c r="C271" s="7">
         <v>503</v>
@@ -12411,10 +12395,10 @@
         <v>12</v>
       </c>
       <c r="I271" s="12" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
       <c r="J271" s="12" t="s">
-        <v>1478</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="272" spans="1:10" x14ac:dyDescent="0.35">
@@ -12422,7 +12406,7 @@
         <v>210</v>
       </c>
       <c r="B272" s="1" t="s">
-        <v>1236</v>
+        <v>1233</v>
       </c>
       <c r="C272" s="7">
         <v>570</v>
@@ -12443,7 +12427,7 @@
         <v>12</v>
       </c>
       <c r="I272" s="12" t="s">
-        <v>1434</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="273" spans="1:10" x14ac:dyDescent="0.35">
@@ -12466,13 +12450,13 @@
         <v>1035</v>
       </c>
       <c r="G273" s="7" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="H273" s="7" t="s">
         <v>66</v>
       </c>
       <c r="I273" s="12" t="s">
-        <v>1449</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="274" spans="1:10" x14ac:dyDescent="0.35">
@@ -12495,13 +12479,13 @@
         <v>354</v>
       </c>
       <c r="G274" s="7" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="H274" s="7" t="s">
         <v>66</v>
       </c>
       <c r="I274" s="12" t="s">
-        <v>1535</v>
+        <v>1530</v>
       </c>
     </row>
     <row r="275" spans="1:10" x14ac:dyDescent="0.35">
@@ -12524,13 +12508,13 @@
         <v>357</v>
       </c>
       <c r="G275" s="7" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="H275" s="7" t="s">
         <v>66</v>
       </c>
       <c r="I275" s="12" t="s">
-        <v>1498</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="276" spans="1:10" x14ac:dyDescent="0.35">
@@ -12611,7 +12595,7 @@
         <v>99</v>
       </c>
       <c r="I278" s="12" t="s">
-        <v>1580</v>
+        <v>1575</v>
       </c>
     </row>
     <row r="279" spans="1:10" x14ac:dyDescent="0.35">
@@ -12640,10 +12624,10 @@
         <v>99</v>
       </c>
       <c r="I279" s="12" t="s">
-        <v>1585</v>
+        <v>1580</v>
       </c>
       <c r="J279" s="12" t="s">
-        <v>1584</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="280" spans="1:10" x14ac:dyDescent="0.35">
@@ -12747,10 +12731,10 @@
         <v>511</v>
       </c>
       <c r="I283" s="12" t="s">
-        <v>1525</v>
+        <v>1520</v>
       </c>
       <c r="J283" s="12" t="s">
-        <v>1524</v>
+        <v>1519</v>
       </c>
     </row>
     <row r="284" spans="1:10" x14ac:dyDescent="0.35">
@@ -12803,7 +12787,7 @@
         <v>197</v>
       </c>
       <c r="I285" s="12" t="s">
-        <v>1502</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="286" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -12832,7 +12816,7 @@
         <v>66</v>
       </c>
       <c r="I286" s="12" t="s">
-        <v>1415</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="287" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -12887,7 +12871,7 @@
         <v>197</v>
       </c>
       <c r="I288" s="12" t="s">
-        <v>1455</v>
+        <v>1452</v>
       </c>
     </row>
     <row r="289" spans="1:10" x14ac:dyDescent="0.35">
@@ -13011,15 +12995,15 @@
         <v>12</v>
       </c>
       <c r="I293" s="12" t="s">
-        <v>1553</v>
+        <v>1548</v>
       </c>
       <c r="J293" s="12" t="s">
-        <v>1552</v>
+        <v>1547</v>
       </c>
     </row>
     <row r="294" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
-        <v>1241</v>
+        <v>1238</v>
       </c>
       <c r="B294" s="1" t="s">
         <v>1085</v>
@@ -13095,10 +13079,10 @@
         <v>99</v>
       </c>
       <c r="I296" s="12" t="s">
-        <v>1501</v>
+        <v>1496</v>
       </c>
       <c r="J296" s="12" t="s">
-        <v>1595</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="297" spans="1:10" x14ac:dyDescent="0.35">
@@ -13121,16 +13105,16 @@
         <v>1058</v>
       </c>
       <c r="G297" s="7" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="H297" s="7" t="s">
         <v>66</v>
       </c>
       <c r="I297" s="12" t="s">
-        <v>1543</v>
+        <v>1538</v>
       </c>
       <c r="J297" s="12" t="s">
-        <v>1542</v>
+        <v>1537</v>
       </c>
     </row>
     <row r="298" spans="1:10" x14ac:dyDescent="0.35">
@@ -13159,10 +13143,10 @@
         <v>66</v>
       </c>
       <c r="I298" s="12" t="s">
-        <v>1476</v>
+        <v>1473</v>
       </c>
       <c r="J298" s="12" t="s">
-        <v>1475</v>
+        <v>1472</v>
       </c>
     </row>
     <row r="299" spans="1:10" x14ac:dyDescent="0.35">
@@ -13191,10 +13175,10 @@
         <v>512</v>
       </c>
       <c r="I299" s="12" t="s">
-        <v>1379</v>
+        <v>1376</v>
       </c>
       <c r="J299" s="12" t="s">
-        <v>1380</v>
+        <v>1377</v>
       </c>
     </row>
     <row r="300" spans="1:10" x14ac:dyDescent="0.35">
@@ -13223,10 +13207,10 @@
         <v>510</v>
       </c>
       <c r="I300" s="12" t="s">
-        <v>1459</v>
+        <v>1456</v>
       </c>
       <c r="J300" s="12" t="s">
-        <v>1458</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="301" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -13255,7 +13239,7 @@
         <v>510</v>
       </c>
       <c r="I301" s="12" t="s">
-        <v>1492</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="302" spans="1:10" x14ac:dyDescent="0.35">
@@ -13310,10 +13294,10 @@
         <v>12</v>
       </c>
       <c r="I303" s="12" t="s">
-        <v>1494</v>
+        <v>1491</v>
       </c>
       <c r="J303" s="12" t="s">
-        <v>1493</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="304" spans="1:10" x14ac:dyDescent="0.35">
@@ -13442,7 +13426,7 @@
         <v>1106</v>
       </c>
       <c r="G309" s="7" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="H309" s="7" t="s">
         <v>66</v>
@@ -13470,7 +13454,7 @@
     </row>
     <row r="311" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
-        <v>1238</v>
+        <v>1235</v>
       </c>
       <c r="B311" s="1" t="s">
         <v>1114</v>
@@ -13560,7 +13544,7 @@
         <v>1124</v>
       </c>
       <c r="G314" s="7" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="H314" s="7" t="s">
         <v>66</v>
@@ -13609,7 +13593,7 @@
         <v>1132</v>
       </c>
       <c r="G316" s="7" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="H316" s="7" t="s">
         <v>66</v>
@@ -13637,7 +13621,7 @@
     </row>
     <row r="318" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
       <c r="B318" s="1" t="s">
         <v>1139</v>
@@ -13683,7 +13667,7 @@
     </row>
     <row r="320" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
-        <v>1234</v>
+        <v>1231</v>
       </c>
       <c r="B320" s="1" t="s">
         <v>1146</v>
@@ -13707,7 +13691,7 @@
         <v>12</v>
       </c>
       <c r="I320" s="12" t="s">
-        <v>1548</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="321" spans="1:10" x14ac:dyDescent="0.35">
@@ -13736,7 +13720,7 @@
         <v>66</v>
       </c>
       <c r="I321" s="12" t="s">
-        <v>1539</v>
+        <v>1534</v>
       </c>
     </row>
     <row r="322" spans="1:10" x14ac:dyDescent="0.35">
@@ -13744,7 +13728,7 @@
         <v>1153</v>
       </c>
       <c r="B322" s="1" t="s">
-        <v>1270</v>
+        <v>1267</v>
       </c>
       <c r="C322" s="7">
         <v>269</v>
@@ -13765,10 +13749,10 @@
         <v>66</v>
       </c>
       <c r="I322" s="12" t="s">
-        <v>1443</v>
+        <v>1440</v>
       </c>
       <c r="J322" s="12" t="s">
-        <v>1442</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="323" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -13797,7 +13781,7 @@
         <v>99</v>
       </c>
       <c r="I323" s="12" t="s">
-        <v>1567</v>
+        <v>1562</v>
       </c>
     </row>
     <row r="324" spans="1:10" x14ac:dyDescent="0.35">
@@ -13823,7 +13807,7 @@
         <v>512</v>
       </c>
       <c r="I324" s="12" t="s">
-        <v>1480</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="325" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -13852,7 +13836,7 @@
         <v>66</v>
       </c>
       <c r="I325" s="12" t="s">
-        <v>1447</v>
+        <v>1444</v>
       </c>
     </row>
     <row r="326" spans="1:10" x14ac:dyDescent="0.35">
@@ -13881,10 +13865,10 @@
         <v>12</v>
       </c>
       <c r="I326" s="12" t="s">
-        <v>1545</v>
+        <v>1540</v>
       </c>
       <c r="J326" s="12" t="s">
-        <v>1544</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="327" spans="1:10" x14ac:dyDescent="0.35">
@@ -13901,7 +13885,7 @@
         <v>200</v>
       </c>
       <c r="E327" s="7" t="s">
-        <v>1257</v>
+        <v>1254</v>
       </c>
       <c r="F327" s="7" t="s">
         <v>1170</v>
@@ -13910,7 +13894,7 @@
         <v>99</v>
       </c>
       <c r="I327" s="12" t="s">
-        <v>1568</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="328" spans="1:10" x14ac:dyDescent="0.35">
@@ -13927,7 +13911,7 @@
         <v>1700</v>
       </c>
       <c r="E328" s="12" t="s">
-        <v>1288</v>
+        <v>1285</v>
       </c>
       <c r="F328" s="7" t="s">
         <v>1172</v>
@@ -13936,7 +13920,7 @@
         <v>510</v>
       </c>
       <c r="I328" s="12" t="s">
-        <v>1387</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="329" spans="1:10" x14ac:dyDescent="0.35">
@@ -13959,7 +13943,7 @@
         <v>66</v>
       </c>
       <c r="I329" s="12" t="s">
-        <v>1460</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="330" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -13985,7 +13969,7 @@
         <v>99</v>
       </c>
       <c r="I330" s="12" t="s">
-        <v>1390</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="331" spans="1:10" x14ac:dyDescent="0.35">
@@ -14008,13 +13992,13 @@
         <v>1185</v>
       </c>
       <c r="G331" s="7" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="H331" s="7" t="s">
         <v>66</v>
       </c>
       <c r="I331" s="12" t="s">
-        <v>1506</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="332" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -14043,10 +14027,10 @@
         <v>510</v>
       </c>
       <c r="I332" s="12" t="s">
-        <v>1511</v>
+        <v>1506</v>
       </c>
       <c r="J332" s="12" t="s">
-        <v>1510</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="333" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -14063,33 +14047,33 @@
         <v>130</v>
       </c>
       <c r="E333" s="7" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="F333" s="7" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="H333" s="7" t="s">
         <v>99</v>
       </c>
       <c r="I333" s="12" t="s">
-        <v>1582</v>
+        <v>1577</v>
       </c>
       <c r="J333" s="12" t="s">
-        <v>1583</v>
-      </c>
-    </row>
-    <row r="334" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>1578</v>
+      </c>
+    </row>
+    <row r="334" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
-        <v>1192</v>
+        <v>1194</v>
       </c>
       <c r="B334" s="1" t="s">
-        <v>18</v>
+        <v>1197</v>
       </c>
       <c r="C334" s="7">
-        <v>269</v>
+        <v>729</v>
       </c>
       <c r="D334" s="7">
-        <v>150</v>
+        <v>350</v>
       </c>
       <c r="E334" s="7" t="s">
         <v>1196</v>
@@ -14098,27 +14082,21 @@
         <v>1195</v>
       </c>
       <c r="H334" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="I334" s="12" t="s">
-        <v>1500</v>
-      </c>
-      <c r="J334" s="12" t="s">
-        <v>1499</v>
-      </c>
-    </row>
-    <row r="335" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="335" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
-        <v>1197</v>
+        <v>1200</v>
       </c>
       <c r="B335" s="1" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="C335" s="7">
-        <v>729</v>
+        <v>1299</v>
       </c>
       <c r="D335" s="7">
-        <v>350</v>
+        <v>650</v>
       </c>
       <c r="E335" s="7" t="s">
         <v>1199</v>
@@ -14127,47 +14105,50 @@
         <v>1198</v>
       </c>
       <c r="H335" s="7" t="s">
-        <v>197</v>
+        <v>66</v>
+      </c>
+      <c r="I335" s="12" t="s">
+        <v>1525</v>
       </c>
     </row>
     <row r="336" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A336" s="1" t="s">
+        <v>1202</v>
+      </c>
+      <c r="B336" s="1" t="s">
         <v>1203</v>
       </c>
-      <c r="B336" s="1" t="s">
+      <c r="C336" s="7">
+        <v>350</v>
+      </c>
+      <c r="D336" s="7">
+        <v>200</v>
+      </c>
+      <c r="E336" s="7" t="s">
+        <v>1205</v>
+      </c>
+      <c r="F336" s="7" t="s">
         <v>1204</v>
-      </c>
-      <c r="C336" s="7">
-        <v>1299</v>
-      </c>
-      <c r="D336" s="7">
-        <v>650</v>
-      </c>
-      <c r="E336" s="7" t="s">
-        <v>1202</v>
-      </c>
-      <c r="F336" s="7" t="s">
-        <v>1201</v>
       </c>
       <c r="H336" s="7" t="s">
         <v>66</v>
       </c>
       <c r="I336" s="12" t="s">
-        <v>1530</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="337" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A337" s="1" t="s">
-        <v>1205</v>
-      </c>
-      <c r="B337" s="1" t="s">
         <v>1206</v>
       </c>
+      <c r="B337" s="1">
+        <v>126</v>
+      </c>
       <c r="C337" s="7">
-        <v>350</v>
+        <v>247</v>
       </c>
       <c r="D337" s="7">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="E337" s="7" t="s">
         <v>1208</v>
@@ -14175,80 +14156,77 @@
       <c r="F337" s="7" t="s">
         <v>1207</v>
       </c>
+      <c r="G337" s="7" t="s">
+        <v>917</v>
+      </c>
       <c r="H337" s="7" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="I337" s="12" t="s">
-        <v>1448</v>
+        <v>1542</v>
+      </c>
+      <c r="J337" s="12" t="s">
+        <v>1541</v>
       </c>
     </row>
     <row r="338" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A338" s="1" t="s">
+        <v>1211</v>
+      </c>
+      <c r="B338" s="1" t="s">
+        <v>1212</v>
+      </c>
+      <c r="C338" s="7">
+        <v>150</v>
+      </c>
+      <c r="D338" s="7">
+        <v>100</v>
+      </c>
+      <c r="E338" s="7" t="s">
+        <v>1210</v>
+      </c>
+      <c r="F338" s="7" t="s">
         <v>1209</v>
       </c>
-      <c r="B338" s="1">
-        <v>126</v>
-      </c>
-      <c r="C338" s="7">
-        <v>247</v>
-      </c>
-      <c r="D338" s="7">
-        <v>120</v>
-      </c>
-      <c r="E338" s="7" t="s">
-        <v>1211</v>
-      </c>
-      <c r="F338" s="7" t="s">
-        <v>1210</v>
-      </c>
-      <c r="G338" s="7" t="s">
-        <v>917</v>
-      </c>
       <c r="H338" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I338" s="12" t="s">
-        <v>1547</v>
-      </c>
-      <c r="J338" s="12" t="s">
-        <v>1546</v>
-      </c>
-    </row>
-    <row r="339" spans="1:10" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="339" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A339" s="1" t="s">
+        <v>1213</v>
+      </c>
+      <c r="B339" s="1" t="s">
         <v>1214</v>
       </c>
-      <c r="B339" s="1" t="s">
+      <c r="C339" s="7">
+        <v>349</v>
+      </c>
+      <c r="D339" s="7">
+        <v>200</v>
+      </c>
+      <c r="E339" s="7" t="s">
+        <v>1216</v>
+      </c>
+      <c r="F339" s="7" t="s">
         <v>1215</v>
-      </c>
-      <c r="C339" s="7">
-        <v>150</v>
-      </c>
-      <c r="D339" s="7">
-        <v>100</v>
-      </c>
-      <c r="E339" s="7" t="s">
-        <v>1213</v>
-      </c>
-      <c r="F339" s="7" t="s">
-        <v>1212</v>
       </c>
       <c r="H339" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="340" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A340" s="1" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="B340" s="1" t="s">
-        <v>1217</v>
+        <v>1220</v>
       </c>
       <c r="C340" s="7">
-        <v>349</v>
+        <v>800</v>
       </c>
       <c r="D340" s="7">
-        <v>200</v>
+        <v>750</v>
       </c>
       <c r="E340" s="7" t="s">
         <v>1219</v>
@@ -14257,21 +14235,27 @@
         <v>1218</v>
       </c>
       <c r="H340" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="341" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+        <v>510</v>
+      </c>
+      <c r="I340" s="12" t="s">
+        <v>1402</v>
+      </c>
+      <c r="J340" s="12" t="s">
+        <v>1401</v>
+      </c>
+    </row>
+    <row r="341" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A341" s="1" t="s">
-        <v>1220</v>
+        <v>1223</v>
       </c>
       <c r="B341" s="1" t="s">
-        <v>1223</v>
+        <v>1224</v>
       </c>
       <c r="C341" s="7">
-        <v>800</v>
+        <v>200</v>
       </c>
       <c r="D341" s="7">
-        <v>750</v>
+        <v>170</v>
       </c>
       <c r="E341" s="7" t="s">
         <v>1222</v>
@@ -14280,65 +14264,62 @@
         <v>1221</v>
       </c>
       <c r="H341" s="7" t="s">
-        <v>510</v>
+        <v>66</v>
       </c>
       <c r="I341" s="12" t="s">
-        <v>1405</v>
+        <v>1454</v>
       </c>
       <c r="J341" s="12" t="s">
-        <v>1404</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="342" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A342" s="1" t="s">
+        <v>1273</v>
+      </c>
+      <c r="B342" s="1" t="s">
         <v>1226</v>
       </c>
-      <c r="B342" s="1" t="s">
+      <c r="C342" s="7">
+        <v>399</v>
+      </c>
+      <c r="D342" s="7">
+        <v>250</v>
+      </c>
+      <c r="E342" s="7" t="s">
+        <v>1228</v>
+      </c>
+      <c r="F342" s="7" t="s">
         <v>1227</v>
       </c>
-      <c r="C342" s="7">
-        <v>200</v>
-      </c>
-      <c r="D342" s="7">
-        <v>170</v>
-      </c>
-      <c r="E342" s="7" t="s">
-        <v>1225</v>
-      </c>
-      <c r="F342" s="7" t="s">
-        <v>1224</v>
+      <c r="G342" s="7" t="s">
+        <v>1272</v>
       </c>
       <c r="H342" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I342" s="12" t="s">
-        <v>1457</v>
-      </c>
-      <c r="J342" s="12" t="s">
-        <v>1456</v>
-      </c>
     </row>
     <row r="343" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A343" s="1" t="s">
-        <v>1276</v>
+        <v>1274</v>
       </c>
       <c r="B343" s="1" t="s">
-        <v>1229</v>
+        <v>1225</v>
       </c>
       <c r="C343" s="7">
         <v>399</v>
       </c>
       <c r="D343" s="7">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="E343" s="7" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="F343" s="7" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
       <c r="G343" s="7" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="H343" s="7" t="s">
         <v>66</v>
@@ -14346,28 +14327,28 @@
     </row>
     <row r="344" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A344" s="1" t="s">
-        <v>1277</v>
+        <v>1239</v>
       </c>
       <c r="B344" s="1" t="s">
-        <v>1228</v>
+        <v>1245</v>
       </c>
       <c r="C344" s="7">
-        <v>399</v>
+        <v>170</v>
       </c>
       <c r="D344" s="7">
-        <v>230</v>
+        <v>150</v>
       </c>
       <c r="E344" s="7" t="s">
-        <v>1233</v>
+        <v>1241</v>
       </c>
       <c r="F344" s="7" t="s">
-        <v>1232</v>
+        <v>1240</v>
       </c>
       <c r="G344" s="7" t="s">
-        <v>1275</v>
+        <v>917</v>
       </c>
       <c r="H344" s="7" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
     </row>
     <row r="345" spans="1:10" x14ac:dyDescent="0.35">
@@ -14375,13 +14356,13 @@
         <v>1242</v>
       </c>
       <c r="B345" s="1" t="s">
-        <v>1248</v>
+        <v>1246</v>
       </c>
       <c r="C345" s="7">
-        <v>170</v>
+        <v>262</v>
       </c>
       <c r="D345" s="7">
-        <v>150</v>
+        <v>190</v>
       </c>
       <c r="E345" s="7" t="s">
         <v>1244</v>
@@ -14398,22 +14379,22 @@
     </row>
     <row r="346" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A346" s="1" t="s">
-        <v>1245</v>
+        <v>1247</v>
       </c>
       <c r="B346" s="1" t="s">
+        <v>1257</v>
+      </c>
+      <c r="C346" s="7">
+        <v>468</v>
+      </c>
+      <c r="D346" s="7">
+        <v>255</v>
+      </c>
+      <c r="E346" s="7" t="s">
         <v>1249</v>
       </c>
-      <c r="C346" s="7">
-        <v>262</v>
-      </c>
-      <c r="D346" s="7">
-        <v>190</v>
-      </c>
-      <c r="E346" s="7" t="s">
-        <v>1247</v>
-      </c>
       <c r="F346" s="7" t="s">
-        <v>1246</v>
+        <v>1248</v>
       </c>
       <c r="G346" s="7" t="s">
         <v>917</v>
@@ -14427,13 +14408,13 @@
         <v>1250</v>
       </c>
       <c r="B347" s="1" t="s">
-        <v>1260</v>
+        <v>9</v>
       </c>
       <c r="C347" s="7">
-        <v>468</v>
+        <v>299</v>
       </c>
       <c r="D347" s="7">
-        <v>255</v>
+        <v>150</v>
       </c>
       <c r="E347" s="7" t="s">
         <v>1252</v>
@@ -14450,22 +14431,22 @@
     </row>
     <row r="348" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A348" s="1" t="s">
-        <v>1253</v>
+        <v>1255</v>
       </c>
       <c r="B348" s="1" t="s">
-        <v>9</v>
+        <v>1256</v>
       </c>
       <c r="C348" s="7">
-        <v>299</v>
+        <v>447</v>
       </c>
       <c r="D348" s="7">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="E348" s="7" t="s">
-        <v>1255</v>
+        <v>1258</v>
       </c>
       <c r="F348" s="7" t="s">
-        <v>1254</v>
+        <v>1259</v>
       </c>
       <c r="G348" s="7" t="s">
         <v>917</v>
@@ -14474,47 +14455,47 @@
         <v>12</v>
       </c>
     </row>
-    <row r="349" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A349" s="1" t="s">
-        <v>1258</v>
+        <v>1260</v>
       </c>
       <c r="B349" s="1" t="s">
-        <v>1259</v>
+        <v>1283</v>
       </c>
       <c r="C349" s="7">
-        <v>447</v>
-      </c>
-      <c r="D349" s="7">
-        <v>250</v>
-      </c>
-      <c r="E349" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="E349" s="12" t="s">
+        <v>1282</v>
+      </c>
+      <c r="F349" s="7" t="s">
         <v>1261</v>
       </c>
-      <c r="F349" s="7" t="s">
-        <v>1262</v>
-      </c>
-      <c r="G349" s="7" t="s">
-        <v>917</v>
-      </c>
       <c r="H349" s="7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="350" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="350" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A350" s="1" t="s">
-        <v>1263</v>
+        <v>1268</v>
       </c>
       <c r="B350" s="1" t="s">
-        <v>1286</v>
+        <v>1269</v>
       </c>
       <c r="C350" s="7">
-        <v>350</v>
-      </c>
-      <c r="E350" s="12" t="s">
-        <v>1285</v>
+        <v>200</v>
+      </c>
+      <c r="D350" s="7">
+        <v>120</v>
+      </c>
+      <c r="E350" s="7" t="s">
+        <v>1271</v>
       </c>
       <c r="F350" s="7" t="s">
-        <v>1264</v>
+        <v>1270</v>
+      </c>
+      <c r="G350" s="7" t="s">
+        <v>419</v>
       </c>
       <c r="H350" s="7" t="s">
         <v>66</v>
@@ -14522,22 +14503,22 @@
     </row>
     <row r="351" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A351" s="1" t="s">
-        <v>1271</v>
+        <v>1277</v>
       </c>
       <c r="B351" s="1" t="s">
-        <v>1272</v>
+        <v>1278</v>
       </c>
       <c r="C351" s="7">
-        <v>200</v>
+        <v>147</v>
       </c>
       <c r="D351" s="7">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="E351" s="7" t="s">
-        <v>1274</v>
+        <v>1280</v>
       </c>
       <c r="F351" s="7" t="s">
-        <v>1273</v>
+        <v>1279</v>
       </c>
       <c r="G351" s="7" t="s">
         <v>419</v>
@@ -14546,50 +14527,53 @@
         <v>66</v>
       </c>
     </row>
-    <row r="352" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A352" s="1" t="s">
-        <v>1280</v>
+        <v>1287</v>
       </c>
       <c r="B352" s="1" t="s">
-        <v>1281</v>
+        <v>1288</v>
       </c>
       <c r="C352" s="7">
-        <v>147</v>
+        <v>899</v>
       </c>
       <c r="D352" s="7">
-        <v>100</v>
-      </c>
-      <c r="E352" s="7" t="s">
-        <v>1283</v>
-      </c>
-      <c r="F352" s="7" t="s">
-        <v>1282</v>
+        <v>485</v>
+      </c>
+      <c r="E352" s="12" t="s">
+        <v>1290</v>
+      </c>
+      <c r="F352" s="12" t="s">
+        <v>1289</v>
       </c>
       <c r="G352" s="7" t="s">
-        <v>419</v>
+        <v>859</v>
       </c>
       <c r="H352" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="353" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>511</v>
+      </c>
+      <c r="I352" s="12" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="353" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A353" s="1" t="s">
-        <v>1290</v>
+        <v>1291</v>
       </c>
       <c r="B353" s="1" t="s">
-        <v>1291</v>
+        <v>1292</v>
       </c>
       <c r="C353" s="7">
-        <v>899</v>
+        <v>1050</v>
       </c>
       <c r="D353" s="7">
-        <v>485</v>
+        <v>600</v>
       </c>
       <c r="E353" s="12" t="s">
+        <v>1294</v>
+      </c>
+      <c r="F353" s="12" t="s">
         <v>1293</v>
-      </c>
-      <c r="F353" s="12" t="s">
-        <v>1292</v>
       </c>
       <c r="G353" s="7" t="s">
         <v>859</v>
@@ -14598,59 +14582,59 @@
         <v>511</v>
       </c>
       <c r="I353" s="12" t="s">
-        <v>1446</v>
+        <v>1418</v>
+      </c>
+      <c r="J353" s="12" t="s">
+        <v>1419</v>
       </c>
     </row>
     <row r="354" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A354" s="1" t="s">
-        <v>1294</v>
+        <v>1295</v>
       </c>
       <c r="B354" s="1" t="s">
-        <v>1295</v>
+        <v>1296</v>
       </c>
       <c r="C354" s="7">
-        <v>1050</v>
+        <v>1084</v>
       </c>
       <c r="D354" s="7">
-        <v>600</v>
+        <v>650</v>
       </c>
       <c r="E354" s="12" t="s">
+        <v>1298</v>
+      </c>
+      <c r="F354" s="12" t="s">
         <v>1297</v>
-      </c>
-      <c r="F354" s="12" t="s">
-        <v>1296</v>
       </c>
       <c r="G354" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H354" s="7" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="I354" s="12" t="s">
-        <v>1421</v>
-      </c>
-      <c r="J354" s="12" t="s">
-        <v>1422</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="355" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A355" s="1" t="s">
-        <v>1298</v>
+        <v>1301</v>
       </c>
       <c r="B355" s="1" t="s">
-        <v>1299</v>
+        <v>1302</v>
       </c>
       <c r="C355" s="7">
-        <v>1084</v>
+        <v>1265</v>
       </c>
       <c r="D355" s="7">
         <v>650</v>
       </c>
       <c r="E355" s="12" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="F355" s="12" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="G355" s="7" t="s">
         <v>859</v>
@@ -14659,44 +14643,47 @@
         <v>510</v>
       </c>
       <c r="I355" s="12" t="s">
-        <v>1418</v>
-      </c>
-    </row>
-    <row r="356" spans="1:10" x14ac:dyDescent="0.35">
+        <v>1416</v>
+      </c>
+    </row>
+    <row r="356" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A356" s="1" t="s">
+        <v>1318</v>
+      </c>
+      <c r="B356" s="1" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C356" s="7">
+        <v>1225</v>
+      </c>
+      <c r="D356" s="7">
+        <v>700</v>
+      </c>
+      <c r="E356" s="12" t="s">
         <v>1304</v>
       </c>
-      <c r="B356" s="1" t="s">
-        <v>1305</v>
-      </c>
-      <c r="C356" s="7">
-        <v>1265</v>
-      </c>
-      <c r="D356" s="7">
-        <v>650</v>
-      </c>
-      <c r="E356" s="12" t="s">
+      <c r="F356" s="12" t="s">
         <v>1303</v>
-      </c>
-      <c r="F356" s="12" t="s">
-        <v>1302</v>
       </c>
       <c r="G356" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H356" s="7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="I356" s="12" t="s">
-        <v>1419</v>
-      </c>
-    </row>
-    <row r="357" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+        <v>1406</v>
+      </c>
+      <c r="J356" s="12" t="s">
+        <v>1407</v>
+      </c>
+    </row>
+    <row r="357" spans="1:10" ht="87" x14ac:dyDescent="0.35">
       <c r="A357" s="1" t="s">
-        <v>1321</v>
+        <v>1317</v>
       </c>
       <c r="B357" s="1" t="s">
-        <v>1318</v>
+        <v>1316</v>
       </c>
       <c r="C357" s="7">
         <v>1225</v>
@@ -14705,10 +14692,10 @@
         <v>700</v>
       </c>
       <c r="E357" s="12" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="F357" s="12" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="G357" s="7" t="s">
         <v>859</v>
@@ -14717,62 +14704,62 @@
         <v>511</v>
       </c>
       <c r="I357" s="12" t="s">
+        <v>1408</v>
+      </c>
+      <c r="J357" s="12" t="s">
         <v>1409</v>
       </c>
-      <c r="J357" s="12" t="s">
-        <v>1410</v>
-      </c>
-    </row>
-    <row r="358" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+    </row>
+    <row r="358" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A358" s="1" t="s">
-        <v>1320</v>
+        <v>1565</v>
       </c>
       <c r="B358" s="1" t="s">
-        <v>1319</v>
+        <v>1566</v>
       </c>
       <c r="C358" s="7">
-        <v>1225</v>
+        <v>590</v>
       </c>
       <c r="D358" s="7">
-        <v>700</v>
+        <v>400</v>
       </c>
       <c r="E358" s="12" t="s">
-        <v>1309</v>
+        <v>1567</v>
       </c>
       <c r="F358" s="12" t="s">
-        <v>1308</v>
+        <v>1568</v>
       </c>
       <c r="G358" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H358" s="7" t="s">
-        <v>511</v>
+        <v>66</v>
       </c>
       <c r="I358" s="12" t="s">
-        <v>1411</v>
+        <v>1569</v>
       </c>
       <c r="J358" s="12" t="s">
-        <v>1412</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="359" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A359" s="1" t="s">
-        <v>1570</v>
+        <v>1309</v>
       </c>
       <c r="B359" s="1" t="s">
-        <v>1571</v>
+        <v>1310</v>
       </c>
       <c r="C359" s="7">
-        <v>590</v>
+        <v>535</v>
       </c>
       <c r="D359" s="7">
         <v>400</v>
       </c>
       <c r="E359" s="12" t="s">
-        <v>1572</v>
+        <v>1308</v>
       </c>
       <c r="F359" s="12" t="s">
-        <v>1573</v>
+        <v>1307</v>
       </c>
       <c r="G359" s="7" t="s">
         <v>859</v>
@@ -14781,62 +14768,56 @@
         <v>66</v>
       </c>
       <c r="I359" s="12" t="s">
-        <v>1574</v>
+        <v>1536</v>
       </c>
       <c r="J359" s="12" t="s">
-        <v>1575</v>
-      </c>
-    </row>
-    <row r="360" spans="1:10" x14ac:dyDescent="0.35">
+        <v>1535</v>
+      </c>
+    </row>
+    <row r="360" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A360" s="1" t="s">
+        <v>1323</v>
+      </c>
+      <c r="B360" s="1" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C360" s="7">
+        <v>614</v>
+      </c>
+      <c r="D360" s="7">
+        <v>375</v>
+      </c>
+      <c r="E360" s="12" t="s">
         <v>1312</v>
       </c>
-      <c r="B360" s="1" t="s">
-        <v>1313</v>
-      </c>
-      <c r="C360" s="7">
-        <v>535</v>
-      </c>
-      <c r="D360" s="7">
-        <v>400</v>
-      </c>
-      <c r="E360" s="12" t="s">
+      <c r="F360" s="12" t="s">
         <v>1311</v>
-      </c>
-      <c r="F360" s="12" t="s">
-        <v>1310</v>
       </c>
       <c r="G360" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H360" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="I360" s="12" t="s">
-        <v>1541</v>
-      </c>
-      <c r="J360" s="12" t="s">
-        <v>1540</v>
-      </c>
-    </row>
-    <row r="361" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="361" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A361" s="1" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B361" s="1" t="s">
         <v>1326</v>
       </c>
-      <c r="B361" s="1" t="s">
-        <v>1327</v>
-      </c>
       <c r="C361" s="7">
-        <v>614</v>
+        <v>946</v>
       </c>
       <c r="D361" s="7">
-        <v>375</v>
+        <v>575</v>
       </c>
       <c r="E361" s="12" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="F361" s="12" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="G361" s="7" t="s">
         <v>859</v>
@@ -14844,25 +14825,31 @@
       <c r="H361" s="7" t="s">
         <v>511</v>
       </c>
-    </row>
-    <row r="362" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="I361" s="12" t="s">
+        <v>1518</v>
+      </c>
+      <c r="J361" s="12" t="s">
+        <v>1517</v>
+      </c>
+    </row>
+    <row r="362" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A362" s="1" t="s">
-        <v>1328</v>
+        <v>1319</v>
       </c>
       <c r="B362" s="1" t="s">
-        <v>1329</v>
+        <v>1320</v>
       </c>
       <c r="C362" s="7">
-        <v>946</v>
+        <v>1174</v>
       </c>
       <c r="D362" s="7">
-        <v>575</v>
+        <v>700</v>
       </c>
       <c r="E362" s="12" t="s">
-        <v>1317</v>
+        <v>1322</v>
       </c>
       <c r="F362" s="12" t="s">
-        <v>1316</v>
+        <v>1321</v>
       </c>
       <c r="G362" s="7" t="s">
         <v>859</v>
@@ -14871,56 +14858,53 @@
         <v>511</v>
       </c>
       <c r="I362" s="12" t="s">
-        <v>1523</v>
+        <v>1405</v>
       </c>
       <c r="J362" s="12" t="s">
-        <v>1522</v>
-      </c>
-    </row>
-    <row r="363" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="363" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A363" s="1" t="s">
-        <v>1322</v>
+        <v>1327</v>
       </c>
       <c r="B363" s="1" t="s">
-        <v>1323</v>
+        <v>1328</v>
       </c>
       <c r="C363" s="7">
-        <v>1174</v>
+        <v>1395</v>
       </c>
       <c r="D363" s="7">
-        <v>700</v>
+        <v>920</v>
       </c>
       <c r="E363" s="12" t="s">
-        <v>1325</v>
+        <v>1330</v>
       </c>
       <c r="F363" s="12" t="s">
-        <v>1324</v>
+        <v>1329</v>
       </c>
       <c r="G363" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H363" s="7" t="s">
-        <v>511</v>
+        <v>66</v>
       </c>
       <c r="I363" s="12" t="s">
-        <v>1408</v>
-      </c>
-      <c r="J363" s="12" t="s">
-        <v>1407</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="364" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
-        <v>1330</v>
+        <v>1511</v>
       </c>
       <c r="B364" s="1" t="s">
         <v>1331</v>
       </c>
       <c r="C364" s="7">
-        <v>1395</v>
+        <v>488</v>
       </c>
       <c r="D364" s="7">
-        <v>920</v>
+        <v>400</v>
       </c>
       <c r="E364" s="12" t="s">
         <v>1333</v>
@@ -14932,24 +14916,27 @@
         <v>859</v>
       </c>
       <c r="H364" s="7" t="s">
-        <v>66</v>
+        <v>511</v>
       </c>
       <c r="I364" s="12" t="s">
-        <v>1397</v>
-      </c>
-    </row>
-    <row r="365" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+        <v>1468</v>
+      </c>
+      <c r="J364" s="12" t="s">
+        <v>1512</v>
+      </c>
+    </row>
+    <row r="365" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
-        <v>1516</v>
+        <v>1334</v>
       </c>
       <c r="B365" s="1" t="s">
-        <v>1334</v>
+        <v>1337</v>
       </c>
       <c r="C365" s="7">
-        <v>488</v>
+        <v>554</v>
       </c>
       <c r="D365" s="7">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="E365" s="12" t="s">
         <v>1336</v>
@@ -14961,152 +14948,152 @@
         <v>859</v>
       </c>
       <c r="H365" s="7" t="s">
-        <v>511</v>
+        <v>12</v>
       </c>
       <c r="I365" s="12" t="s">
-        <v>1471</v>
+        <v>1574</v>
       </c>
       <c r="J365" s="12" t="s">
-        <v>1517</v>
-      </c>
-    </row>
-    <row r="366" spans="1:10" x14ac:dyDescent="0.35">
+        <v>1573</v>
+      </c>
+    </row>
+    <row r="366" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A366" s="1" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B366" s="1" t="s">
+        <v>1341</v>
+      </c>
+      <c r="C366" s="7">
+        <v>398</v>
+      </c>
+      <c r="D366" s="7">
+        <v>250</v>
+      </c>
+      <c r="E366" s="12" t="s">
         <v>1340</v>
       </c>
-      <c r="C366" s="7">
-        <v>554</v>
-      </c>
-      <c r="D366" s="7">
-        <v>200</v>
-      </c>
-      <c r="E366" s="12" t="s">
+      <c r="F366" s="12" t="s">
         <v>1339</v>
-      </c>
-      <c r="F366" s="12" t="s">
-        <v>1338</v>
       </c>
       <c r="G366" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H366" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I366" s="12" t="s">
-        <v>1579</v>
-      </c>
-      <c r="J366" s="12" t="s">
-        <v>1578</v>
-      </c>
-    </row>
-    <row r="367" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="367" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A367" s="1" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B367" s="1" t="s">
+        <v>1343</v>
+      </c>
+      <c r="C367" s="7">
+        <v>399</v>
+      </c>
+      <c r="D367" s="7">
+        <v>100</v>
+      </c>
+      <c r="E367" s="12" t="s">
+        <v>1345</v>
+      </c>
+      <c r="F367" s="12" t="s">
         <v>1344</v>
-      </c>
-      <c r="C367" s="7">
-        <v>398</v>
-      </c>
-      <c r="D367" s="7">
-        <v>250</v>
-      </c>
-      <c r="E367" s="12" t="s">
-        <v>1343</v>
-      </c>
-      <c r="F367" s="12" t="s">
-        <v>1342</v>
       </c>
       <c r="G367" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H367" s="7" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="368" spans="1:10" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+      <c r="I367" s="12" t="s">
+        <v>1532</v>
+      </c>
+    </row>
+    <row r="368" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A368" s="1" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
       <c r="B368" s="1" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="C368" s="7">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D368" s="7">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="E368" s="12" t="s">
+        <v>1349</v>
+      </c>
+      <c r="F368" s="12" t="s">
         <v>1348</v>
-      </c>
-      <c r="F368" s="12" t="s">
-        <v>1347</v>
       </c>
       <c r="G368" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H368" s="7" t="s">
-        <v>66</v>
+        <v>197</v>
       </c>
       <c r="I368" s="12" t="s">
-        <v>1537</v>
-      </c>
-    </row>
-    <row r="369" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>1426</v>
+      </c>
+      <c r="J368" s="12" t="s">
+        <v>1427</v>
+      </c>
+    </row>
+    <row r="369" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A369" s="1" t="s">
-        <v>1349</v>
+        <v>1350</v>
       </c>
       <c r="B369" s="1" t="s">
-        <v>1350</v>
+        <v>1351</v>
       </c>
       <c r="C369" s="7">
-        <v>397</v>
+        <v>350</v>
       </c>
       <c r="D369" s="7">
         <v>300</v>
       </c>
       <c r="E369" s="12" t="s">
+        <v>1353</v>
+      </c>
+      <c r="F369" s="12" t="s">
         <v>1352</v>
-      </c>
-      <c r="F369" s="12" t="s">
-        <v>1351</v>
       </c>
       <c r="G369" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H369" s="7" t="s">
-        <v>197</v>
+        <v>66</v>
       </c>
       <c r="I369" s="12" t="s">
-        <v>1429</v>
+        <v>1527</v>
       </c>
       <c r="J369" s="12" t="s">
-        <v>1430</v>
-      </c>
-    </row>
-    <row r="370" spans="1:10" x14ac:dyDescent="0.35">
+        <v>1526</v>
+      </c>
+    </row>
+    <row r="370" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A370" s="1" t="s">
-        <v>1353</v>
+        <v>1356</v>
       </c>
       <c r="B370" s="1" t="s">
-        <v>1354</v>
+        <v>1357</v>
       </c>
       <c r="C370" s="7">
-        <v>350</v>
+        <v>385</v>
       </c>
       <c r="D370" s="7">
         <v>300</v>
       </c>
       <c r="E370" s="12" t="s">
-        <v>1356</v>
+        <v>1355</v>
       </c>
       <c r="F370" s="12" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="G370" s="7" t="s">
         <v>859</v>
@@ -15115,30 +15102,27 @@
         <v>66</v>
       </c>
       <c r="I370" s="12" t="s">
-        <v>1532</v>
-      </c>
-      <c r="J370" s="12" t="s">
-        <v>1531</v>
-      </c>
-    </row>
-    <row r="371" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+        <v>1422</v>
+      </c>
+    </row>
+    <row r="371" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A371" s="1" t="s">
         <v>1359</v>
       </c>
       <c r="B371" s="1" t="s">
+        <v>1358</v>
+      </c>
+      <c r="C371" s="7">
+        <v>1690</v>
+      </c>
+      <c r="D371" s="7">
+        <v>1090</v>
+      </c>
+      <c r="E371" s="12" t="s">
+        <v>1421</v>
+      </c>
+      <c r="F371" s="12" t="s">
         <v>1360</v>
-      </c>
-      <c r="C371" s="7">
-        <v>385</v>
-      </c>
-      <c r="D371" s="7">
-        <v>300</v>
-      </c>
-      <c r="E371" s="12" t="s">
-        <v>1358</v>
-      </c>
-      <c r="F371" s="12" t="s">
-        <v>1357</v>
       </c>
       <c r="G371" s="7" t="s">
         <v>859</v>
@@ -15147,136 +15131,107 @@
         <v>66</v>
       </c>
       <c r="I371" s="12" t="s">
-        <v>1425</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="372" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A372" s="1" t="s">
+        <v>1363</v>
+      </c>
+      <c r="B372" s="1" t="s">
+        <v>1364</v>
+      </c>
+      <c r="C372" s="7">
+        <v>1999</v>
+      </c>
+      <c r="D372" s="7">
+        <v>800</v>
+      </c>
+      <c r="E372" s="12" t="s">
         <v>1362</v>
       </c>
-      <c r="B372" s="1" t="s">
+      <c r="F372" s="12" t="s">
         <v>1361</v>
-      </c>
-      <c r="C372" s="7">
-        <v>1690</v>
-      </c>
-      <c r="D372" s="7">
-        <v>1090</v>
-      </c>
-      <c r="E372" s="12" t="s">
-        <v>1424</v>
-      </c>
-      <c r="F372" s="12" t="s">
-        <v>1363</v>
       </c>
       <c r="G372" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H372" s="7" t="s">
-        <v>66</v>
+        <v>197</v>
       </c>
       <c r="I372" s="12" t="s">
-        <v>1394</v>
-      </c>
-    </row>
-    <row r="373" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>1399</v>
+      </c>
+    </row>
+    <row r="373" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A373" s="1" t="s">
-        <v>1366</v>
+        <v>1368</v>
       </c>
       <c r="B373" s="1" t="s">
         <v>1367</v>
       </c>
       <c r="C373" s="7">
-        <v>1999</v>
+        <v>4699</v>
       </c>
       <c r="D373" s="7">
-        <v>800</v>
+        <v>2832</v>
       </c>
       <c r="E373" s="12" t="s">
+        <v>1366</v>
+      </c>
+      <c r="F373" s="12" t="s">
         <v>1365</v>
-      </c>
-      <c r="F373" s="12" t="s">
-        <v>1364</v>
       </c>
       <c r="G373" s="7" t="s">
         <v>859</v>
       </c>
       <c r="H373" s="7" t="s">
-        <v>197</v>
+        <v>510</v>
       </c>
       <c r="I373" s="12" t="s">
-        <v>1402</v>
-      </c>
-    </row>
-    <row r="374" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>1386</v>
+      </c>
+      <c r="J373" s="12" t="s">
+        <v>1385</v>
+      </c>
+    </row>
+    <row r="374" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A374" s="1" t="s">
-        <v>1371</v>
+        <v>1369</v>
       </c>
       <c r="B374" s="1" t="s">
         <v>1370</v>
       </c>
       <c r="C374" s="7">
-        <v>4699</v>
+        <v>349</v>
       </c>
       <c r="D374" s="7">
-        <v>2832</v>
+        <v>295</v>
       </c>
       <c r="E374" s="12" t="s">
-        <v>1369</v>
+        <v>1372</v>
       </c>
       <c r="F374" s="12" t="s">
-        <v>1368</v>
+        <v>1371</v>
       </c>
       <c r="G374" s="7" t="s">
-        <v>859</v>
+        <v>419</v>
       </c>
       <c r="H374" s="7" t="s">
-        <v>510</v>
+        <v>66</v>
       </c>
       <c r="I374" s="12" t="s">
-        <v>1389</v>
+        <v>1479</v>
       </c>
       <c r="J374" s="12" t="s">
-        <v>1388</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="375" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A375" s="1" t="s">
-        <v>1372</v>
-      </c>
-      <c r="B375" s="1" t="s">
-        <v>1373</v>
-      </c>
-      <c r="C375" s="7">
-        <v>349</v>
-      </c>
-      <c r="D375" s="7">
-        <v>295</v>
-      </c>
-      <c r="E375" s="12" t="s">
-        <v>1375</v>
-      </c>
-      <c r="F375" s="12" t="s">
-        <v>1374</v>
-      </c>
-      <c r="G375" s="7" t="s">
-        <v>419</v>
-      </c>
-      <c r="H375" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="I375" s="12" t="s">
-        <v>1482</v>
-      </c>
-      <c r="J375" s="12" t="s">
-        <v>1481</v>
-      </c>
-    </row>
-    <row r="376" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A376" s="13" t="s">
-        <v>1591</v>
-      </c>
-      <c r="B376" s="1"/>
+      <c r="A375" s="13" t="s">
+        <v>1586</v>
+      </c>
+      <c r="B375" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -15285,52 +15240,52 @@
     <hyperlink ref="F60" r:id="rId3"/>
     <hyperlink ref="E271" r:id="rId4"/>
     <hyperlink ref="E60" r:id="rId5"/>
-    <hyperlink ref="E350" r:id="rId6"/>
+    <hyperlink ref="E349" r:id="rId6"/>
     <hyperlink ref="E253" r:id="rId7"/>
     <hyperlink ref="E328" r:id="rId8"/>
     <hyperlink ref="E152" r:id="rId9"/>
-    <hyperlink ref="F353" r:id="rId10" location="&amp;gid=1&amp;pid=1"/>
-    <hyperlink ref="E353" r:id="rId11"/>
-    <hyperlink ref="F354" r:id="rId12" location="&amp;gid=1&amp;pid=1"/>
-    <hyperlink ref="E354" r:id="rId13"/>
-    <hyperlink ref="F355" r:id="rId14" location="&amp;gid=1&amp;pid=1"/>
-    <hyperlink ref="E355" r:id="rId15"/>
-    <hyperlink ref="F356" r:id="rId16"/>
-    <hyperlink ref="E356" r:id="rId17"/>
-    <hyperlink ref="F357" r:id="rId18"/>
-    <hyperlink ref="E357" r:id="rId19"/>
-    <hyperlink ref="F358" display="https://www.mercadolibre.com.mx/epicentro-audishako-max-02-restaurador-de-bajos-para-auto-subwoofer-para-carro-pickups-y-suv-accesorios-para-auto-audio-diseno-en-relieve-3d-incluye-dash-remoto-control-de-bajos/p/MLM64640099?pdp_filters=item_id:MLM46970202"/>
-    <hyperlink ref="E358" r:id="rId20"/>
-    <hyperlink ref="F360" r:id="rId21"/>
-    <hyperlink ref="E360" r:id="rId22"/>
-    <hyperlink ref="F361" r:id="rId23"/>
-    <hyperlink ref="E361" r:id="rId24"/>
-    <hyperlink ref="F362" r:id="rId25"/>
-    <hyperlink ref="E362" r:id="rId26"/>
-    <hyperlink ref="F364" r:id="rId27"/>
-    <hyperlink ref="E364" r:id="rId28"/>
-    <hyperlink ref="F365" r:id="rId29" location="reviews"/>
-    <hyperlink ref="E365" r:id="rId30"/>
-    <hyperlink ref="F366" r:id="rId31"/>
-    <hyperlink ref="E366" r:id="rId32"/>
-    <hyperlink ref="F367" r:id="rId33"/>
-    <hyperlink ref="E367" r:id="rId34"/>
-    <hyperlink ref="F368" r:id="rId35"/>
-    <hyperlink ref="E368" r:id="rId36"/>
-    <hyperlink ref="F369" r:id="rId37"/>
-    <hyperlink ref="E369" r:id="rId38"/>
-    <hyperlink ref="F370" r:id="rId39"/>
-    <hyperlink ref="E370" r:id="rId40"/>
-    <hyperlink ref="F371" r:id="rId41"/>
-    <hyperlink ref="E371" r:id="rId42"/>
-    <hyperlink ref="F372" r:id="rId43"/>
-    <hyperlink ref="E372" r:id="rId44"/>
-    <hyperlink ref="F373" r:id="rId45"/>
-    <hyperlink ref="E373" r:id="rId46"/>
-    <hyperlink ref="F374" r:id="rId47"/>
-    <hyperlink ref="E374" r:id="rId48"/>
-    <hyperlink ref="F375" r:id="rId49"/>
-    <hyperlink ref="E375" r:id="rId50"/>
+    <hyperlink ref="F352" r:id="rId10" location="&amp;gid=1&amp;pid=1"/>
+    <hyperlink ref="E352" r:id="rId11"/>
+    <hyperlink ref="F353" r:id="rId12" location="&amp;gid=1&amp;pid=1"/>
+    <hyperlink ref="E353" r:id="rId13"/>
+    <hyperlink ref="F354" r:id="rId14" location="&amp;gid=1&amp;pid=1"/>
+    <hyperlink ref="E354" r:id="rId15"/>
+    <hyperlink ref="F355" r:id="rId16"/>
+    <hyperlink ref="E355" r:id="rId17"/>
+    <hyperlink ref="F356" r:id="rId18"/>
+    <hyperlink ref="E356" r:id="rId19"/>
+    <hyperlink ref="F357" display="https://www.mercadolibre.com.mx/epicentro-audishako-max-02-restaurador-de-bajos-para-auto-subwoofer-para-carro-pickups-y-suv-accesorios-para-auto-audio-diseno-en-relieve-3d-incluye-dash-remoto-control-de-bajos/p/MLM64640099?pdp_filters=item_id:MLM46970202"/>
+    <hyperlink ref="E357" r:id="rId20"/>
+    <hyperlink ref="F359" r:id="rId21"/>
+    <hyperlink ref="E359" r:id="rId22"/>
+    <hyperlink ref="F360" r:id="rId23"/>
+    <hyperlink ref="E360" r:id="rId24"/>
+    <hyperlink ref="F361" r:id="rId25"/>
+    <hyperlink ref="E361" r:id="rId26"/>
+    <hyperlink ref="F363" r:id="rId27"/>
+    <hyperlink ref="E363" r:id="rId28"/>
+    <hyperlink ref="F364" r:id="rId29" location="reviews"/>
+    <hyperlink ref="E364" r:id="rId30"/>
+    <hyperlink ref="F365" r:id="rId31"/>
+    <hyperlink ref="E365" r:id="rId32"/>
+    <hyperlink ref="F366" r:id="rId33"/>
+    <hyperlink ref="E366" r:id="rId34"/>
+    <hyperlink ref="F367" r:id="rId35"/>
+    <hyperlink ref="E367" r:id="rId36"/>
+    <hyperlink ref="F368" r:id="rId37"/>
+    <hyperlink ref="E368" r:id="rId38"/>
+    <hyperlink ref="F369" r:id="rId39"/>
+    <hyperlink ref="E369" r:id="rId40"/>
+    <hyperlink ref="F370" r:id="rId41"/>
+    <hyperlink ref="E370" r:id="rId42"/>
+    <hyperlink ref="F371" r:id="rId43"/>
+    <hyperlink ref="E371" r:id="rId44"/>
+    <hyperlink ref="F372" r:id="rId45"/>
+    <hyperlink ref="E372" r:id="rId46"/>
+    <hyperlink ref="F373" r:id="rId47"/>
+    <hyperlink ref="E373" r:id="rId48"/>
+    <hyperlink ref="F374" r:id="rId49"/>
+    <hyperlink ref="E374" r:id="rId50"/>
     <hyperlink ref="I72" display="https://http2.mlstatic.com/D_NQ_NP_2X_977864-MLA82522530268_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_728802-MLA82808708997_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_714871-MLA82808836891_032025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I299" r:id="rId51"/>
     <hyperlink ref="J299" r:id="rId52"/>
@@ -15341,48 +15296,48 @@
     <hyperlink ref="I67" display="https://http2.mlstatic.com/D_NQ_NP_2X_754117-MLA87918629604_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_955266-MLA88256438081_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_924778-MLA88256272783_072025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I265" display="https://http2.mlstatic.com/D_NQ_NP_2X_651538-MLA109474609027_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_786870-MLA109384870397_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_877937-MLA109385877631_032026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I328" display="https://http2.mlstatic.com/D_NQ_NP_2X_659872-MLA110558100656_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_654212-MLA110558217136_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_728798-MLA110558100602_052026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J374" r:id="rId54"/>
-    <hyperlink ref="I374" r:id="rId55"/>
+    <hyperlink ref="J373" r:id="rId54"/>
+    <hyperlink ref="I373" r:id="rId55"/>
     <hyperlink ref="I330" display="https://http2.mlstatic.com/D_NQ_NP_2X_704682-MLA112632086794_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_648062-MLA114215908179_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_721338-MLA112631444306_062026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="E250" r:id="rId56"/>
     <hyperlink ref="I250" r:id="rId57"/>
     <hyperlink ref="J250" r:id="rId58"/>
     <hyperlink ref="I36" r:id="rId59"/>
-    <hyperlink ref="I372" display="https://http2.mlstatic.com/D_NQ_NP_2X_870766-MLA111944165952_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_637261-MLA111944285568_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_835091-MLA112882459449_062026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I371" display="https://http2.mlstatic.com/D_NQ_NP_2X_870766-MLA111944165952_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_637261-MLA111944285568_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_835091-MLA112882459449_062026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="J60" r:id="rId60"/>
     <hyperlink ref="I60" display="https://http2.mlstatic.com/D_NQ_NP_2X_650019-MLA112598239078_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_694102-MLA111420836191_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_960139-MLA111232526403_052026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I364" r:id="rId61"/>
+    <hyperlink ref="I363" r:id="rId61"/>
     <hyperlink ref="I225" display="https://http2.mlstatic.com/D_NQ_NP_2X_761866-MLA76203783381_052024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_967910-MLA76082310461_042024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_699850-MLA76082339489_042024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="J32" r:id="rId62"/>
     <hyperlink ref="I32" display="https://http2.mlstatic.com/D_NQ_NP_2X_937988-MLA100214376229_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_839463-MLA100214244569_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_878239-MLA100214347283_122025-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I101" display="https://http2.mlstatic.com/D_NQ_NP_2X_853469-MLA73479850047_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_636371-MLA72966055893_112023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_647337-MLA74448293715_022024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="I373" display="https://http2.mlstatic.com/D_NQ_NP_2X_838661-MLA114043475512_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_997422-MLA111845686244_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_946430-MLA112856485647_062026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I372" display="https://http2.mlstatic.com/D_NQ_NP_2X_838661-MLA114043475512_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_997422-MLA111845686244_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_946430-MLA112856485647_062026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I146" display="https://http2.mlstatic.com/D_NQ_NP_2X_700050-MLA90330537717_082025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_810830-MLA92985348779_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_611435-MLA103169335415_122025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="J341" r:id="rId63"/>
-    <hyperlink ref="I341" display="https://http2.mlstatic.com/D_NQ_NP_2X_972461-MLA108765590667_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_959062-MLA111287287492_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_702439-MLA108999676116_032026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="J340" r:id="rId63"/>
+    <hyperlink ref="I340" display="https://http2.mlstatic.com/D_NQ_NP_2X_972461-MLA108765590667_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_959062-MLA111287287492_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_702439-MLA108999676116_032026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I244" display="https://http2.mlstatic.com/D_NQ_NP_2X_772336-MLA83215360667_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_641687-MLA82926894938_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_686941-MLA80851161221_112024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J362" r:id="rId64"/>
-    <hyperlink ref="I362" display="https://http2.mlstatic.com/D_NQ_NP_2X_654570-MLA114163554383_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_820669-MLA112176540320_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_827402-MLA113697495744_072026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J357" r:id="rId65"/>
-    <hyperlink ref="I357" display="https://http2.mlstatic.com/D_NQ_NP_2X_622982-MLA91998379772_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_918567-MLA93316673763_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_951409-MLA93316693351_092025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="I358" r:id="rId66"/>
-    <hyperlink ref="J358" r:id="rId67"/>
+    <hyperlink ref="J361" r:id="rId64"/>
+    <hyperlink ref="I361" display="https://http2.mlstatic.com/D_NQ_NP_2X_654570-MLA114163554383_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_820669-MLA112176540320_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_827402-MLA113697495744_072026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="J356" r:id="rId65"/>
+    <hyperlink ref="I356" display="https://http2.mlstatic.com/D_NQ_NP_2X_622982-MLA91998379772_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_918567-MLA93316673763_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_951409-MLA93316693351_092025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
+    <hyperlink ref="I357" r:id="rId66"/>
+    <hyperlink ref="J357" r:id="rId67"/>
     <hyperlink ref="J169" r:id="rId68"/>
     <hyperlink ref="I169" display="https://http2.mlstatic.com/D_NQ_NP_2X_630634-MLA83929492736_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_826427-MLA83875691856_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_778506-MLA83875632066_042025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I286" display="https://http2.mlstatic.com/D_NQ_NP_2X_601798-MLA74779553000_032024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_784677-MLA71729912500_092023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_982997-MLA73375012815_122023-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="J56" r:id="rId69"/>
     <hyperlink ref="I56" r:id="rId70"/>
-    <hyperlink ref="I355" r:id="rId71"/>
-    <hyperlink ref="I356" r:id="rId72"/>
+    <hyperlink ref="I354" r:id="rId71"/>
+    <hyperlink ref="I355" r:id="rId72"/>
     <hyperlink ref="I132" r:id="rId73"/>
-    <hyperlink ref="I354" r:id="rId74"/>
-    <hyperlink ref="J354" r:id="rId75"/>
-    <hyperlink ref="I371" display="https://http2.mlstatic.com/D_NQ_NP_2X_730160-MLA112550162587_062026-F.webp;http://http2.mlstatic.com/D_NQ_NP_2X_748872-MLA113290799753_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_824232-MLA112954608093_062026-F.webp;https://http2.mlstatic.com/D_NQ"/>
+    <hyperlink ref="I353" r:id="rId74"/>
+    <hyperlink ref="J353" r:id="rId75"/>
+    <hyperlink ref="I370" display="https://http2.mlstatic.com/D_NQ_NP_2X_730160-MLA112550162587_062026-F.webp;http://http2.mlstatic.com/D_NQ_NP_2X_748872-MLA113290799753_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_824232-MLA112954608093_062026-F.webp;https://http2.mlstatic.com/D_NQ"/>
     <hyperlink ref="I107" r:id="rId76"/>
     <hyperlink ref="I2" display="https://http2.mlstatic.com/D_NQ_NP_2X_644970-MLA111138624893_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_618974-MLA113557256809_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_849248-MLA111414716285_052026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I11" r:id="rId77"/>
-    <hyperlink ref="I369" r:id="rId78"/>
-    <hyperlink ref="J369" r:id="rId79"/>
+    <hyperlink ref="I368" r:id="rId78"/>
+    <hyperlink ref="J368" r:id="rId79"/>
     <hyperlink ref="E145" r:id="rId80"/>
     <hyperlink ref="I145" r:id="rId81"/>
     <hyperlink ref="J180" r:id="rId82"/>
@@ -15400,11 +15355,11 @@
     <hyperlink ref="I322" r:id="rId94"/>
     <hyperlink ref="J54" r:id="rId95"/>
     <hyperlink ref="I54" r:id="rId96"/>
-    <hyperlink ref="I353" r:id="rId97"/>
+    <hyperlink ref="I352" r:id="rId97"/>
     <hyperlink ref="I325" r:id="rId98"/>
-    <hyperlink ref="J366" r:id="rId99"/>
-    <hyperlink ref="I366" display="https://http2.mlstatic.com/D_NQ_NP_2X_967252-MLA112857017004_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_802434-MLA114058497103_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_904877-MLA112857136140_072026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I337" display="https://http2.mlstatic.com/D_NQ_NP_2X_871513-MLA105683275105_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_921467-MLA106225093215_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_768089-MLA111241397693_052026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="J365" r:id="rId99"/>
+    <hyperlink ref="I365" display="https://http2.mlstatic.com/D_NQ_NP_2X_967252-MLA112857017004_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_802434-MLA114058497103_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_904877-MLA112857136140_072026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I336" display="https://http2.mlstatic.com/D_NQ_NP_2X_871513-MLA105683275105_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_921467-MLA106225093215_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_768089-MLA111241397693_052026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I273" r:id="rId100"/>
     <hyperlink ref="J268" r:id="rId101"/>
     <hyperlink ref="I268" display="https://http2.mlstatic.com/D_NQ_NP_2X_723996-MLA101839595031_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_648298-MLA100279286785_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_899562-MLA105452243109_012026-F.webp;https://http2.mlstatic.com/D_N"/>
@@ -15412,8 +15367,8 @@
     <hyperlink ref="I106" display="https://http2.mlstatic.com/D_NQ_NP_2X_986480-MLA92403239851_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_992851-MLA91999385090_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_790783-MLA94732447073_102025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I185" display="https://http2.mlstatic.com/D_NQ_NP_2X_714527-MLA94159366454_102025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_847366-MLA97737335743_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_618907-MLA100261323194_122025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
     <hyperlink ref="I288" r:id="rId103"/>
-    <hyperlink ref="J342" r:id="rId104"/>
-    <hyperlink ref="I342" r:id="rId105"/>
+    <hyperlink ref="J341" r:id="rId104"/>
+    <hyperlink ref="I341" r:id="rId105"/>
     <hyperlink ref="J300" r:id="rId106"/>
     <hyperlink ref="I300" r:id="rId107"/>
     <hyperlink ref="I329" display="https://http2.mlstatic.com/D_NQ_NP_2X_886751-MLA110760597980_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_722285-MLA111072136212_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_745568-MLA111456288976_052026-F.webp;https://http2.mlstatic.com/D_N"/>
@@ -15427,7 +15382,7 @@
     <hyperlink ref="I197" display="https://http2.mlstatic.com/D_NQ_NP_2X_882824-MLA78038279945_072024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_628505-MLA80605999965_112024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_605405-MLA79717879214_102024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="J108" r:id="rId115"/>
     <hyperlink ref="I108" r:id="rId116"/>
-    <hyperlink ref="I365" r:id="rId117"/>
+    <hyperlink ref="I364" r:id="rId117"/>
     <hyperlink ref="I174" display="https://http2.mlstatic.com/D_NQ_NP_2X_671282-MLA88303913955_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_751626-MLA88304056333_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_928886-MLA111461620111_052026-F.webp;https://http2.mlstatic.com/D_NQ_"/>
     <hyperlink ref="I85" r:id="rId118"/>
     <hyperlink ref="I212" r:id="rId119"/>
@@ -15437,8 +15392,8 @@
     <hyperlink ref="J271" r:id="rId122"/>
     <hyperlink ref="I271" r:id="rId123"/>
     <hyperlink ref="I324" r:id="rId124"/>
-    <hyperlink ref="J375" r:id="rId125"/>
-    <hyperlink ref="I375" r:id="rId126"/>
+    <hyperlink ref="J374" r:id="rId125"/>
+    <hyperlink ref="I374" r:id="rId126"/>
     <hyperlink ref="J53" r:id="rId127"/>
     <hyperlink ref="I53" r:id="rId128"/>
     <hyperlink ref="I222" display="https://http2.mlstatic.com/D_NQ_NP_2X_931197-MLA111097282025_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_647752-MLA86304062244_062025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_697099-MLA86808814199_062025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
@@ -15455,99 +15410,97 @@
     <hyperlink ref="J48" r:id="rId134"/>
     <hyperlink ref="I48" display="https://http2.mlstatic.com/D_NQ_NP_2X_615383-MLA106283983813_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_637244-MLA106762003457_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_647036-MLA106069021004_022026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I275" r:id="rId135"/>
-    <hyperlink ref="J334" r:id="rId136"/>
-    <hyperlink ref="I334" display="https://http2.mlstatic.com/D_NQ_NP_2X_694390-MLA103915605591_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_901157-MLA112027651816_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_930408-MLA112027361550_062026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I296" display="https://http2.mlstatic.com/D_NQ_NP_2X_877410-MLA86700953698_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_621602-MLA110823348827_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_945418-MLA86701516062_072025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="I285" r:id="rId137"/>
+    <hyperlink ref="I285" r:id="rId136"/>
     <hyperlink ref="I3" display="https://http2.mlstatic.com/D_NQ_NP_2X_652387-MLA81262109420_122024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_964100-MLA74205385415_012024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_663926-MLA71594815900_092023-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J52" r:id="rId138"/>
+    <hyperlink ref="J52" r:id="rId137"/>
     <hyperlink ref="I52" display="https://http2.mlstatic.com/D_NQ_NP_2X_787566-MLA112208805453_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_610420-MLA108420590498_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_778316-MLA108420330866_032026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I331" display="https://http2.mlstatic.com/D_NQ_NP_2X_811172-MLA108871819192_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_673692-MLA109653928111_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_807085-MLA109742422391_032026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I210" display="https://http2.mlstatic.com/D_NQ_NP_2X_787733-MLA73258839528_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_702415-MLA111282425851_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_934591-MLA108763618671_032026-F.webp;https://http2.mlstatic.com/D_NQ"/>
     <hyperlink ref="I65" display="https://http2.mlstatic.com/D_NQ_NP_2X_822004-MLA83792590685_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_922399-MLA83499949924_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_741644-MLA73913804094_012024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="I205" r:id="rId139"/>
-    <hyperlink ref="J332" r:id="rId140"/>
-    <hyperlink ref="I332" r:id="rId141"/>
+    <hyperlink ref="I205" r:id="rId138"/>
+    <hyperlink ref="J332" r:id="rId139"/>
+    <hyperlink ref="I332" r:id="rId140"/>
     <hyperlink ref="I143" display="https://http2.mlstatic.com/D_NQ_NP_2X_951908-MLA106095526036_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_697058-MLA92029170496_092025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_770689-MLA112170606647_052026-F.webp;https://http2.mlstatic.com/D_NQ"/>
-    <hyperlink ref="J143" r:id="rId142"/>
-    <hyperlink ref="J87" r:id="rId143"/>
-    <hyperlink ref="I87" r:id="rId144"/>
-    <hyperlink ref="J365" r:id="rId145"/>
-    <hyperlink ref="J235" r:id="rId146"/>
+    <hyperlink ref="J143" r:id="rId141"/>
+    <hyperlink ref="J87" r:id="rId142"/>
+    <hyperlink ref="I87" r:id="rId143"/>
+    <hyperlink ref="J364" r:id="rId144"/>
+    <hyperlink ref="J235" r:id="rId145"/>
     <hyperlink ref="I235" display="https://http2.mlstatic.com/D_NQ_NP_2X_786831-MLA112508605409_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_945451-MLA106951088919_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_942407-MLA79868078780_102024-F.webp;https://http2.mlstatic.com/D_NQ"/>
-    <hyperlink ref="J25" r:id="rId147"/>
-    <hyperlink ref="I156" r:id="rId148"/>
-    <hyperlink ref="J283" r:id="rId149"/>
-    <hyperlink ref="I283" r:id="rId150"/>
-    <hyperlink ref="I147" r:id="rId151"/>
-    <hyperlink ref="J167" r:id="rId152"/>
+    <hyperlink ref="J25" r:id="rId146"/>
+    <hyperlink ref="I156" r:id="rId147"/>
+    <hyperlink ref="J283" r:id="rId148"/>
+    <hyperlink ref="I283" r:id="rId149"/>
+    <hyperlink ref="I147" r:id="rId150"/>
+    <hyperlink ref="J167" r:id="rId151"/>
     <hyperlink ref="I167" display="https://http2.mlstatic.com/D_NQ_NP_2X_949414-MLA115597206229_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_781530-MLA115596590455_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_794977-MLA113865153424_072026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I242" r:id="rId153"/>
-    <hyperlink ref="I336" r:id="rId154"/>
-    <hyperlink ref="J370" r:id="rId155"/>
-    <hyperlink ref="I370" r:id="rId156"/>
+    <hyperlink ref="I242" r:id="rId152"/>
+    <hyperlink ref="I335" r:id="rId153"/>
+    <hyperlink ref="J369" r:id="rId154"/>
+    <hyperlink ref="I369" r:id="rId155"/>
     <hyperlink ref="I113" display="https://http2.mlstatic.com/D_NQ_NP_2X_602967-MLA106207657120_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_937184-MLA99857184303_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_615655-MLA93805615686_102025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="J113" r:id="rId157"/>
+    <hyperlink ref="J113" r:id="rId156"/>
     <hyperlink ref="I274" display="https://http2.mlstatic.com/D_NQ_NP_2X_811367-MLA96964641173_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_724534-MLA95972455447_102025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_862711-MLA94582890276_102025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="I188" r:id="rId158"/>
-    <hyperlink ref="I368" r:id="rId159"/>
+    <hyperlink ref="I188" r:id="rId157"/>
+    <hyperlink ref="I367" r:id="rId158"/>
     <hyperlink ref="I112" display="https://http2.mlstatic.com/D_NQ_NP_2X_832809-MLA100859657141_122025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_651615-MLA104572148023_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_683702-MLA104248384382_012026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I321" r:id="rId160"/>
-    <hyperlink ref="J360" r:id="rId161"/>
-    <hyperlink ref="I360" display="https://http2.mlstatic.com/D_NQ_NP_2X_986254-MLA113898749317_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_998498-MLA115220256263_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_611119-MLA113912677208_072026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I321" r:id="rId159"/>
+    <hyperlink ref="J359" r:id="rId160"/>
+    <hyperlink ref="I359" display="https://http2.mlstatic.com/D_NQ_NP_2X_986254-MLA113898749317_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_998498-MLA115220256263_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_611119-MLA113912677208_072026-F.webp;https://http2.mlstatic.com/D_N"/>
     <hyperlink ref="I297" display="https://http2.mlstatic.com/D_NQ_NP_2X_672294-MLA110281902509_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_995715-MLA110918042491_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_936537-MLA110364709430_052026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J297" r:id="rId162"/>
-    <hyperlink ref="J326" r:id="rId163"/>
+    <hyperlink ref="J297" r:id="rId161"/>
+    <hyperlink ref="J326" r:id="rId162"/>
     <hyperlink ref="I326" display="https://http2.mlstatic.com/D_NQ_NP_2X_623123-MLA111040290746_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_934760-MLA111878498611_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_790070-MLA112661729675_062026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J338" r:id="rId164"/>
-    <hyperlink ref="I338" display="https://http2.mlstatic.com/D_NQ_NP_2X_637815-MLA110916194519_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_643077-MLA110749031212_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_708016-MLA112321199072_062026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I320" r:id="rId165"/>
-    <hyperlink ref="I122" r:id="rId166"/>
-    <hyperlink ref="J55" r:id="rId167"/>
+    <hyperlink ref="J337" r:id="rId163"/>
+    <hyperlink ref="I337" display="https://http2.mlstatic.com/D_NQ_NP_2X_637815-MLA110916194519_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_643077-MLA110749031212_052026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_708016-MLA112321199072_062026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="I320" r:id="rId164"/>
+    <hyperlink ref="I122" r:id="rId165"/>
+    <hyperlink ref="J55" r:id="rId166"/>
     <hyperlink ref="I55" display="https://http2.mlstatic.com/D_NQ_NP_2X_707272-MLA81406001662_122024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_992452-MLA71699440818_092023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_616985-MLA84032409756_052025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J293" r:id="rId168"/>
+    <hyperlink ref="J293" r:id="rId167"/>
     <hyperlink ref="I293" display="https://http2.mlstatic.com/D_NQ_NP_2X_699847-MLA83204192108_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_847455-MLA79932861627_102024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_823994-MLA70105011582_062023-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="J247" r:id="rId169"/>
+    <hyperlink ref="J247" r:id="rId168"/>
     <hyperlink ref="I247" display="https://http2.mlstatic.com/D_NQ_NP_2X_896395-MLA74651133358_022024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_757231-MLA73307952803_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_773664-MLA113844190574_072026-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="I269" r:id="rId170"/>
-    <hyperlink ref="J214" r:id="rId171"/>
+    <hyperlink ref="I269" r:id="rId169"/>
+    <hyperlink ref="J214" r:id="rId170"/>
     <hyperlink ref="I214" display="https://http2.mlstatic.com/D_NQ_NP_2X_857704-MLA105910693631_012026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_785878-MLA115684445439_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_732723-MLA114610870605_072026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="I124" r:id="rId172"/>
+    <hyperlink ref="I124" r:id="rId171"/>
     <hyperlink ref="I139" display="https://http2.mlstatic.com/D_NQ_NP_2X_731885-MLA81735782871_012025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_877502-MLA81736505623_012025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_739624-MLA81735782869_012025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
     <hyperlink ref="I151" display="https://http2.mlstatic.com/D_NQ_NP_2X_852777-MLA73231184100_122023-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_953229-MLA74068746840_012024-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_727505-MLA74823139724_032024-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="I163" r:id="rId173"/>
-    <hyperlink ref="J163" r:id="rId174"/>
-    <hyperlink ref="F111" r:id="rId175" location="reviews"/>
-    <hyperlink ref="I111" r:id="rId176"/>
-    <hyperlink ref="I323" r:id="rId177"/>
-    <hyperlink ref="I327" r:id="rId178"/>
+    <hyperlink ref="I163" r:id="rId172"/>
+    <hyperlink ref="J163" r:id="rId173"/>
+    <hyperlink ref="F111" r:id="rId174" location="reviews"/>
+    <hyperlink ref="I111" r:id="rId175"/>
+    <hyperlink ref="I323" r:id="rId176"/>
+    <hyperlink ref="I327" r:id="rId177"/>
     <hyperlink ref="I102" display="https://http2.mlstatic.com/D_NQ_NP_2X_701490-MLA108653774761_032026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_910611-MLA87584829978_072025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_761367-MLA87718920709_072025-F.webp;https://http2.mlstatic.com/D_NQ_"/>
-    <hyperlink ref="E359" r:id="rId179"/>
-    <hyperlink ref="F359" r:id="rId180"/>
-    <hyperlink ref="I359" display="https://http2.mlstatic.com/D_NQ_NP_2X_957897-MLA114152946760_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_988648-MLA114781488773_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_938364-MLA113693419924_072026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J359" r:id="rId181"/>
-    <hyperlink ref="E231" r:id="rId182"/>
-    <hyperlink ref="I231" r:id="rId183"/>
-    <hyperlink ref="I278" r:id="rId184"/>
-    <hyperlink ref="F29" r:id="rId185"/>
+    <hyperlink ref="E358" r:id="rId178"/>
+    <hyperlink ref="F358" r:id="rId179"/>
+    <hyperlink ref="I358" display="https://http2.mlstatic.com/D_NQ_NP_2X_957897-MLA114152946760_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_988648-MLA114781488773_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_938364-MLA113693419924_072026-F.webp;https://http2.mlstatic.com/D_N"/>
+    <hyperlink ref="J358" r:id="rId180"/>
+    <hyperlink ref="E231" r:id="rId181"/>
+    <hyperlink ref="I231" r:id="rId182"/>
+    <hyperlink ref="I278" r:id="rId183"/>
+    <hyperlink ref="F29" r:id="rId184"/>
     <hyperlink ref="I333" display="https://http2.mlstatic.com/D_NQ_NP_2X_661292-MLA98293086467_112025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_907390-MLA106707175024_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_876338-MLA108047534008_032026-F.webp;https://http2.mlstatic.com/D_NQ"/>
-    <hyperlink ref="J333" r:id="rId186"/>
-    <hyperlink ref="J279" r:id="rId187"/>
+    <hyperlink ref="J333" r:id="rId185"/>
+    <hyperlink ref="J279" r:id="rId186"/>
     <hyperlink ref="I279" display="https://http2.mlstatic.com/D_NQ_NP_2X_609731-MLA83282009211_032025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_965155-MLA83841127402_042025-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_758965-MLA85304541601_052025-F.webp;https://http2.mlstatic.com/D_NQ_N"/>
-    <hyperlink ref="I162" r:id="rId188"/>
-    <hyperlink ref="J162" r:id="rId189"/>
-    <hyperlink ref="I141" r:id="rId190"/>
-    <hyperlink ref="J142" r:id="rId191"/>
+    <hyperlink ref="I162" r:id="rId187"/>
+    <hyperlink ref="J162" r:id="rId188"/>
+    <hyperlink ref="I141" r:id="rId189"/>
+    <hyperlink ref="J142" r:id="rId190"/>
     <hyperlink ref="I142" display="https://http2.mlstatic.com/D_NQ_NP_2X_863418-MLA109994960812_042026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_927650-MLA105811665406_022026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_743624-MLA105810281830_022026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="J86" r:id="rId192"/>
+    <hyperlink ref="J86" r:id="rId191"/>
     <hyperlink ref="I86" display="https://http2.mlstatic.com/D_NQ_NP_2X_929447-MLA114868215933_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_688697-MLA113791320300_072026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_631693-MLA113790881904_072026-F.webp;https://http2.mlstatic.com/D_N"/>
-    <hyperlink ref="F86" r:id="rId193"/>
-    <hyperlink ref="J296" r:id="rId194"/>
+    <hyperlink ref="F86" r:id="rId192"/>
+    <hyperlink ref="J296" r:id="rId193"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId195"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId194"/>
   <tableParts count="1">
-    <tablePart r:id="rId196"/>
+    <tablePart r:id="rId195"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualiza proyecto (2 modificados, 2 eliminados, 1 nuevo): download_log.txt, productos.xlsx, reporte_urls_invalidas.csv
</commit_message>
<xml_diff>
--- a/datos/productos.xlsx
+++ b/datos/productos.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2486" uniqueCount="1660">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2488" uniqueCount="1662">
   <si>
     <t>Nombre</t>
   </si>
@@ -4980,9 +4980,6 @@
     <t>https://articulo.mercadolibre.com.mx/MLM-5261216182-funda-para-volante-fibra-de-carbono-gama-alta-forma-d-negro-_JM?quantity=1&amp;sid=purchases</t>
   </si>
   <si>
-    <t>https://http2.mlstatic.com/D_NQ_NP_2X_647314-MLA112718039093_062026-F.webp;;https://http2.mlstatic.com/D_NQ_NP_2X_893993-MLA114600687014_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_679978-MLA113117754927_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_992169-MLA113116577615_062026-F.webp</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pistola para Pintar Inalámbrica </t>
   </si>
   <si>
@@ -4996,9 +4993,6 @@
   </si>
   <si>
     <t>2 PIEZA</t>
-  </si>
-  <si>
-    <t>https://http2.mlstatic.com/D_766480-MLM74144490966_012024-N.jpg;https://http2.mlstatic.com/D_969489-MLM74157311644_012024-N.jpg</t>
   </si>
   <si>
     <t>Tiras Trasera Luces Direccionales Secuencial Drl Auto</t>
@@ -5015,6 +5009,18 @@
   </si>
   <si>
     <t>Par de Faros led, Luces Decorativas Led Blancas Y Amarilla para Auto/Carro</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_647314-MLA112718039093_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_893993-MLA114600687014_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_679978-MLA113117754927_062026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_992169-MLA113116577615_062026-F.webp</t>
+  </si>
+  <si>
+    <t>http://panchochacharas.netlify.app/Imagenes/WhatsApp Image 2026-09-06 at 5.24.25 PM.jpeg</t>
+  </si>
+  <si>
+    <t>Soporte Celular Impermeable Fácil Uso Para Gorra, Bicicleta, Motocicleta</t>
+  </si>
+  <si>
+    <t>https://http2.mlstatic.com/D_NQ_NP_2X_740027-CBT97828404288_112025-F.webp</t>
   </si>
 </sst>
 </file>
@@ -5176,8 +5182,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:J377" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J377"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:J378" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J378">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="AUTOMOVIL"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState ref="A2:H342">
     <sortCondition ref="A1:A342"/>
   </sortState>
@@ -5482,7 +5494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J377"/>
+  <dimension ref="A1:J378"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="70" style="1" customWidth="1"/>
@@ -5528,7 +5540,7 @@
         <v>1259</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="11.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="11.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>1433</v>
       </c>
@@ -5557,7 +5569,7 @@
         <v>1437</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>982</v>
       </c>
@@ -5587,7 +5599,7 @@
       </c>
       <c r="J3" s="12"/>
     </row>
-    <row r="4" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>984</v>
       </c>
@@ -5616,7 +5628,7 @@
         <v>1367</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>533</v>
       </c>
@@ -5639,7 +5651,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>136</v>
       </c>
@@ -5668,7 +5680,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>357</v>
       </c>
@@ -5691,7 +5703,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>795</v>
       </c>
@@ -5717,7 +5729,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>90</v>
       </c>
@@ -5743,7 +5755,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" ht="72.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>637</v>
       </c>
@@ -5769,7 +5781,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>794</v>
       </c>
@@ -5795,7 +5807,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>208</v>
       </c>
@@ -5824,7 +5836,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" ht="72.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>687</v>
       </c>
@@ -5850,7 +5862,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>886</v>
       </c>
@@ -5873,7 +5885,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>576</v>
       </c>
@@ -5899,7 +5911,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>907</v>
       </c>
@@ -5922,7 +5934,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>95</v>
       </c>
@@ -5945,7 +5957,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>789</v>
       </c>
@@ -5968,7 +5980,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>700</v>
       </c>
@@ -5994,7 +6006,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>523</v>
       </c>
@@ -6017,7 +6029,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>726</v>
       </c>
@@ -6040,7 +6052,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>702</v>
       </c>
@@ -6066,7 +6078,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>478</v>
       </c>
@@ -6089,7 +6101,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>478</v>
       </c>
@@ -6112,7 +6124,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>478</v>
       </c>
@@ -6135,7 +6147,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>445</v>
       </c>
@@ -6164,7 +6176,7 @@
         <v>1579</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>97</v>
       </c>
@@ -6196,7 +6208,7 @@
         <v>1580</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>783</v>
       </c>
@@ -6222,7 +6234,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>772</v>
       </c>
@@ -6248,7 +6260,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>100</v>
       </c>
@@ -6271,7 +6283,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>773</v>
       </c>
@@ -6300,7 +6312,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>782</v>
       </c>
@@ -6326,7 +6338,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>774</v>
       </c>
@@ -6358,7 +6370,7 @@
         <v>1572</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>777</v>
       </c>
@@ -6384,7 +6396,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>775</v>
       </c>
@@ -6413,7 +6425,7 @@
         <v>1544</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>776</v>
       </c>
@@ -6436,7 +6448,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>971</v>
       </c>
@@ -6465,7 +6477,7 @@
         <v>1275</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>1187</v>
       </c>
@@ -6491,7 +6503,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>915</v>
       </c>
@@ -6514,7 +6526,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>543</v>
       </c>
@@ -6537,7 +6549,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>841</v>
       </c>
@@ -6566,7 +6578,7 @@
         <v>1521</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>68</v>
       </c>
@@ -6586,7 +6598,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>162</v>
       </c>
@@ -6609,7 +6621,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>140</v>
       </c>
@@ -6635,7 +6647,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>848</v>
       </c>
@@ -6658,7 +6670,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>853</v>
       </c>
@@ -6681,7 +6693,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>849</v>
       </c>
@@ -6704,7 +6716,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>849</v>
       </c>
@@ -6727,7 +6739,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>418</v>
       </c>
@@ -6759,7 +6771,7 @@
         <v>1573</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>173</v>
       </c>
@@ -6785,7 +6797,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>301</v>
       </c>
@@ -6811,7 +6823,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>164</v>
       </c>
@@ -6834,7 +6846,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>745</v>
       </c>
@@ -6866,7 +6878,7 @@
         <v>1368</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>744</v>
       </c>
@@ -6898,7 +6910,7 @@
         <v>1351</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>407</v>
       </c>
@@ -6930,7 +6942,7 @@
         <v>1318</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>191</v>
       </c>
@@ -6962,7 +6974,7 @@
         <v>1568</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>749</v>
       </c>
@@ -6994,7 +7006,7 @@
         <v>1295</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>893</v>
       </c>
@@ -7017,7 +7029,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>733</v>
       </c>
@@ -7040,7 +7052,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>973</v>
       </c>
@@ -7072,7 +7084,7 @@
         <v>1277</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>304</v>
       </c>
@@ -7098,7 +7110,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>889</v>
       </c>
@@ -7121,7 +7133,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>786</v>
       </c>
@@ -7147,7 +7159,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>861</v>
       </c>
@@ -7173,7 +7185,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>978</v>
       </c>
@@ -7205,7 +7217,7 @@
         <v>1266</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>105</v>
       </c>
@@ -7234,7 +7246,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>684</v>
       </c>
@@ -7257,7 +7269,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>620</v>
       </c>
@@ -7283,7 +7295,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>308</v>
       </c>
@@ -7312,7 +7324,7 @@
         <v>1313</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>361</v>
       </c>
@@ -7338,7 +7350,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>821</v>
       </c>
@@ -7370,7 +7382,7 @@
         <v>1586</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>337</v>
       </c>
@@ -7393,7 +7405,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>333</v>
       </c>
@@ -7422,7 +7434,7 @@
         <v>1314</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>364</v>
       </c>
@@ -7451,7 +7463,7 @@
         <v>1358</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>723</v>
       </c>
@@ -7477,7 +7489,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>711</v>
       </c>
@@ -7500,7 +7512,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>722</v>
       </c>
@@ -7523,7 +7535,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>947</v>
       </c>
@@ -7549,7 +7561,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="79" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>708</v>
       </c>
@@ -7575,7 +7587,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="80" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>520</v>
       </c>
@@ -7598,7 +7610,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>514</v>
       </c>
@@ -7621,7 +7633,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>953</v>
       </c>
@@ -7647,7 +7659,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="83" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>961</v>
       </c>
@@ -7673,7 +7685,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="84" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>282</v>
       </c>
@@ -7702,7 +7714,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="85" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>545</v>
       </c>
@@ -7731,7 +7743,7 @@
         <v>1582</v>
       </c>
     </row>
-    <row r="86" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>1177</v>
       </c>
@@ -7763,7 +7775,7 @@
         <v>1376</v>
       </c>
     </row>
-    <row r="87" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>825</v>
       </c>
@@ -7789,7 +7801,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" ht="58" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>595</v>
       </c>
@@ -7815,7 +7827,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="89" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>626</v>
       </c>
@@ -7841,7 +7853,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="90" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>669</v>
       </c>
@@ -7864,7 +7876,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="91" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>201</v>
       </c>
@@ -7890,7 +7902,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="92" spans="1:10" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:10" ht="72.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>555</v>
       </c>
@@ -7916,7 +7928,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>592</v>
       </c>
@@ -7945,7 +7957,7 @@
         <v>1551</v>
       </c>
     </row>
-    <row r="94" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>590</v>
       </c>
@@ -7977,7 +7989,7 @@
         <v>1557</v>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>590</v>
       </c>
@@ -8006,7 +8018,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>276</v>
       </c>
@@ -8032,7 +8044,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="97" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>178</v>
       </c>
@@ -8058,7 +8070,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="98" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>213</v>
       </c>
@@ -8087,7 +8099,7 @@
         <v>1546</v>
       </c>
     </row>
-    <row r="99" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>154</v>
       </c>
@@ -8113,7 +8125,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="100" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>414</v>
       </c>
@@ -8142,7 +8154,7 @@
         <v>1596</v>
       </c>
     </row>
-    <row r="101" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>837</v>
       </c>
@@ -8168,7 +8180,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="102" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>182</v>
       </c>
@@ -8194,7 +8206,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="103" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>918</v>
       </c>
@@ -8220,7 +8232,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="104" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>311</v>
       </c>
@@ -8249,7 +8261,7 @@
         <v>1325</v>
       </c>
     </row>
-    <row r="105" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>919</v>
       </c>
@@ -8283,10 +8295,10 @@
     </row>
     <row r="106" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
-        <v>1659</v>
+        <v>1657</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="C106" s="7">
         <v>199</v>
@@ -8295,7 +8307,7 @@
         <v>150</v>
       </c>
       <c r="E106" s="12" t="s">
-        <v>1654</v>
+        <v>1659</v>
       </c>
       <c r="G106" s="7" t="s">
         <v>863</v>
@@ -8304,10 +8316,10 @@
         <v>476</v>
       </c>
       <c r="I106" s="12" t="s">
-        <v>1658</v>
-      </c>
-    </row>
-    <row r="107" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1656</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>458</v>
       </c>
@@ -8336,7 +8348,7 @@
         <v>1541</v>
       </c>
     </row>
-    <row r="108" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>472</v>
       </c>
@@ -8365,7 +8377,7 @@
         <v>1550</v>
       </c>
     </row>
-    <row r="109" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>368</v>
       </c>
@@ -8397,7 +8409,7 @@
         <v>1390</v>
       </c>
     </row>
-    <row r="110" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>804</v>
       </c>
@@ -8426,7 +8438,7 @@
         <v>1543</v>
       </c>
     </row>
-    <row r="111" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>800</v>
       </c>
@@ -8452,7 +8464,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="112" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>372</v>
       </c>
@@ -8484,7 +8496,7 @@
         <v>1354</v>
       </c>
     </row>
-    <row r="113" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>1514</v>
       </c>
@@ -8516,7 +8528,7 @@
         <v>1518</v>
       </c>
     </row>
-    <row r="114" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>644</v>
       </c>
@@ -8542,7 +8554,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="115" spans="1:10" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:10" ht="58" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>672</v>
       </c>
@@ -8568,7 +8580,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="116" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>630</v>
       </c>
@@ -8594,7 +8606,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="117" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>652</v>
       </c>
@@ -8617,7 +8629,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="118" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>8</v>
       </c>
@@ -8646,7 +8658,7 @@
         <v>1399</v>
       </c>
     </row>
-    <row r="119" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>461</v>
       </c>
@@ -8669,7 +8681,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="120" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>639</v>
       </c>
@@ -8695,7 +8707,7 @@
         <v>1406</v>
       </c>
     </row>
-    <row r="121" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>510</v>
       </c>
@@ -8718,7 +8730,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="122" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>214</v>
       </c>
@@ -8741,7 +8753,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="123" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>217</v>
       </c>
@@ -8767,7 +8779,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="124" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>220</v>
       </c>
@@ -8793,7 +8805,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="125" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>339</v>
       </c>
@@ -8819,7 +8831,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="126" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>343</v>
       </c>
@@ -8845,7 +8857,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="127" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>70</v>
       </c>
@@ -8871,12 +8883,12 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="128" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>1631</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>1651</v>
+        <v>1650</v>
       </c>
       <c r="C128" s="7">
         <v>1356</v>
@@ -8900,7 +8912,7 @@
         <v>1299</v>
       </c>
     </row>
-    <row r="129" spans="1:10" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:10" ht="58" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>904</v>
       </c>
@@ -8923,7 +8935,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="130" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>396</v>
       </c>
@@ -8949,7 +8961,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="131" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>73</v>
       </c>
@@ -8975,7 +8987,7 @@
         <v>1363</v>
       </c>
     </row>
-    <row r="132" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>256</v>
       </c>
@@ -9004,7 +9016,7 @@
         <v>1529</v>
       </c>
     </row>
-    <row r="133" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>1178</v>
       </c>
@@ -9036,7 +9048,7 @@
         <v>1334</v>
       </c>
     </row>
-    <row r="134" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>76</v>
       </c>
@@ -9059,7 +9071,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="135" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>79</v>
       </c>
@@ -9088,7 +9100,7 @@
         <v>1569</v>
       </c>
     </row>
-    <row r="136" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>81</v>
       </c>
@@ -9111,7 +9123,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="137" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>422</v>
       </c>
@@ -9137,7 +9149,7 @@
         <v>1428</v>
       </c>
     </row>
-    <row r="138" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>436</v>
       </c>
@@ -9166,7 +9178,7 @@
         <v>1429</v>
       </c>
     </row>
-    <row r="139" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>432</v>
       </c>
@@ -9195,7 +9207,7 @@
         <v>1598</v>
       </c>
     </row>
-    <row r="140" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>223</v>
       </c>
@@ -9221,7 +9233,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="141" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>84</v>
       </c>
@@ -9337,7 +9349,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="145" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>145</v>
       </c>
@@ -9366,7 +9378,7 @@
         <v>1332</v>
       </c>
     </row>
-    <row r="146" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>148</v>
       </c>
@@ -9392,7 +9404,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="147" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>151</v>
       </c>
@@ -9421,7 +9433,7 @@
         <v>1408</v>
       </c>
     </row>
-    <row r="148" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>557</v>
       </c>
@@ -9447,7 +9459,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="149" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>1523</v>
       </c>
@@ -9473,7 +9485,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="150" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>586</v>
       </c>
@@ -9499,7 +9511,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="151" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>428</v>
       </c>
@@ -9551,7 +9563,7 @@
         <v>1380</v>
       </c>
     </row>
-    <row r="153" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>551</v>
       </c>
@@ -9597,7 +9609,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="155" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>658</v>
       </c>
@@ -9623,7 +9635,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="156" spans="1:10" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:10" ht="58" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>656</v>
       </c>
@@ -9646,7 +9658,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="157" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>648</v>
       </c>
@@ -9669,7 +9681,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="158" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>259</v>
       </c>
@@ -9701,7 +9713,7 @@
         <v>1427</v>
       </c>
     </row>
-    <row r="159" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>448</v>
       </c>
@@ -9730,7 +9742,7 @@
         <v>1410</v>
       </c>
     </row>
-    <row r="160" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:10" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>272</v>
       </c>
@@ -9756,7 +9768,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="161" spans="1:10" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:10" ht="15.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>109</v>
       </c>
@@ -9782,7 +9794,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="162" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>59</v>
       </c>
@@ -9840,12 +9852,12 @@
         <v>476</v>
       </c>
     </row>
-    <row r="164" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>1632</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>1651</v>
+        <v>1650</v>
       </c>
       <c r="C164" s="7">
         <v>1526</v>
@@ -9872,7 +9884,7 @@
         <v>1292</v>
       </c>
     </row>
-    <row r="165" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>697</v>
       </c>
@@ -9898,7 +9910,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="166" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>712</v>
       </c>
@@ -9924,7 +9936,7 @@
         <v>1526</v>
       </c>
     </row>
-    <row r="167" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>454</v>
       </c>
@@ -10002,7 +10014,7 @@
         <v>1340</v>
       </c>
     </row>
-    <row r="170" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>583</v>
       </c>
@@ -10033,7 +10045,7 @@
         <v>49</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>1652</v>
+        <v>1651</v>
       </c>
       <c r="C171" s="7">
         <v>250</v>
@@ -10054,7 +10066,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="172" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>502</v>
       </c>
@@ -10077,7 +10089,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="173" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>502</v>
       </c>
@@ -10100,7 +10112,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="174" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>910</v>
       </c>
@@ -10123,7 +10135,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="175" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>870</v>
       </c>
@@ -10146,7 +10158,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="176" spans="1:10" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:10" ht="58" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>680</v>
       </c>
@@ -10172,7 +10184,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="177" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>499</v>
       </c>
@@ -10195,7 +10207,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="178" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>376</v>
       </c>
@@ -10221,7 +10233,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="179" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>769</v>
       </c>
@@ -10250,7 +10262,7 @@
         <v>1326</v>
       </c>
     </row>
-    <row r="180" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>166</v>
       </c>
@@ -10276,7 +10288,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="181" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>318</v>
       </c>
@@ -10302,7 +10314,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="182" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>858</v>
       </c>
@@ -10328,7 +10340,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="183" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:10" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>197</v>
       </c>
@@ -10357,7 +10369,7 @@
         <v>1263</v>
       </c>
     </row>
-    <row r="184" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>522</v>
       </c>
@@ -10380,7 +10392,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="185" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>522</v>
       </c>
@@ -10403,7 +10415,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="186" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>874</v>
       </c>
@@ -10426,7 +10438,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="187" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>876</v>
       </c>
@@ -10449,7 +10461,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="188" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>539</v>
       </c>
@@ -10472,7 +10484,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="189" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>237</v>
       </c>
@@ -10501,7 +10513,7 @@
         <v>1345</v>
       </c>
     </row>
-    <row r="190" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>924</v>
       </c>
@@ -10533,7 +10545,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="191" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>169</v>
       </c>
@@ -10559,7 +10571,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="192" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>17</v>
       </c>
@@ -10585,7 +10597,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="193" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A193" s="1" t="s">
         <v>960</v>
       </c>
@@ -10611,7 +10623,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="194" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>561</v>
       </c>
@@ -10637,7 +10649,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="195" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>675</v>
       </c>
@@ -10663,7 +10675,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="196" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>565</v>
       </c>
@@ -10689,7 +10701,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="197" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>717</v>
       </c>
@@ -10712,7 +10724,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="198" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>21</v>
       </c>
@@ -10741,7 +10753,7 @@
         <v>1372</v>
       </c>
     </row>
-    <row r="199" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>321</v>
       </c>
@@ -10767,7 +10779,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="200" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>548</v>
       </c>
@@ -10790,7 +10802,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="201" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>263</v>
       </c>
@@ -10819,7 +10831,7 @@
         <v>1593</v>
       </c>
     </row>
-    <row r="202" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>379</v>
       </c>
@@ -10877,7 +10889,7 @@
         <v>1371</v>
       </c>
     </row>
-    <row r="204" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>465</v>
       </c>
@@ -10903,7 +10915,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="205" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>13</v>
       </c>
@@ -10932,7 +10944,7 @@
         <v>1342</v>
       </c>
     </row>
-    <row r="206" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>765</v>
       </c>
@@ -10955,7 +10967,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="207" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>469</v>
       </c>
@@ -10987,7 +10999,7 @@
         <v>1566</v>
       </c>
     </row>
-    <row r="208" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>604</v>
       </c>
@@ -11013,7 +11025,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="209" spans="1:9" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:9" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>604</v>
       </c>
@@ -11039,7 +11051,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="210" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:9" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>604</v>
       </c>
@@ -11065,7 +11077,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="211" spans="1:9" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:9" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
         <v>614</v>
       </c>
@@ -11091,7 +11103,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="212" spans="1:9" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:9" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A212" s="1" t="s">
         <v>941</v>
       </c>
@@ -11117,7 +11129,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="213" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:9" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>813</v>
       </c>
@@ -11143,7 +11155,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="214" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:9" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>796</v>
       </c>
@@ -11198,7 +11210,7 @@
         <v>1353</v>
       </c>
     </row>
-    <row r="216" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:9" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>348</v>
       </c>
@@ -11221,7 +11233,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="217" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:9" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>266</v>
       </c>
@@ -11247,7 +11259,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="218" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:9" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
         <v>279</v>
       </c>
@@ -11276,7 +11288,7 @@
         <v>1279</v>
       </c>
     </row>
-    <row r="219" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:9" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
         <v>65</v>
       </c>
@@ -11305,7 +11317,7 @@
         <v>1561</v>
       </c>
     </row>
-    <row r="220" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:9" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>615</v>
       </c>
@@ -11334,7 +11346,7 @@
         <v>1555</v>
       </c>
     </row>
-    <row r="221" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:9" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>730</v>
       </c>
@@ -11360,7 +11372,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="222" spans="1:9" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:9" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>1175</v>
       </c>
@@ -11386,7 +11398,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="223" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:9" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>942</v>
       </c>
@@ -11415,7 +11427,7 @@
         <v>1562</v>
       </c>
     </row>
-    <row r="224" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:9" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>945</v>
       </c>
@@ -11444,7 +11456,7 @@
         <v>1418</v>
       </c>
     </row>
-    <row r="225" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>616</v>
       </c>
@@ -11473,7 +11485,7 @@
         <v>1539</v>
       </c>
     </row>
-    <row r="226" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>289</v>
       </c>
@@ -11499,7 +11511,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="227" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>324</v>
       </c>
@@ -11525,7 +11537,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="228" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>205</v>
       </c>
@@ -11557,7 +11569,7 @@
         <v>1378</v>
       </c>
     </row>
-    <row r="229" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>240</v>
       </c>
@@ -11583,7 +11595,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="230" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>933</v>
       </c>
@@ -11609,7 +11621,7 @@
         <v>1311</v>
       </c>
     </row>
-    <row r="231" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>400</v>
       </c>
@@ -11632,7 +11644,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="232" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>487</v>
       </c>
@@ -11655,7 +11667,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="233" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>600</v>
       </c>
@@ -11681,7 +11693,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="234" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A234" s="1" t="s">
         <v>227</v>
       </c>
@@ -11707,7 +11719,7 @@
         <v>1387</v>
       </c>
     </row>
-    <row r="235" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A235" s="1" t="s">
         <v>116</v>
       </c>
@@ -11733,7 +11745,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="236" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A236" s="1" t="s">
         <v>119</v>
       </c>
@@ -11762,7 +11774,7 @@
         <v>1285</v>
       </c>
     </row>
-    <row r="237" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A237" s="1" t="s">
         <v>122</v>
       </c>
@@ -11794,7 +11806,7 @@
         <v>1337</v>
       </c>
     </row>
-    <row r="238" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A238" s="1" t="s">
         <v>664</v>
       </c>
@@ -11820,7 +11832,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="239" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A239" s="1" t="s">
         <v>352</v>
       </c>
@@ -11852,7 +11864,7 @@
         <v>1570</v>
       </c>
     </row>
-    <row r="240" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
         <v>832</v>
       </c>
@@ -11875,7 +11887,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="241" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
         <v>962</v>
       </c>
@@ -11907,7 +11919,7 @@
         <v>1576</v>
       </c>
     </row>
-    <row r="242" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>403</v>
       </c>
@@ -11939,7 +11951,7 @@
         <v>1274</v>
       </c>
     </row>
-    <row r="243" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>244</v>
       </c>
@@ -11965,7 +11977,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="244" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>689</v>
       </c>
@@ -11988,7 +12000,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="245" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
         <v>269</v>
       </c>
@@ -12011,7 +12023,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="246" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
         <v>572</v>
       </c>
@@ -12034,7 +12046,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="247" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>693</v>
       </c>
@@ -12060,7 +12072,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="248" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>382</v>
       </c>
@@ -12089,7 +12101,7 @@
         <v>1513</v>
       </c>
     </row>
-    <row r="249" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>934</v>
       </c>
@@ -12115,7 +12127,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="250" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
         <v>808</v>
       </c>
@@ -12141,7 +12153,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="251" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
         <v>247</v>
       </c>
@@ -12170,7 +12182,7 @@
         <v>1310</v>
       </c>
     </row>
-    <row r="252" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
         <v>230</v>
       </c>
@@ -12202,7 +12214,7 @@
         <v>1356</v>
       </c>
     </row>
-    <row r="253" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
         <v>327</v>
       </c>
@@ -12228,7 +12240,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="254" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
         <v>1149</v>
       </c>
@@ -12251,7 +12263,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="255" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
         <v>882</v>
       </c>
@@ -12274,7 +12286,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="256" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
         <v>234</v>
       </c>
@@ -12297,7 +12309,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="257" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A257" s="1" t="s">
         <v>929</v>
       </c>
@@ -12329,7 +12341,7 @@
         <v>1571</v>
       </c>
     </row>
-    <row r="258" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
         <v>385</v>
       </c>
@@ -12355,7 +12367,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="259" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
         <v>250</v>
       </c>
@@ -12384,7 +12396,7 @@
         <v>1316</v>
       </c>
     </row>
-    <row r="260" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
         <v>253</v>
       </c>
@@ -12416,7 +12428,7 @@
         <v>1322</v>
       </c>
     </row>
-    <row r="261" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
         <v>753</v>
       </c>
@@ -12445,7 +12457,7 @@
         <v>1404</v>
       </c>
     </row>
-    <row r="262" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
         <v>411</v>
       </c>
@@ -12471,7 +12483,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="263" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A263" s="1" t="s">
         <v>188</v>
       </c>
@@ -12503,7 +12515,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="264" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
         <v>194</v>
       </c>
@@ -12532,7 +12544,7 @@
         <v>1309</v>
       </c>
     </row>
-    <row r="265" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
         <v>389</v>
       </c>
@@ -12558,7 +12570,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="266" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
         <v>938</v>
       </c>
@@ -12584,7 +12596,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="267" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
         <v>937</v>
       </c>
@@ -12613,7 +12625,7 @@
         <v>1420</v>
       </c>
     </row>
-    <row r="268" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
         <v>936</v>
       </c>
@@ -12645,7 +12657,7 @@
         <v>1424</v>
       </c>
     </row>
-    <row r="269" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
         <v>766</v>
       </c>
@@ -12674,7 +12686,7 @@
         <v>1554</v>
       </c>
     </row>
-    <row r="270" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A270" s="2" t="s">
         <v>935</v>
       </c>
@@ -12697,7 +12709,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="271" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
         <v>767</v>
       </c>
@@ -12725,10 +12737,10 @@
     </row>
     <row r="272" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A272" s="1" t="s">
-        <v>1655</v>
+        <v>1653</v>
       </c>
       <c r="B272" s="1" t="s">
-        <v>1656</v>
+        <v>1654</v>
       </c>
       <c r="C272" s="7">
         <v>290</v>
@@ -12737,7 +12749,7 @@
         <v>150</v>
       </c>
       <c r="E272" s="13" t="s">
-        <v>1657</v>
+        <v>1655</v>
       </c>
       <c r="G272" s="7" t="s">
         <v>863</v>
@@ -12752,7 +12764,7 @@
         <v>1382</v>
       </c>
     </row>
-    <row r="273" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A273" s="1" t="s">
         <v>330</v>
       </c>
@@ -12776,7 +12788,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="274" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A274" s="1" t="s">
         <v>185</v>
       </c>
@@ -12805,7 +12817,7 @@
         <v>1366</v>
       </c>
     </row>
-    <row r="275" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A275" s="1" t="s">
         <v>293</v>
       </c>
@@ -12834,7 +12846,7 @@
         <v>1294</v>
       </c>
     </row>
-    <row r="276" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A276" s="1" t="s">
         <v>159</v>
       </c>
@@ -12860,7 +12872,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="277" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A277" s="1" t="s">
         <v>393</v>
       </c>
@@ -12889,7 +12901,7 @@
         <v>1327</v>
       </c>
     </row>
-    <row r="278" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A278" s="1" t="s">
         <v>566</v>
       </c>
@@ -12915,7 +12927,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="279" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A279" s="1" t="s">
         <v>899</v>
       </c>
@@ -12938,7 +12950,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="280" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A280" s="1" t="s">
         <v>507</v>
       </c>
@@ -12961,7 +12973,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="281" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A281" s="1" t="s">
         <v>530</v>
       </c>
@@ -12984,7 +12996,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="282" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A282" s="1" t="s">
         <v>737</v>
       </c>
@@ -13016,7 +13028,7 @@
         <v>1401</v>
       </c>
     </row>
-    <row r="283" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>1150</v>
       </c>
@@ -13042,7 +13054,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="284" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A284" s="1" t="s">
         <v>985</v>
       </c>
@@ -13068,7 +13080,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="285" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A285" s="1" t="s">
         <v>989</v>
       </c>
@@ -13100,7 +13112,7 @@
         <v>1432</v>
       </c>
     </row>
-    <row r="286" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>993</v>
       </c>
@@ -13132,7 +13144,7 @@
         <v>1394</v>
       </c>
     </row>
-    <row r="287" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A287" s="1" t="s">
         <v>1070</v>
       </c>
@@ -13164,7 +13176,7 @@
         <v>1343</v>
       </c>
     </row>
-    <row r="288" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
         <v>998</v>
       </c>
@@ -13196,7 +13208,7 @@
         <v>1262</v>
       </c>
     </row>
-    <row r="289" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A289" s="1" t="s">
         <v>1002</v>
       </c>
@@ -13228,7 +13240,7 @@
         <v>1585</v>
       </c>
     </row>
-    <row r="290" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A290" s="1" t="s">
         <v>1006</v>
       </c>
@@ -13257,7 +13269,7 @@
         <v>1360</v>
       </c>
     </row>
-    <row r="291" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A291" s="1" t="s">
         <v>1008</v>
       </c>
@@ -13283,7 +13295,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="292" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A292" s="1" t="s">
         <v>1014</v>
       </c>
@@ -13315,7 +13327,7 @@
         <v>1361</v>
       </c>
     </row>
-    <row r="293" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A293" s="1" t="s">
         <v>1018</v>
       </c>
@@ -13341,7 +13353,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="294" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
         <v>1026</v>
       </c>
@@ -13361,7 +13373,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="295" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
         <v>1028</v>
       </c>
@@ -13381,7 +13393,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="296" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
         <v>1032</v>
       </c>
@@ -13404,7 +13416,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="297" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
         <v>1036</v>
       </c>
@@ -13424,7 +13436,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="298" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
         <v>1040</v>
       </c>
@@ -13444,7 +13456,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="299" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>1147</v>
       </c>
@@ -13470,7 +13482,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="300" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
         <v>1047</v>
       </c>
@@ -13496,7 +13508,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="301" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
         <v>1051</v>
       </c>
@@ -13516,7 +13528,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="302" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>1055</v>
       </c>
@@ -13542,7 +13554,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="303" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>1059</v>
       </c>
@@ -13565,7 +13577,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="304" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
         <v>1063</v>
       </c>
@@ -13585,7 +13597,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="305" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
         <v>1176</v>
       </c>
@@ -13608,7 +13620,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="306" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>1143</v>
       </c>
@@ -13637,7 +13649,7 @@
         <v>1398</v>
       </c>
     </row>
-    <row r="307" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>1074</v>
       </c>
@@ -13669,7 +13681,7 @@
         <v>1597</v>
       </c>
     </row>
-    <row r="308" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>1077</v>
       </c>
@@ -13701,7 +13713,7 @@
         <v>1584</v>
       </c>
     </row>
-    <row r="309" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>1080</v>
       </c>
@@ -13730,7 +13742,7 @@
         <v>1563</v>
       </c>
     </row>
-    <row r="310" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
         <v>1083</v>
       </c>
@@ -13762,7 +13774,7 @@
         <v>1396</v>
       </c>
     </row>
-    <row r="311" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
         <v>1088</v>
       </c>
@@ -13791,7 +13803,7 @@
         <v>1578</v>
       </c>
     </row>
-    <row r="312" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A312" s="1" t="s">
         <v>1090</v>
       </c>
@@ -13820,7 +13832,7 @@
         <v>1587</v>
       </c>
     </row>
-    <row r="313" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A313" s="1" t="s">
         <v>1091</v>
       </c>
@@ -13843,7 +13855,7 @@
         <v>1331</v>
       </c>
     </row>
-    <row r="314" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
         <v>1630</v>
       </c>
@@ -13872,7 +13884,7 @@
         <v>1272</v>
       </c>
     </row>
-    <row r="315" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
         <v>1099</v>
       </c>
@@ -13904,7 +13916,7 @@
         <v>1540</v>
       </c>
     </row>
-    <row r="316" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A316" s="1" t="s">
         <v>1104</v>
       </c>
@@ -13936,7 +13948,7 @@
         <v>1373</v>
       </c>
     </row>
-    <row r="317" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A317" s="1" t="s">
         <v>1107</v>
       </c>
@@ -13965,7 +13977,7 @@
         <v>1423</v>
       </c>
     </row>
-    <row r="318" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
         <v>1110</v>
       </c>
@@ -13988,7 +14000,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="319" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
         <v>1600</v>
       </c>
@@ -14017,7 +14029,7 @@
         <v>1581</v>
       </c>
     </row>
-    <row r="320" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
         <v>1117</v>
       </c>
@@ -14043,7 +14055,7 @@
         <v>1321</v>
       </c>
     </row>
-    <row r="321" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
         <v>1123</v>
       </c>
@@ -14072,7 +14084,7 @@
         <v>1588</v>
       </c>
     </row>
-    <row r="322" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
         <v>1125</v>
       </c>
@@ -14101,7 +14113,7 @@
         <v>1534</v>
       </c>
     </row>
-    <row r="323" spans="1:10" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:10" ht="72.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>1129</v>
       </c>
@@ -14130,7 +14142,7 @@
         <v>1283</v>
       </c>
     </row>
-    <row r="324" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>1135</v>
       </c>
@@ -14159,7 +14171,7 @@
         <v>1328</v>
       </c>
     </row>
-    <row r="325" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
         <v>1185</v>
       </c>
@@ -14185,7 +14197,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="326" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>1186</v>
       </c>
@@ -14211,7 +14223,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="327" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>1151</v>
       </c>
@@ -14240,7 +14252,7 @@
         <v>1574</v>
       </c>
     </row>
-    <row r="328" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A328" s="1" t="s">
         <v>1154</v>
       </c>
@@ -14266,7 +14278,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="329" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A329" s="1" t="s">
         <v>1159</v>
       </c>
@@ -14292,7 +14304,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="330" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A330" s="1" t="s">
         <v>1162</v>
       </c>
@@ -14318,7 +14330,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="331" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A331" s="1" t="s">
         <v>1167</v>
       </c>
@@ -14344,7 +14356,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="332" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A332" s="1" t="s">
         <v>1172</v>
       </c>
@@ -14364,7 +14376,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="333" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A333" s="1" t="s">
         <v>1180</v>
       </c>
@@ -14421,7 +14433,7 @@
     </row>
     <row r="335" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
-        <v>1649</v>
+        <v>1648</v>
       </c>
       <c r="B335" s="1" t="s">
         <v>1199</v>
@@ -14445,13 +14457,13 @@
         <v>476</v>
       </c>
       <c r="I335" s="12" t="s">
-        <v>1650</v>
+        <v>1649</v>
       </c>
       <c r="J335" s="12" t="s">
         <v>1300</v>
       </c>
     </row>
-    <row r="336" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A336" s="1" t="s">
         <v>1202</v>
       </c>
@@ -14483,7 +14495,7 @@
         <v>1525</v>
       </c>
     </row>
-    <row r="337" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A337" s="1" t="s">
         <v>1208</v>
       </c>
@@ -14515,7 +14527,7 @@
         <v>1537</v>
       </c>
     </row>
-    <row r="338" spans="1:10" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:10" ht="58" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A338" s="1" t="s">
         <v>1629</v>
       </c>
@@ -14547,7 +14559,7 @@
         <v>1289</v>
       </c>
     </row>
-    <row r="339" spans="1:10" ht="87" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:10" ht="87" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A339" s="1" t="s">
         <v>1628</v>
       </c>
@@ -14579,7 +14591,7 @@
         <v>1291</v>
       </c>
     </row>
-    <row r="340" spans="1:10" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:10" ht="72.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A340" s="1" t="s">
         <v>1221</v>
       </c>
@@ -14611,7 +14623,7 @@
         <v>1567</v>
       </c>
     </row>
-    <row r="341" spans="1:10" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:10" ht="72.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A341" s="1" t="s">
         <v>1627</v>
       </c>
@@ -14643,7 +14655,7 @@
         <v>1286</v>
       </c>
     </row>
-    <row r="342" spans="1:10" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:10" ht="58" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A342" s="1" t="s">
         <v>1223</v>
       </c>
@@ -14672,7 +14684,7 @@
         <v>1536</v>
       </c>
     </row>
-    <row r="343" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A343" s="1" t="s">
         <v>1227</v>
       </c>
@@ -14736,7 +14748,7 @@
         <v>1575</v>
       </c>
     </row>
-    <row r="345" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A345" s="1" t="s">
         <v>1235</v>
       </c>
@@ -14768,7 +14780,7 @@
         <v>1307</v>
       </c>
     </row>
-    <row r="346" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A346" s="1" t="s">
         <v>1239</v>
       </c>
@@ -14800,7 +14812,7 @@
         <v>1388</v>
       </c>
     </row>
-    <row r="347" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A347" s="1" t="s">
         <v>1244</v>
       </c>
@@ -14832,7 +14844,7 @@
         <v>1565</v>
       </c>
     </row>
-    <row r="348" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A348" s="1" t="s">
         <v>1248</v>
       </c>
@@ -14861,7 +14873,7 @@
         <v>1281</v>
       </c>
     </row>
-    <row r="349" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A349" s="1" t="s">
         <v>1253</v>
       </c>
@@ -14893,7 +14905,7 @@
         <v>1270</v>
       </c>
     </row>
-    <row r="350" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A350" s="1" t="s">
         <v>1254</v>
       </c>
@@ -14925,7 +14937,7 @@
         <v>1349</v>
       </c>
     </row>
-    <row r="351" spans="1:10" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:10" ht="58" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A351" s="1" t="s">
         <v>1438</v>
       </c>
@@ -14957,7 +14969,7 @@
         <v>1592</v>
       </c>
     </row>
-    <row r="352" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A352" s="1" t="s">
         <v>1443</v>
       </c>
@@ -14989,7 +15001,7 @@
         <v>1530</v>
       </c>
     </row>
-    <row r="353" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A353" s="1" t="s">
         <v>1447</v>
       </c>
@@ -15018,7 +15030,7 @@
         <v>1451</v>
       </c>
     </row>
-    <row r="354" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A354" s="1" t="s">
         <v>1452</v>
       </c>
@@ -15047,7 +15059,7 @@
         <v>1455</v>
       </c>
     </row>
-    <row r="355" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A355" s="1" t="s">
         <v>1458</v>
       </c>
@@ -15073,7 +15085,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="356" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:10" ht="29" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A356" s="1" t="s">
         <v>1462</v>
       </c>
@@ -15105,7 +15117,7 @@
         <v>1466</v>
       </c>
     </row>
-    <row r="357" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:10" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A357" s="1" t="s">
         <v>1468</v>
       </c>
@@ -15134,7 +15146,7 @@
         <v>1471</v>
       </c>
     </row>
-    <row r="358" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A358" s="1" t="s">
         <v>1472</v>
       </c>
@@ -15166,7 +15178,7 @@
         <v>1564</v>
       </c>
     </row>
-    <row r="359" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A359" s="1" t="s">
         <v>1477</v>
       </c>
@@ -15198,7 +15210,7 @@
         <v>1589</v>
       </c>
     </row>
-    <row r="360" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A360" s="1" t="s">
         <v>1482</v>
       </c>
@@ -15224,7 +15236,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="361" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A361" s="1" t="s">
         <v>1486</v>
       </c>
@@ -15250,7 +15262,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="362" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A362" s="1" t="s">
         <v>1492</v>
       </c>
@@ -15276,7 +15288,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="363" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A363" s="1" t="s">
         <v>1493</v>
       </c>
@@ -15302,7 +15314,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="364" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:10" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
         <v>1498</v>
       </c>
@@ -15331,7 +15343,7 @@
         <v>1502</v>
       </c>
     </row>
-    <row r="365" spans="1:10" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:10" ht="23.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
         <v>1503</v>
       </c>
@@ -15363,7 +15375,7 @@
         <v>1548</v>
       </c>
     </row>
-    <row r="366" spans="1:10" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:10" ht="15.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A366" s="1" t="s">
         <v>1508</v>
       </c>
@@ -15389,7 +15401,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="367" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A367" s="1" t="s">
         <v>1590</v>
       </c>
@@ -15413,7 +15425,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="368" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A368" s="1" t="s">
         <v>1601</v>
       </c>
@@ -15437,7 +15449,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="369" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A369" s="1" t="s">
         <v>1601</v>
       </c>
@@ -15463,7 +15475,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="370" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A370" s="1" t="s">
         <v>1605</v>
       </c>
@@ -15489,7 +15501,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="371" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A371" s="1" t="s">
         <v>1616</v>
       </c>
@@ -15515,7 +15527,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="372" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A372" s="1" t="s">
         <v>1610</v>
       </c>
@@ -15541,7 +15553,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="373" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A373" s="1" t="s">
         <v>1617</v>
       </c>
@@ -15567,7 +15579,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="374" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A374" s="1" t="s">
         <v>1622</v>
       </c>
@@ -15596,7 +15608,7 @@
         <v>1625</v>
       </c>
     </row>
-    <row r="375" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A375" s="1" t="s">
         <v>1633</v>
       </c>
@@ -15628,7 +15640,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="376" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A376" s="1" t="s">
         <v>1639</v>
       </c>
@@ -15660,7 +15672,7 @@
         <v>1644</v>
       </c>
     </row>
-    <row r="377" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A377" s="1" t="s">
         <v>1645</v>
       </c>
@@ -15686,10 +15698,25 @@
         <v>476</v>
       </c>
       <c r="I377" s="12" t="s">
-        <v>1648</v>
+        <v>1658</v>
       </c>
       <c r="J377" s="12" t="s">
         <v>1644</v>
+      </c>
+    </row>
+    <row r="378" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A378" s="1" t="s">
+        <v>1660</v>
+      </c>
+      <c r="B378" s="1"/>
+      <c r="C378" s="7">
+        <v>190</v>
+      </c>
+      <c r="D378" s="7">
+        <v>150</v>
+      </c>
+      <c r="E378" s="12" t="s">
+        <v>1661</v>
       </c>
     </row>
   </sheetData>
@@ -16051,16 +16078,17 @@
     <hyperlink ref="J376" r:id="rId278"/>
     <hyperlink ref="E377" r:id="rId279"/>
     <hyperlink ref="F377" r:id="rId280"/>
-    <hyperlink ref="I377" display="https://http2.mlstatic.com/D_NQ_NP_2X_647314-MLA112718039093_062026-F.webp;;https://http2.mlstatic.com/D_NQ_NP_2X_893993-MLA114600687014_082026-F.webp;https://http2.mlstatic.com/D_NQ_NP_2X_679978-MLA113117754927_062026-F.webp;https://http2.mlstatic.com/D_"/>
+    <hyperlink ref="I377"/>
     <hyperlink ref="J377" r:id="rId281"/>
     <hyperlink ref="E106" r:id="rId282"/>
     <hyperlink ref="E272" r:id="rId283"/>
     <hyperlink ref="I106" r:id="rId284"/>
+    <hyperlink ref="E378" r:id="rId285"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId285"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId286"/>
   <tableParts count="1">
-    <tablePart r:id="rId286"/>
+    <tablePart r:id="rId287"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>